<commit_message>
WeatherHistory update – 2026-09-07 11:00 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5655,21 +5655,21 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>28.8</v>
+        <v>28.5</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G178" s="7" t="n">
         <v>12</v>
@@ -5690,11 +5690,11 @@
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
@@ -5713,13 +5713,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>26.9</v>
+        <v>26.7</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -5727,10 +5727,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>1.8</v>
+        <v>3.7</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -5742,13 +5742,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>26.8</v>
+        <v>27</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -5756,10 +5756,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>4.7</v>
+        <v>0.4</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -5771,24 +5771,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>26.8</v>
+        <v>28.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -5800,27 +5800,56 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>27.5</v>
+        <v>28.8</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -5841,7 +5870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10983,24 +11012,24 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>28</v>
+        <v>29.4</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>5.6</v>
+        <v>1.3</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>11.3</v>
+        <v>11.8</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -11012,13 +11041,13 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
@@ -11026,10 +11055,10 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>26.2</v>
+        <v>29.7</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8.9</v>
+        <v>8.4</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -11041,13 +11070,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>19.8</v>
+        <v>19.2</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>0.1</v>
+        <v>33.1</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -11055,10 +11084,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>26.9</v>
+        <v>58.5</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>5</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -11070,24 +11099,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>18.1</v>
+        <v>17.1</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>48.8</v>
+        <v>3.3</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>6.1</v>
+        <v>11.6</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -11099,24 +11128,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -11128,27 +11157,56 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18.8</v>
+        <v>19.5</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E183" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F183" s="4" t="n">
         <v>1.8</v>
       </c>
-      <c r="E183" s="4" t="inlineStr">
-        <is>
-          <t>JV</t>
-        </is>
-      </c>
-      <c r="F183" s="4" t="n">
-        <v>0.4</v>
-      </c>
       <c r="G183" s="4" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -11169,7 +11227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16311,17 +16369,17 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>26.3</v>
+        <v>26.2</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
@@ -16346,7 +16404,7 @@
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
@@ -16369,13 +16427,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>23.3</v>
+        <v>23.1</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -16383,10 +16441,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -16398,13 +16456,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>4.9</v>
+        <v>5.6</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -16427,13 +16485,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>23.9</v>
+        <v>24.8</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -16456,17 +16514,17 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>24.2</v>
+        <v>23.5</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.3</v>
+        <v>5.6</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
@@ -16477,6 +16535,35 @@
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -16497,7 +16584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21639,24 +21726,24 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>27.7</v>
+        <v>28.2</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>10.6</v>
+        <v>21.2</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>10.7</v>
+        <v>9.5</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -21668,10 +21755,10 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="D179" s="4" t="n">
         <v>2.7</v>
@@ -21682,10 +21769,10 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>27.5</v>
+        <v>33</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>8</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -21697,24 +21784,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>24.2</v>
+        <v>23.9</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>2.8</v>
+        <v>22.8</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>2.7</v>
+        <v>4.2</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>76</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -21726,13 +21813,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>22.6</v>
+        <v>21.7</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -21740,10 +21827,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>43.8</v>
+        <v>77.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>6.7</v>
+        <v>2.7</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -21755,13 +21842,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>21.4</v>
+        <v>22.3</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.1</v>
+        <v>3.2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -21769,10 +21856,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>39.6</v>
+        <v>24.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -21784,27 +21871,56 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>22.1</v>
+        <v>20.2</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>1.3</v>
+        <v>60.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.8</v>
+        <v>4.8</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -21825,7 +21941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26967,13 +27083,13 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>17.6</v>
+        <v>19.5</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
@@ -26981,10 +27097,10 @@
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>15.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>10.2</v>
+        <v>10.9</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -26996,24 +27112,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="D179" s="4" t="n">
         <v>1.9</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>12.1</v>
+        <v>16.3</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -27025,13 +27141,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>1.8</v>
+        <v>10.6</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1.9</v>
+        <v>3.2</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -27039,10 +27155,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>88.2</v>
+        <v>90.3</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -27054,24 +27170,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>8.4</v>
+        <v>10</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>50.2</v>
+        <v>36.9</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>6</v>
+        <v>7.6</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -27083,24 +27199,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>7.4</v>
+        <v>10.6</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>48.6</v>
+        <v>7.2</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>6.2</v>
+        <v>11.1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -27112,27 +27228,56 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>8.4</v>
+        <v>10</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>15.6</v>
+        <v>2</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>10.1</v>
+        <v>11.8</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -27153,7 +27298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28786,24 +28931,24 @@
         <v>46272</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>14.4</v>
+        <v>17</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="D57" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>52.7</v>
+        <v>49.6</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>5.7</v>
+        <v>6</v>
       </c>
       <c r="H57" s="10">
         <f>SUM(C51:C57)</f>
@@ -28815,13 +28960,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>18.1</v>
+        <v>17.7</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -28829,10 +28974,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>13.3</v>
+        <v>0.3</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -28844,13 +28989,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>19.2</v>
+        <v>19.5</v>
       </c>
       <c r="C59" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -28858,10 +29003,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -28873,24 +29018,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>17.2</v>
+        <v>16.6</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>1.7</v>
+        <v>2.7</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>59.6</v>
+        <v>57.8</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>4.8</v>
+        <v>5.1</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -28902,24 +29047,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.2</v>
+        <v>14.1</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>28.6</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
         <v>1.7</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>97.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.3</v>
+        <v>3.2</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -28931,27 +29076,56 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>100</v>
+        <v>54.9</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H63" s="10">
+        <f>SUM(C57:C63)</f>
         <v/>
       </c>
     </row>
@@ -28972,7 +29146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30605,24 +30779,24 @@
         <v>46272</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>14.2</v>
+        <v>16.6</v>
       </c>
       <c r="C57" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>57.6</v>
+        <v>48.6</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>5.1</v>
+        <v>6.2</v>
       </c>
       <c r="H57" s="10">
         <f>SUM(C51:C57)</f>
@@ -30634,13 +30808,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>18</v>
+        <v>18.1</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -30648,10 +30822,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>21.9</v>
+        <v>0.6</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>9.4</v>
+        <v>11.9</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -30663,13 +30837,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>19.1</v>
+        <v>20.2</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>5.2</v>
+        <v>6.3</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -30677,10 +30851,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>18</v>
+        <v>8.5</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>11</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -30692,13 +30866,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>14.4</v>
+        <v>15.1</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>4.1</v>
+        <v>2.7</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -30706,10 +30880,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>98</v>
+        <v>93.2</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -30721,24 +30895,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>11.5</v>
+        <v>14.6</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>25.6</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>100</v>
+        <v>44.9</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>6.6</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -30750,27 +30924,56 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.3</v>
+        <v>13.6</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>87.3</v>
+        <v>31.6</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>1.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H63" s="10">
+        <f>SUM(C57:C63)</f>
         <v/>
       </c>
     </row>
@@ -30791,7 +30994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32424,24 +32627,24 @@
         <v>46272</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>15.7</v>
+        <v>17.7</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>44.1</v>
+        <v>52.6</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>6.7</v>
+        <v>5.7</v>
       </c>
       <c r="H57" s="10">
         <f>SUM(C51:C57)</f>
@@ -32453,13 +32656,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>19.3</v>
+        <v>19.4</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -32467,10 +32670,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>22.3</v>
+        <v>1</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>11.9</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -32482,13 +32685,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>20.5</v>
+        <v>21</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>3.6</v>
+        <v>0.6</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -32496,10 +32699,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>25.8</v>
+        <v>7.6</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>8.9</v>
+        <v>11.1</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -32511,24 +32714,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>14.8</v>
+        <v>15.3</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>97.8</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -32540,13 +32743,13 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.4</v>
+        <v>15.6</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>20.3</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -32554,10 +32757,10 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>98.2</v>
+        <v>54.7</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.2</v>
+        <v>5.4</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -32569,27 +32772,56 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.4</v>
+        <v>15.5</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>3.8</v>
+        <v>2.3</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>94.5</v>
+        <v>47.8</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0.7</v>
+        <v>6.3</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H63" s="10">
+        <f>SUM(C57:C63)</f>
         <v/>
       </c>
     </row>
@@ -32610,7 +32842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34243,13 +34475,13 @@
         <v>46272</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>14.4</v>
+        <v>16.1</v>
       </c>
       <c r="C57" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
@@ -34257,10 +34489,10 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>50.1</v>
+        <v>61.4</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>6</v>
+        <v>4.6</v>
       </c>
       <c r="H57" s="10">
         <f>SUM(C51:C57)</f>
@@ -34272,7 +34504,7 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>17.4</v>
+        <v>17.3</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
@@ -34286,10 +34518,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>10.4</v>
+        <v>0.3</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -34301,13 +34533,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>18.9</v>
+        <v>19.4</v>
       </c>
       <c r="C59" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -34315,10 +34547,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>2.1</v>
+        <v>0.1</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -34330,13 +34562,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.7</v>
+        <v>15.9</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>3.8</v>
+        <v>9.9</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -34344,7 +34576,7 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>65</v>
+        <v>64.7</v>
       </c>
       <c r="G60" s="7" t="n">
         <v>4.2</v>
@@ -34359,13 +34591,13 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>12.2</v>
+        <v>13.8</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>18.8</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -34373,10 +34605,10 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.8</v>
+        <v>73.8</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -34388,27 +34620,56 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.2</v>
+        <v>13.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>100</v>
+        <v>54.9</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H63" s="10">
+        <f>SUM(C57:C63)</f>
         <v/>
       </c>
     </row>
@@ -34429,7 +34690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36062,13 +36323,13 @@
         <v>46272</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>15.7</v>
+        <v>18.1</v>
       </c>
       <c r="C57" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
@@ -36076,10 +36337,10 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>44.9</v>
+        <v>52.6</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>6.6</v>
+        <v>5.7</v>
       </c>
       <c r="H57" s="10">
         <f>SUM(C51:C57)</f>
@@ -36091,24 +36352,24 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>18.9</v>
+        <v>0.3</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>12</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -36120,13 +36381,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>21</v>
+        <v>21.3</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -36134,10 +36395,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>9</v>
+        <v>3.7</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -36149,24 +36410,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.6</v>
+        <v>16.8</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>4.2</v>
+        <v>0</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>1.4</v>
+        <v>2.5</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>93.2</v>
+        <v>75.2</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.8</v>
+        <v>3</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -36178,24 +36439,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.7</v>
+        <v>15.3</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>16.6</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.8</v>
+        <v>72.3</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -36207,27 +36468,56 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.4</v>
+        <v>15.8</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>13.8</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>99</v>
+        <v>56.6</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0.1</v>
+        <v>5.2</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H63" s="10">
+        <f>SUM(C57:C63)</f>
         <v/>
       </c>
     </row>
@@ -36248,7 +36538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37881,13 +38171,13 @@
         <v>46272</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>11.9</v>
+        <v>14.1</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
@@ -37895,10 +38185,10 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>48.2</v>
+        <v>53.5</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>6.2</v>
+        <v>5.6</v>
       </c>
       <c r="H57" s="10">
         <f>SUM(C51:C57)</f>
@@ -37910,13 +38200,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>15.1</v>
+        <v>15</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -37924,10 +38214,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>14.4</v>
+        <v>1.3</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>10.3</v>
+        <v>11.8</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -37939,13 +38229,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>16</v>
+        <v>16.9</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -37953,10 +38243,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>7.4</v>
+        <v>2.5</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11.1</v>
+        <v>11.7</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -37968,13 +38258,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>10.7</v>
+        <v>11.5</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>6.1</v>
+        <v>2</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -37982,10 +38272,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>88.09999999999999</v>
+        <v>89</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -37997,24 +38287,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>11.8</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>15.5</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>98.59999999999999</v>
+        <v>80.5</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.2</v>
+        <v>2.3</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -38026,27 +38316,56 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>7.7</v>
+        <v>10.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>7.6</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>94.90000000000001</v>
+        <v>60.9</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0.6</v>
+        <v>4.7</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H63" s="10">
+        <f>SUM(C57:C63)</f>
         <v/>
       </c>
     </row>
@@ -38067,7 +38386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43209,24 +43528,24 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>25.9</v>
+        <v>28.1</v>
       </c>
       <c r="C178" s="7" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>37</v>
+        <v>45.2</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>7.6</v>
+        <v>6.6</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -43238,24 +43557,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>25.9</v>
+        <v>25.3</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>3.7</v>
+        <v>11.2</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>16.1</v>
+        <v>18.6</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -43267,24 +43586,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>21.6</v>
+        <v>21.5</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>25.3</v>
+        <v>62.5</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>87.90000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -43296,24 +43615,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>20.9</v>
+        <v>21.2</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>74.8</v>
+        <v>99.2</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>3</v>
+        <v>0.1</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -43325,24 +43644,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>18.9</v>
+        <v>20.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>55.9</v>
+        <v>19.9</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>5.3</v>
+        <v>9.6</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -43354,27 +43673,56 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18.5</v>
+        <v>20.1</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>1.8</v>
+        <v>4.4</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>42.4</v>
+        <v>66</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>6.9</v>
+        <v>4.1</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -43395,7 +43743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45028,13 +45376,13 @@
         <v>46272</v>
       </c>
       <c r="B57" s="4" t="n">
-        <v>13.3</v>
+        <v>15.2</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
@@ -45042,10 +45390,10 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>69.2</v>
+        <v>50.8</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>3.7</v>
+        <v>5.9</v>
       </c>
       <c r="H57" s="10">
         <f>SUM(C51:C57)</f>
@@ -45057,24 +45405,24 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>17.4</v>
+        <v>17.9</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>39.6</v>
+        <v>8.4</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>7.2</v>
+        <v>11</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -45086,24 +45434,24 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>15.7</v>
+        <v>17.3</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>9.4</v>
+        <v>26.4</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>1.3</v>
+        <v>3.8</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>83.2</v>
+        <v>70.5</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -45115,24 +45463,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>12.5</v>
+        <v>12.3</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>1.9</v>
+        <v>3.5</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>77</v>
+        <v>70.7</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>2.8</v>
+        <v>3.5</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -45144,13 +45492,13 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="C61" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -45158,10 +45506,10 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>97.8</v>
+        <v>49.2</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.3</v>
+        <v>6.1</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -45173,13 +45521,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.3</v>
+        <v>13.1</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>0.9</v>
+        <v>2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -45187,13 +45535,42 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>76.8</v>
+        <v>58.6</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2.8</v>
+        <v>5</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H63" s="10">
+        <f>SUM(C57:C63)</f>
         <v/>
       </c>
     </row>
@@ -45214,7 +45591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -50356,24 +50733,24 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>27.3</v>
+        <v>27.7</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -50391,18 +50768,18 @@
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>1.2</v>
+        <v>5.9</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>11.9</v>
+        <v>11.3</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -50414,13 +50791,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>26.7</v>
+        <v>26.9</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -50428,10 +50805,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>0.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -50443,24 +50820,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>26.1</v>
+        <v>28.2</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>5.7</v>
+        <v>2.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>50.4</v>
+        <v>10.2</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>6</v>
+        <v>10.8</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -50472,24 +50849,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>0</v>
+        <v>11.8</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.3</v>
+        <v>4.2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>48</v>
+        <v>46.7</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -50501,13 +50878,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>25.1</v>
+        <v>26.9</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -50515,13 +50892,42 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>34.8</v>
+        <v>13.5</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>7.8</v>
+        <v>10.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -50542,7 +50948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -55684,13 +56090,13 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>24.9</v>
+        <v>25.8</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
@@ -55698,10 +56104,10 @@
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>8</v>
+        <v>7.2</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -55716,21 +56122,21 @@
         <v>23.5</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>0</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>11.9</v>
+        <v>26.2</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>10.6</v>
+        <v>8.9</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -55742,13 +56148,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>18.8</v>
+        <v>17.8</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>5.3</v>
+        <v>4.7</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -55756,10 +56162,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>29.9</v>
+        <v>61.7</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>8.4</v>
+        <v>4.6</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -55771,13 +56177,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>14.8</v>
+        <v>14.6</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -55785,10 +56191,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>27</v>
+        <v>2.1</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>11.7</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -55800,24 +56206,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.9</v>
+        <v>16.4</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -55829,27 +56235,56 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.9</v>
+        <v>15.8</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -55870,7 +56305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61012,13 +61447,13 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>15.1</v>
+        <v>13.2</v>
       </c>
       <c r="C178" s="7" t="n">
-        <v>30.6</v>
+        <v>16.7</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
@@ -61026,10 +61461,10 @@
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>97.40000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -61041,24 +61476,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>13.7</v>
+        <v>12</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>11.9</v>
+        <v>26</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>93.2</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -61070,13 +61505,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>12.3</v>
+        <v>12.6</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -61084,10 +61519,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>65.5</v>
+        <v>29.2</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>4.1</v>
+        <v>8.5</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -61099,7 +61534,7 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>11.5</v>
+        <v>11.1</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
@@ -61109,14 +61544,14 @@
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -61128,13 +61563,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -61142,10 +61577,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>58</v>
+        <v>89.7</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>5</v>
+        <v>1.2</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -61157,13 +61592,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -61171,13 +61606,42 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>97</v>
+        <v>92.7</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -61198,7 +61662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66340,24 +66804,24 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>23.9</v>
+        <v>25.9</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>23.1</v>
+        <v>31.7</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -66369,24 +66833,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>24.2</v>
+        <v>23.9</v>
       </c>
       <c r="C179" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>33.2</v>
+        <v>3.1</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8</v>
+        <v>11.6</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -66398,13 +66862,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>21.5</v>
+        <v>21.1</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>28.4</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -66412,7 +66876,7 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>63.6</v>
+        <v>63</v>
       </c>
       <c r="G180" s="7" t="n">
         <v>4.4</v>
@@ -66427,21 +66891,21 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>16.1</v>
+        <v>16.2</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>78.90000000000001</v>
+        <v>62.2</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>5.6</v>
+        <v>4.5</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>99.59999999999999</v>
+        <v>99.8</v>
       </c>
       <c r="G181" s="4" t="n">
         <v>0</v>
@@ -66456,13 +66920,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>15.1</v>
+        <v>16.4</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>6.9</v>
+        <v>15.2</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.5</v>
+        <v>4.3</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -66470,10 +66934,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>92.40000000000001</v>
+        <v>51.2</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>0.9</v>
+        <v>5.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -66485,13 +66949,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.3</v>
+        <v>17.9</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -66499,13 +66963,42 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>77.09999999999999</v>
+        <v>58.4</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>2.7</v>
+        <v>5</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -66526,7 +67019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -71668,7 +72161,7 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>25.2</v>
+        <v>27.4</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
@@ -71678,14 +72171,14 @@
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>13.5</v>
+        <v>21.3</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -71697,7 +72190,7 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>26.4</v>
+        <v>26.2</v>
       </c>
       <c r="C179" s="4" t="n">
         <v>0</v>
@@ -71711,10 +72204,10 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>31.2</v>
+        <v>3.4</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>11.6</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -71726,13 +72219,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>22.8</v>
+        <v>22.4</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>23.7</v>
+        <v>60.2</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -71740,10 +72233,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>62.3</v>
+        <v>61.9</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -71755,13 +72248,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>18.8</v>
+        <v>19.3</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>73</v>
+        <v>42.2</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -71769,10 +72262,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>99</v>
+        <v>99.8</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -71784,24 +72277,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>17.1</v>
+        <v>19.2</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>13.8</v>
+        <v>28.8</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>95.90000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>0.5</v>
+        <v>3.7</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -71813,13 +72306,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>17.1</v>
+        <v>18.8</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -71827,13 +72320,42 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>73.40000000000001</v>
+        <v>55.9</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>3.2</v>
+        <v>5.3</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -71854,7 +72376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -76996,7 +77518,7 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>22.3</v>
+        <v>24.4</v>
       </c>
       <c r="C178" s="7" t="n">
         <v>0</v>
@@ -77006,14 +77528,14 @@
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>8.6</v>
+        <v>2.9</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>11</v>
+        <v>11.7</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -77025,13 +77547,13 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>23</v>
+        <v>22.7</v>
       </c>
       <c r="C179" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
@@ -77039,10 +77561,10 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -77054,13 +77576,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>22</v>
+        <v>21.7</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -77068,10 +77590,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>6.2</v>
+        <v>46</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>11.3</v>
+        <v>6.5</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -77083,24 +77605,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>16.5</v>
+        <v>18.7</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>54.3</v>
+        <v>10.7</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>88.8</v>
+        <v>86.3</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -77112,13 +77634,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>14.3</v>
+        <v>16.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>28.9</v>
+        <v>24.6</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -77126,10 +77648,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>63.3</v>
+        <v>94.3</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>4.4</v>
+        <v>0.7</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -77141,13 +77663,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>14.3</v>
+        <v>16.1</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -77155,13 +77677,42 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>43.8</v>
+        <v>66.8</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>6.7</v>
+        <v>4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>
@@ -77182,7 +77733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82324,24 +82875,24 @@
         <v>46272</v>
       </c>
       <c r="B178" s="7" t="n">
-        <v>18.7</v>
+        <v>19.7</v>
       </c>
       <c r="C178" s="7" t="n">
-        <v>10.9</v>
+        <v>0.6</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F178" s="7" t="n">
-        <v>40.3</v>
+        <v>39.4</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="H178" s="12">
         <f>SUM(C172:C178)</f>
@@ -82353,24 +82904,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>18.7</v>
+        <v>19.3</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>4.5</v>
+        <v>3.3</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>37.6</v>
+        <v>20.4</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>7.5</v>
+        <v>9.6</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -82382,13 +82933,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>22.7</v>
+        <v>23.1</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -82396,10 +82947,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>96.7</v>
+        <v>97.8</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -82411,24 +82962,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>10.8</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>50.8</v>
+        <v>77.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>5.9</v>
+        <v>2.7</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -82440,24 +82991,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>10.3</v>
+        <v>12</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>3.5</v>
+        <v>0.3</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>48</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>6.2</v>
+        <v>3.2</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -82469,27 +83020,56 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>10.7</v>
+        <v>12.1</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>6.3</v>
+        <v>0.4</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>85.5</v>
+        <v>61.1</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>1.7</v>
+        <v>4.7</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C184" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="G184" s="7" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H184" s="12">
+        <f>SUM(C178:C184)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-08 10:16 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5684,17 +5684,17 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>27.2</v>
+        <v>28</v>
       </c>
       <c r="C179" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
@@ -5727,10 +5727,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -5742,24 +5742,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>27</v>
+        <v>27.2</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.7</v>
+        <v>3.2</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -5771,7 +5771,7 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>28.8</v>
+        <v>28.4</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
@@ -5785,7 +5785,7 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G182" s="7" t="n">
         <v>12</v>
@@ -5800,24 +5800,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>28.8</v>
+        <v>28.9</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>4.9</v>
+        <v>7.6</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -5829,13 +5829,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>27.7</v>
+        <v>28.3</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -5843,13 +5843,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>32.4</v>
+        <v>11.3</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.1</v>
+        <v>10.6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -5870,7 +5899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11041,24 +11070,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>26.3</v>
+        <v>28</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>0.9</v>
+        <v>3.2</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>29.7</v>
+        <v>55.1</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8.4</v>
+        <v>5.4</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -11070,10 +11099,10 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>19.2</v>
+        <v>19.6</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>33.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D180" s="7" t="n">
         <v>3.2</v>
@@ -11084,10 +11113,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>58.5</v>
+        <v>56.6</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -11099,13 +11128,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>17.1</v>
+        <v>18.4</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -11113,10 +11142,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>3.3</v>
+        <v>11.2</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>11.6</v>
+        <v>10.7</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -11128,24 +11157,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.8</v>
+        <v>19.6</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>6.5</v>
+        <v>11.2</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.2</v>
+        <v>10.7</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -11163,7 +11192,7 @@
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -11171,10 +11200,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>1.8</v>
+        <v>23.8</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.8</v>
+        <v>9.1</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -11186,7 +11215,7 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>19.4</v>
+        <v>20.2</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
@@ -11200,13 +11229,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>2</v>
+        <v>28.3</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.8</v>
+        <v>8.6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -11227,7 +11285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16398,13 +16456,13 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>24.2</v>
+        <v>24.5</v>
       </c>
       <c r="C179" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>8.6</v>
+        <v>7.6</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
@@ -16427,7 +16485,7 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
@@ -16441,7 +16499,7 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G180" s="7" t="n">
         <v>12</v>
@@ -16456,13 +16514,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>23.7</v>
+        <v>23.6</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>5.6</v>
+        <v>6.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -16485,13 +16543,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>24.8</v>
+        <v>24.2</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.2</v>
+        <v>4.9</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -16514,13 +16572,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>23.5</v>
+        <v>24.6</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>5.6</v>
+        <v>4.5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -16543,13 +16601,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>24</v>
+        <v>24.6</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>5</v>
+        <v>3.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -16557,13 +16615,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>12</v>
+        <v>10.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -16584,7 +16671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21755,24 +21842,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>25.9</v>
+        <v>26.6</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>33</v>
+        <v>52.6</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8</v>
+        <v>5.7</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -21784,13 +21871,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>23.9</v>
+        <v>24.1</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>22.8</v>
+        <v>21</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -21798,10 +21885,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>79.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -21813,24 +21900,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>21.7</v>
+        <v>22.3</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0.8</v>
+        <v>3.2</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>4.6</v>
+        <v>5.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>77.5</v>
+        <v>49.8</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>2.7</v>
+        <v>6</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -21842,13 +21929,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>22.3</v>
+        <v>21</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -21856,10 +21943,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>24.8</v>
+        <v>34.6</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>9</v>
+        <v>7.8</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -21871,13 +21958,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>20.2</v>
+        <v>21.7</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>14.5</v>
+        <v>0.2</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -21885,10 +21972,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>60.3</v>
+        <v>17.2</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>4.8</v>
+        <v>9.9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -21900,13 +21987,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>21.8</v>
+        <v>22.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -21914,13 +22001,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>10.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -21941,7 +22057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27112,24 +27228,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>16.9</v>
+        <v>17.3</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>16.3</v>
+        <v>46.8</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>10</v>
+        <v>6.4</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -27141,24 +27257,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>10.9</v>
+        <v>10.2</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>10.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>90.3</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -27170,13 +27286,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.4</v>
+        <v>3.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -27184,10 +27300,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>36.9</v>
+        <v>22.2</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>7.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -27199,13 +27315,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>10.6</v>
+        <v>8.6</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -27213,10 +27329,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>7.2</v>
+        <v>5.5</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -27228,21 +27344,21 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>10</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="G183" s="4" t="n">
         <v>11.8</v>
@@ -27257,13 +27373,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>10.9</v>
+        <v>9.5</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -27271,13 +27387,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>3.9</v>
+        <v>60.1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.5</v>
+        <v>4.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -27298,7 +27443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28960,21 +29105,21 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>17.7</v>
+        <v>20.2</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="G58" s="7" t="n">
         <v>12</v>
@@ -28992,14 +29137,14 @@
         <v>19.5</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
@@ -29018,24 +29163,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>16.6</v>
+        <v>15.7</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>2.7</v>
+        <v>19.7</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>57.8</v>
+        <v>90.5</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>5.1</v>
+        <v>1.1</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -29047,13 +29192,13 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>14.1</v>
+        <v>13.8</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -29061,10 +29206,10 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>73.59999999999999</v>
+        <v>99.8</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -29076,24 +29221,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>14</v>
+        <v>14.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>54.9</v>
+        <v>83.2</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.4</v>
+        <v>2</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -29105,27 +29250,56 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>14</v>
+        <v>14.7</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>88.7</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>12</v>
+        <v>1.4</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H64" s="12">
+        <f>SUM(C58:C64)</f>
         <v/>
       </c>
     </row>
@@ -29146,7 +29320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30808,13 +30982,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>18.1</v>
+        <v>21.3</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -30822,10 +30996,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -30837,13 +31011,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>20.2</v>
+        <v>20</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>6.3</v>
+        <v>35.1</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -30851,10 +31025,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>8.5</v>
+        <v>18.5</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -30866,13 +31040,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.1</v>
+        <v>14.6</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>2.7</v>
+        <v>6.7</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -30880,10 +31054,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>93.2</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -30895,24 +31069,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>14.6</v>
+        <v>13.2</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>15.4</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>44.9</v>
+        <v>100</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>6.6</v>
+        <v>0</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -30924,24 +31098,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>13.6</v>
+        <v>12.8</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>31.6</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>1.2</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -30953,27 +31127,56 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>37.5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>12</v>
+        <v>7.5</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H64" s="12">
+        <f>SUM(C58:C64)</f>
         <v/>
       </c>
     </row>
@@ -30994,7 +31197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32656,13 +32859,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>19.4</v>
+        <v>21.5</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -32670,7 +32873,7 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="G58" s="7" t="n">
         <v>11.9</v>
@@ -32685,13 +32888,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>21</v>
+        <v>20.6</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0.6</v>
+        <v>14.1</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -32699,10 +32902,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>7.6</v>
+        <v>14</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11.1</v>
+        <v>10.3</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -32714,24 +32917,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.3</v>
+        <v>14.5</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>0.2</v>
+        <v>2.4</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>93.40000000000001</v>
+        <v>95.8</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -32743,24 +32946,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>15.6</v>
+        <v>14.1</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>18.8</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>54.7</v>
+        <v>99.8</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -32772,24 +32975,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>15.5</v>
+        <v>13.9</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.3</v>
+        <v>3</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>47.8</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>6.3</v>
+        <v>0.6</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -32801,27 +33004,56 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>14.9</v>
+        <v>13</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>60.5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>12</v>
+        <v>4.7</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H64" s="12">
+        <f>SUM(C58:C64)</f>
         <v/>
       </c>
     </row>
@@ -32842,7 +33074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34504,13 +34736,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>17.3</v>
+        <v>19.7</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -34518,7 +34750,7 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G58" s="7" t="n">
         <v>12</v>
@@ -34533,13 +34765,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>19.4</v>
+        <v>19.5</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0</v>
+        <v>4.4</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -34547,7 +34779,7 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="G59" s="4" t="n">
         <v>12</v>
@@ -34562,24 +34794,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.9</v>
+        <v>15</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>9.9</v>
+        <v>19.1</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>64.7</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>4.2</v>
+        <v>1.2</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -34591,24 +34823,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.8</v>
+        <v>12.9</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>9.9</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>73.8</v>
+        <v>99.8</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -34620,13 +34852,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -34634,10 +34866,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>54.9</v>
+        <v>91.8</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.4</v>
+        <v>1</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -34649,13 +34881,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.5</v>
+        <v>12.9</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -34663,13 +34895,42 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>12</v>
+        <v>1.2</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H64" s="12">
+        <f>SUM(C58:C64)</f>
         <v/>
       </c>
     </row>
@@ -34690,7 +34951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36352,13 +36613,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>19.1</v>
+        <v>21.8</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -36384,10 +36645,10 @@
         <v>21.3</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -36395,10 +36656,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>3.7</v>
+        <v>8.6</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11.6</v>
+        <v>11</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -36410,24 +36671,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>16.8</v>
+        <v>15.9</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>75.2</v>
+        <v>94.7</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>3</v>
+        <v>0.6</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -36439,24 +36700,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>15.3</v>
+        <v>14.6</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>17.4</v>
       </c>
       <c r="D61" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>72.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>3.3</v>
+        <v>0.1</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -36468,24 +36729,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>15.8</v>
+        <v>15.2</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>56.6</v>
+        <v>73.2</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.2</v>
+        <v>3.2</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -36497,27 +36758,56 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>15.3</v>
+        <v>13.8</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>12</v>
+        <v>0.6</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H64" s="12">
+        <f>SUM(C58:C64)</f>
         <v/>
       </c>
     </row>
@@ -36538,7 +36828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38200,13 +38490,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>15</v>
+        <v>17.2</v>
       </c>
       <c r="C58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -38214,10 +38504,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>1.3</v>
+        <v>0.1</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -38229,10 +38519,10 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0</v>
+        <v>13.1</v>
       </c>
       <c r="D59" s="4" t="n">
         <v>2.9</v>
@@ -38243,10 +38533,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>2.5</v>
+        <v>5.8</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11.7</v>
+        <v>11.3</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -38258,13 +38548,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>11.5</v>
+        <v>11.1</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>2</v>
+        <v>5.4</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -38272,10 +38562,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>89</v>
+        <v>94.3</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -38287,24 +38577,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>11.8</v>
+        <v>10.1</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>20.1</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>80.5</v>
+        <v>100</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -38316,24 +38606,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>10.7</v>
+        <v>10.4</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>10.9</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>60.9</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>4.7</v>
+        <v>0.1</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -38345,27 +38635,56 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>10.8</v>
+        <v>10</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>1.4</v>
+        <v>99</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>11.8</v>
+        <v>0.1</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H64" s="12">
+        <f>SUM(C58:C64)</f>
         <v/>
       </c>
     </row>
@@ -38386,7 +38705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43557,24 +43876,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>25.3</v>
+        <v>27.1</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>11.2</v>
+        <v>10.4</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>18.6</v>
+        <v>51.1</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>5.9</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -43589,10 +43908,10 @@
         <v>21.5</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>62.5</v>
+        <v>37.8</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -43600,10 +43919,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>84.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -43615,24 +43934,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>21.2</v>
+        <v>19.2</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>99.2</v>
+        <v>80.2</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0.1</v>
+        <v>2.4</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -43644,24 +43963,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>20.8</v>
+        <v>19</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>0.8</v>
+        <v>7.3</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>0.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>19.9</v>
+        <v>59.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>9.6</v>
+        <v>4.8</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -43673,24 +43992,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>20.1</v>
+        <v>19.3</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>4.4</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
         <v>0.3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>66</v>
+        <v>24.6</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>4.1</v>
+        <v>9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -43702,13 +44021,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>20</v>
+        <v>19.2</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -43716,13 +44035,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>21.6</v>
+        <v>28.5</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -43743,7 +44091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45405,13 +45753,13 @@
         <v>46273</v>
       </c>
       <c r="B58" s="7" t="n">
-        <v>17.9</v>
+        <v>21.4</v>
       </c>
       <c r="C58" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D58" s="7" t="n">
-        <v>4</v>
+        <v>4.4</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
@@ -45419,10 +45767,10 @@
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>8.4</v>
+        <v>10.3</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>11</v>
+        <v>10.8</v>
       </c>
       <c r="H58" s="12">
         <f>SUM(C52:C58)</f>
@@ -45434,13 +45782,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>17.3</v>
+        <v>16.4</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>26.4</v>
+        <v>15</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -45448,10 +45796,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>70.5</v>
+        <v>65.3</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -45463,13 +45811,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -45477,10 +45825,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>70.7</v>
+        <v>63.6</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>3.5</v>
+        <v>4.4</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -45492,24 +45840,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>11.7</v>
+        <v>12.1</v>
       </c>
       <c r="C61" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>49.2</v>
+        <v>34</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>6.1</v>
+        <v>7.9</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -45521,24 +45869,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>58.6</v>
+        <v>78.3</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5</v>
+        <v>2.6</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -45550,27 +45898,56 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13</v>
+        <v>12.2</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>35.8</v>
+        <v>25.6</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>7.7</v>
+        <v>8.9</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H64" s="12">
+        <f>SUM(C58:C64)</f>
         <v/>
       </c>
     </row>
@@ -45591,7 +45968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -50762,13 +51139,13 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>26.8</v>
+        <v>27.2</v>
       </c>
       <c r="C179" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
@@ -50776,10 +51153,10 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>5.9</v>
+        <v>0.1</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>11.3</v>
+        <v>12</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -50791,24 +51168,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>26.9</v>
+        <v>27</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -50820,13 +51197,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>28.2</v>
+        <v>28.8</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.3</v>
+        <v>5.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -50834,10 +51211,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>10.2</v>
+        <v>10.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -50849,13 +51226,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>26.1</v>
+        <v>26.5</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -50863,10 +51240,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>46.7</v>
+        <v>12.3</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>6.4</v>
+        <v>10.5</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -50878,13 +51255,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>26.9</v>
+        <v>26</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -50892,10 +51269,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>13.5</v>
+        <v>37.9</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>10.4</v>
+        <v>7.5</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -50907,27 +51284,56 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>24.4</v>
+        <v>25.6</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>5.9</v>
+        <v>1.8</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.3</v>
+        <v>4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>70.09999999999999</v>
+        <v>24.6</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>3.6</v>
+        <v>9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -50948,7 +51354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56119,13 +56525,13 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>23.5</v>
+        <v>25.7</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>1.1</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
@@ -56133,10 +56539,10 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>26.2</v>
+        <v>45.6</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8.9</v>
+        <v>6.5</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -56151,10 +56557,10 @@
         <v>17.8</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>3.2</v>
+        <v>4.6</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -56162,10 +56568,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>61.7</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -56177,13 +56583,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>14.6</v>
+        <v>14.7</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -56191,7 +56597,7 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="G181" s="4" t="n">
         <v>11.7</v>
@@ -56206,13 +56612,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -56220,10 +56626,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -56235,13 +56641,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>15.8</v>
+        <v>16.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -56249,10 +56655,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -56264,27 +56670,56 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>16.9</v>
+        <v>17.9</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>21.7</v>
+        <v>61</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.4</v>
+        <v>4.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -56305,7 +56740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61476,13 +61911,13 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>12</v>
+        <v>12.9</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>26</v>
+        <v>11.9</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
@@ -61490,10 +61925,10 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>90.90000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -61505,24 +61940,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>12.6</v>
+        <v>11.5</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>2.7</v>
+        <v>1</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>29.2</v>
+        <v>61.6</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>8.5</v>
+        <v>4.6</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -61534,24 +61969,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>11.1</v>
+        <v>11.7</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>25</v>
+        <v>20.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -61563,24 +61998,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>11.3</v>
+        <v>10.7</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>4.7</v>
+        <v>3.2</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>0.9</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>89.7</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -61592,24 +62027,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>7.5</v>
+        <v>5.7</v>
       </c>
       <c r="D183" s="4" t="n">
         <v>1.4</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>92.7</v>
+        <v>98</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -61621,27 +62056,56 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>12.4</v>
+        <v>12.8</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>4.2</v>
+        <v>6.2</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>100</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="G184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -61662,7 +62126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66833,24 +67297,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>23.9</v>
+        <v>25.8</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>3.1</v>
+        <v>0.1</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -66862,10 +67326,10 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>21.1</v>
+        <v>20.6</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>68.09999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="D180" s="7" t="n">
         <v>3.5</v>
@@ -66876,10 +67340,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>63</v>
+        <v>73.8</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>4.4</v>
+        <v>3.1</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -66894,10 +67358,10 @@
         <v>16.2</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>62.2</v>
+        <v>48.1</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>4.5</v>
+        <v>7.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -66905,10 +67369,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>99.8</v>
+        <v>98.8</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -66920,24 +67384,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.4</v>
+        <v>16.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>15.2</v>
+        <v>21.6</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>51.2</v>
+        <v>76.3</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>5.9</v>
+        <v>2.8</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -66949,13 +67413,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -66963,10 +67427,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>58.4</v>
+        <v>73.5</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -66978,13 +67442,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -66992,13 +67456,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.8</v>
+        <v>11</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -67019,7 +67512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -72190,24 +72683,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>26.2</v>
+        <v>28.1</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>3.4</v>
+        <v>0.1</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -72219,24 +72712,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>22.4</v>
+        <v>21.9</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>60.2</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>61.9</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>4.6</v>
+        <v>3.1</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -72248,24 +72741,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>19.3</v>
+        <v>19.4</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>42.2</v>
+        <v>60.5</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.4</v>
+        <v>3.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>99.8</v>
+        <v>99.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -72277,13 +72770,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.2</v>
+        <v>19.5</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>28.8</v>
+        <v>22.4</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -72291,10 +72784,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>69.5</v>
+        <v>82.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>3.7</v>
+        <v>2.1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -72309,7 +72802,7 @@
         <v>18.8</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D183" s="4" t="n">
         <v>1.6</v>
@@ -72320,10 +72813,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>55.9</v>
+        <v>63.1</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>5.3</v>
+        <v>4.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -72335,13 +72828,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>19.1</v>
+        <v>18.9</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -72349,13 +72842,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>13.3</v>
+        <v>20.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.4</v>
+        <v>9.5</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -72376,7 +72898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -77547,24 +78069,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>22.7</v>
+        <v>24.5</v>
       </c>
       <c r="C179" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>10</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -77576,13 +78098,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -77590,10 +78112,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>46</v>
+        <v>53.6</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>6.5</v>
+        <v>5.6</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -77608,18 +78130,18 @@
         <v>18.7</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>10.7</v>
+        <v>37.6</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>86.3</v>
+        <v>86.7</v>
       </c>
       <c r="G181" s="4" t="n">
         <v>1.6</v>
@@ -77634,13 +78156,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.8</v>
+        <v>17.6</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>24.6</v>
+        <v>39.7</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -77648,10 +78170,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>94.3</v>
+        <v>82.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>0.7</v>
+        <v>2.1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -77663,24 +78185,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.1</v>
+        <v>16.2</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.1</v>
+        <v>2.6</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.9</v>
+        <v>2.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>66.8</v>
+        <v>77.2</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>4</v>
+        <v>2.7</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -77692,13 +78214,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>16.1</v>
+        <v>14.7</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.2</v>
+        <v>4.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -77706,13 +78228,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>25.6</v>
+        <v>85.8</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.9</v>
+        <v>1.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>
@@ -77733,7 +78284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82904,24 +83455,24 @@
         <v>46273</v>
       </c>
       <c r="B179" s="4" t="n">
-        <v>19.3</v>
+        <v>20.5</v>
       </c>
       <c r="C179" s="4" t="n">
-        <v>3.3</v>
+        <v>5.2</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>20.4</v>
+        <v>32.5</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>9.6</v>
+        <v>8.1</v>
       </c>
       <c r="H179" s="10">
         <f>SUM(C173:C179)</f>
@@ -82933,24 +83484,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>12.5</v>
+        <v>12.2</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>23.1</v>
+        <v>24.6</v>
       </c>
       <c r="D180" s="7" t="n">
         <v>1.7</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>97.8</v>
+        <v>96.8</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -82962,24 +83513,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>10.8</v>
+        <v>10.3</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>77.5</v>
+        <v>46.3</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>2.7</v>
+        <v>6.4</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -82991,24 +83542,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>0.3</v>
+        <v>2.5</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>73.59999999999999</v>
+        <v>93</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>3.2</v>
+        <v>0.8</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -83020,10 +83571,10 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="D183" s="4" t="n">
         <v>0.6</v>
@@ -83034,10 +83585,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>61.1</v>
+        <v>65.2</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -83049,13 +83600,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>13.1</v>
+        <v>11.8</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -83063,13 +83614,42 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>32.2</v>
+        <v>47.1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.1</v>
+        <v>6.3</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B185" s="4" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H185" s="10">
+        <f>SUM(C179:C185)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-09 10:22 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5713,24 +5713,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>26.7</v>
+        <v>27.5</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.9</v>
+        <v>4.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -5742,21 +5742,21 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G181" s="4" t="n">
         <v>11.9</v>
@@ -5771,13 +5771,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>28.4</v>
+        <v>28.1</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -5785,10 +5785,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -5800,24 +5800,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>28.9</v>
+        <v>28.5</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>7.6</v>
+        <v>5.1</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -5829,24 +5829,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>28.3</v>
+        <v>28.2</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>11.3</v>
+        <v>33.8</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.6</v>
+        <v>7.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -5858,27 +5858,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>27.1</v>
+        <v>25.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>10.9</v>
+        <v>26.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -5899,7 +5928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11099,24 +11128,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>19.6</v>
+        <v>20.5</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.2</v>
+        <v>4.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>56.6</v>
+        <v>24.8</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>5.2</v>
+        <v>9</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -11128,13 +11157,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -11142,10 +11171,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>11.2</v>
+        <v>20.9</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>10.7</v>
+        <v>9.5</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -11157,24 +11186,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.6</v>
+        <v>20.1</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>11.2</v>
+        <v>12.4</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -11186,13 +11215,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -11200,10 +11229,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>23.8</v>
+        <v>0.6</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9.1</v>
+        <v>11.9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -11215,7 +11244,7 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>20.2</v>
+        <v>20.4</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
@@ -11229,10 +11258,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>28.3</v>
+        <v>1.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.6</v>
+        <v>11.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -11244,27 +11273,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>21.8</v>
+        <v>23</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -11285,7 +11343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16485,21 +16543,21 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>6.6</v>
+        <v>5.8</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G180" s="7" t="n">
         <v>12</v>
@@ -16520,7 +16578,7 @@
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -16543,13 +16601,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>24.2</v>
+        <v>24.1</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>4.9</v>
+        <v>5.7</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -16572,7 +16630,7 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>24.6</v>
+        <v>24.2</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
@@ -16601,7 +16659,7 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>24.6</v>
+        <v>24.7</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
@@ -16615,10 +16673,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>10.8</v>
+        <v>14.5</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.7</v>
+        <v>10.3</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -16630,27 +16688,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>24.4</v>
+        <v>24</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -16671,7 +16758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21871,24 +21958,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>24.1</v>
+        <v>23.2</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>21</v>
+        <v>10.1</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>4.3</v>
+        <v>7.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>74.7</v>
+        <v>63.3</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>3</v>
+        <v>4.4</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -21900,24 +21987,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>22.3</v>
+        <v>21</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>3.2</v>
+        <v>37.7</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>49.8</v>
+        <v>62.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -21929,10 +22016,10 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>21</v>
+        <v>20.6</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>2</v>
+        <v>5.2</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>2.9</v>
@@ -21943,10 +22030,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>34.6</v>
+        <v>42.3</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -21958,24 +22045,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>17.2</v>
+        <v>43.5</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9.9</v>
+        <v>6.8</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -21987,13 +22074,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>22.1</v>
+        <v>21.7</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -22001,10 +22088,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>30.3</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.9</v>
+        <v>8.4</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -22016,13 +22103,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>22</v>
+        <v>22.3</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -22030,13 +22117,42 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>27.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -22057,7 +22173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27257,24 +27373,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>10.2</v>
+        <v>10.5</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.1</v>
+        <v>4.3</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>94.90000000000001</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -27286,24 +27402,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>9.4</v>
+        <v>7.3</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0</v>
+        <v>16.2</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>3.3</v>
+        <v>4.2</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>22.2</v>
+        <v>40.3</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -27315,13 +27431,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2</v>
+        <v>3.7</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -27329,10 +27445,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>5.5</v>
+        <v>16</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.3</v>
+        <v>10.1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -27350,7 +27466,7 @@
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -27358,10 +27474,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>1.9</v>
+        <v>14.6</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.8</v>
+        <v>10.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -27373,13 +27489,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>9.5</v>
+        <v>10.8</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -27387,10 +27503,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>60.1</v>
+        <v>49.6</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -27402,27 +27518,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>24.6</v>
+        <v>18.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -27443,7 +27588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29134,24 +29279,24 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>19.5</v>
+        <v>21.6</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -29163,13 +29308,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>19.7</v>
+        <v>22.7</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -29177,10 +29322,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>90.5</v>
+        <v>89.5</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -29192,24 +29337,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.8</v>
+        <v>13</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>11.6</v>
+        <v>20.9</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.8</v>
+        <v>98</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -29221,13 +29366,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>14.7</v>
+        <v>13.1</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -29235,10 +29380,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>83.2</v>
+        <v>67.2</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -29250,24 +29395,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>14.7</v>
+        <v>13</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>88.7</v>
+        <v>15.8</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>1.4</v>
+        <v>10.1</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -29279,27 +29424,56 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.3</v>
+        <v>13.7</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>48.4</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>6.2</v>
+        <v>3.2</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(C59:C65)</f>
         <v/>
       </c>
     </row>
@@ -29320,7 +29494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31011,24 +31185,24 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>20</v>
+        <v>22.4</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>35.1</v>
+        <v>22.6</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>18.5</v>
+        <v>28.2</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -31040,13 +31214,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>14.6</v>
+        <v>14.9</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>6.7</v>
+        <v>5.9</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -31054,10 +31228,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>96.09999999999999</v>
+        <v>88</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -31069,24 +31243,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.2</v>
+        <v>12.1</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>15.4</v>
+        <v>17.9</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>100</v>
+        <v>88.5</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -31098,24 +31272,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.8</v>
+        <v>11.1</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>90.40000000000001</v>
+        <v>52</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>1.2</v>
+        <v>5.8</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -31127,24 +31301,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.7</v>
+        <v>12.2</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>37.5</v>
+        <v>25.2</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -31156,27 +31330,56 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.1</v>
+        <v>12.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>19.7</v>
+        <v>84</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>9.6</v>
+        <v>1.9</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(C59:C65)</f>
         <v/>
       </c>
     </row>
@@ -31197,7 +31400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32888,13 +33091,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>20.6</v>
+        <v>22.7</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>14.1</v>
+        <v>5.2</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -32902,10 +33105,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>14</v>
+        <v>24.6</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>10.3</v>
+        <v>9</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -32917,13 +33120,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>14.5</v>
+        <v>15.2</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>2.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -32931,10 +33134,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>95.8</v>
+        <v>90.8</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -32946,24 +33149,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>14.1</v>
+        <v>12.7</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>18.8</v>
+        <v>17</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.8</v>
+        <v>97.3</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -32975,13 +33178,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>13.9</v>
+        <v>11.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -32989,10 +33192,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>95.09999999999999</v>
+        <v>60.1</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0.6</v>
+        <v>4.8</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -33004,24 +33207,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13</v>
+        <v>12.9</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>1.9</v>
+        <v>0.9</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>60.5</v>
+        <v>26</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4.7</v>
+        <v>8.9</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -33033,27 +33236,56 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.1</v>
+        <v>13</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>26.4</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(C59:C65)</f>
         <v/>
       </c>
     </row>
@@ -33074,7 +33306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34765,13 +34997,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>19.5</v>
+        <v>21.3</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>4.4</v>
+        <v>10.5</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -34779,7 +35011,7 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G59" s="4" t="n">
         <v>12</v>
@@ -34794,24 +35026,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>19.1</v>
+        <v>34.7</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>89.90000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -34823,24 +35055,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>12.9</v>
+        <v>11.7</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>9.9</v>
+        <v>15.5</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.3</v>
+        <v>3.3</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.8</v>
+        <v>98.3</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -34852,24 +35084,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>13.9</v>
+        <v>11.5</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>9.5</v>
+        <v>0.2</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.6</v>
+        <v>4.2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>91.8</v>
+        <v>66.8</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -34881,24 +35113,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.9</v>
+        <v>12.2</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2.9</v>
+        <v>1.6</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>90</v>
+        <v>6.1</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>1.2</v>
+        <v>11.3</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -34910,13 +35142,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.5</v>
+        <v>13.6</v>
       </c>
       <c r="C64" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -34924,13 +35156,42 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>67.59999999999999</v>
+        <v>94</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.9</v>
+        <v>0.7</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(C59:C65)</f>
         <v/>
       </c>
     </row>
@@ -34951,7 +35212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36642,13 +36903,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>21.3</v>
+        <v>23.2</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>6.7</v>
+        <v>3.6</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -36656,10 +36917,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>8.6</v>
+        <v>19.8</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11</v>
+        <v>9.6</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -36671,13 +36932,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.9</v>
+        <v>16.5</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>2.2</v>
+        <v>6</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -36685,10 +36946,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>94.7</v>
+        <v>88.7</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -36700,24 +36961,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>14.6</v>
+        <v>13.3</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>17.4</v>
+        <v>13.6</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.40000000000001</v>
+        <v>88.3</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.1</v>
+        <v>1.4</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -36729,24 +36990,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>15.2</v>
+        <v>12.4</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>5.5</v>
+        <v>0.2</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>73.2</v>
+        <v>62.1</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>3.2</v>
+        <v>4.5</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -36758,24 +37019,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.8</v>
+        <v>13</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>1.3</v>
+        <v>0.1</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>94.90000000000001</v>
+        <v>21.3</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.6</v>
+        <v>9.4</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -36787,27 +37048,56 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.1</v>
+        <v>13.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>18.8</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>0</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(C59:C65)</f>
         <v/>
       </c>
     </row>
@@ -36828,7 +37118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38519,13 +38809,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>16.8</v>
+        <v>18.8</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>13.1</v>
+        <v>4.6</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -38533,10 +38823,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>5.8</v>
+        <v>12.4</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -38548,13 +38838,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>11.1</v>
+        <v>11.6</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>5.4</v>
+        <v>6.9</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -38562,10 +38852,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>94.3</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -38577,17 +38867,17 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>20.1</v>
+        <v>13.3</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.3</v>
+        <v>2.1</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
@@ -38606,13 +38896,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>10.4</v>
+        <v>8.1</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>10.9</v>
+        <v>0.2</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -38620,10 +38910,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>99.40000000000001</v>
+        <v>60</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0.1</v>
+        <v>4.8</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -38635,24 +38925,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>10</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>99</v>
+        <v>35.5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.1</v>
+        <v>7.7</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -38667,24 +38957,53 @@
         <v>9.800000000000001</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.7</v>
+        <v>1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>18.6</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(C59:C65)</f>
         <v/>
       </c>
     </row>
@@ -38705,7 +39024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43905,24 +44224,24 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>21.5</v>
+        <v>22</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>37.8</v>
+        <v>20.4</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>90.8</v>
+        <v>94</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -43934,24 +44253,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>19.2</v>
+        <v>18.6</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>13.7</v>
+        <v>11</v>
       </c>
       <c r="D181" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E181" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F181" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="G181" s="4" t="n">
         <v>1.3</v>
-      </c>
-      <c r="E181" s="4" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="F181" s="4" t="n">
-        <v>80.2</v>
-      </c>
-      <c r="G181" s="4" t="n">
-        <v>2.4</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -43963,24 +44282,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>7.3</v>
+        <v>1.4</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>59.8</v>
+        <v>69.7</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -43992,24 +44311,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>19.3</v>
+        <v>19.7</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>24.6</v>
+        <v>24.2</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -44021,10 +44340,10 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>19.2</v>
+        <v>19.7</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>0.3</v>
@@ -44035,10 +44354,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>28.5</v>
+        <v>51</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.6</v>
+        <v>5.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -44050,27 +44369,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20.3</v>
+        <v>20.6</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>38.3</v>
+        <v>33.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7.4</v>
+        <v>8</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -44091,7 +44439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45782,13 +46130,13 @@
         <v>46274</v>
       </c>
       <c r="B59" s="4" t="n">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="C59" s="4" t="n">
-        <v>15</v>
+        <v>23.6</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -45796,10 +46144,10 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>65.3</v>
+        <v>88.8</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>4.2</v>
+        <v>1.3</v>
       </c>
       <c r="H59" s="10">
         <f>SUM(C53:C59)</f>
@@ -45811,13 +46159,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>12.4</v>
+        <v>12.2</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -45825,10 +46173,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>63.6</v>
+        <v>87</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>4.4</v>
+        <v>1.6</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -45840,24 +46188,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>12.1</v>
+        <v>11.4</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>34</v>
+        <v>87.5</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>7.9</v>
+        <v>1.5</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -45869,24 +46217,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.7</v>
+        <v>11.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.5</v>
+        <v>1.1</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>78.3</v>
+        <v>47.3</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2.6</v>
+        <v>6.3</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -45898,13 +46246,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.2</v>
+        <v>13.9</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -45912,10 +46260,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>25.6</v>
+        <v>67</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>8.9</v>
+        <v>4</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -45927,13 +46275,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.8</v>
+        <v>12.9</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -45941,13 +46289,42 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>70.5</v>
+        <v>59.4</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.5</v>
+        <v>4.9</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H65" s="10">
+        <f>SUM(C59:C65)</f>
         <v/>
       </c>
     </row>
@@ -45968,7 +46345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51168,13 +51545,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>27</v>
+        <v>28.2</v>
       </c>
       <c r="C180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -51182,10 +51559,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>0.3</v>
+        <v>1.7</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -51197,24 +51574,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>28.8</v>
+        <v>29.2</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>5.4</v>
+        <v>6.7</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>10.5</v>
+        <v>24.4</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>10.7</v>
+        <v>9.1</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -51226,24 +51603,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>26.5</v>
+        <v>26.7</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>11.6</v>
+        <v>32.1</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.5</v>
+        <v>5.3</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>12.3</v>
+        <v>23.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>10.5</v>
+        <v>9.1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -51255,13 +51632,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>26</v>
+        <v>25.4</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -51269,10 +51646,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>37.9</v>
+        <v>67.8</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>7.5</v>
+        <v>3.9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -51284,24 +51661,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>25.6</v>
+        <v>26.3</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>24.6</v>
+        <v>6.5</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9</v>
+        <v>11.2</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -51313,27 +51690,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>25.8</v>
+        <v>26</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>5.7</v>
+        <v>2.9</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>16.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10</v>
+        <v>10.8</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -51354,7 +51760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56554,13 +56960,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>17.8</v>
+        <v>18.6</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -56568,10 +56974,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>64.59999999999999</v>
+        <v>57</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -56583,7 +56989,7 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>14.7</v>
+        <v>14.6</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
@@ -56597,10 +57003,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>2.6</v>
+        <v>12.3</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>11.7</v>
+        <v>10.5</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -56612,13 +57018,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.3</v>
+        <v>16.6</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.9</v>
+        <v>3.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -56626,10 +57032,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0.6</v>
+        <v>8.9</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.9</v>
+        <v>10.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -56641,13 +57047,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.3</v>
+        <v>16.4</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -56655,10 +57061,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>3.3</v>
+        <v>1.1</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.6</v>
+        <v>11.9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -56676,18 +57082,18 @@
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>61</v>
+        <v>1.6</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>4.7</v>
+        <v>11.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -56699,13 +57105,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>18.6</v>
+        <v>20</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -56713,13 +57119,42 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>6.8</v>
+        <v>3.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -56740,7 +57175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61940,13 +62375,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -61954,10 +62389,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>61.6</v>
+        <v>41</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>4.6</v>
+        <v>7.1</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -61969,24 +62404,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D181" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>20.5</v>
+        <v>50.6</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>9.5</v>
+        <v>5.9</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -61998,21 +62433,21 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>10.7</v>
+        <v>12.1</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>3.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>92.40000000000001</v>
+        <v>92.2</v>
       </c>
       <c r="G182" s="7" t="n">
         <v>0.9</v>
@@ -62027,13 +62462,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>11.9</v>
+        <v>12.1</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>5.7</v>
+        <v>7</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -62041,10 +62476,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -62056,24 +62491,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>6.2</v>
+        <v>2.7</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>99.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -62085,13 +62520,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>11.9</v>
+        <v>11</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -62099,13 +62534,42 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>95</v>
+        <v>91.7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -62126,7 +62590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67326,13 +67790,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>20.6</v>
+        <v>21.8</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>70.8</v>
+        <v>35.7</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -67340,10 +67804,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>73.8</v>
+        <v>89.2</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>3.1</v>
+        <v>1.3</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -67355,24 +67819,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>16.2</v>
+        <v>17.3</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>48.1</v>
+        <v>61.3</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>98.8</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -67387,21 +67851,21 @@
         <v>16.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>21.6</v>
+        <v>50</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.8</v>
+        <v>5.2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>76.3</v>
+        <v>87.2</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>2.8</v>
+        <v>1.5</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -67413,13 +67877,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18</v>
+        <v>18.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -67427,10 +67891,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>73.5</v>
+        <v>38.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>3.2</v>
+        <v>7.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -67442,24 +67906,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>18.3</v>
+        <v>17.2</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>19.7</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11</v>
+        <v>9.6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -67471,13 +67935,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>18.4</v>
+        <v>18.1</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -67485,13 +67949,42 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>41</v>
+        <v>46.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7.1</v>
+        <v>6.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -67512,7 +68005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -72712,13 +73205,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>21.9</v>
+        <v>23.3</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>84.40000000000001</v>
+        <v>23.5</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -72726,10 +73219,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>74.40000000000001</v>
+        <v>93.2</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>3.1</v>
+        <v>0.8</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -72741,13 +73234,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>19.4</v>
+        <v>20.7</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>60.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -72755,7 +73248,7 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>99.5</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="G181" s="4" t="n">
         <v>0.1</v>
@@ -72770,13 +73263,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.5</v>
+        <v>19.3</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>22.4</v>
+        <v>21.1</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -72784,10 +73277,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>82.8</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>2.1</v>
+        <v>1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -72799,10 +73292,10 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18.8</v>
+        <v>18.9</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
         <v>1.6</v>
@@ -72813,10 +73306,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>63.1</v>
+        <v>43.4</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>4.4</v>
+        <v>6.8</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -72828,24 +73321,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>18.9</v>
+        <v>18.2</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>20.9</v>
+        <v>19.5</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -72857,27 +73350,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>18.9</v>
+        <v>19.4</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.4</v>
+        <v>1.1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>31.1</v>
+        <v>46.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>6.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -72898,7 +73420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -78098,13 +78620,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>21.5</v>
+        <v>22.7</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>2.1</v>
+        <v>0.5</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -78112,10 +78634,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>53.6</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -78127,24 +78649,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>18.7</v>
+        <v>20.4</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>37.6</v>
+        <v>35</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>86.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>1.6</v>
+        <v>3.4</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -78156,24 +78678,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>17.6</v>
+        <v>17.7</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>39.7</v>
+        <v>60.8</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>82.8</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -78185,24 +78707,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.2</v>
+        <v>15.7</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.2</v>
+        <v>4.6</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>77.2</v>
+        <v>30.7</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>2.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -78214,13 +78736,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>14.7</v>
+        <v>15</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>4.7</v>
+        <v>3.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -78228,10 +78750,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>85.8</v>
+        <v>11.5</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>1.7</v>
+        <v>10.6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -78243,13 +78765,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>5.6</v>
+        <v>2.5</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -78257,13 +78779,42 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>13.3</v>
+        <v>63.1</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.4</v>
+        <v>4.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>
@@ -78284,7 +78835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83484,13 +84035,13 @@
         <v>46274</v>
       </c>
       <c r="B180" s="7" t="n">
-        <v>12.2</v>
+        <v>10.6</v>
       </c>
       <c r="C180" s="7" t="n">
-        <v>24.6</v>
+        <v>9.9</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
@@ -83498,10 +84049,10 @@
         </is>
       </c>
       <c r="F180" s="7" t="n">
-        <v>96.8</v>
+        <v>99.3</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="H180" s="12">
         <f>SUM(C174:C180)</f>
@@ -83513,24 +84064,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>46.3</v>
+        <v>95.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>6.4</v>
+        <v>0.5</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -83542,24 +84093,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>2.5</v>
+        <v>0.2</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>93</v>
+        <v>70.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>0.8</v>
+        <v>3.5</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -83571,24 +84122,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>65.2</v>
+        <v>19.5</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>4.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -83600,13 +84151,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>11.8</v>
+        <v>13.4</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -83614,10 +84165,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>47.1</v>
+        <v>62.7</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>6.3</v>
+        <v>4.5</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -83629,27 +84180,56 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>12.8</v>
+        <v>14.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>36.3</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7.6</v>
+        <v>2.8</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H186" s="12">
+        <f>SUM(C180:C186)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-10 10:14 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5742,13 +5742,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>27</v>
+        <v>28.2</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -5756,10 +5756,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>0.5</v>
+        <v>2.2</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -5771,13 +5771,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -5785,10 +5785,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -5800,24 +5800,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>28.5</v>
+        <v>28.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.1</v>
+        <v>3.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>5.1</v>
+        <v>8.5</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.4</v>
+        <v>11</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -5829,24 +5829,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>28.2</v>
+        <v>27.4</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>33.8</v>
+        <v>10.6</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>7.9</v>
+        <v>10.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -5858,24 +5858,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>2.4</v>
+        <v>5.3</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>26.9</v>
+        <v>11.7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>10.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -5887,13 +5887,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.4</v>
+        <v>23.9</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>11.7</v>
+        <v>1.4</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -5901,13 +5901,42 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>53.1</v>
+        <v>28.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>5.6</v>
+        <v>8.6</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -5928,7 +5957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11157,24 +11186,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>18.3</v>
+        <v>20.4</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>20.9</v>
+        <v>18</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>9.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -11186,7 +11215,7 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>20.1</v>
+        <v>19.6</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
@@ -11200,10 +11229,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>12.4</v>
+        <v>0.2</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -11215,13 +11244,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -11229,10 +11258,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>0.6</v>
+        <v>5.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.9</v>
+        <v>11.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -11244,21 +11273,21 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>20.4</v>
+        <v>20.6</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="G184" s="7" t="n">
         <v>11.8</v>
@@ -11273,24 +11302,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23</v>
+        <v>21.9</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>0.6</v>
+        <v>20.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11.9</v>
+        <v>9.5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -11302,27 +11331,56 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>24.9</v>
+        <v>23.7</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>0.8</v>
+        <v>7.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.9</v>
+        <v>11.1</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -11343,7 +11401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16572,17 +16630,17 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>23.6</v>
+        <v>23.9</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
@@ -16601,13 +16659,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>24.1</v>
+        <v>24.2</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -16630,13 +16688,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>4.5</v>
+        <v>5.7</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -16659,24 +16717,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.3</v>
+        <v>12</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -16688,13 +16746,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3.9</v>
+        <v>3.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -16702,10 +16760,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -16717,13 +16775,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>23.3</v>
+        <v>22.5</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -16731,13 +16789,42 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>7.2</v>
+        <v>6.6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -16758,7 +16845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21990,21 +22077,21 @@
         <v>21</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>37.7</v>
+        <v>4.6</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>62.5</v>
+        <v>45</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>4.5</v>
+        <v>6.6</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -22019,7 +22106,7 @@
         <v>20.6</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>5.2</v>
+        <v>2.9</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>2.9</v>
@@ -22030,10 +22117,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>42.3</v>
+        <v>41.9</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -22045,24 +22132,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>21.5</v>
+        <v>22.1</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>43.5</v>
+        <v>6.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>6.8</v>
+        <v>11.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -22074,13 +22161,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>21.7</v>
+        <v>21.4</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -22088,10 +22175,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>30.3</v>
+        <v>39.2</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.4</v>
+        <v>7.3</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -22103,13 +22190,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>22.3</v>
+        <v>22.1</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -22117,10 +22204,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>58.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.9</v>
+        <v>5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -22132,13 +22219,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.4</v>
+        <v>21.9</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -22146,13 +22233,42 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>11.9</v>
+        <v>55.8</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.6</v>
+        <v>5.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -22173,7 +22289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27402,24 +27518,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>7.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>16.2</v>
+        <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>40.3</v>
+        <v>5.3</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>7.2</v>
+        <v>11.4</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -27431,13 +27547,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -27445,10 +27561,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>16</v>
+        <v>30.3</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>10.1</v>
+        <v>8.4</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -27460,13 +27576,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -27474,10 +27590,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>14.6</v>
+        <v>11</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>10.2</v>
+        <v>10.7</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -27489,13 +27605,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -27503,10 +27619,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>49.6</v>
+        <v>1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>6</v>
+        <v>11.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -27518,24 +27634,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>18.2</v>
+        <v>53.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -27547,27 +27663,56 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>12.5</v>
+        <v>13.8</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -27588,7 +27733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29308,24 +29453,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.6</v>
+        <v>16.1</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>22.7</v>
+        <v>0.4</v>
       </c>
       <c r="D60" s="7" t="n">
         <v>2.2</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>89.5</v>
+        <v>77</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.3</v>
+        <v>2.8</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -29337,24 +29482,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13</v>
+        <v>13.8</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>20.9</v>
+        <v>17.7</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>98</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -29366,24 +29511,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>13.1</v>
+        <v>12.3</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.6</v>
+        <v>4.2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>67.2</v>
+        <v>63.6</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -29401,18 +29546,18 @@
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>15.8</v>
+        <v>3.9</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>10.1</v>
+        <v>11.5</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -29424,13 +29569,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -29438,10 +29583,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>73.40000000000001</v>
+        <v>46.1</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.2</v>
+        <v>6.5</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -29453,27 +29598,56 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>6.3</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.6</v>
+        <v>0.9</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>69.5</v>
+        <v>45.1</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>3.7</v>
+        <v>6.6</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H66" s="12">
+        <f>SUM(C60:C66)</f>
         <v/>
       </c>
     </row>
@@ -29494,7 +29668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31214,13 +31388,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>5.9</v>
+        <v>0.5</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -31228,10 +31402,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>88</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -31243,24 +31417,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>17.9</v>
+        <v>32.9</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>88.5</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -31272,24 +31446,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>52</v>
+        <v>56.4</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.8</v>
+        <v>5.2</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -31301,10 +31475,10 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.2</v>
+        <v>12</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>0.9</v>
@@ -31315,10 +31489,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>25.2</v>
+        <v>24</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -31330,24 +31504,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>12.8</v>
+        <v>13.5</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>4.3</v>
+        <v>0.3</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>84</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -31359,27 +31533,56 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.8</v>
+        <v>14</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>79.5</v>
+        <v>41.2</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>2.5</v>
+        <v>7.1</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H66" s="12">
+        <f>SUM(C60:C66)</f>
         <v/>
       </c>
     </row>
@@ -31400,7 +31603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33120,24 +33323,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>15.2</v>
+        <v>16.1</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>1.9</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>90.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -33149,13 +33352,13 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>12.7</v>
+        <v>13.3</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>17</v>
+        <v>36.3</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -33163,10 +33366,10 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>97.3</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -33178,24 +33381,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>60.1</v>
+        <v>33.4</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>4.8</v>
+        <v>8</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -33207,24 +33410,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>8.9</v>
+        <v>12</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -33236,24 +33439,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13</v>
+        <v>14.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>94.90000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>0.6</v>
+        <v>2.8</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -33265,27 +33468,56 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.9</v>
+        <v>15.8</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>57</v>
+        <v>22.3</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>5.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H66" s="12">
+        <f>SUM(C60:C66)</f>
         <v/>
       </c>
     </row>
@@ -33306,7 +33538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35026,24 +35258,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>34.7</v>
+        <v>0</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>86.2</v>
+        <v>86.5</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -35055,13 +35287,13 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>11.7</v>
+        <v>12.6</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>15.5</v>
+        <v>30.8</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -35069,10 +35301,10 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>98.3</v>
+        <v>94.2</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -35084,24 +35316,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.5</v>
+        <v>10.8</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.2</v>
+        <v>4.7</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>66.8</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -35113,24 +35345,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.2</v>
+        <v>12.4</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>6.1</v>
+        <v>2.5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>11.3</v>
+        <v>11.7</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -35142,13 +35374,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.6</v>
+        <v>14.4</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.8</v>
+        <v>1.3</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -35156,10 +35388,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>94</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>0.7</v>
+        <v>3.9</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -35171,27 +35403,56 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2.6</v>
+        <v>0.5</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>81.59999999999999</v>
+        <v>36.7</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>2.2</v>
+        <v>7.6</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H66" s="12">
+        <f>SUM(C60:C66)</f>
         <v/>
       </c>
     </row>
@@ -35212,7 +35473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36932,24 +37193,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>16.5</v>
+        <v>17.6</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>6</v>
+        <v>1.6</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>88.7</v>
+        <v>92</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -36961,24 +37222,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.3</v>
+        <v>13.8</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>13.6</v>
+        <v>23.4</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>88.3</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -36990,13 +37251,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.4</v>
+        <v>12.6</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.4</v>
+        <v>2.7</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -37004,10 +37265,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>62.1</v>
+        <v>55</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -37019,24 +37280,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13</v>
+        <v>12.7</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>21.3</v>
+        <v>1.9</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>9.4</v>
+        <v>11.8</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -37048,13 +37309,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.1</v>
+        <v>15.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -37062,10 +37323,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>99.59999999999999</v>
+        <v>71.3</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -37077,13 +37338,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -37091,13 +37352,42 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>32</v>
+        <v>23.6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H66" s="12">
+        <f>SUM(C60:C66)</f>
         <v/>
       </c>
     </row>
@@ -37118,7 +37408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38838,13 +39128,13 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>11.6</v>
+        <v>13.1</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>6.9</v>
+        <v>0.6</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
@@ -38852,10 +39142,10 @@
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>89.40000000000001</v>
+        <v>91.2</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -38867,13 +39157,13 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>9</v>
+        <v>9.6</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>13.3</v>
+        <v>28.9</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -38896,24 +39186,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>8.1</v>
+        <v>7.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>60</v>
+        <v>51.1</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>4.8</v>
+        <v>5.9</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -38925,13 +39215,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -38939,10 +39229,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>35.5</v>
+        <v>1</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>7.7</v>
+        <v>11.9</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -38954,24 +39244,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>99.40000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>0.1</v>
+        <v>3.4</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -38983,27 +39273,56 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>11.1</v>
+        <v>11.8</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>79.5</v>
+        <v>26.9</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>2.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H66" s="12">
+        <f>SUM(C60:C66)</f>
         <v/>
       </c>
     </row>
@@ -39024,7 +39343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44253,13 +44572,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>18.6</v>
+        <v>19.1</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -44267,10 +44586,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>89</v>
+        <v>76.2</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>1.3</v>
+        <v>2.9</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -44282,24 +44601,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.8</v>
+        <v>20</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>1.4</v>
+        <v>4.7</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>69.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -44311,13 +44630,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>19.7</v>
+        <v>19.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -44325,10 +44644,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>24.2</v>
+        <v>22.1</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -44340,24 +44659,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>19.7</v>
+        <v>19.4</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>51</v>
+        <v>51.7</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -44369,24 +44688,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20.6</v>
+        <v>21.1</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>33.2</v>
+        <v>25</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -44398,13 +44717,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>20.5</v>
+        <v>21.8</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -44412,13 +44731,42 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>44.1</v>
+        <v>20.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>6.7</v>
+        <v>9.6</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -44439,7 +44787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46159,24 +46507,24 @@
         <v>46275</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>12.2</v>
+        <v>13.2</v>
       </c>
       <c r="C60" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>87</v>
+        <v>93.2</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="H60" s="12">
         <f>SUM(C54:C60)</f>
@@ -46188,24 +46536,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>11.4</v>
+        <v>9.9</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="D61" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G61" s="4" t="n">
         <v>1.9</v>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="G61" s="4" t="n">
-        <v>1.5</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -46217,24 +46565,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.7</v>
+        <v>11.4</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>47.3</v>
+        <v>37.6</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>6.3</v>
+        <v>7.5</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -46246,10 +46594,10 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.9</v>
+        <v>13.7</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>2.1</v>
+        <v>0.3</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>1.9</v>
@@ -46260,10 +46608,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>67</v>
+        <v>61.7</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -46275,24 +46623,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>12.9</v>
+        <v>14.2</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>5</v>
+        <v>2.7</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>59.4</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>4.9</v>
+        <v>4.2</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -46304,27 +46652,56 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>11.2</v>
+        <v>14.1</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>32.2</v>
+        <v>41</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>8.1</v>
+        <v>7.1</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H66" s="12">
+        <f>SUM(C60:C66)</f>
         <v/>
       </c>
     </row>
@@ -46345,7 +46722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51574,13 +51951,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>29.2</v>
+        <v>29.8</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>6.7</v>
+        <v>7.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -51588,10 +51965,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>24.4</v>
+        <v>31.1</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>9.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -51603,13 +51980,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>26.7</v>
+        <v>27</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>32.1</v>
+        <v>11.4</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.3</v>
+        <v>4.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -51617,7 +51994,7 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>23.8</v>
+        <v>24.4</v>
       </c>
       <c r="G182" s="7" t="n">
         <v>9.1</v>
@@ -51632,13 +52009,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>25.4</v>
+        <v>26.4</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>3.8</v>
+        <v>3</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3</v>
+        <v>5.6</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -51646,10 +52023,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>67.8</v>
+        <v>61.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -51661,13 +52038,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>26.3</v>
+        <v>26.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -51675,10 +52052,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>6.5</v>
+        <v>17.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.2</v>
+        <v>9.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -51690,24 +52067,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>53.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.8</v>
+        <v>5.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -51719,27 +52096,56 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>16.4</v>
+        <v>32.4</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10</v>
+        <v>8.1</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -51760,7 +52166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56989,13 +57395,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>14.6</v>
+        <v>17.5</v>
       </c>
       <c r="C181" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -57003,10 +57409,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>12.3</v>
+        <v>16.4</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -57018,7 +57424,7 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.6</v>
+        <v>16.7</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
@@ -57032,10 +57438,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>8.9</v>
+        <v>1.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>10.9</v>
+        <v>11.8</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -57047,13 +57453,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.8</v>
+        <v>3.7</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -57061,10 +57467,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>1.1</v>
+        <v>17.8</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.9</v>
+        <v>9.9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -57076,13 +57482,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>17.9</v>
+        <v>17.8</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -57090,7 +57496,7 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="G184" s="7" t="n">
         <v>11.8</v>
@@ -57105,13 +57511,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20</v>
+        <v>18.8</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -57119,10 +57525,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>3.9</v>
+        <v>36.1</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11.5</v>
+        <v>7.7</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -57134,13 +57540,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.4</v>
+        <v>19.8</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -57148,13 +57554,42 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>0</v>
+        <v>9.9</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>12</v>
+        <v>10.8</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -57175,7 +57610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62404,24 +62839,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>12</v>
+        <v>12.8</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>50.6</v>
+        <v>66.8</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>5.9</v>
+        <v>4</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -62433,24 +62868,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>12.1</v>
+        <v>10.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>14.1</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>92.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>0.9</v>
+        <v>2.1</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -62462,24 +62897,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>12.1</v>
+        <v>11.5</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>7</v>
+        <v>20.3</v>
       </c>
       <c r="D183" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E183" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F183" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="G183" s="4" t="n">
         <v>1.1</v>
-      </c>
-      <c r="E183" s="4" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="F183" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="G183" s="4" t="n">
-        <v>0.1</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -62491,10 +62926,10 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>1.7</v>
@@ -62505,10 +62940,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>88</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -62520,24 +62955,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>91.7</v>
+        <v>99.8</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -62549,27 +62984,56 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>11.6</v>
+        <v>14.3</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>99.2</v>
+        <v>97.8</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -62590,7 +63054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67819,24 +68283,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>61.3</v>
+        <v>85</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>6.8</v>
+        <v>8.4</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>99.59999999999999</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -67848,13 +68312,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.8</v>
+        <v>16.9</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>50</v>
+        <v>37.4</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -67862,10 +68326,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>87.2</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -67877,13 +68341,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18.3</v>
+        <v>17.8</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -67891,10 +68355,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>38.3</v>
+        <v>18</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>7.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -67912,18 +68376,18 @@
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>19.7</v>
+        <v>15.6</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -67935,10 +68399,10 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>1.5</v>
@@ -67949,10 +68413,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>46.9</v>
+        <v>33.6</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>6.4</v>
+        <v>8</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -67964,27 +68428,56 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>18.1</v>
+        <v>18.8</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>5.1</v>
+        <v>4.5</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -68005,7 +68498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -73234,13 +73727,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>20.7</v>
+        <v>20.3</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>88.40000000000001</v>
+        <v>60.6</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -73248,10 +73741,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>98.90000000000001</v>
+        <v>97.5</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -73263,13 +73756,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.3</v>
+        <v>18.4</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>21.1</v>
+        <v>31.6</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -73277,10 +73770,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>91.40000000000001</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -73292,13 +73785,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18.9</v>
+        <v>18.1</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.6</v>
+        <v>2.9</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -73306,10 +73799,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>43.4</v>
+        <v>16.1</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>6.8</v>
+        <v>10.1</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -73321,24 +73814,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>18.2</v>
+        <v>18</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>19.5</v>
+        <v>25.6</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -73350,24 +73843,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>19.4</v>
+        <v>19.7</v>
       </c>
       <c r="C185" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" s="4" t="n">
         <v>1.5</v>
       </c>
-      <c r="D185" s="4" t="n">
-        <v>1.1</v>
-      </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
           <t>Z</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>46.5</v>
+        <v>41</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -73379,13 +73872,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>19.3</v>
+        <v>21</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -73393,13 +73886,42 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>15.2</v>
+        <v>4.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.2</v>
+        <v>11.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -73420,7 +73942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -78649,13 +79171,13 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>20.4</v>
+        <v>21.9</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>35</v>
+        <v>32.3</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
@@ -78663,10 +79185,10 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>71.40000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>3.4</v>
+        <v>0.9</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -78678,13 +79200,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>60.8</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -78692,10 +79214,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>74.09999999999999</v>
+        <v>59</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>3.1</v>
+        <v>4.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -78707,13 +79229,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>15.7</v>
+        <v>14.9</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>4.6</v>
+        <v>5.7</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -78721,10 +79243,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>30.7</v>
+        <v>27.8</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -78736,13 +79258,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>15</v>
+        <v>14.4</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -78750,10 +79272,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>11.5</v>
+        <v>1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.6</v>
+        <v>11.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -78765,13 +79287,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>14.8</v>
+        <v>15.7</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -78779,10 +79301,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>63.1</v>
+        <v>53.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>4.4</v>
+        <v>5.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -78794,13 +79316,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>15.3</v>
+        <v>17.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.5</v>
+        <v>2.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -78808,13 +79330,42 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>20.7</v>
+        <v>2.4</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>9.5</v>
+        <v>11.7</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>
@@ -78835,7 +79386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H186"/>
+  <dimension ref="A1:H187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84064,24 +84615,24 @@
         <v>46275</v>
       </c>
       <c r="B181" s="4" t="n">
-        <v>10.4</v>
+        <v>10.8</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>3.5</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>95.5</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="H181" s="10">
         <f>SUM(C175:C181)</f>
@@ -84096,10 +84647,10 @@
         <v>11.5</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>0.2</v>
+        <v>2.1</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -84107,10 +84658,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>70.8</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -84122,24 +84673,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>19.5</v>
+        <v>24.9</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -84151,24 +84702,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>13.4</v>
+        <v>12.5</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>62.7</v>
+        <v>26.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>4.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -84180,13 +84731,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>14.2</v>
+        <v>15.9</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -84194,10 +84745,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>76.59999999999999</v>
+        <v>26.8</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>2.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -84209,27 +84760,56 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>15.1</v>
+        <v>17.1</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>19.5</v>
+        <v>1.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>11.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B187" s="4" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H187" s="10">
+        <f>SUM(C181:C187)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-11 10:12 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5771,13 +5771,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>28.2</v>
+        <v>29.5</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -5785,10 +5785,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0.4</v>
+        <v>2.1</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -5800,13 +5800,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>28.3</v>
+        <v>28.6</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -5814,10 +5814,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>8.5</v>
+        <v>6.6</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -5829,13 +5829,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>27.4</v>
+        <v>27</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.4</v>
+        <v>3.2</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.5</v>
+        <v>3.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -5843,10 +5843,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>10.6</v>
+        <v>16.5</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.7</v>
+        <v>10</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -5858,13 +5858,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>24.6</v>
+        <v>24.4</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>5.3</v>
+        <v>2.9</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>11.7</v>
+        <v>29.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.6</v>
+        <v>8.5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -5887,24 +5887,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>23.9</v>
+        <v>23.2</v>
       </c>
       <c r="C186" s="7" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D186" s="7" t="n">
         <v>1.4</v>
       </c>
-      <c r="D186" s="7" t="n">
-        <v>1.3</v>
-      </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>28.7</v>
+        <v>59.4</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8.6</v>
+        <v>4.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -5916,10 +5916,10 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>24.6</v>
+        <v>23.6</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="D187" s="4" t="n">
         <v>1.7</v>
@@ -5930,13 +5930,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>6.5</v>
+        <v>11.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.2</v>
+        <v>10.6</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -5957,7 +5986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11215,21 +11244,21 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>19.6</v>
+        <v>21.9</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G182" s="7" t="n">
         <v>12</v>
@@ -11244,7 +11273,7 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>19.5</v>
+        <v>19.7</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
@@ -11258,10 +11287,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>5.3</v>
+        <v>2.8</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -11273,13 +11302,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>20.6</v>
+        <v>21</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -11287,10 +11316,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -11302,24 +11331,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>21.9</v>
+        <v>22.2</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>20.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9.5</v>
+        <v>11</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -11331,24 +11360,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>23.7</v>
+        <v>24.8</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>7.2</v>
+        <v>18.6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -11360,13 +11389,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.5</v>
+        <v>23.8</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -11374,13 +11403,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>3.3</v>
+        <v>12.5</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.6</v>
+        <v>10.5</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -11401,7 +11459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16659,21 +16717,21 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>24.2</v>
+        <v>24.5</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G182" s="7" t="n">
         <v>12</v>
@@ -16688,13 +16746,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -16717,21 +16775,21 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>24.6</v>
+        <v>24.5</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.9</v>
+        <v>6.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G184" s="7" t="n">
         <v>12</v>
@@ -16746,24 +16804,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.7</v>
+        <v>23.9</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3.3</v>
+        <v>7.7</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>0.6</v>
+        <v>7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11.9</v>
+        <v>11.2</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -16775,13 +16833,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.5</v>
+        <v>22.8</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>6.1</v>
+        <v>8.4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -16789,10 +16847,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>6.6</v>
+        <v>38.5</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.2</v>
+        <v>7.4</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -16804,13 +16862,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>6.9</v>
+        <v>9.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -16818,13 +16876,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -16845,7 +16932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22103,24 +22190,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>20.6</v>
+        <v>22.9</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>41.9</v>
+        <v>43.1</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -22132,24 +22219,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>22.1</v>
+        <v>22.6</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -22161,13 +22248,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>21.4</v>
+        <v>22.9</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -22175,10 +22262,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>39.2</v>
+        <v>26.3</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>7.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -22190,7 +22277,7 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>22.1</v>
+        <v>22.9</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
@@ -22204,10 +22291,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>58.2</v>
+        <v>27.7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -22219,10 +22306,10 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.9</v>
+        <v>22.6</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>1.2</v>
@@ -22233,10 +22320,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>55.8</v>
+        <v>8.6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>5.3</v>
+        <v>11</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -22248,27 +22335,56 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>49.4</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>6.1</v>
+        <v>3.7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -22289,7 +22405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27547,24 +27663,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>30.3</v>
+        <v>26.3</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -27576,7 +27692,7 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
@@ -27590,10 +27706,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>10.7</v>
+        <v>10.3</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -27605,13 +27721,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -27619,10 +27735,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -27634,13 +27750,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>11.7</v>
+        <v>11.4</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.3</v>
+        <v>2.1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -27648,10 +27764,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>53.3</v>
+        <v>27.1</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>5.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -27663,24 +27779,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>13.8</v>
+        <v>12.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>0</v>
+        <v>12.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>12</v>
+        <v>10.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -27692,27 +27808,56 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>10.6</v>
+        <v>11.4</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>6</v>
+        <v>38.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.3</v>
+        <v>7.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -27733,7 +27878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29482,24 +29627,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.8</v>
+        <v>14.3</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>17.7</v>
+        <v>5.8</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>93.90000000000001</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.7</v>
+        <v>2.4</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -29511,24 +29656,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>63.6</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>4.4</v>
+        <v>1.3</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -29540,24 +29685,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>3.9</v>
+        <v>46.1</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>11.5</v>
+        <v>6.5</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -29569,24 +29714,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.1</v>
+        <v>11.9</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0.3</v>
+        <v>3.5</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>46.1</v>
+        <v>82</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>6.5</v>
+        <v>2.2</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -29598,24 +29743,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>15</v>
+        <v>13.5</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>45.1</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>6.6</v>
+        <v>3.9</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -29627,13 +29772,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>6.9</v>
+        <v>10.3</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -29641,13 +29786,42 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>21.1</v>
+        <v>78.3</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>9.5</v>
+        <v>2.6</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H67" s="10">
+        <f>SUM(C61:C67)</f>
         <v/>
       </c>
     </row>
@@ -29668,7 +29842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31417,24 +31591,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>12.2</v>
+        <v>11.4</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>32.9</v>
+        <v>3.9</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -31446,24 +31620,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.3</v>
+        <v>11</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>56.4</v>
+        <v>39.6</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.2</v>
+        <v>7.2</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -31475,24 +31649,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12</v>
+        <v>12.8</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>24</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>9.1</v>
+        <v>2.8</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -31504,24 +31678,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.5</v>
+        <v>13.3</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0.3</v>
+        <v>6.1</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>86.90000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -31533,13 +31707,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14</v>
+        <v>13.8</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.1</v>
+        <v>2.5</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -31547,10 +31721,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>41.2</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -31562,13 +31736,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.3</v>
+        <v>12.9</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>3.2</v>
+        <v>12.5</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -31576,13 +31750,42 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>28.7</v>
+        <v>75</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>8.6</v>
+        <v>3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H67" s="10">
+        <f>SUM(C61:C67)</f>
         <v/>
       </c>
     </row>
@@ -31603,7 +31806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33352,24 +33555,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.3</v>
+        <v>12.2</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>36.3</v>
+        <v>9</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>99.09999999999999</v>
+        <v>97.5</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -33381,24 +33584,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.5</v>
+        <v>10.8</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>33.4</v>
+        <v>34.7</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -33413,21 +33616,21 @@
         <v>12.8</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>55.2</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>12</v>
+        <v>5.4</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -33439,13 +33642,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.8</v>
+        <v>13.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>1.3</v>
+        <v>3.3</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -33453,10 +33656,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>76.3</v>
+        <v>69.3</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.8</v>
+        <v>3.7</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -33468,24 +33671,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>15.8</v>
+        <v>14.5</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>22.3</v>
+        <v>49.6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>6</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -33497,27 +33700,56 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>17.2</v>
+        <v>13.6</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>1.1</v>
+        <v>2.1</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>3.1</v>
+        <v>2.3</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>38.3</v>
+        <v>66.2</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>7.4</v>
+        <v>4.1</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="H67" s="10">
+        <f>SUM(C61:C67)</f>
         <v/>
       </c>
     </row>
@@ -33538,7 +33770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35287,24 +35519,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>12.6</v>
+        <v>12.2</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>30.8</v>
+        <v>6.3</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>94.2</v>
+        <v>89.8</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -35319,21 +35551,21 @@
         <v>10.8</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>4.7</v>
+        <v>6.7</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>65.90000000000001</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -35345,13 +35577,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.4</v>
+        <v>12.9</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -35359,10 +35591,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>2.5</v>
+        <v>45</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>11.7</v>
+        <v>6.6</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -35374,24 +35606,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.4</v>
+        <v>11.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0.1</v>
+        <v>4.2</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>67.40000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.9</v>
+        <v>2.6</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -35403,13 +35635,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>15</v>
+        <v>13.7</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -35417,10 +35649,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>36.7</v>
+        <v>62.5</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>7.6</v>
+        <v>4.5</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -35432,13 +35664,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>16.3</v>
+        <v>13.5</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>1.8</v>
+        <v>15.3</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -35446,13 +35678,42 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>21.7</v>
+        <v>81</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>9.4</v>
+        <v>2.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H67" s="10">
+        <f>SUM(C61:C67)</f>
         <v/>
       </c>
     </row>
@@ -35473,7 +35734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37222,24 +37483,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>13.8</v>
+        <v>13</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>23.4</v>
+        <v>3</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>95.40000000000001</v>
+        <v>97.3</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -37251,10 +37512,10 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.6</v>
+        <v>11.8</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
         <v>2.7</v>
@@ -37265,10 +37526,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>55</v>
+        <v>40.9</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.4</v>
+        <v>7.1</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -37280,24 +37541,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.7</v>
+        <v>12.9</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0.9</v>
+        <v>1.8</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>1.9</v>
+        <v>52.9</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>11.8</v>
+        <v>5.7</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -37309,24 +37570,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>15.1</v>
+        <v>13.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="D64" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>71.3</v>
+        <v>73.2</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -37338,13 +37599,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>16</v>
+        <v>13.4</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -37352,10 +37613,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>23.6</v>
+        <v>61.7</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>4.6</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -37367,27 +37628,56 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>17.1</v>
+        <v>14.1</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>39.8</v>
+        <v>70.7</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>7.2</v>
+        <v>3.5</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H67" s="10">
+        <f>SUM(C61:C67)</f>
         <v/>
       </c>
     </row>
@@ -37408,7 +37698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39157,24 +39447,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>28.9</v>
+        <v>7.7</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>100</v>
+        <v>99.5</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -39186,13 +39476,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -39200,10 +39490,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>51.1</v>
+        <v>53.5</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -39215,24 +39505,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>11.9</v>
+        <v>5.4</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -39244,13 +39534,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>10.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0.7</v>
+        <v>6</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -39258,10 +39548,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>71.7</v>
+        <v>79.5</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.4</v>
+        <v>2.5</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -39273,24 +39563,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>11.8</v>
+        <v>10.7</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>26.9</v>
+        <v>89</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -39302,13 +39592,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>12.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -39316,13 +39606,42 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>47.5</v>
+        <v>73.7</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>6.3</v>
+        <v>3.2</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H67" s="10">
+        <f>SUM(C61:C67)</f>
         <v/>
       </c>
     </row>
@@ -39343,7 +39662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44601,24 +44920,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>20</v>
+        <v>21.9</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>4.7</v>
+        <v>2.3</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>67.90000000000001</v>
+        <v>56.2</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>3.9</v>
+        <v>5.3</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -44630,13 +44949,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>19.3</v>
+        <v>20.1</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -44644,10 +44963,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>22.1</v>
+        <v>39</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -44659,24 +44978,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>19.4</v>
+        <v>20.4</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>51.7</v>
+        <v>66.8</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>5.8</v>
+        <v>4</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -44688,13 +45007,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -44702,10 +45021,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>25</v>
+        <v>49.6</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -44717,13 +45036,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.8</v>
+        <v>21.5</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -44731,10 +45050,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>20.3</v>
+        <v>37.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>9.6</v>
+        <v>7.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -44746,27 +45065,56 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.9</v>
+        <v>21.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>57.8</v>
+        <v>81</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>5.1</v>
+        <v>2.3</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -44787,7 +45135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46536,24 +46884,24 @@
         <v>46276</v>
       </c>
       <c r="B61" s="4" t="n">
-        <v>9.9</v>
+        <v>10.3</v>
       </c>
       <c r="C61" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>83.90000000000001</v>
+        <v>58.1</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>1.9</v>
+        <v>5</v>
       </c>
       <c r="H61" s="10">
         <f>SUM(C55:C61)</f>
@@ -46565,24 +46913,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>37.6</v>
+        <v>47.1</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>7.5</v>
+        <v>6.3</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -46594,24 +46942,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.7</v>
+        <v>12.4</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.3</v>
+        <v>7.2</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>61.7</v>
+        <v>93.7</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4.6</v>
+        <v>0.8</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -46623,24 +46971,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.2</v>
+        <v>13.9</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>2.7</v>
+        <v>1.9</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>65.40000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>4.2</v>
+        <v>2.6</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -46652,13 +47000,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.1</v>
+        <v>13.5</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -46666,10 +47014,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>41</v>
+        <v>52.5</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>7.1</v>
+        <v>5.7</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -46681,27 +47029,56 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.2</v>
+        <v>12.5</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>3.7</v>
+        <v>1.9</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>18.4</v>
+        <v>59.2</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>4.9</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H67" s="10">
+        <f>SUM(C61:C67)</f>
         <v/>
       </c>
     </row>
@@ -46722,7 +47099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51980,24 +52357,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>27</v>
+        <v>27.7</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>11.4</v>
+        <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>4.6</v>
+        <v>3</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>24.4</v>
+        <v>28.1</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -52009,24 +52386,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>26.4</v>
+        <v>25.9</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>3</v>
+        <v>12.2</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>5.6</v>
+        <v>2.9</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>61.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>4.6</v>
+        <v>2.7</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -52038,24 +52415,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>26.1</v>
+        <v>26.4</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>4.9</v>
+        <v>5.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>17.9</v>
+        <v>22.1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -52067,24 +52444,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>25.9</v>
+        <v>26.3</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>53.5</v>
+        <v>31.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>5.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -52096,24 +52473,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>26.1</v>
+        <v>26</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>32.4</v>
+        <v>9.4</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8.1</v>
+        <v>10.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -52125,27 +52502,56 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>25.7</v>
+        <v>25.4</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -52166,7 +52572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -57424,13 +57830,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.7</v>
+        <v>19.4</v>
       </c>
       <c r="C182" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -57438,10 +57844,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -57453,13 +57859,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.5</v>
+        <v>16.7</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -57467,7 +57873,7 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="G183" s="4" t="n">
         <v>9.9</v>
@@ -57482,13 +57888,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>17.8</v>
+        <v>18.4</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.4</v>
+        <v>3.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -57496,10 +57902,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1.4</v>
+        <v>4.1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.8</v>
+        <v>11.5</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -57511,13 +57917,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>18.8</v>
+        <v>19.9</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -57525,10 +57931,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>36.1</v>
+        <v>13.7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7.7</v>
+        <v>10.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -57540,13 +57946,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>19.8</v>
+        <v>22.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -57554,10 +57960,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>9.9</v>
+        <v>5.9</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.8</v>
+        <v>11.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -57569,13 +57975,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>17.9</v>
+        <v>19.8</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -57583,13 +57989,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>12</v>
+        <v>11.2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -57610,7 +58045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62868,13 +63303,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>10.8</v>
+        <v>11.4</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>14.1</v>
+        <v>0.5</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -62882,10 +63317,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>82.09999999999999</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -62897,13 +63332,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>11.5</v>
+        <v>11.2</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>20.3</v>
+        <v>15.9</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -62911,10 +63346,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>91</v>
+        <v>88.7</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -62932,18 +63367,18 @@
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>94.09999999999999</v>
+        <v>52.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>0.7</v>
+        <v>5.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -62955,10 +63390,10 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>11.4</v>
+        <v>11.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>3.8</v>
+        <v>1.9</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>0.6</v>
@@ -62969,10 +63404,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>99.8</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -62984,10 +63419,10 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>12.5</v>
+        <v>12.2</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>14.3</v>
+        <v>17.5</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>1.2</v>
@@ -62998,10 +63433,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>97.8</v>
+        <v>96.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -63013,10 +63448,10 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>5.2</v>
+        <v>6.2</v>
       </c>
       <c r="D187" s="4" t="n">
         <v>1.7</v>
@@ -63027,13 +63462,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>83.09999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -63054,7 +63518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68312,13 +68776,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>16.9</v>
+        <v>17.4</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>37.4</v>
+        <v>0.4</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -68326,10 +68790,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>88.59999999999999</v>
+        <v>84.7</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -68341,13 +68805,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>17.8</v>
+        <v>17.2</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>4.6</v>
+        <v>3.8</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -68355,10 +68819,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -68370,7 +68834,7 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>17.2</v>
+        <v>17.5</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
@@ -68384,10 +68848,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>15.6</v>
+        <v>25</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -68399,24 +68863,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>33.6</v>
+        <v>44.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8</v>
+        <v>6.7</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -68434,7 +68898,7 @@
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -68442,10 +68906,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -68457,13 +68921,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>18.8</v>
+        <v>17</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>9</v>
+        <v>11.5</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -68471,13 +68935,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>34.5</v>
+        <v>46.5</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>7.9</v>
+        <v>6.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -68498,7 +68991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -73756,13 +74249,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>18.4</v>
+        <v>18.8</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>31.6</v>
+        <v>6.1</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -73770,10 +74263,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>90.40000000000001</v>
+        <v>95</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -73785,13 +74278,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.9</v>
+        <v>2.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -73799,7 +74292,7 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>16.1</v>
+        <v>15.8</v>
       </c>
       <c r="G183" s="4" t="n">
         <v>10.1</v>
@@ -73814,24 +74307,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>25.6</v>
+        <v>21.7</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -73843,13 +74336,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -73857,10 +74350,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>41</v>
+        <v>58.4</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7.1</v>
+        <v>5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -73872,13 +74365,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21</v>
+        <v>21.1</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -73886,10 +74379,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>4.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.5</v>
+        <v>11</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -73901,13 +74394,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.2</v>
+        <v>19.4</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>17</v>
+        <v>10.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -73915,13 +74408,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>18.4</v>
+        <v>55.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>5.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -73942,7 +74464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -79200,24 +79722,24 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>17.6</v>
+        <v>17.2</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>70.90000000000001</v>
+        <v>2.8</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3.1</v>
+        <v>3.7</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>59</v>
+        <v>54.2</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>4.9</v>
+        <v>5.5</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -79229,13 +79751,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>5.7</v>
+        <v>5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -79243,10 +79765,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>27.8</v>
+        <v>25.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -79258,13 +79780,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>14.4</v>
+        <v>15.3</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -79272,10 +79794,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1</v>
+        <v>10.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.9</v>
+        <v>10.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -79287,13 +79809,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>15.7</v>
+        <v>16.4</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -79301,10 +79823,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>53.5</v>
+        <v>63.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>5.6</v>
+        <v>4.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -79316,13 +79838,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -79330,10 +79852,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>2.4</v>
+        <v>12.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.7</v>
+        <v>10.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -79345,27 +79867,56 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>18.8</v>
+        <v>17.5</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.5</v>
+        <v>4.1</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>0.4</v>
+        <v>46.9</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>12</v>
+        <v>6.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>
@@ -79386,7 +79937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84644,13 +85195,13 @@
         <v>46276</v>
       </c>
       <c r="B182" s="7" t="n">
-        <v>11.5</v>
+        <v>12.6</v>
       </c>
       <c r="C182" s="7" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
@@ -84658,10 +85209,10 @@
         </is>
       </c>
       <c r="F182" s="7" t="n">
-        <v>74.90000000000001</v>
+        <v>38.7</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>3</v>
+        <v>7.4</v>
       </c>
       <c r="H182" s="12">
         <f>SUM(C176:C182)</f>
@@ -84673,7 +85224,7 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>11.7</v>
+        <v>12.1</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
@@ -84683,14 +85234,14 @@
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>24.9</v>
+        <v>35.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9</v>
+        <v>7.8</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -84702,24 +85253,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>12.5</v>
+        <v>14.1</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>26.9</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>3.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -84731,24 +85282,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>15.9</v>
+        <v>14.7</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>26.8</v>
+        <v>50.6</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>5.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -84760,24 +85311,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>17.1</v>
+        <v>15.2</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>1.2</v>
+        <v>14.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.9</v>
+        <v>10.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -84789,13 +85340,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.3</v>
+        <v>12.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>4.3</v>
+        <v>5.4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -84803,13 +85354,42 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>60.1</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>4.8</v>
+        <v>1.7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="11" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="C188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H188" s="12">
+        <f>SUM(C182:C188)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-12 09:46 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5800,24 +5800,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>28.6</v>
+        <v>29.2</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="D183" s="4" t="n">
         <v>3.3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>6.6</v>
+        <v>12.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.2</v>
+        <v>10.5</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -5829,13 +5829,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>27</v>
+        <v>26.7</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -5843,10 +5843,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>16.5</v>
+        <v>14</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -5858,24 +5858,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>24.4</v>
+        <v>23.9</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>2.9</v>
+        <v>12.9</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.9</v>
+        <v>3.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>29.5</v>
+        <v>63.4</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.5</v>
+        <v>4.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -5887,24 +5887,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>23.2</v>
+        <v>24.3</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>6.7</v>
+        <v>0.3</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>59.4</v>
+        <v>29.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>4.9</v>
+        <v>8.4</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -5916,13 +5916,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>23.6</v>
+        <v>24</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -5930,10 +5930,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>11.6</v>
+        <v>9.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>10.6</v>
+        <v>10.8</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -5945,13 +5945,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>24.2</v>
+        <v>24.8</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -5959,13 +5959,42 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>8.4</v>
+        <v>3.7</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11</v>
+        <v>11.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -5986,7 +6015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11273,24 +11302,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>19.7</v>
+        <v>22.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -11302,7 +11331,7 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>21</v>
+        <v>21.5</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
@@ -11316,7 +11345,7 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G184" s="7" t="n">
         <v>11.9</v>
@@ -11331,13 +11360,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>22.2</v>
+        <v>23.6</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -11345,10 +11374,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>18.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -11360,13 +11389,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>24.8</v>
+        <v>24.5</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -11374,10 +11403,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>18.6</v>
+        <v>0</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>12</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -11389,24 +11418,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>23.8</v>
+        <v>21.5</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>12.5</v>
+        <v>7.4</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>10.5</v>
+        <v>11.1</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -11418,27 +11447,56 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22</v>
+        <v>17.7</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>3.7</v>
+        <v>57.4</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.6</v>
+        <v>5.1</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -11459,7 +11517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16746,21 +16804,21 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>24.4</v>
+        <v>24.7</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G183" s="4" t="n">
         <v>12</v>
@@ -16781,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -16789,10 +16847,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>0.1</v>
+        <v>6.3</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>12</v>
+        <v>11.2</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -16804,13 +16862,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.9</v>
+        <v>23.6</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>7.7</v>
+        <v>8.9</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -16818,10 +16876,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>7</v>
+        <v>11.8</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11.2</v>
+        <v>10.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -16839,7 +16897,7 @@
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>8.4</v>
+        <v>9.1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -16847,10 +16905,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>38.5</v>
+        <v>27.9</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>7.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -16862,13 +16920,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -16891,13 +16949,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22.8</v>
+        <v>23</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -16905,13 +16963,42 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -16932,7 +17019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22219,7 +22306,7 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>22.6</v>
+        <v>24.8</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
@@ -22229,14 +22316,14 @@
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>5.4</v>
+        <v>22.5</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>11.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -22248,13 +22335,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>22.9</v>
+        <v>23.3</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -22262,10 +22349,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>26.3</v>
+        <v>43.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>6.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -22277,13 +22364,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>22.9</v>
+        <v>23.5</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.4</v>
+        <v>2.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -22291,10 +22378,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>27.7</v>
+        <v>19.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -22306,13 +22393,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.6</v>
+        <v>23.1</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -22320,10 +22407,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>8.6</v>
+        <v>11.5</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -22338,10 +22425,10 @@
         <v>22.5</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -22349,10 +22436,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>69.09999999999999</v>
+        <v>42</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>3.7</v>
+        <v>7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -22364,27 +22451,56 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22.6</v>
+        <v>22.9</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>68.2</v>
+        <v>53.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>3.8</v>
+        <v>5.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -22405,7 +22521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27692,24 +27808,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>9.9</v>
+        <v>13</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>14</v>
+        <v>22.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>10.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -27721,24 +27837,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>31</v>
+        <v>32.4</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -27750,24 +27866,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>11.4</v>
+        <v>12.9</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>27.1</v>
+        <v>11.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -27779,13 +27895,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>12.4</v>
+        <v>13.1</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -27793,10 +27909,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>12.3</v>
+        <v>2.9</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.5</v>
+        <v>11.7</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -27808,24 +27924,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>11.4</v>
+        <v>12.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>38.1</v>
+        <v>23.2</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>7.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -27837,17 +27953,17 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
@@ -27858,6 +27974,35 @@
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -27878,7 +28023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29656,24 +29801,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>12.4</v>
+        <v>12.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>89.09999999999999</v>
+        <v>58.5</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>1.3</v>
+        <v>5</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -29685,24 +29830,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>46.1</v>
+        <v>56.1</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>6.5</v>
+        <v>5.3</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -29714,24 +29859,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>11.9</v>
+        <v>13.9</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>3.5</v>
+        <v>0.6</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>82</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -29743,24 +29888,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.5</v>
+        <v>13.8</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>67.40000000000001</v>
+        <v>64</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>3.9</v>
+        <v>4.3</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -29772,24 +29917,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.4</v>
+        <v>14.9</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>10.3</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
         <v>1.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>78.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>2.6</v>
+        <v>11</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -29801,27 +29946,56 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>11.8</v>
+        <v>13.4</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.3</v>
+        <v>5.8</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>34.4</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>7.9</v>
+        <v>3.5</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(C62:C68)</f>
         <v/>
       </c>
     </row>
@@ -29842,7 +30016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31620,24 +31794,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11</v>
+        <v>12.3</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>39.6</v>
+        <v>53.3</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>7.2</v>
+        <v>5.6</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -31649,13 +31823,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.8</v>
+        <v>13.1</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -31663,10 +31837,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>76.40000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>2.8</v>
+        <v>3.5</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -31678,13 +31852,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.3</v>
+        <v>14.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>6.1</v>
+        <v>8.6</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -31692,10 +31866,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>89.7</v>
+        <v>79.3</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -31707,13 +31881,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.8</v>
+        <v>12.9</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -31721,10 +31895,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>71.90000000000001</v>
+        <v>51</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>3.4</v>
+        <v>5.9</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -31736,24 +31910,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>12.9</v>
+        <v>14.3</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>12.5</v>
+        <v>6.5</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>75</v>
+        <v>44.9</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>3</v>
+        <v>6.6</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -31765,27 +31939,56 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>11.1</v>
+        <v>13.9</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.9</v>
+        <v>4.2</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(C62:C68)</f>
         <v/>
       </c>
     </row>
@@ -31806,7 +32009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33584,21 +33787,21 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>34.7</v>
+        <v>35.1</v>
       </c>
       <c r="G62" s="7" t="n">
         <v>7.8</v>
@@ -33613,10 +33816,10 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>2</v>
@@ -33627,10 +33830,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>55.2</v>
+        <v>60.2</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -33642,13 +33845,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.1</v>
+        <v>14.2</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>3.3</v>
+        <v>6.9</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -33656,10 +33859,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>69.3</v>
+        <v>77</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.7</v>
+        <v>2.8</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -33671,10 +33874,10 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.5</v>
+        <v>13.8</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>1.8</v>
@@ -33685,10 +33888,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>49.6</v>
+        <v>13.7</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>6</v>
+        <v>10.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -33700,24 +33903,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>13.6</v>
+        <v>15.3</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>2.1</v>
+        <v>0.6</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>66.2</v>
+        <v>39.5</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>4.1</v>
+        <v>7.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -33729,27 +33932,56 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>11.4</v>
+        <v>13.7</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0</v>
+        <v>12.3</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>52.1</v>
+        <v>71.5</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>5.7</v>
+        <v>3.4</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(C62:C68)</f>
         <v/>
       </c>
     </row>
@@ -33770,7 +34002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35548,13 +35780,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>10.8</v>
+        <v>11.5</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>6.7</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -35562,10 +35794,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>79.90000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2.4</v>
+        <v>3.4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -35577,24 +35809,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.9</v>
+        <v>12.4</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>45</v>
+        <v>60.6</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>6.6</v>
+        <v>4.7</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -35606,13 +35838,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>11.8</v>
+        <v>13.7</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -35620,10 +35852,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>78.09999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -35635,24 +35867,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>62.5</v>
+        <v>49.2</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -35664,13 +35896,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>13.5</v>
+        <v>14.2</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>15.3</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -35678,10 +35910,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>81</v>
+        <v>6.2</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>2.3</v>
+        <v>11.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -35693,27 +35925,56 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>11.2</v>
+        <v>12.4</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>29.9</v>
+        <v>63.5</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>8.4</v>
+        <v>4.4</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(C62:C68)</f>
         <v/>
       </c>
     </row>
@@ -35734,7 +35995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37512,24 +37773,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.8</v>
+        <v>12.9</v>
       </c>
       <c r="C62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>40.9</v>
+        <v>30.4</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>7.1</v>
+        <v>8.4</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -37541,7 +37802,7 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.9</v>
+        <v>13.2</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
@@ -37555,10 +37816,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>52.9</v>
+        <v>59.1</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>5.7</v>
+        <v>4.9</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -37570,24 +37831,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.1</v>
+        <v>13.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>2.1</v>
+        <v>5.4</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>73.2</v>
+        <v>79.5</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -37599,24 +37860,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.4</v>
+        <v>13.1</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>61.7</v>
+        <v>23.6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>4.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -37628,24 +37889,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.1</v>
+        <v>15.3</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>70.7</v>
+        <v>18.9</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>3.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -37657,27 +37918,56 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>11.6</v>
+        <v>14.5</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>37.1</v>
+        <v>75</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(C62:C68)</f>
         <v/>
       </c>
     </row>
@@ -37698,7 +37988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39476,24 +39766,24 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
         <v>2.6</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>53.5</v>
+        <v>36.6</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>5.6</v>
+        <v>7.6</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -39508,10 +39798,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>2.6</v>
+        <v>0.8</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -39519,10 +39809,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>55</v>
+        <v>55.8</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -39534,13 +39824,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>10.6</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>6</v>
+        <v>5.2</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -39548,10 +39838,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>79.5</v>
+        <v>81</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -39563,13 +39853,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>10.7</v>
+        <v>10.2</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -39577,10 +39867,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>89</v>
+        <v>56.6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>1.3</v>
+        <v>5.2</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -39592,24 +39882,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>11.7</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>4.3</v>
+        <v>0.1</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>73.7</v>
+        <v>10.3</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>3.2</v>
+        <v>10.8</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -39621,27 +39911,56 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>7.7</v>
+        <v>9.9</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0</v>
+        <v>12.3</v>
       </c>
       <c r="D67" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>72</v>
+        <v>73.8</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(C62:C68)</f>
         <v/>
       </c>
     </row>
@@ -39662,7 +39981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44949,24 +45268,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>20.1</v>
+        <v>21.7</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>39</v>
+        <v>25.5</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>7.3</v>
+        <v>8.9</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -44981,10 +45300,10 @@
         <v>20.4</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -44992,10 +45311,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>66.8</v>
+        <v>73.3</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -45007,13 +45326,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>21.2</v>
+        <v>21.8</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -45021,10 +45340,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>49.6</v>
+        <v>30.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>6</v>
+        <v>8.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -45036,24 +45355,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>37.7</v>
+        <v>35.5</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -45068,21 +45387,21 @@
         <v>21.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>81</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>2.3</v>
+        <v>3.3</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -45094,27 +45413,56 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20.1</v>
+        <v>20.7</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>60</v>
+        <v>51.6</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -45135,7 +45483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46913,13 +47261,13 @@
         <v>46277</v>
       </c>
       <c r="B62" s="7" t="n">
-        <v>11.7</v>
+        <v>13.7</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>4.1</v>
+        <v>1.3</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
@@ -46927,10 +47275,10 @@
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>47.1</v>
+        <v>44</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>6.3</v>
+        <v>6.7</v>
       </c>
       <c r="H62" s="12">
         <f>SUM(C56:C62)</f>
@@ -46942,13 +47290,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.4</v>
+        <v>12.7</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>7.2</v>
+        <v>12.6</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -46956,10 +47304,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>93.7</v>
+        <v>95.5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -46971,24 +47319,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.9</v>
+        <v>13.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>2.2</v>
+        <v>3.1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>78.09999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -47000,24 +47348,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.5</v>
+        <v>11.9</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2.7</v>
+        <v>0.3</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>52.5</v>
+        <v>54.9</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -47029,24 +47377,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>12.5</v>
+        <v>14.8</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>1</v>
+        <v>2.6</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>59.2</v>
+        <v>53.5</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>4.9</v>
+        <v>5.6</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -47058,13 +47406,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>11.8</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -47072,13 +47420,42 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>47.1</v>
+        <v>54.3</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(C62:C68)</f>
         <v/>
       </c>
     </row>
@@ -47099,7 +47476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -52386,24 +52763,24 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>25.9</v>
+        <v>26.2</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>12.2</v>
+        <v>0.5</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>77.40000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -52418,21 +52795,21 @@
         <v>26.4</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>22.1</v>
+        <v>21.7</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -52444,13 +52821,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>26.3</v>
+        <v>26.7</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -52458,10 +52835,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>31.2</v>
+        <v>14.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>10.3</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -52473,13 +52850,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>26</v>
+        <v>26.2</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -52487,10 +52864,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>9.4</v>
+        <v>6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.9</v>
+        <v>11.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -52502,24 +52879,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>25.4</v>
+        <v>26.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>6.9</v>
+        <v>3.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.2</v>
+        <v>11.6</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -52531,13 +52908,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>25.8</v>
+        <v>25.7</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>4.9</v>
+        <v>1.8</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -52545,13 +52922,42 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>50.6</v>
+        <v>7.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.9</v>
+        <v>11.1</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -52572,7 +52978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -57859,13 +58265,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>16.7</v>
+        <v>19.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -57873,10 +58279,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>17.6</v>
+        <v>0.2</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9.9</v>
+        <v>12</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -57888,7 +58294,7 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
@@ -57902,10 +58308,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.5</v>
+        <v>11.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -57917,24 +58323,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>19.9</v>
+        <v>20.7</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>13.7</v>
+        <v>9.4</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.4</v>
+        <v>10.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -57946,13 +58352,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.4</v>
+        <v>21.7</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -57960,10 +58366,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>5.9</v>
+        <v>0.4</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.3</v>
+        <v>12</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -57975,13 +58381,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>19.8</v>
+        <v>18.5</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -57989,10 +58395,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>6.8</v>
+        <v>5.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -58004,13 +58410,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.8</v>
+        <v>14.3</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.7</v>
+        <v>2.6</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -58018,13 +58424,42 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>2.9</v>
+        <v>46.1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.7</v>
+        <v>6.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -58045,7 +58480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63332,13 +63767,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>15.9</v>
+        <v>12.7</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -63346,10 +63781,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>88.7</v>
+        <v>96</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -63361,7 +63796,7 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>12.4</v>
+        <v>11.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
@@ -63371,14 +63806,14 @@
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>52.9</v>
+        <v>15.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>5.7</v>
+        <v>10.1</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -63390,24 +63825,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>11.2</v>
+        <v>12.1</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>97.09999999999999</v>
+        <v>59</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>0.3</v>
+        <v>4.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -63419,24 +63854,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>12.2</v>
+        <v>12.4</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>17.5</v>
+        <v>15.9</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>96.2</v>
+        <v>99.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -63448,13 +63883,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>11.6</v>
+        <v>12.3</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -63462,10 +63897,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>87.7</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -63477,27 +63912,56 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>8.6</v>
+        <v>3.4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>99.7</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -63518,7 +63982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68805,13 +69269,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>17.2</v>
+        <v>18.6</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -68819,7 +69283,7 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>7</v>
+        <v>6.3</v>
       </c>
       <c r="G183" s="4" t="n">
         <v>11.2</v>
@@ -68834,13 +69298,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -68848,10 +69312,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>25</v>
+        <v>36.9</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -68863,24 +69327,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>19</v>
+        <v>19.3</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.2</v>
+        <v>3.8</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>44.3</v>
+        <v>43.6</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -68892,13 +69356,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -68921,13 +69385,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>17</v>
+        <v>19.5</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>11.5</v>
+        <v>0.6</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -68935,10 +69399,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>46.5</v>
+        <v>5.7</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>6.4</v>
+        <v>11.3</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -68950,13 +69414,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.9</v>
+        <v>17.3</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>36.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -68964,13 +69428,42 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>61.5</v>
+        <v>55.6</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>4.6</v>
+        <v>5.3</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -68991,7 +69484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -74278,7 +74771,7 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>18.2</v>
+        <v>20.1</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
@@ -74292,10 +74785,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>15.8</v>
+        <v>4.2</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>10.1</v>
+        <v>11.5</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -74321,10 +74814,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>21.7</v>
+        <v>35.2</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.4</v>
+        <v>7.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -74336,13 +74829,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>1.1</v>
+        <v>6.3</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -74350,10 +74843,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>58.4</v>
+        <v>49.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>5</v>
+        <v>6.1</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -74365,13 +74858,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.1</v>
+        <v>20.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -74379,10 +74872,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>1.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11</v>
+        <v>11.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -74394,24 +74887,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>19.4</v>
+        <v>21.6</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>10.2</v>
+        <v>0.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>55.1</v>
+        <v>3</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>5.4</v>
+        <v>11.6</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -74423,27 +74916,56 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>18.4</v>
+        <v>19</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>42.4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>66.8</v>
+        <v>74.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -74464,7 +74986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -79751,13 +80273,13 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>15</v>
+        <v>15.9</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
@@ -79765,10 +80287,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>25.3</v>
+        <v>1.8</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>9</v>
+        <v>11.8</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -79780,13 +80302,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -79794,10 +80316,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>10.9</v>
+        <v>11.7</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -79809,13 +80331,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>16.4</v>
+        <v>16</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -79823,10 +80345,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>63.5</v>
+        <v>59.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>4.4</v>
+        <v>4.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -79838,13 +80360,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>17.6</v>
+        <v>16.9</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -79852,10 +80374,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>12.7</v>
+        <v>5.5</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.5</v>
+        <v>11.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -79867,10 +80389,10 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>17.5</v>
+        <v>17.8</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
         <v>1.6</v>
@@ -79881,10 +80403,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>46.9</v>
+        <v>0</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>6.4</v>
+        <v>12</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -79896,27 +80418,56 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>15.4</v>
+        <v>17.5</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.3</v>
+        <v>10</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.3</v>
+        <v>1.6</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>73.40000000000001</v>
+        <v>49.6</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>
@@ -79937,7 +80488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -85224,7 +85775,7 @@
         <v>46277</v>
       </c>
       <c r="B183" s="4" t="n">
-        <v>12.1</v>
+        <v>14.3</v>
       </c>
       <c r="C183" s="4" t="n">
         <v>0</v>
@@ -85238,10 +85789,10 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>35.3</v>
+        <v>48.3</v>
       </c>
       <c r="G183" s="4" t="n">
-        <v>7.8</v>
+        <v>6.2</v>
       </c>
       <c r="H183" s="10">
         <f>SUM(C177:C183)</f>
@@ -85256,7 +85807,7 @@
         <v>14.1</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>1.1</v>
@@ -85267,10 +85818,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>67.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -85285,10 +85836,10 @@
         <v>14.7</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.1</v>
+        <v>6.3</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -85296,10 +85847,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>50.6</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>5.9</v>
+        <v>1.8</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -85311,10 +85862,10 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>15.2</v>
+        <v>14.9</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>0.7</v>
@@ -85325,10 +85876,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>14.3</v>
+        <v>25</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.3</v>
+        <v>9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -85340,24 +85891,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.1</v>
+        <v>13.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>5.4</v>
+        <v>21.8</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>85.90000000000001</v>
+        <v>63.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>1.7</v>
+        <v>4.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -85369,7 +85920,7 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>11.6</v>
+        <v>10.3</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
@@ -85383,13 +85934,42 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>45.9</v>
+        <v>40.4</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>6.5</v>
+        <v>7.2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B189" s="4" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H189" s="10">
+        <f>SUM(C183:C189)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-13 10:47 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5829,24 +5829,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>26.7</v>
+        <v>26.5</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.5</v>
+        <v>4.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>14</v>
+        <v>26.1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.3</v>
+        <v>8.9</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -5858,13 +5858,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.9</v>
+        <v>23.5</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>12.9</v>
+        <v>14.3</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>63.4</v>
+        <v>77.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>4.4</v>
+        <v>2.7</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -5887,24 +5887,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>24.3</v>
+        <v>21.8</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0.3</v>
+        <v>10.5</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.6</v>
+        <v>4.4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>29.7</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8.4</v>
+        <v>1.4</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -5916,13 +5916,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>24</v>
+        <v>23.2</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.9</v>
+        <v>4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -5930,10 +5930,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>9.6</v>
+        <v>56.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>10.8</v>
+        <v>5.2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -5945,24 +5945,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>24.8</v>
+        <v>23.2</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.5</v>
+        <v>3.4</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>3.7</v>
+        <v>21.1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.6</v>
+        <v>9.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -5974,13 +5974,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>26.1</v>
+        <v>23.8</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -5988,13 +5988,42 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>27.9</v>
+        <v>14.4</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -6015,7 +6044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11331,24 +11360,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>21.5</v>
+        <v>24.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>0.8</v>
+        <v>2.3</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -11360,7 +11389,7 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.6</v>
+        <v>23.5</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
@@ -11374,10 +11403,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>18.2</v>
+        <v>11.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>10.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -11389,13 +11418,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -11418,24 +11447,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.5</v>
+        <v>21.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>7.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.1</v>
+        <v>10.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -11447,7 +11476,7 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
@@ -11457,14 +11486,14 @@
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>57.4</v>
+        <v>50.4</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.1</v>
+        <v>6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -11476,27 +11505,56 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>18.4</v>
+        <v>17.5</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>26.4</v>
+        <v>44.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>6.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -11517,7 +11575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16833,13 +16891,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>24.5</v>
+        <v>24.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>6.2</v>
+        <v>7.6</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -16847,10 +16905,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>6.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -16862,13 +16920,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.6</v>
+        <v>23.1</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>8.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -16876,10 +16934,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>11.8</v>
+        <v>22.7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -16891,13 +16949,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.8</v>
+        <v>22.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>9.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -16905,10 +16963,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>27.9</v>
+        <v>50.6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>5.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -16920,24 +16978,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.3</v>
+        <v>21.7</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>9.4</v>
+        <v>4.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>0</v>
+        <v>60.3</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>12</v>
+        <v>4.8</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -16949,24 +17007,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>6.2</v>
+        <v>2.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>0</v>
+        <v>12.3</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>12</v>
+        <v>10.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -16978,13 +17036,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>23.6</v>
+        <v>22.7</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -16992,13 +17050,42 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>4.7</v>
+        <v>0.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -17019,7 +17106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22335,24 +22422,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>23.3</v>
+        <v>25.3</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>43.9</v>
+        <v>34.8</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>6.7</v>
+        <v>7.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -22364,24 +22451,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.5</v>
+        <v>23.7</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>19.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -22393,13 +22480,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>23.1</v>
+        <v>24</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.9</v>
+        <v>3.1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -22407,10 +22494,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>11.5</v>
+        <v>7.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -22422,13 +22509,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.5</v>
+        <v>22.7</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -22436,10 +22523,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>42</v>
+        <v>21.7</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>7</v>
+        <v>9.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -22451,24 +22538,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>53.5</v>
+        <v>71.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.6</v>
+        <v>3.4</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -22480,13 +22567,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>21.2</v>
+        <v>19.8</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -22494,13 +22581,42 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>54.9</v>
+        <v>40.4</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>5.4</v>
+        <v>7.2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -22521,7 +22637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27837,24 +27953,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>11.4</v>
+        <v>14.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>32.4</v>
+        <v>21</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>8.1</v>
+        <v>9.5</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -27872,7 +27988,7 @@
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -27880,10 +27996,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>11.3</v>
+        <v>22.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -27895,13 +28011,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>13.1</v>
+        <v>13.5</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -27909,10 +28025,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -27924,13 +28040,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.1</v>
+        <v>12.3</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.4</v>
+        <v>1.9</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -27938,10 +28054,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>23.2</v>
+        <v>29.9</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -27953,24 +28069,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>7.9</v>
+        <v>8.5</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>57.8</v>
+        <v>39</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.1</v>
+        <v>7.3</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -27982,27 +28098,56 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.6</v>
+        <v>1.9</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>31.8</v>
+        <v>46.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>6.4</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -28023,7 +28168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29830,13 +29975,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.8</v>
+        <v>14.4</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -29844,10 +29989,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>56.1</v>
+        <v>80.5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>5.3</v>
+        <v>2.3</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -29859,24 +30004,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.9</v>
+        <v>13.6</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>0.6</v>
+        <v>4.1</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>78.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -29888,24 +30033,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.8</v>
+        <v>14.7</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2</v>
+        <v>4.1</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>64</v>
+        <v>23.9</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>4.3</v>
+        <v>9.1</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -29917,24 +30062,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.9</v>
+        <v>15.5</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>4.9</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -29946,24 +30091,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13.4</v>
+        <v>16.7</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>70.90000000000001</v>
+        <v>34.5</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.5</v>
+        <v>7.9</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -29975,13 +30120,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>14.1</v>
+        <v>15.3</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -29989,13 +30134,42 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>22.9</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H69" s="10">
+        <f>SUM(C63:C69)</f>
         <v/>
       </c>
     </row>
@@ -30016,7 +30190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31823,24 +31997,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.1</v>
+        <v>15.3</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>70.8</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>3.5</v>
+        <v>1.4</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -31852,24 +32026,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.8</v>
+        <v>12.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>8.6</v>
+        <v>6.7</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.7</v>
+        <v>1</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>79.3</v>
+        <v>85.2</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -31881,24 +32055,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>12.9</v>
+        <v>14</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -31910,13 +32084,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.3</v>
+        <v>14.1</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -31924,10 +32098,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>44.9</v>
+        <v>18.8</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>6.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -31939,10 +32113,10 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13.9</v>
+        <v>14.9</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>11.5</v>
+        <v>1.6</v>
       </c>
       <c r="D67" s="4" t="n">
         <v>1.1</v>
@@ -31953,10 +32127,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>65</v>
+        <v>94.7</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.2</v>
+        <v>0.6</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -31968,13 +32142,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.3</v>
+        <v>12.9</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>15.7</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -31982,13 +32156,42 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>68.90000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H69" s="10">
+        <f>SUM(C63:C69)</f>
         <v/>
       </c>
     </row>
@@ -32009,7 +32212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33816,24 +34019,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.2</v>
+        <v>14.7</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>60.2</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4.8</v>
+        <v>1.8</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -33845,24 +34048,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>14.2</v>
+        <v>13.2</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>6.9</v>
+        <v>5.7</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>77</v>
+        <v>91.3</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -33874,24 +34077,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.8</v>
+        <v>14.5</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>1.8</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>13.7</v>
+        <v>32.6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>10.4</v>
+        <v>8.1</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -33903,13 +34106,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.3</v>
+        <v>15</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -33917,10 +34120,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>39.5</v>
+        <v>4.3</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>7.3</v>
+        <v>11.5</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -33932,24 +34135,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13.7</v>
+        <v>15.9</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>12.3</v>
+        <v>1.4</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>71.5</v>
+        <v>77.5</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -33961,27 +34164,56 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>15.9</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>72.5</v>
+        <v>85.2</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>3.3</v>
+        <v>1.8</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H69" s="10">
+        <f>SUM(C63:C69)</f>
         <v/>
       </c>
     </row>
@@ -34002,7 +34234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35809,24 +36041,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.4</v>
+        <v>14</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>1.8</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>60.6</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4.7</v>
+        <v>1.9</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -35838,24 +36070,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>5</v>
+        <v>6.7</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>81.5</v>
+        <v>67.2</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -35867,24 +36099,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.5</v>
+        <v>14.1</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.9</v>
+        <v>4.5</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>49.2</v>
+        <v>35.8</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>6.1</v>
+        <v>7.7</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -35896,24 +36128,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.2</v>
+        <v>15.2</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>6.2</v>
+        <v>7.2</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -35925,24 +36157,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.4</v>
+        <v>16.2</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>63.5</v>
+        <v>28.5</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.4</v>
+        <v>8.6</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -35954,27 +36186,56 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.9</v>
+        <v>15</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>30.9</v>
+        <v>85.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>1.8</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H69" s="10">
+        <f>SUM(C63:C69)</f>
         <v/>
       </c>
     </row>
@@ -35995,7 +36256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37802,24 +38063,24 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>13.2</v>
+        <v>15.3</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>59.1</v>
+        <v>89.8</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4.9</v>
+        <v>1.2</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -37831,13 +38092,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.8</v>
+        <v>13.2</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>5.4</v>
+        <v>1.5</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -37845,10 +38106,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>79.5</v>
+        <v>70.2</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.5</v>
+        <v>3.6</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -37860,13 +38121,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>13.1</v>
+        <v>14.4</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -37874,10 +38135,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>23.6</v>
+        <v>29.9</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -37889,7 +38150,7 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
@@ -37903,10 +38164,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>18.9</v>
+        <v>4.5</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>11.5</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -37918,24 +38179,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>14.5</v>
+        <v>16.1</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>7.8</v>
+        <v>0.2</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>75</v>
+        <v>49.2</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3</v>
+        <v>6.1</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -37947,27 +38208,56 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.6</v>
+        <v>13.9</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>11.1</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>49.4</v>
+        <v>77.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6.1</v>
+        <v>2.7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H69" s="10">
+        <f>SUM(C63:C69)</f>
         <v/>
       </c>
     </row>
@@ -37988,7 +38278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39795,10 +40085,10 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>11.1</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>1.7</v>
@@ -39809,10 +40099,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>55.8</v>
+        <v>95.8</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>5.3</v>
+        <v>0.5</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -39824,13 +40114,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>10.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>5.2</v>
+        <v>4.2</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -39838,10 +40128,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>81</v>
+        <v>95.5</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>2.3</v>
+        <v>0.5</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -39853,21 +40143,21 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>56.6</v>
+        <v>56.3</v>
       </c>
       <c r="G65" s="4" t="n">
         <v>5.2</v>
@@ -39882,13 +40172,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -39896,10 +40186,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>10.3</v>
+        <v>6.1</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>10.8</v>
+        <v>11.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -39911,24 +40201,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>9.9</v>
+        <v>12</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>12.3</v>
+        <v>3</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>73.8</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -39940,27 +40230,56 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>11</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>14.1</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>65</v>
+        <v>97.2</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>4.2</v>
+        <v>0.3</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H69" s="10">
+        <f>SUM(C63:C69)</f>
         <v/>
       </c>
     </row>
@@ -39981,7 +40300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45297,24 +45616,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>20.4</v>
+        <v>22.2</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>73.3</v>
+        <v>76.8</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -45326,13 +45645,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>21.8</v>
+        <v>22.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -45340,10 +45659,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>30.2</v>
+        <v>20.1</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.4</v>
+        <v>9.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -45355,24 +45674,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>35.5</v>
+        <v>48.8</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>7.7</v>
+        <v>6.1</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -45384,13 +45703,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -45398,10 +45717,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>72.09999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>3.3</v>
+        <v>2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -45413,13 +45732,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20.7</v>
+        <v>19.7</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.7</v>
+        <v>12.3</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -45427,10 +45746,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>51.6</v>
+        <v>81</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.8</v>
+        <v>2.3</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -45442,27 +45761,56 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>19.2</v>
+        <v>18.1</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0.7</v>
+        <v>4.5</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>51.4</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>5.8</v>
+        <v>4.2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -45483,7 +45831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47290,13 +47638,13 @@
         <v>46278</v>
       </c>
       <c r="B63" s="4" t="n">
-        <v>12.7</v>
+        <v>13.7</v>
       </c>
       <c r="C63" s="4" t="n">
-        <v>12.6</v>
+        <v>17.6</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -47304,10 +47652,10 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>95.5</v>
+        <v>87.2</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H63" s="10">
         <f>SUM(C57:C63)</f>
@@ -47322,21 +47670,21 @@
         <v>13.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>67.2</v>
+        <v>61.1</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -47348,24 +47696,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>54.9</v>
+        <v>11.5</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>5.4</v>
+        <v>10.6</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -47377,13 +47725,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.8</v>
+        <v>13.8</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -47391,10 +47739,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>53.5</v>
+        <v>58.8</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -47406,13 +47754,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>11.8</v>
+        <v>12.4</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -47420,10 +47768,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>54.3</v>
+        <v>62.3</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -47435,27 +47783,56 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>11.3</v>
+        <v>11</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>50.6</v>
+        <v>89.8</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>5.9</v>
+        <v>1.2</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H69" s="10">
+        <f>SUM(C63:C69)</f>
         <v/>
       </c>
     </row>
@@ -47476,7 +47853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -52792,13 +53169,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>26.4</v>
+        <v>26.7</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>4.8</v>
+        <v>5.2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -52806,10 +53183,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>21.7</v>
+        <v>10.8</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>9.4</v>
+        <v>10.7</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -52821,24 +53198,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>26.7</v>
+        <v>26.3</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>4.9</v>
+        <v>4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>14.3</v>
+        <v>31.7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -52850,24 +53227,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>6</v>
+        <v>11.4</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.3</v>
+        <v>10.6</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -52879,24 +53256,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>26.1</v>
+        <v>26</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>3.1</v>
+        <v>7.2</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.6</v>
+        <v>11.1</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -52908,24 +53285,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>25.7</v>
+        <v>25.1</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.2</v>
+        <v>2.2</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.8</v>
+        <v>3.7</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>7.8</v>
+        <v>19.1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -52937,13 +53314,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>25.1</v>
+        <v>25.4</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0.1</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.8</v>
+        <v>4.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -52951,13 +53328,42 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>6.8</v>
+        <v>7.6</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -52978,7 +53384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -58294,24 +58700,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>18.6</v>
+        <v>20.7</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.4</v>
+        <v>4.6</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -58323,13 +58729,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -58337,10 +58743,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>9.4</v>
+        <v>4.4</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.9</v>
+        <v>11.5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -58352,13 +58758,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.7</v>
+        <v>22</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -58366,10 +58772,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -58381,13 +58787,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>18.5</v>
+        <v>18.2</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -58395,10 +58801,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>5.1</v>
+        <v>1.9</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -58410,13 +58816,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -58424,10 +58830,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>46.1</v>
+        <v>23.4</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>6.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -58439,13 +58845,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>14.5</v>
+        <v>15.4</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -58453,13 +58859,42 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>35.6</v>
+        <v>48.6</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.7</v>
+        <v>6.2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -58480,7 +58915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63796,21 +64231,21 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>11.1</v>
+        <v>12.4</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>15.9</v>
+        <v>15.6</v>
       </c>
       <c r="G184" s="7" t="n">
         <v>10.1</v>
@@ -63825,10 +64260,10 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>12.1</v>
+        <v>12.5</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>12.2</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>1</v>
@@ -63839,10 +64274,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>59</v>
+        <v>86.8</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>4.9</v>
+        <v>1.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -63854,24 +64289,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>12.4</v>
+        <v>14</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>15.9</v>
+        <v>30.1</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>99.2</v>
+        <v>98.5</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -63883,13 +64318,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -63897,10 +64332,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>90.40000000000001</v>
+        <v>88.3</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -63912,24 +64347,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>3.4</v>
+        <v>4.6</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>96.09999999999999</v>
+        <v>93.7</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -63941,27 +64376,56 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>11.1</v>
+        <v>10.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>5</v>
+        <v>6.9</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>91.90000000000001</v>
+        <v>97.3</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -63982,7 +64446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69298,24 +69762,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>17.6</v>
+        <v>20</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>36.9</v>
+        <v>50.1</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>7.6</v>
+        <v>6</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -69327,13 +69791,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>3.8</v>
+        <v>9.1</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -69341,10 +69805,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>43.6</v>
+        <v>48.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -69356,24 +69820,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>19</v>
+        <v>18.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.3</v>
+        <v>3.4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -69385,13 +69849,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>19.5</v>
+        <v>17.5</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -69399,10 +69863,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>5.7</v>
+        <v>15.2</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.3</v>
+        <v>10.2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -69414,13 +69878,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.3</v>
+        <v>18.4</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>36.9</v>
+        <v>27.4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.7</v>
+        <v>2.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -69428,10 +69892,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>55.6</v>
+        <v>60.4</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.3</v>
+        <v>4.8</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -69443,10 +69907,10 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>16</v>
+        <v>16.4</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>6</v>
+        <v>13.4</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>2</v>
@@ -69457,13 +69921,42 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>74.40000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>3.1</v>
+        <v>2.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -69484,7 +69977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -74800,24 +75293,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>19</v>
+        <v>21.2</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>35.2</v>
+        <v>47</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>7.8</v>
+        <v>6.4</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -74829,24 +75322,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="C185" s="4" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="G185" s="4" t="n">
         <v>6.3</v>
-      </c>
-      <c r="D185" s="4" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E185" s="4" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="F185" s="4" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="G185" s="4" t="n">
-        <v>6.1</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -74858,24 +75351,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>20.4</v>
+        <v>19.6</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>1.2</v>
+        <v>6.4</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.9</v>
+        <v>11.2</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -74887,24 +75380,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.6</v>
+        <v>19.3</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>3</v>
+        <v>13.5</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.6</v>
+        <v>10.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -74916,13 +75409,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>42.4</v>
+        <v>26.8</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -74930,10 +75423,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>74.8</v>
+        <v>53.1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>3</v>
+        <v>5.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -74945,27 +75438,56 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>2.6</v>
+        <v>12.5</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>67</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -74986,7 +75508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80302,13 +80824,13 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>15.1</v>
+        <v>17.1</v>
       </c>
       <c r="C184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
@@ -80316,10 +80838,10 @@
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>11.7</v>
+        <v>10</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>10.6</v>
+        <v>10.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -80331,24 +80853,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>16</v>
+        <v>15.6</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>59.5</v>
+        <v>63.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>4.9</v>
+        <v>4.3</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -80360,13 +80882,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>16.9</v>
+        <v>15.9</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.7</v>
+        <v>4.4</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -80374,10 +80896,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>5.5</v>
+        <v>26.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -80389,13 +80911,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>17.8</v>
+        <v>15.8</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -80403,10 +80925,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -80418,13 +80940,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -80432,10 +80954,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>49.6</v>
+        <v>27</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -80447,27 +80969,56 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>16.1</v>
+        <v>15.5</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>7.2</v>
+        <v>11.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.6</v>
+        <v>2.7</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>62.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>4.5</v>
+        <v>2.8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>
@@ -80488,7 +81039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -85804,24 +86355,24 @@
         <v>46278</v>
       </c>
       <c r="B184" s="7" t="n">
-        <v>14.1</v>
+        <v>16.3</v>
       </c>
       <c r="C184" s="7" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F184" s="7" t="n">
-        <v>73.7</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="H184" s="12">
         <f>SUM(C178:C184)</f>
@@ -85833,13 +86384,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>14.7</v>
+        <v>14.4</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>6.3</v>
+        <v>8.1</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -85847,10 +86398,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>85.40000000000001</v>
+        <v>79.7</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -85862,13 +86413,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>14.9</v>
+        <v>15.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -85876,10 +86427,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>25</v>
+        <v>17.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>9</v>
+        <v>9.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -85891,13 +86442,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>13.1</v>
+        <v>13.4</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>21.8</v>
+        <v>19.1</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -85905,10 +86456,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>63.1</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>4.4</v>
+        <v>2.7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -85920,13 +86471,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -85934,10 +86485,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>40.4</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>7.2</v>
+        <v>0.2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -85952,10 +86503,10 @@
         <v>10.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -85963,13 +86514,42 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>59.4</v>
+        <v>74.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>4.9</v>
+        <v>3.1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="11" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C190" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="n">
+        <v>87.3</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H190" s="12">
+        <f>SUM(C184:C190)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-14 11:13 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5858,13 +5858,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.5</v>
+        <v>24.4</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>14.3</v>
+        <v>2.4</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3.3</v>
+        <v>4.2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>77.2</v>
+        <v>55.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>2.7</v>
+        <v>5.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -5887,24 +5887,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.8</v>
+        <v>22.4</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>10.5</v>
+        <v>6.7</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>4.4</v>
+        <v>3.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>88.40000000000001</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>1.4</v>
+        <v>2.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -5916,13 +5916,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>23.2</v>
+        <v>23.4</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>4</v>
+        <v>6.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -5930,10 +5930,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>56.6</v>
+        <v>48.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>5.2</v>
+        <v>6.2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -5945,24 +5945,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>23.2</v>
+        <v>23.6</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.4</v>
+        <v>2.9</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>21.1</v>
+        <v>1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>9.5</v>
+        <v>11.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -5974,10 +5974,10 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>23.8</v>
+        <v>23.6</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>1.8</v>
@@ -5988,10 +5988,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>14.4</v>
+        <v>39.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>10.3</v>
+        <v>7.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -6003,27 +6003,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>25.1</v>
+        <v>24.7</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1.3</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>27.9</v>
+        <v>17.6</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -6044,7 +6073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11389,13 +11418,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.5</v>
+        <v>26.4</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -11403,10 +11432,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>11.3</v>
+        <v>4.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.6</v>
+        <v>11.5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -11418,17 +11447,17 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>24.7</v>
+        <v>25</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
@@ -11447,13 +11476,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.1</v>
+        <v>20.9</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.2</v>
+        <v>3.2</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -11461,10 +11490,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -11476,13 +11505,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.5</v>
+        <v>17.1</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -11490,10 +11519,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>50.4</v>
+        <v>51.4</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -11505,21 +11534,21 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.5</v>
+        <v>17.1</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>44.5</v>
+        <v>44.1</v>
       </c>
       <c r="G189" s="4" t="n">
         <v>6.7</v>
@@ -11534,27 +11563,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>6.8</v>
+        <v>0.6</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -11575,7 +11633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16920,13 +16978,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.1</v>
+        <v>23.4</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -16934,10 +16992,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>22.7</v>
+        <v>18.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -16949,13 +17007,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -16963,10 +17021,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>50.6</v>
+        <v>46.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -16978,13 +17036,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.7</v>
+        <v>22.5</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -16992,10 +17050,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>60.3</v>
+        <v>61.9</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -17007,13 +17065,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22</v>
+        <v>22.6</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.2</v>
+        <v>5.6</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -17021,10 +17079,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>12.3</v>
+        <v>3.1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>10.5</v>
+        <v>11.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -17036,13 +17094,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>22.7</v>
+        <v>22.2</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3.8</v>
+        <v>5.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -17050,7 +17108,7 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G189" s="4" t="n">
         <v>12</v>
@@ -17071,21 +17129,50 @@
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>3.6</v>
+        <v>5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -17106,7 +17193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22451,10 +22538,10 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>23.7</v>
+        <v>25</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>2.2</v>
+        <v>0.4</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>2.6</v>
@@ -22465,10 +22552,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>10.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -22494,10 +22581,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>7.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -22509,24 +22596,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.7</v>
+        <v>23.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>1.7</v>
+        <v>7.6</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.1</v>
+        <v>3.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>21.7</v>
+        <v>35.8</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>9.4</v>
+        <v>7.7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -22538,13 +22625,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20.9</v>
+        <v>20.7</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>4.9</v>
+        <v>4.3</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -22552,10 +22639,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>71.8</v>
+        <v>64.7</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -22567,13 +22654,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>1.3</v>
+        <v>2.1</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -22581,10 +22668,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>40.4</v>
+        <v>57.1</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.2</v>
+        <v>5.1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -22596,27 +22683,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>21.3</v>
+        <v>20.8</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>3.1</v>
+        <v>1.6</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>60.3</v>
+        <v>6.6</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.8</v>
+        <v>11.2</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -22637,7 +22753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27982,24 +28098,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>12.9</v>
+        <v>15.8</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>22.9</v>
+        <v>5.2</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>11.4</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -28011,24 +28127,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>3.8</v>
+        <v>4.8</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -28040,21 +28156,21 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.3</v>
+        <v>11.6</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>1.9</v>
+        <v>14</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.3</v>
+        <v>2.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>29.9</v>
+        <v>30</v>
       </c>
       <c r="G187" s="4" t="n">
         <v>8.4</v>
@@ -28069,13 +28185,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -28083,10 +28199,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>39</v>
+        <v>44.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>7.3</v>
+        <v>6.7</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -28098,24 +28214,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>8.1</v>
+        <v>7.5</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>46.5</v>
+        <v>40.8</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -28127,27 +28243,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>30.4</v>
+        <v>21.9</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.4</v>
+        <v>9.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -28168,7 +28313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30004,24 +30149,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.6</v>
+        <v>13.5</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>4.1</v>
+        <v>1.7</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>69.5</v>
+        <v>54.3</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.7</v>
+        <v>5.5</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -30033,24 +30178,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>4.1</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>23.9</v>
+        <v>30.2</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>9.1</v>
+        <v>8.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -30062,13 +30207,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.5</v>
+        <v>15.8</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -30076,10 +30221,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>4.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.4</v>
+        <v>10.8</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -30091,24 +30236,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>16.7</v>
+        <v>15.8</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>34.5</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>7.9</v>
+        <v>3.6</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -30120,24 +30265,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>15.3</v>
+        <v>14.6</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>3.8</v>
+        <v>1.2</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>88.09999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -30149,27 +30294,56 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14.5</v>
+        <v>14.7</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>56.2</v>
+        <v>41</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>5.3</v>
+        <v>7.1</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H70" s="12">
+        <f>SUM(C64:C70)</f>
         <v/>
       </c>
     </row>
@@ -30190,7 +30364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32026,13 +32200,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>12.8</v>
+        <v>15.3</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>6.7</v>
+        <v>1.4</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -32040,10 +32214,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>85.2</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>1.8</v>
+        <v>4.1</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -32055,10 +32229,10 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14</v>
+        <v>14.6</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>1.5</v>
@@ -32069,10 +32243,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>48</v>
+        <v>45.6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -32084,13 +32258,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.1</v>
+        <v>14.7</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -32098,10 +32272,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>18.8</v>
+        <v>8.6</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>11</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -32113,24 +32287,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>14.9</v>
+        <v>12.4</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>1.6</v>
+        <v>4.2</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>94.7</v>
+        <v>63.1</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>0.6</v>
+        <v>4.4</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -32142,24 +32316,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.9</v>
+        <v>12.2</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>15.7</v>
+        <v>4.5</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>83.40000000000001</v>
+        <v>99.8</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -32171,13 +32345,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.7</v>
+        <v>12.5</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0.2</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2.2</v>
+        <v>1.7</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -32185,13 +32359,42 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>44.1</v>
+        <v>31.1</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>6.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H70" s="12">
+        <f>SUM(C64:C70)</f>
         <v/>
       </c>
     </row>
@@ -32212,7 +32415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34048,24 +34251,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.2</v>
+        <v>14.8</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>5.7</v>
+        <v>0.4</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>91.3</v>
+        <v>47.5</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>1</v>
+        <v>6.3</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -34077,13 +34280,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.5</v>
+        <v>14.9</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2.6</v>
+        <v>0.6</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -34091,10 +34294,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>32.6</v>
+        <v>38.4</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -34106,13 +34309,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15</v>
+        <v>15.3</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -34120,10 +34323,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>4.3</v>
+        <v>5.8</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -34135,13 +34338,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>15.9</v>
+        <v>13.6</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -34149,10 +34352,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>77.5</v>
+        <v>59.8</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>2.7</v>
+        <v>4.8</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -34164,13 +34367,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.5</v>
+        <v>12.2</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>15.9</v>
+        <v>6</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2</v>
+        <v>0.9</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -34178,10 +34381,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>85.2</v>
+        <v>85.5</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -34193,27 +34396,56 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>33</v>
+        <v>32.6</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H70" s="12">
+        <f>SUM(C64:C70)</f>
         <v/>
       </c>
     </row>
@@ -34234,7 +34466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36070,24 +36302,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.5</v>
+        <v>14.2</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>6.7</v>
+        <v>0.4</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>67.2</v>
+        <v>52.3</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.9</v>
+        <v>5.7</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -36102,10 +36334,10 @@
         <v>14.1</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>4.5</v>
+        <v>7.9</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -36113,10 +36345,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>35.8</v>
+        <v>46.3</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>7.7</v>
+        <v>6.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -36128,13 +36360,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.2</v>
+        <v>15.4</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -36142,10 +36374,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -36157,13 +36389,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>16.2</v>
+        <v>15.3</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.1</v>
+        <v>6.2</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -36171,10 +36403,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>28.5</v>
+        <v>43.8</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>8.6</v>
+        <v>6.7</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -36186,24 +36418,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>15</v>
+        <v>13.8</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>3.6</v>
+        <v>1.1</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>85.3</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -36215,13 +36447,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14.5</v>
+        <v>13.8</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.2</v>
+        <v>2.3</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -36229,13 +36461,42 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>57.2</v>
+        <v>65</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>5.1</v>
+        <v>4.2</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H70" s="12">
+        <f>SUM(C64:C70)</f>
         <v/>
       </c>
     </row>
@@ -36256,7 +36517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38092,24 +38353,24 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.2</v>
+        <v>15.1</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>1.5</v>
+        <v>0.3</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>70.2</v>
+        <v>50.4</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3.6</v>
+        <v>6</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -38121,13 +38382,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.4</v>
+        <v>14.7</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -38135,10 +38396,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>29.9</v>
+        <v>23.4</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>8.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -38150,13 +38411,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.2</v>
+        <v>15.5</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -38164,10 +38425,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -38179,24 +38440,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>16.1</v>
+        <v>14.4</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>49.2</v>
+        <v>61.1</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -38208,24 +38469,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.9</v>
+        <v>13.4</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>11.1</v>
+        <v>5.3</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.7</v>
+        <v>0.9</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>77.3</v>
+        <v>81</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -38237,7 +38498,7 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.9</v>
+        <v>13.2</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
@@ -38247,17 +38508,46 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>41.2</v>
+        <v>38.7</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H70" s="12">
+        <f>SUM(C64:C70)</f>
         <v/>
       </c>
     </row>
@@ -38278,7 +38568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40114,13 +40404,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.9</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>4.2</v>
+        <v>0.4</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -40128,10 +40418,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>95.5</v>
+        <v>48.9</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>0.5</v>
+        <v>6.1</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -40143,24 +40433,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>1.7</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>56.3</v>
+        <v>55.3</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -40172,13 +40462,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -40186,10 +40476,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>6.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.3</v>
+        <v>10.9</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -40201,13 +40491,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12</v>
+        <v>9.6</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>3</v>
+        <v>4.3</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -40215,10 +40505,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>83.40000000000001</v>
+        <v>69</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>2</v>
+        <v>3.7</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -40230,21 +40520,21 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>11</v>
+        <v>9.9</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>14.1</v>
+        <v>4.4</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>97.2</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G68" s="7" t="n">
         <v>0.3</v>
@@ -40259,13 +40549,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>9.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -40273,13 +40563,42 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>84.2</v>
+        <v>43.6</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>1.9</v>
+        <v>6.8</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H70" s="12">
+        <f>SUM(C64:C70)</f>
         <v/>
       </c>
     </row>
@@ -40300,7 +40619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45645,24 +45964,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>22.2</v>
+        <v>24.1</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>20.1</v>
+        <v>16.3</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>9.6</v>
+        <v>10</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -45674,24 +45993,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.1</v>
+        <v>21.3</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>48.8</v>
+        <v>30.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>6.1</v>
+        <v>8.4</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -45703,24 +46022,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.2</v>
+        <v>20.9</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>4.2</v>
+        <v>27.3</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>83.59999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -45732,24 +46051,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>19.7</v>
+        <v>20</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>12.3</v>
+        <v>6.4</v>
       </c>
       <c r="D188" s="7" t="n">
         <v>0.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>81</v>
+        <v>62.1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2.3</v>
+        <v>4.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -45761,24 +46080,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>18.1</v>
+        <v>19.3</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>4.5</v>
+        <v>0.5</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>65.40000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>4.2</v>
+        <v>3.4</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -45790,27 +46109,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
       <c r="C190" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="D190" s="7" t="n">
-        <v>0.5</v>
-      </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
           <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>77.8</v>
+        <v>41.2</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>2.7</v>
+        <v>7.1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -45831,7 +46179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47667,13 +48015,13 @@
         <v>46279</v>
       </c>
       <c r="B64" s="7" t="n">
-        <v>13.1</v>
+        <v>13.4</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>5</v>
+        <v>0.1</v>
       </c>
       <c r="D64" s="7" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
@@ -47681,10 +48029,10 @@
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>61.1</v>
+        <v>32.1</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>4.7</v>
+        <v>8.1</v>
       </c>
       <c r="H64" s="12">
         <f>SUM(C58:C64)</f>
@@ -47696,13 +48044,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -47710,10 +48058,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>11.5</v>
+        <v>6.7</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>10.6</v>
+        <v>11.2</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -47725,10 +48073,10 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>13.8</v>
+        <v>14.8</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>2.5</v>
+        <v>13.6</v>
       </c>
       <c r="D66" s="7" t="n">
         <v>3.7</v>
@@ -47739,10 +48087,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>58.8</v>
+        <v>72.5</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>4.9</v>
+        <v>3.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -47754,24 +48102,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.4</v>
+        <v>13</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>62.3</v>
+        <v>76.3</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.5</v>
+        <v>2.8</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -47783,24 +48131,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>89.8</v>
+        <v>44.5</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>1.2</v>
+        <v>6.7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -47812,13 +48160,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -47826,13 +48174,42 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>61.9</v>
+        <v>41</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>4.6</v>
+        <v>7.1</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>81</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H70" s="12">
+        <f>SUM(C64:C70)</f>
         <v/>
       </c>
     </row>
@@ -47853,7 +48230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -53198,24 +53575,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>26.3</v>
+        <v>26.6</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>31.7</v>
+        <v>22.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -53227,13 +53604,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>26.1</v>
+        <v>26.2</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.7</v>
+        <v>4.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -53241,7 +53618,7 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="G186" s="7" t="n">
         <v>10.6</v>
@@ -53259,21 +53636,21 @@
         <v>26</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>7.2</v>
+        <v>5.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -53285,10 +53662,10 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>25.1</v>
+        <v>25.2</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>2.2</v>
+        <v>0.5</v>
       </c>
       <c r="D188" s="7" t="n">
         <v>3.7</v>
@@ -53299,10 +53676,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>19.1</v>
+        <v>20.7</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -53314,13 +53691,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>25.4</v>
+        <v>24.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -53328,10 +53705,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>7.6</v>
+        <v>45.9</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>11.1</v>
+        <v>6.5</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -53343,27 +53720,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>25.7</v>
+        <v>24.8</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>76.2</v>
+        <v>20.1</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>2.9</v>
+        <v>9.6</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -53384,7 +53790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -58729,13 +59135,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20.5</v>
+        <v>23.5</v>
       </c>
       <c r="C185" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3.1</v>
+        <v>3.7</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -58743,10 +59149,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>4.4</v>
+        <v>7.5</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>11.5</v>
+        <v>11.1</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -58758,13 +59164,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -58772,10 +59178,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -58787,13 +59193,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>18.2</v>
+        <v>17.7</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -58801,10 +59207,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -58816,13 +59222,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>14.2</v>
+        <v>14</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -58830,10 +59236,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>23.4</v>
+        <v>53.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>5.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -58845,13 +59251,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>15.4</v>
+        <v>14.6</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -58859,10 +59265,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>48.6</v>
+        <v>30.3</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>6.2</v>
+        <v>8.4</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -58874,13 +59280,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>15.2</v>
+        <v>14.8</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -58888,13 +59294,42 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>1.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.9</v>
+        <v>11</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -58915,7 +59350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64260,13 +64695,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>12.5</v>
+        <v>13.1</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>12.2</v>
+        <v>13.6</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -64274,10 +64709,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>86.8</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -64289,24 +64724,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>14</v>
+        <v>14.2</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>30.1</v>
+        <v>26.2</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>98.5</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -64318,24 +64753,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.2</v>
+        <v>12.7</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>6.1</v>
+        <v>4.4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>88.3</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -64347,24 +64782,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.2</v>
+        <v>10.9</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>4.6</v>
+        <v>2.2</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>93.7</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -64376,13 +64811,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>10.9</v>
+        <v>11.3</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>6.9</v>
+        <v>4.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -64390,10 +64825,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>97.3</v>
+        <v>93.8</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -64408,24 +64843,53 @@
         <v>11.4</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>96.40000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -64446,7 +64910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69791,13 +70255,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>19.2</v>
+        <v>19.7</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>9.1</v>
+        <v>1.7</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -69805,10 +70269,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>48.9</v>
+        <v>13.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>6.1</v>
+        <v>10.3</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -69820,13 +70284,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -69834,7 +70298,7 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="G186" s="7" t="n">
         <v>11.5</v>
@@ -69849,13 +70313,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>17.5</v>
+        <v>18.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -69863,10 +70327,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>15.2</v>
+        <v>4.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>10.2</v>
+        <v>11.5</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -69878,13 +70342,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>18.4</v>
+        <v>17.5</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>27.4</v>
+        <v>55.8</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.3</v>
+        <v>3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -69892,10 +70356,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>60.4</v>
+        <v>78.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>4.8</v>
+        <v>2.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -69907,24 +70371,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>16.4</v>
+        <v>16.7</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>13.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>80.5</v>
+        <v>90</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -69936,27 +70400,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>16.8</v>
+        <v>18.1</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>63.3</v>
+        <v>48.8</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -69977,7 +70470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -75322,13 +75815,13 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>20.1</v>
+        <v>20.6</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>14.1</v>
+        <v>1.8</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
@@ -75336,10 +75829,10 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>47.9</v>
+        <v>13.9</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>6.3</v>
+        <v>10.3</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -75357,7 +75850,7 @@
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -75365,10 +75858,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -75380,21 +75873,21 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>19.3</v>
+        <v>20</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>13.5</v>
+        <v>13.1</v>
       </c>
       <c r="G187" s="4" t="n">
         <v>10.4</v>
@@ -75409,13 +75902,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>19.6</v>
+        <v>19</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>26.8</v>
+        <v>31.1</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -75423,10 +75916,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>53.1</v>
+        <v>75.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.6</v>
+        <v>2.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -75438,24 +75931,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.6</v>
+        <v>18.2</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>12.5</v>
+        <v>7.9</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>96.09999999999999</v>
+        <v>83.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -75467,27 +75960,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.1</v>
+        <v>18.9</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>45.1</v>
+        <v>48</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -75508,7 +76030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80853,24 +81375,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>15.6</v>
+        <v>17.2</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>2.9</v>
+        <v>0.9</v>
       </c>
       <c r="D185" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>63.9</v>
+        <v>51</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>4.3</v>
+        <v>5.9</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -80888,7 +81410,7 @@
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -80896,10 +81418,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>26.7</v>
+        <v>28.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -80911,24 +81433,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>15.8</v>
+        <v>16.4</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>5.8</v>
+        <v>18.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -80940,13 +81462,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.6</v>
+        <v>17.1</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>4</v>
+        <v>5.3</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -80954,10 +81476,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>27</v>
+        <v>33.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -80969,13 +81491,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>15.5</v>
+        <v>14.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>11.7</v>
+        <v>26</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.7</v>
+        <v>1.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -80983,10 +81505,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>76.59999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -80998,27 +81520,56 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1</v>
+        <v>2.1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>20.3</v>
+        <v>43</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.6</v>
+        <v>6.8</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>
@@ -81039,7 +81590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -86384,24 +86935,24 @@
         <v>46279</v>
       </c>
       <c r="B185" s="4" t="n">
-        <v>14.4</v>
+        <v>15.1</v>
       </c>
       <c r="C185" s="4" t="n">
-        <v>8.1</v>
+        <v>1</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>1.4</v>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>79.7</v>
+        <v>53</v>
       </c>
       <c r="G185" s="4" t="n">
-        <v>2.4</v>
+        <v>5.6</v>
       </c>
       <c r="H185" s="10">
         <f>SUM(C179:C185)</f>
@@ -86413,7 +86964,7 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>15.4</v>
+        <v>15.7</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
@@ -86427,7 +86978,7 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>17.7</v>
+        <v>17.9</v>
       </c>
       <c r="G186" s="7" t="n">
         <v>9.9</v>
@@ -86442,24 +86993,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>19.1</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>77.09999999999999</v>
+        <v>72</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -86471,24 +87022,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>3.2</v>
+        <v>1.1</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>98.59999999999999</v>
+        <v>94</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -86500,13 +87051,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>10.9</v>
+        <v>10.4</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -86514,10 +87065,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>74.2</v>
+        <v>91.8</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -86529,13 +87080,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>12</v>
+        <v>11.2</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -86543,13 +87094,42 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>87.3</v>
+        <v>44.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>1.5</v>
+        <v>6.6</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B191" s="4" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H191" s="10">
+        <f>SUM(C185:C191)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-15 10:40 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5887,24 +5887,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.4</v>
+        <v>20.7</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>6.7</v>
+        <v>13.4</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>78.90000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -5916,13 +5916,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>23.4</v>
+        <v>22.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -5930,10 +5930,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>48.6</v>
+        <v>69</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>6.2</v>
+        <v>3.7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -5945,24 +5945,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>23.6</v>
+        <v>22.7</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.9</v>
+        <v>5.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -5977,7 +5977,7 @@
         <v>23.6</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>1.8</v>
@@ -5988,10 +5988,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>39.5</v>
+        <v>16.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.3</v>
+        <v>10.1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -6003,13 +6003,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.7</v>
+        <v>24.1</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -6017,10 +6017,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>17.6</v>
+        <v>14</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.9</v>
+        <v>10.3</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -6032,27 +6032,56 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>25.9</v>
+        <v>24.4</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0.3</v>
+        <v>1.6</v>
       </c>
       <c r="D191" s="4" t="n">
         <v>1.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>50</v>
+        <v>40.4</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6</v>
+        <v>7.2</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -6073,7 +6102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11447,13 +11476,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>25</v>
+        <v>27.1</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -11476,24 +11505,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>20.9</v>
+        <v>19.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3.2</v>
+        <v>2.2</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>7.5</v>
+        <v>51</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.1</v>
+        <v>5.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -11505,24 +11534,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>51.4</v>
+        <v>56.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.8</v>
+        <v>5.2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -11534,24 +11563,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>44.1</v>
+        <v>29.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>6.7</v>
+        <v>8.5</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -11563,24 +11592,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.5</v>
+        <v>17.9</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>0.6</v>
+        <v>27.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -11592,27 +11621,56 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20.6</v>
+        <v>21.3</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>3.7</v>
+        <v>20.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.6</v>
+        <v>9.5</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -11633,7 +11691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17007,13 +17065,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.6</v>
+        <v>22.8</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>7.9</v>
+        <v>6.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -17021,10 +17079,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>46.2</v>
+        <v>76.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>6.5</v>
+        <v>2.8</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -17036,24 +17094,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.5</v>
+        <v>22.3</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>2.8</v>
+        <v>0.5</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>61.9</v>
+        <v>62.8</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -17071,7 +17129,7 @@
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>5.6</v>
+        <v>7.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -17079,10 +17137,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>3.1</v>
+        <v>26.2</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.6</v>
+        <v>8.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -17094,13 +17152,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>5.8</v>
+        <v>7.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -17123,13 +17181,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.9</v>
+        <v>22.5</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -17137,10 +17195,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -17152,27 +17210,56 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n">
         <v>23.4</v>
       </c>
-      <c r="C191" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D191" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E191" s="4" t="inlineStr">
-        <is>
-          <t>SV</t>
-        </is>
-      </c>
-      <c r="F191" s="4" t="n">
-        <v>2.3</v>
-      </c>
       <c r="G191" s="4" t="n">
-        <v>11.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -17193,7 +17280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22567,24 +22654,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>24</v>
+        <v>25.7</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>12</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -22596,13 +22683,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>7.6</v>
+        <v>11.8</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3.3</v>
+        <v>2.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -22610,10 +22697,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>35.8</v>
+        <v>33.2</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -22625,24 +22712,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20.7</v>
+        <v>20.8</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>4.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.2</v>
+        <v>4.4</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>64.7</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>4.2</v>
+        <v>2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -22654,13 +22741,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>2.1</v>
+        <v>0.3</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.8</v>
+        <v>3.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -22668,10 +22755,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>57.1</v>
+        <v>89.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>5.1</v>
+        <v>1.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -22683,13 +22770,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>20.8</v>
+        <v>20.3</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -22697,10 +22784,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>6.6</v>
+        <v>3.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.2</v>
+        <v>11.6</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -22712,27 +22799,56 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>24.4</v>
+        <v>46.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.1</v>
+        <v>6.4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -22753,7 +22869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28127,24 +28243,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>13.7</v>
+        <v>15.6</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>4.8</v>
+        <v>6.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.4</v>
+        <v>11.2</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -28156,24 +28272,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>11.6</v>
+        <v>12.6</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>14</v>
+        <v>2.9</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>30</v>
+        <v>19.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>8.4</v>
+        <v>9.6</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -28185,13 +28301,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>8.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3</v>
+        <v>3.8</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -28199,10 +28315,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>44.5</v>
+        <v>47</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>6.7</v>
+        <v>6.4</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -28214,24 +28330,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>40.8</v>
+        <v>35.1</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.1</v>
+        <v>7.8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -28243,13 +28359,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -28257,10 +28373,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>21.9</v>
+        <v>20.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.4</v>
+        <v>9.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -28272,13 +28388,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>10.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -28286,13 +28402,42 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>9.6</v>
+        <v>44.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>10.8</v>
+        <v>6.6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -28313,7 +28458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30178,13 +30323,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.5</v>
+        <v>16.1</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -30192,10 +30337,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>30.2</v>
+        <v>31.4</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -30207,7 +30352,7 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.8</v>
+        <v>16</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
@@ -30221,10 +30366,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>11.4</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -30239,10 +30384,10 @@
         <v>15.8</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>2.5</v>
+        <v>20.8</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -30250,10 +30395,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>70.09999999999999</v>
+        <v>41.4</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.6</v>
+        <v>7</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -30265,13 +30410,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>14.6</v>
+        <v>15.5</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -30279,10 +30424,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>87.7</v>
+        <v>40.1</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>1.5</v>
+        <v>7.2</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -30294,24 +30439,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14.7</v>
+        <v>17.4</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>41</v>
+        <v>69.3</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>7.1</v>
+        <v>3.7</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -30323,27 +30468,56 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>14.3</v>
+        <v>17.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>66.40000000000001</v>
+        <v>42.2</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4</v>
+        <v>6.9</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H71" s="10">
+        <f>SUM(C65:C71)</f>
         <v/>
       </c>
     </row>
@@ -30364,7 +30538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32229,24 +32403,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.6</v>
+        <v>15.3</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>45.6</v>
+        <v>15.3</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>6.5</v>
+        <v>10.2</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -32258,13 +32432,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.7</v>
+        <v>15.1</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>0</v>
+        <v>16.4</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -32272,10 +32446,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>8.6</v>
+        <v>22.9</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -32287,24 +32461,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.4</v>
+        <v>12.7</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>4.2</v>
+        <v>28.9</v>
       </c>
       <c r="D67" s="4" t="n">
         <v>1.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>63.1</v>
+        <v>82.8</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.4</v>
+        <v>2.1</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -32316,24 +32490,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.2</v>
+        <v>13.6</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>4.5</v>
+        <v>0.6</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>99.8</v>
+        <v>92.8</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -32345,24 +32519,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.5</v>
+        <v>14.2</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.2</v>
+        <v>6.7</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>31.1</v>
+        <v>88.3</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -32374,13 +32548,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12.8</v>
+        <v>14.7</v>
       </c>
       <c r="C70" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -32388,13 +32562,42 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>60.9</v>
+        <v>87.5</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.7</v>
+        <v>1.5</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H71" s="10">
+        <f>SUM(C65:C71)</f>
         <v/>
       </c>
     </row>
@@ -32415,7 +32618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34280,24 +34483,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.9</v>
+        <v>16</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>38.4</v>
+        <v>21</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>7.4</v>
+        <v>9.5</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -34309,13 +34512,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.3</v>
+        <v>15.6</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -34323,10 +34526,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>5.8</v>
+        <v>12.7</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -34338,13 +34541,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13.6</v>
+        <v>13.1</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>1.3</v>
+        <v>24.7</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -34352,10 +34555,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>59.8</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.8</v>
+        <v>3.5</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -34367,24 +34570,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.2</v>
+        <v>14.1</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>85.5</v>
+        <v>78.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>1.7</v>
+        <v>2.6</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -34396,24 +34599,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.9</v>
+        <v>15.4</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2.3</v>
+        <v>0.5</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>32.6</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.1</v>
+        <v>1.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -34425,27 +34628,56 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>14.3</v>
+        <v>15.4</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>59</v>
+        <v>47.1</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.9</v>
+        <v>6.3</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H71" s="10">
+        <f>SUM(C65:C71)</f>
         <v/>
       </c>
     </row>
@@ -34466,7 +34698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36331,24 +36563,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.1</v>
+        <v>15.4</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>7.9</v>
+        <v>1.4</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>46.3</v>
+        <v>41</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -36360,13 +36592,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -36374,10 +36606,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>6.3</v>
+        <v>13.9</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.2</v>
+        <v>10.3</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -36392,21 +36624,21 @@
         <v>15.3</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>6.2</v>
+        <v>10.5</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>43.8</v>
+        <v>52</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -36418,13 +36650,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.8</v>
+        <v>15</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -36432,10 +36664,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>81.40000000000001</v>
+        <v>49.4</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>2.2</v>
+        <v>6.1</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -36447,13 +36679,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>13.8</v>
+        <v>17.1</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>2.3</v>
+        <v>1.6</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -36461,10 +36693,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>65</v>
+        <v>78.5</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>4.2</v>
+        <v>2.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -36476,27 +36708,56 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>14.6</v>
+        <v>16.1</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>66.2</v>
+        <v>44.7</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.1</v>
+        <v>6.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H71" s="10">
+        <f>SUM(C65:C71)</f>
         <v/>
       </c>
     </row>
@@ -36517,7 +36778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38382,24 +38643,24 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>14.7</v>
+        <v>16.8</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>23.4</v>
+        <v>11.4</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -38411,13 +38672,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.5</v>
+        <v>15.7</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -38425,10 +38686,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>5.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>11.3</v>
+        <v>10.8</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -38440,24 +38701,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>14.4</v>
+        <v>13.9</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0.9</v>
+        <v>9.1</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>61.1</v>
+        <v>64.8</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -38469,24 +38730,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.4</v>
+        <v>14.8</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>5.3</v>
+        <v>4.8</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>2.3</v>
+        <v>3.7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -38498,24 +38759,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>13.2</v>
+        <v>15</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2</v>
+        <v>0.9</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>38.7</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>7.4</v>
+        <v>1.5</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -38527,13 +38788,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>13.9</v>
+        <v>15.4</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -38541,13 +38802,42 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>60</v>
+        <v>58.6</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H71" s="10">
+        <f>SUM(C65:C71)</f>
         <v/>
       </c>
     </row>
@@ -38568,7 +38858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40433,13 +40723,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>11.2</v>
+        <v>12.7</v>
       </c>
       <c r="C65" s="4" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -40447,10 +40737,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>55.3</v>
+        <v>13.8</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>5.4</v>
+        <v>10.3</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -40462,10 +40752,10 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D66" s="7" t="n">
         <v>2.3</v>
@@ -40476,10 +40766,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>20.6</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>10.9</v>
+        <v>9.5</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -40491,24 +40781,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>4.3</v>
+        <v>21.5</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>69</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -40520,13 +40810,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>9.9</v>
+        <v>11.2</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>4.4</v>
+        <v>3.5</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -40534,10 +40824,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>97.09999999999999</v>
+        <v>95.5</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -40549,24 +40839,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>12.3</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>6.3</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>43.6</v>
+        <v>89.5</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>6.8</v>
+        <v>1.3</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -40578,27 +40868,56 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>10.6</v>
+        <v>11.9</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>1.3</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>67</v>
+        <v>65.8</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H71" s="10">
+        <f>SUM(C65:C71)</f>
         <v/>
       </c>
     </row>
@@ -40619,7 +40938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45993,24 +46312,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>21.3</v>
+        <v>23.2</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>30.2</v>
+        <v>19.6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8.4</v>
+        <v>9.6</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -46022,24 +46341,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>20.9</v>
+        <v>21.4</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>27.3</v>
+        <v>6.7</v>
       </c>
       <c r="D187" s="4" t="n">
         <v>1.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>71.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -46051,24 +46370,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>6.4</v>
+        <v>17.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>62.1</v>
+        <v>83.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>4.5</v>
+        <v>2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -46080,13 +46399,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>19.3</v>
+        <v>19.6</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0.5</v>
+        <v>3.3</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -46094,10 +46413,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>71.3</v>
+        <v>85</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>3.4</v>
+        <v>1.8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -46109,24 +46428,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>19</v>
+        <v>19.4</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>41.2</v>
+        <v>59.4</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>7.1</v>
+        <v>4.9</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -46138,7 +46457,7 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20.1</v>
+        <v>19.7</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
@@ -46148,17 +46467,46 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>44.9</v>
+        <v>67.8</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.6</v>
+        <v>3.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -46179,7 +46527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48044,13 +48392,13 @@
         <v>46280</v>
       </c>
       <c r="B65" s="4" t="n">
-        <v>12.3</v>
+        <v>15</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -48058,10 +48406,10 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>6.7</v>
+        <v>2.6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>11.2</v>
+        <v>11.7</v>
       </c>
       <c r="H65" s="10">
         <f>SUM(C59:C65)</f>
@@ -48073,13 +48421,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>13.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -48087,10 +48435,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>72.5</v>
+        <v>74.2</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -48102,24 +48450,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13</v>
+        <v>12.8</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>1.7</v>
+        <v>4</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>76.3</v>
+        <v>68.2</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -48131,24 +48479,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>11.8</v>
+        <v>12.1</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>44.5</v>
+        <v>57.5</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6.7</v>
+        <v>5.1</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -48160,24 +48508,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>11.2</v>
+        <v>12.5</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>41</v>
+        <v>7.8</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>7.1</v>
+        <v>11.1</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -48189,13 +48537,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12.7</v>
+        <v>11.7</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.4</v>
+        <v>4.3</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -48203,13 +48551,42 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>81</v>
+        <v>75.8</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H71" s="10">
+        <f>SUM(C65:C71)</f>
         <v/>
       </c>
     </row>
@@ -48230,7 +48607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -53604,24 +53981,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>26.2</v>
+        <v>26.6</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>1.8</v>
+        <v>0.5</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>4.6</v>
+        <v>5.9</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>11.8</v>
+        <v>5.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>10.6</v>
+        <v>11.3</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -53633,24 +54010,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>5.6</v>
+        <v>7.6</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -53662,13 +54039,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>25.2</v>
+        <v>25.7</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.7</v>
+        <v>4.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -53676,10 +54053,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>20.7</v>
+        <v>36.3</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>9.5</v>
+        <v>7.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -53691,24 +54068,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>24.9</v>
+        <v>23.6</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0.7</v>
+        <v>15.5</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>4.5</v>
+        <v>6.2</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>45.9</v>
+        <v>70.3</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>6.5</v>
+        <v>3.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -53720,24 +54097,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.8</v>
+        <v>22.5</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.1</v>
+        <v>1.8</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2</v>
+        <v>4.1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>20.1</v>
+        <v>31.9</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -53749,27 +54126,56 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>25.1</v>
+        <v>22.9</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0.7</v>
+        <v>2.4</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>8.6</v>
+        <v>21.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11</v>
+        <v>9.4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -53790,7 +54196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -59164,24 +59570,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>22.5</v>
+        <v>24</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.9</v>
+        <v>5.2</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -59193,13 +59599,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>17.7</v>
+        <v>17.2</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>4.9</v>
+        <v>4.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -59207,10 +59613,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>2.6</v>
+        <v>33.8</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.7</v>
+        <v>7.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -59222,24 +59628,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>14</v>
+        <v>14.3</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.2</v>
+        <v>4.1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>53.5</v>
+        <v>42.2</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.6</v>
+        <v>6.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -59251,13 +59657,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -59265,10 +59671,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>30.3</v>
+        <v>49.6</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8.4</v>
+        <v>6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -59280,13 +59686,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>14.8</v>
+        <v>14.2</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -59294,10 +59700,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>12.3</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -59309,13 +59715,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -59323,13 +59729,42 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>0.6</v>
+        <v>17.8</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.9</v>
+        <v>9.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -59350,7 +59785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64724,24 +65159,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>14.2</v>
+        <v>12.1</v>
       </c>
       <c r="C186" s="7" t="n">
-        <v>26.2</v>
+        <v>12.3</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>92.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>0.9</v>
+        <v>2.1</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -64753,24 +65188,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.7</v>
+        <v>10.7</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>4.4</v>
+        <v>9.5</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>96.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -64782,24 +65217,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>2.2</v>
+        <v>5.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>98.59999999999999</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0.2</v>
+        <v>1.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -64811,7 +65246,7 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>11.3</v>
+        <v>12.1</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>4.7</v>
@@ -64821,11 +65256,11 @@
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>93.8</v>
+        <v>94</v>
       </c>
       <c r="G189" s="4" t="n">
         <v>0.7</v>
@@ -64840,13 +65275,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>11.4</v>
+        <v>12.4</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>9.9</v>
+        <v>14</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -64854,10 +65289,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>94.2</v>
+        <v>97.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -64869,13 +65304,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>10.7</v>
+        <v>11.6</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -64883,13 +65318,42 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>93.5</v>
+        <v>95.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -64910,7 +65374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -70284,13 +70748,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>18.5</v>
+        <v>20.1</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>3.2</v>
+        <v>2.6</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -70298,10 +70762,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>4.4</v>
+        <v>0</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -70313,13 +70777,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>18.1</v>
+        <v>18.4</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -70327,10 +70791,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>4.1</v>
+        <v>2.8</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -70342,13 +70806,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.5</v>
+        <v>18.2</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>55.8</v>
+        <v>45.8</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -70356,10 +70820,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>78.5</v>
+        <v>79.2</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -70371,10 +70835,10 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>16.7</v>
+        <v>17.7</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>37</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>2.2</v>
@@ -70385,10 +70849,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>90</v>
+        <v>94.7</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -70400,13 +70864,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.1</v>
+        <v>17.6</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.6</v>
+        <v>9.4</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -70414,10 +70878,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>48.8</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>6.1</v>
+        <v>1.9</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -70429,13 +70893,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18</v>
+        <v>18.2</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -70443,13 +70907,42 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>35.7</v>
+        <v>29.3</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7.7</v>
+        <v>8.5</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -70470,7 +70963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -75844,24 +76337,24 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>19.6</v>
+        <v>21.9</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -75873,13 +76366,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>20</v>
+        <v>20.3</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -75887,10 +76380,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>13.1</v>
+        <v>3.5</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>10.4</v>
+        <v>11.6</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -75902,13 +76395,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>31.1</v>
+        <v>25.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -75916,10 +76409,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>75.8</v>
+        <v>71</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -75931,13 +76424,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>18.2</v>
+        <v>19.1</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>7.9</v>
+        <v>26.8</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -75945,10 +76438,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>83.2</v>
+        <v>96.8</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -75960,13 +76453,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.9</v>
+        <v>18.3</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>1.3</v>
+        <v>10.6</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -75974,10 +76467,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>48</v>
+        <v>71.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>6.2</v>
+        <v>3.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -75989,13 +76482,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>19.3</v>
+        <v>19</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -76003,13 +76496,42 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>40</v>
+        <v>27.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -76030,7 +76552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81404,13 +81926,13 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>15.9</v>
+        <v>17.4</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
@@ -81418,10 +81940,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>28.7</v>
+        <v>1.7</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8.6</v>
+        <v>11.8</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -81439,7 +81961,7 @@
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -81447,10 +81969,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>18.1</v>
+        <v>8.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>11</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -81462,13 +81984,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.1</v>
+        <v>17.9</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>5.3</v>
+        <v>0.5</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -81476,10 +81998,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>33.8</v>
+        <v>11.9</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>7.9</v>
+        <v>10.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -81491,13 +82013,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>14.9</v>
+        <v>16.2</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>26</v>
+        <v>10.9</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -81505,10 +82027,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>86.3</v>
+        <v>74.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.6</v>
+        <v>3.1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -81520,24 +82042,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>15.6</v>
+        <v>16.1</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>43</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>6.8</v>
+        <v>2</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -81549,13 +82071,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>15.7</v>
+        <v>16.8</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -81563,13 +82085,42 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>10.4</v>
+        <v>41.8</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>10.8</v>
+        <v>7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>
@@ -81590,7 +82141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -86964,7 +87515,7 @@
         <v>46280</v>
       </c>
       <c r="B186" s="7" t="n">
-        <v>15.7</v>
+        <v>17.9</v>
       </c>
       <c r="C186" s="7" t="n">
         <v>0</v>
@@ -86978,10 +87529,10 @@
         </is>
       </c>
       <c r="F186" s="7" t="n">
-        <v>17.9</v>
+        <v>10.3</v>
       </c>
       <c r="G186" s="7" t="n">
-        <v>9.9</v>
+        <v>10.8</v>
       </c>
       <c r="H186" s="12">
         <f>SUM(C180:C186)</f>
@@ -86993,24 +87544,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>70.90000000000001</v>
+        <v>36.4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>72</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>3.4</v>
+        <v>3.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -87022,24 +87573,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.6</v>
+        <v>11.2</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>1.1</v>
+        <v>5.6</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>94</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -87051,24 +87602,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>10.4</v>
+        <v>10.8</v>
       </c>
       <c r="C189" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D189" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="D189" s="4" t="n">
-        <v>0.6</v>
-      </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>91.8</v>
+        <v>94.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -87080,13 +87631,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -87094,10 +87645,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>44.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>6.6</v>
+        <v>2.9</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -87109,13 +87660,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>12.8</v>
+        <v>12.4</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0.1</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -87123,13 +87674,42 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>54.9</v>
+        <v>60.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>5.4</v>
+        <v>4.7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="11" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C192" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="n">
+        <v>78.7</v>
+      </c>
+      <c r="G192" s="7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H192" s="12">
+        <f>SUM(C186:C192)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-16 10:28 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5916,24 +5916,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.1</v>
+        <v>22.7</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>69</v>
+        <v>50.8</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>3.7</v>
+        <v>5.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -5951,7 +5951,7 @@
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G188" s="7" t="n">
         <v>12</v>
@@ -5974,24 +5974,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>23.6</v>
+        <v>23.4</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>16.2</v>
+        <v>19.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -6003,10 +6003,10 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.1</v>
+        <v>24.6</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1.4</v>
@@ -6017,10 +6017,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>14</v>
+        <v>27.4</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -6032,24 +6032,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>24.4</v>
+        <v>26.2</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>40.4</v>
+        <v>27.1</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -6061,27 +6061,56 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.8</v>
+        <v>26.9</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>50.4</v>
+        <v>5.1</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6</v>
+        <v>11.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -6102,7 +6131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11505,24 +11534,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>19.1</v>
+        <v>19.5</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>7.2</v>
+        <v>6.5</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>51</v>
+        <v>67.7</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>5.9</v>
+        <v>3.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -11534,13 +11563,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.4</v>
+        <v>17.7</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -11548,10 +11577,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>56.5</v>
+        <v>28.9</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.2</v>
+        <v>8.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -11563,21 +11592,21 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.2</v>
+        <v>17.7</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>29.5</v>
+        <v>29</v>
       </c>
       <c r="G189" s="4" t="n">
         <v>8.5</v>
@@ -11592,24 +11621,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>17.9</v>
+        <v>18.1</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>27.5</v>
+        <v>9</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -11621,24 +11650,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>21.3</v>
+        <v>20</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>20.7</v>
+        <v>17.4</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -11650,7 +11679,7 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.6</v>
+        <v>22.7</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
@@ -11660,17 +11689,46 @@
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>19.1</v>
+        <v>14.2</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -11691,7 +11749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17094,13 +17152,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.3</v>
+        <v>22.7</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3.9</v>
+        <v>4.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -17108,10 +17166,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>62.8</v>
+        <v>42.9</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>4.5</v>
+        <v>6.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -17126,10 +17184,10 @@
         <v>22.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -17137,10 +17195,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>26.2</v>
+        <v>5.7</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>8.9</v>
+        <v>11.3</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -17152,13 +17210,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -17166,10 +17224,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>12</v>
+        <v>10.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -17181,13 +17239,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.5</v>
+        <v>22.9</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -17195,10 +17253,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -17210,13 +17268,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>22.6</v>
+        <v>23.3</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>6.2</v>
+        <v>5.1</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -17224,10 +17282,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>23.4</v>
+        <v>9.4</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -17239,13 +17297,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.5</v>
+        <v>23.2</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -17253,13 +17311,42 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>30.9</v>
+        <v>18.9</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -17280,7 +17367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22683,13 +22770,13 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>22.9</v>
+        <v>24.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>11.8</v>
+        <v>3</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
@@ -22697,10 +22784,10 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>33.2</v>
+        <v>39.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>8</v>
+        <v>7.3</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -22712,24 +22799,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>83.09999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -22741,13 +22828,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>19.8</v>
+        <v>21.7</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0.3</v>
+        <v>10.8</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3.3</v>
+        <v>3.9</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -22755,10 +22842,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>89.5</v>
+        <v>56.1</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.3</v>
+        <v>5.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -22770,13 +22857,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>20.3</v>
+        <v>21.5</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -22784,10 +22871,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>3.5</v>
+        <v>16.8</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.6</v>
+        <v>10</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -22799,13 +22886,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -22813,10 +22900,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>46.7</v>
+        <v>36.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.4</v>
+        <v>7.6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -22828,13 +22915,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.1</v>
+        <v>23.3</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -22842,13 +22929,42 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>45.7</v>
+        <v>68.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.5</v>
+        <v>3.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -22869,7 +22985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28272,24 +28388,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>12.6</v>
+        <v>13.8</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>2.9</v>
+        <v>1.3</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>19.6</v>
+        <v>34.9</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>9.6</v>
+        <v>7.8</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -28301,13 +28417,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -28315,10 +28431,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>47</v>
+        <v>28.2</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>6.4</v>
+        <v>8.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -28330,24 +28446,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>7.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>35.1</v>
+        <v>33.7</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -28359,13 +28475,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -28373,10 +28489,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>20.7</v>
+        <v>25.4</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -28388,13 +28504,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>11.8</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -28402,10 +28518,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>44.9</v>
+        <v>44.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -28417,27 +28533,56 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>10.8</v>
+        <v>11.7</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>46.9</v>
+        <v>42.2</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.4</v>
+        <v>6.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -28458,7 +28603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30352,24 +30497,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>16</v>
+        <v>17.5</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>11.4</v>
+        <v>16.4</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>10.6</v>
+        <v>10</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -30381,13 +30526,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>15.8</v>
+        <v>14.8</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>20.8</v>
+        <v>12.5</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -30395,10 +30540,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>41.4</v>
+        <v>46.7</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>7</v>
+        <v>6.4</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -30410,13 +30555,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>15.5</v>
+        <v>13.6</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -30424,10 +30569,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>40.1</v>
+        <v>48.6</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>7.2</v>
+        <v>6.2</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -30439,24 +30584,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>17.4</v>
+        <v>15.7</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>69.3</v>
+        <v>33.4</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>3.7</v>
+        <v>8</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -30468,24 +30613,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>17.5</v>
+        <v>15.9</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.2</v>
+        <v>1.4</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>1.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>42.2</v>
+        <v>37.1</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -30497,27 +30642,56 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.7</v>
+        <v>13.5</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>2.8</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>64.7</v>
+        <v>35.4</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>4.2</v>
+        <v>7.8</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H72" s="12">
+        <f>SUM(C66:C72)</f>
         <v/>
       </c>
     </row>
@@ -30538,7 +30712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32432,24 +32606,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.1</v>
+        <v>17.7</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>16.4</v>
+        <v>1.6</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>22.9</v>
+        <v>48.7</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>6.2</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -32461,10 +32635,10 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>28.9</v>
+        <v>27.2</v>
       </c>
       <c r="D67" s="4" t="n">
         <v>1.2</v>
@@ -32475,10 +32649,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>82.8</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -32490,24 +32664,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.6</v>
+        <v>12.5</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>92.8</v>
+        <v>76.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>0.9</v>
+        <v>2.8</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -32519,24 +32693,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14.2</v>
+        <v>13.5</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>6.7</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>88.3</v>
+        <v>14.1</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>1.4</v>
+        <v>10.3</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -32548,13 +32722,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.5</v>
+        <v>3.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -32562,10 +32736,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>87.5</v>
+        <v>57.2</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>1.5</v>
+        <v>5.1</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -32577,27 +32751,56 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.8</v>
+        <v>11.3</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>6.4</v>
+        <v>10.6</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>69.7</v>
+        <v>48.4</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>3.6</v>
+        <v>6.2</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H72" s="12">
+        <f>SUM(C66:C72)</f>
         <v/>
       </c>
     </row>
@@ -32618,7 +32821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34512,13 +34715,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.6</v>
+        <v>17.4</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -34526,10 +34729,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>12.7</v>
+        <v>32</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>10.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -34541,24 +34744,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>24.7</v>
+        <v>17.7</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>71.09999999999999</v>
+        <v>57.9</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.5</v>
+        <v>5.1</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -34570,24 +34773,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>14.1</v>
+        <v>13.2</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>78.3</v>
+        <v>52.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>2.6</v>
+        <v>5.7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -34599,24 +34802,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.4</v>
+        <v>14.6</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>0.5</v>
+        <v>1.7</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>86.90000000000001</v>
+        <v>22.1</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>1.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -34628,24 +34831,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.4</v>
+        <v>16</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.2</v>
+        <v>2.7</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>47.1</v>
+        <v>45.1</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -34657,13 +34860,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.7</v>
+        <v>10.3</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1.7</v>
+        <v>7.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -34671,13 +34874,42 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>59</v>
+        <v>50.4</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>4.9</v>
+        <v>6</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H72" s="12">
+        <f>SUM(C66:C72)</f>
         <v/>
       </c>
     </row>
@@ -34698,7 +34930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36592,13 +36824,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.6</v>
+        <v>16.7</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -36606,10 +36838,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>13.9</v>
+        <v>16.9</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -36621,24 +36853,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>15.3</v>
+        <v>14.1</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>10.5</v>
+        <v>17.7</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>52</v>
+        <v>57.4</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>5.8</v>
+        <v>5.1</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -36650,13 +36882,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>15</v>
+        <v>13.2</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -36664,10 +36896,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>49.4</v>
+        <v>54.8</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -36679,24 +36911,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>17.1</v>
+        <v>15</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>78.5</v>
+        <v>44.3</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>2.6</v>
+        <v>6.7</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -36708,24 +36940,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.1</v>
+        <v>15.8</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>1.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>44.7</v>
+        <v>43.2</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -36737,13 +36969,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.3</v>
+        <v>12.1</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0.9</v>
+        <v>2.7</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -36751,13 +36983,42 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>72.2</v>
+        <v>36.7</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>3.3</v>
+        <v>7.6</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H72" s="12">
+        <f>SUM(C66:C72)</f>
         <v/>
       </c>
     </row>
@@ -36778,7 +37039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38672,24 +38933,24 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>15.7</v>
+        <v>17.5</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>21</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>10.8</v>
+        <v>9.5</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -38701,13 +38962,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13.9</v>
+        <v>13.5</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>9.1</v>
+        <v>5.6</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -38715,10 +38976,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>64.8</v>
+        <v>45.8</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.2</v>
+        <v>6.5</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -38730,24 +38991,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>14.8</v>
+        <v>13.9</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>69</v>
+        <v>50.6</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>3.7</v>
+        <v>5.9</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -38759,24 +39020,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15</v>
+        <v>15.2</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>87.90000000000001</v>
+        <v>16.6</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -38788,13 +39049,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.4</v>
+        <v>15.8</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -38802,10 +39063,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>58.6</v>
+        <v>28.5</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>5</v>
+        <v>8.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -38817,27 +39078,56 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.5</v>
+        <v>11.4</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0.1</v>
+        <v>2.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2.9</v>
+        <v>4.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>49.2</v>
+        <v>42.8</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H72" s="12">
+        <f>SUM(C66:C72)</f>
         <v/>
       </c>
     </row>
@@ -38858,7 +39148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40752,13 +41042,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>11.9</v>
+        <v>13.5</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -40766,10 +41056,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>20.6</v>
+        <v>40</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>9.5</v>
+        <v>7.2</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -40781,13 +41071,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>9.5</v>
+        <v>8.9</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>21.5</v>
+        <v>16.2</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -40795,10 +41085,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>79.40000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>2.5</v>
+        <v>5.8</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -40810,24 +41100,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>11.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>95.5</v>
+        <v>49.9</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -40839,24 +41129,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.3</v>
+        <v>11.1</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>6.3</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>89.5</v>
+        <v>23</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>1.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -40868,24 +41158,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>65.8</v>
+        <v>56.2</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.1</v>
+        <v>5.3</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -40897,13 +41187,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>8.4</v>
+        <v>6.9</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1.7</v>
+        <v>6.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.1</v>
+        <v>4.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -40911,13 +41201,42 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>60.7</v>
+        <v>72.2</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>4.7</v>
+        <v>3.3</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H72" s="12">
+        <f>SUM(C66:C72)</f>
         <v/>
       </c>
     </row>
@@ -40938,7 +41257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46341,24 +46660,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>21.4</v>
+        <v>23.8</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>6.7</v>
+        <v>5</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>4.1</v>
+        <v>4.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -46370,13 +46689,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20.1</v>
+        <v>20.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>17.9</v>
+        <v>14.2</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -46384,10 +46703,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>83.5</v>
+        <v>76</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2</v>
+        <v>2.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -46399,24 +46718,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>19.6</v>
+        <v>21</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>3.3</v>
+        <v>6.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>85</v>
+        <v>45.1</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.8</v>
+        <v>6.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -46428,24 +46747,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>19.4</v>
+        <v>19.9</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>59.4</v>
+        <v>29.1</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.9</v>
+        <v>8.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -46457,7 +46776,7 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>19.7</v>
+        <v>21</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
@@ -46467,14 +46786,14 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>67.8</v>
+        <v>60</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>3.9</v>
+        <v>4.8</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -46486,7 +46805,7 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>20.6</v>
+        <v>21.7</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
@@ -46496,17 +46815,46 @@
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>44.9</v>
+        <v>58.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.6</v>
+        <v>5</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -46527,7 +46875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48421,13 +48769,13 @@
         <v>46281</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>14.5</v>
+        <v>16.7</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>13.6</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
@@ -48435,10 +48783,10 @@
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>74.2</v>
+        <v>77.5</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="H66" s="12">
         <f>SUM(C60:C66)</f>
@@ -48450,13 +48798,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.8</v>
+        <v>12.1</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>4</v>
+        <v>1.4</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -48464,10 +48812,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>68.2</v>
+        <v>60.6</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>3.8</v>
+        <v>4.7</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -48479,24 +48827,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.2</v>
+        <v>3.1</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>57.5</v>
+        <v>43.2</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>5.1</v>
+        <v>6.8</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -48508,24 +48856,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.5</v>
+        <v>12.3</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>7.8</v>
+        <v>38.1</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>11.1</v>
+        <v>7.4</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -48537,13 +48885,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>11.7</v>
+        <v>13</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>4.3</v>
+        <v>6.4</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -48551,10 +48899,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>75.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -48566,13 +48914,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>3.7</v>
+        <v>1.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -48580,13 +48928,42 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>28.7</v>
+        <v>45.1</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>8.6</v>
+        <v>6.6</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H72" s="12">
+        <f>SUM(C66:C72)</f>
         <v/>
       </c>
     </row>
@@ -48607,7 +48984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -54010,24 +54387,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>25.9</v>
+        <v>26.1</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>7.6</v>
+        <v>1.1</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.1</v>
+        <v>11.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -54039,13 +54416,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>25.7</v>
+        <v>25.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.1</v>
+        <v>5.7</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -54053,10 +54430,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>36.3</v>
+        <v>51.9</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>7.6</v>
+        <v>5.8</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -54068,10 +54445,10 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>23.6</v>
+        <v>25.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>15.5</v>
+        <v>2.9</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>6.2</v>
@@ -54082,7 +54459,7 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>70.3</v>
+        <v>69.8</v>
       </c>
       <c r="G189" s="4" t="n">
         <v>3.6</v>
@@ -54097,24 +54474,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.5</v>
+        <v>24.8</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>1.8</v>
+        <v>5.5</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>31.9</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>3.2</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -54126,24 +54503,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>22.9</v>
+        <v>25.1</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>21.9</v>
+        <v>49.6</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.4</v>
+        <v>6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -54155,27 +54532,56 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.9</v>
+        <v>25.4</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>4</v>
+        <v>0.3</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>35.9</v>
+        <v>23.2</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>7.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -54196,7 +54602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -59599,24 +60005,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>17.2</v>
+        <v>18.7</v>
       </c>
       <c r="C187" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D187" s="4" t="n">
         <v>4.2</v>
       </c>
-      <c r="D187" s="4" t="n">
-        <v>4.3</v>
-      </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>33.8</v>
+        <v>51.2</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>7.9</v>
+        <v>5.9</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -59628,10 +60034,10 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>14.3</v>
+        <v>14.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.8</v>
+        <v>5.5</v>
       </c>
       <c r="D188" s="7" t="n">
         <v>4.1</v>
@@ -59642,10 +60048,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>42.2</v>
+        <v>53.9</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>6.9</v>
+        <v>5.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -59657,13 +60063,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>15</v>
+        <v>14.4</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.5</v>
+        <v>3.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -59671,10 +60077,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>49.6</v>
+        <v>29.6</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>6</v>
+        <v>8.4</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -59686,13 +60092,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>14.2</v>
+        <v>15.2</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -59700,10 +60106,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>12.3</v>
+        <v>5.8</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10.5</v>
+        <v>11.3</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -59715,13 +60121,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18</v>
+        <v>17.8</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -59729,10 +60135,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>17.8</v>
+        <v>13.3</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.9</v>
+        <v>10.4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -59744,13 +60150,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.6</v>
+        <v>19.3</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -59758,13 +60164,42 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>19.6</v>
+        <v>36.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.6</v>
+        <v>7.6</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -59785,7 +60220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65188,24 +65623,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>10.7</v>
+        <v>12.8</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>79.09999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -65217,24 +65652,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>5.9</v>
+        <v>7.4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>86.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -65246,21 +65681,21 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>12.1</v>
+        <v>11.5</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>4.7</v>
+        <v>15.7</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>0.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>94</v>
+        <v>94.5</v>
       </c>
       <c r="G189" s="4" t="n">
         <v>0.7</v>
@@ -65275,13 +65710,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>12.4</v>
+        <v>12.8</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>14</v>
+        <v>9.6</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -65289,10 +65724,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>97.7</v>
+        <v>96.8</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -65304,7 +65739,7 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>11.2</v>
@@ -65318,10 +65753,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>95.7</v>
+        <v>93.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -65336,10 +65771,10 @@
         <v>12.4</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>3.3</v>
+        <v>2.2</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -65347,13 +65782,42 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>83.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>99.3</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -65374,7 +65838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -70777,24 +71241,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>18.4</v>
+        <v>20.3</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>2.8</v>
+        <v>6.5</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.7</v>
+        <v>11.2</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -70806,13 +71270,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>18.2</v>
+        <v>17.3</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>45.8</v>
+        <v>61.3</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -70820,10 +71284,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>79.2</v>
+        <v>87</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -70835,24 +71299,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.7</v>
+        <v>16.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>37</v>
+        <v>37.5</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>94.7</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -70864,13 +71328,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>17.6</v>
+        <v>18.6</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>9.4</v>
+        <v>1.6</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.8</v>
+        <v>1.2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -70878,10 +71342,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>84.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>1.9</v>
+        <v>4.1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -70899,18 +71363,18 @@
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>29.3</v>
+        <v>64</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>8.5</v>
+        <v>4.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -70922,27 +71386,56 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>17.9</v>
+        <v>19.4</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.1</v>
+        <v>2.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>30.6</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>3.6</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -70963,7 +71456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -76366,24 +76859,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>20.3</v>
+        <v>22.1</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>3.5</v>
+        <v>5.3</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -76395,13 +76888,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>19.8</v>
+        <v>19.2</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>25.9</v>
+        <v>55.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -76409,10 +76902,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>71</v>
+        <v>77.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -76424,13 +76917,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>19.1</v>
+        <v>18.7</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>26.8</v>
+        <v>32.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -76438,10 +76931,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>96.8</v>
+        <v>87.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -76453,24 +76946,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.3</v>
+        <v>19.7</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>10.6</v>
+        <v>2</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>71.7</v>
+        <v>62.1</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -76482,13 +76975,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>19</v>
+        <v>20.1</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -76496,10 +76989,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>27.7</v>
+        <v>49.2</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -76511,27 +77004,56 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.2</v>
+        <v>20.9</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>52</v>
+        <v>71.7</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.8</v>
+        <v>3.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -76552,7 +77074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81955,24 +82477,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>16.4</v>
+        <v>18.6</v>
       </c>
       <c r="C187" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>8.1</v>
+        <v>0</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -81984,10 +82506,10 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.5</v>
+        <v>5.8</v>
       </c>
       <c r="D188" s="7" t="n">
         <v>2.3</v>
@@ -81998,10 +82520,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>11.9</v>
+        <v>28.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>10.6</v>
+        <v>8.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -82013,13 +82535,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>16.2</v>
+        <v>17</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>10.9</v>
+        <v>10.6</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -82027,10 +82549,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>74.2</v>
+        <v>60.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>3.1</v>
+        <v>4.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -82042,13 +82564,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>16.1</v>
+        <v>17.7</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>5.2</v>
+        <v>1.6</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.3</v>
+        <v>1.1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -82056,10 +82578,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>83.40000000000001</v>
+        <v>46.9</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>2</v>
+        <v>6.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -82071,24 +82593,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>16.8</v>
+        <v>17.6</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>41.8</v>
+        <v>51</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7</v>
+        <v>5.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -82100,13 +82622,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>15.8</v>
+        <v>17.2</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4.2</v>
+        <v>3.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -82114,13 +82636,42 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>34.4</v>
+        <v>72.7</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>7.9</v>
+        <v>3.3</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>
@@ -82141,7 +82692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -87544,24 +88095,24 @@
         <v>46281</v>
       </c>
       <c r="B187" s="4" t="n">
-        <v>13.9</v>
+        <v>13.2</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>36.4</v>
+        <v>21.4</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>67.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="G187" s="4" t="n">
-        <v>3.9</v>
+        <v>1.6</v>
       </c>
       <c r="H187" s="10">
         <f>SUM(C181:C187)</f>
@@ -87573,24 +88124,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>11.2</v>
+        <v>11.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>5.6</v>
+        <v>1.4</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>96.59999999999999</v>
+        <v>93</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -87602,13 +88153,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>10.8</v>
+        <v>11.4</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>2</v>
+        <v>0.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -87616,10 +88167,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>94.5</v>
+        <v>66.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>0.7</v>
+        <v>4</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -87631,13 +88182,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>10.9</v>
+        <v>11.9</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -87645,10 +88196,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>75.59999999999999</v>
+        <v>63.1</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>2.9</v>
+        <v>4.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -87660,13 +88211,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>12.4</v>
+        <v>13.8</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -87674,10 +88225,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>60.5</v>
+        <v>75</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4.7</v>
+        <v>3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -87689,27 +88240,56 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>12.8</v>
+        <v>13.7</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>78.7</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B193" s="4" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H193" s="10">
+        <f>SUM(C187:C193)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-17 10:38 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5945,13 +5945,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22.7</v>
+        <v>23.5</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>5.7</v>
+        <v>4.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -5974,13 +5974,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -5988,10 +5988,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>19.2</v>
+        <v>37.9</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -6003,24 +6003,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.6</v>
+        <v>24.3</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>27.4</v>
+        <v>21.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -6032,24 +6032,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>26.2</v>
+        <v>25.8</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>27.1</v>
+        <v>34.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -6061,24 +6061,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>26.9</v>
+        <v>25.4</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>5.1</v>
+        <v>27.9</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>11.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -6090,13 +6090,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>25.2</v>
+        <v>24</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>3.8</v>
+        <v>0.7</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -6104,13 +6104,42 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>39.6</v>
+        <v>23.2</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>7.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -6131,7 +6160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11563,13 +11592,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.7</v>
+        <v>18.8</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -11577,10 +11606,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>28.9</v>
+        <v>54.7</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>8.5</v>
+        <v>5.4</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -11592,7 +11621,7 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
@@ -11606,10 +11635,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>29</v>
+        <v>28.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -11621,24 +11650,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.1</v>
+        <v>18.6</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>9</v>
+        <v>15.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10.9</v>
+        <v>10.1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -11650,13 +11679,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20</v>
+        <v>19.3</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -11664,10 +11693,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>17.4</v>
+        <v>6.2</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.9</v>
+        <v>11.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -11679,7 +11708,7 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.7</v>
+        <v>22</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
@@ -11689,14 +11718,14 @@
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>14.2</v>
+        <v>23</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>10.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -11708,13 +11737,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23.7</v>
+        <v>21.1</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -11722,13 +11751,42 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>6.2</v>
+        <v>1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -11749,7 +11807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17181,24 +17239,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22.6</v>
+        <v>22.8</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>5.7</v>
+        <v>1.1</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -17210,13 +17268,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -17224,10 +17282,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>11.4</v>
+        <v>8.9</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>10.6</v>
+        <v>10.9</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -17239,13 +17297,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.9</v>
+        <v>22.7</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>6.8</v>
+        <v>7.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -17253,10 +17311,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>0</v>
+        <v>19.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>12</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -17268,13 +17326,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>23.3</v>
+        <v>23.1</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>5.1</v>
+        <v>5.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -17282,10 +17340,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>9.4</v>
+        <v>0.6</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>10.9</v>
+        <v>11.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -17297,13 +17355,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.2</v>
+        <v>22.4</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -17311,10 +17369,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>18.9</v>
+        <v>43.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -17326,27 +17384,56 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>24.1</v>
+        <v>21.8</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>6</v>
+        <v>17.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.3</v>
+        <v>9.9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -17367,7 +17454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22799,24 +22886,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>22</v>
+        <v>23.5</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>9.4</v>
+        <v>4.3</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>71.2</v>
+        <v>55.6</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>3.5</v>
+        <v>5.3</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -22828,24 +22915,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>10.8</v>
+        <v>7.1</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3.9</v>
+        <v>4.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>56.1</v>
+        <v>47.9</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>5.3</v>
+        <v>6.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -22857,13 +22944,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>21.5</v>
+        <v>22.1</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.5</v>
+        <v>3.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -22871,10 +22958,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>16.8</v>
+        <v>5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10</v>
+        <v>11.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -22886,13 +22973,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>22</v>
+        <v>22.1</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -22900,10 +22987,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>36.5</v>
+        <v>42.8</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7.6</v>
+        <v>6.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -22915,13 +23002,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.3</v>
+        <v>22.9</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -22929,10 +23016,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>68.5</v>
+        <v>70.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -22944,27 +23031,56 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>24.1</v>
+        <v>21.5</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.3</v>
+        <v>2.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>0.8</v>
+        <v>40.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.9</v>
+        <v>7.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -22985,7 +23101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28417,24 +28533,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>9.6</v>
+        <v>11.5</v>
       </c>
       <c r="C188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>28.2</v>
+        <v>79.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>8.6</v>
+        <v>2.4</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -28446,13 +28562,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -28460,10 +28576,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>33.7</v>
+        <v>40.4</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8</v>
+        <v>7.2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -28475,13 +28591,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>9</v>
+        <v>10.3</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -28489,10 +28605,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>25.4</v>
+        <v>10.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9</v>
+        <v>10.7</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -28510,7 +28626,7 @@
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -28518,10 +28634,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>44.5</v>
+        <v>45.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -28533,13 +28649,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>11.7</v>
+        <v>11</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -28547,10 +28663,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>42.2</v>
+        <v>52</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.9</v>
+        <v>5.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -28562,27 +28678,56 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="C193" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G193" s="4" t="n">
         <v>11.5</v>
-      </c>
-      <c r="C193" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D193" s="4" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E193" s="4" t="inlineStr">
-        <is>
-          <t>JZ</t>
-        </is>
-      </c>
-      <c r="F193" s="4" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="G193" s="4" t="n">
-        <v>11.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -28603,7 +28748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30526,24 +30671,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>12.5</v>
+        <v>17.1</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.2</v>
+        <v>3.1</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>46.7</v>
+        <v>64.7</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>6.4</v>
+        <v>4.2</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -30555,24 +30700,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.6</v>
+        <v>14.4</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>48.6</v>
+        <v>36.6</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6.2</v>
+        <v>7.6</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -30584,24 +30729,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.7</v>
+        <v>15.1</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>0.9</v>
+        <v>1.9</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>33.4</v>
+        <v>18.4</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -30613,13 +30758,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.9</v>
+        <v>15.7</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -30627,10 +30772,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>37.1</v>
+        <v>55.3</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>7.5</v>
+        <v>5.4</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -30645,21 +30790,21 @@
         <v>13.5</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>35.4</v>
+        <v>68.5</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.8</v>
+        <v>3.8</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -30671,13 +30816,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -30685,13 +30830,42 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>40.2</v>
+        <v>17.2</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>7.2</v>
+        <v>9.9</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(C67:C73)</f>
         <v/>
       </c>
     </row>
@@ -30712,7 +30886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32635,24 +32809,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.4</v>
+        <v>12.7</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>27.2</v>
+        <v>0.2</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>77.40000000000001</v>
+        <v>54.7</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>2.7</v>
+        <v>5.4</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -32664,7 +32838,7 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.5</v>
+        <v>12.8</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
@@ -32678,10 +32852,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>76.3</v>
+        <v>50.2</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>2.8</v>
+        <v>6</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -32693,13 +32867,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>13.5</v>
+        <v>13.9</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -32707,10 +32881,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>14.1</v>
+        <v>31.2</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>10.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -32722,10 +32896,10 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>1.8</v>
@@ -32736,10 +32910,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>57.2</v>
+        <v>44.7</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>5.1</v>
+        <v>6.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -32754,10 +32928,10 @@
         <v>11.3</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>10.6</v>
+        <v>11.7</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2.9</v>
+        <v>2.2</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -32765,10 +32939,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>48.4</v>
+        <v>66</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6.2</v>
+        <v>4.1</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -32780,27 +32954,56 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>2.9</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>60.6</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4.7</v>
+        <v>1</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(C67:C73)</f>
         <v/>
       </c>
     </row>
@@ -32821,7 +33024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34744,13 +34947,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.7</v>
+        <v>14</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>17.7</v>
+        <v>0</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -34758,10 +34961,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>57.9</v>
+        <v>53.2</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -34773,24 +34976,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.2</v>
+        <v>14</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>52.3</v>
+        <v>30.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>5.7</v>
+        <v>8.4</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -34802,13 +35005,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14.6</v>
+        <v>15.1</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -34816,10 +35019,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>22.1</v>
+        <v>28.4</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -34831,13 +35034,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16</v>
+        <v>16.4</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>2.7</v>
+        <v>0.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -34845,10 +35048,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>45.1</v>
+        <v>61.5</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>6.6</v>
+        <v>4.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -34860,10 +35063,10 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>10.3</v>
+        <v>11.2</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>7.5</v>
+        <v>5.7</v>
       </c>
       <c r="D71" s="4" t="n">
         <v>4.4</v>
@@ -34874,10 +35077,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>50.4</v>
+        <v>55.1</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6</v>
+        <v>5.4</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -34889,13 +35092,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.8</v>
+        <v>4.4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -34903,13 +35106,42 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>60.3</v>
+        <v>63.9</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4.8</v>
+        <v>4.3</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(C67:C73)</f>
         <v/>
       </c>
     </row>
@@ -34930,7 +35162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36853,13 +37085,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>14.1</v>
+        <v>13.3</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>17.7</v>
+        <v>5.9</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -36867,10 +37099,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>57.4</v>
+        <v>73.3</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>5.1</v>
+        <v>3.2</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -36882,24 +37114,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.2</v>
+        <v>13.9</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>54.8</v>
+        <v>48.7</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>5.4</v>
+        <v>6.2</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -36911,13 +37143,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15</v>
+        <v>14.6</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -36925,10 +37157,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>44.3</v>
+        <v>27.6</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>6.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -36940,13 +37172,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -36954,10 +37186,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>43.2</v>
+        <v>51.6</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -36969,13 +37201,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.1</v>
+        <v>12.8</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -36983,10 +37215,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>36.7</v>
+        <v>44.3</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -37001,10 +37233,10 @@
         <v>9.4</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -37012,13 +37244,42 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>50.4</v>
+        <v>42.4</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(C67:C73)</f>
         <v/>
       </c>
     </row>
@@ -37039,7 +37300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38962,24 +39223,24 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>13.5</v>
+        <v>15.6</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>5.6</v>
+        <v>0.2</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>45.8</v>
+        <v>63.9</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>6.5</v>
+        <v>4.3</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -38991,13 +39252,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.9</v>
+        <v>14.9</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -39005,10 +39266,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>50.6</v>
+        <v>29.9</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>5.9</v>
+        <v>8.4</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -39020,24 +39281,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.2</v>
+        <v>15.6</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.4</v>
+        <v>2.3</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>16.6</v>
+        <v>22</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -39049,24 +39310,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.8</v>
+        <v>16.4</v>
       </c>
       <c r="C70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D70" s="7" t="n">
-        <v>1.4</v>
-      </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>28.5</v>
+        <v>50.8</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>8.6</v>
+        <v>5.9</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -39078,13 +39339,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.4</v>
+        <v>12.2</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.4</v>
+        <v>3.7</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -39092,10 +39353,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>42.8</v>
+        <v>41.4</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -39107,13 +39368,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.2</v>
+        <v>2.3</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -39121,13 +39382,42 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>45.9</v>
+        <v>51</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>6.5</v>
+        <v>5.9</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(C67:C73)</f>
         <v/>
       </c>
     </row>
@@ -39148,7 +39438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41071,13 +41361,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>8.9</v>
+        <v>10.6</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>16.2</v>
+        <v>0</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -41085,10 +41375,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>51.8</v>
+        <v>65.2</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>5.8</v>
+        <v>4.2</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -41100,13 +41390,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -41114,10 +41404,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>49.9</v>
+        <v>41.6</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -41129,13 +41419,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -41143,10 +41433,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>23</v>
+        <v>28.3</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -41158,24 +41448,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>56.2</v>
+        <v>58</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -41187,13 +41477,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>6.9</v>
+        <v>7.7</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -41201,10 +41491,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>72.2</v>
+        <v>79.5</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -41216,13 +41506,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>5.1</v>
+        <v>4.7</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>4.3</v>
+        <v>5.2</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.4</v>
+        <v>3.4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -41230,13 +41520,42 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>71.5</v>
+        <v>86.5</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(C67:C73)</f>
         <v/>
       </c>
     </row>
@@ -41257,7 +41576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46689,24 +47008,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>20.6</v>
+        <v>22.4</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>14.2</v>
+        <v>4.7</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>76</v>
+        <v>52.4</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2.9</v>
+        <v>5.7</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -46718,24 +47037,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>21</v>
+        <v>20.5</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>6.7</v>
+        <v>4.2</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>45.1</v>
+        <v>51</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -46747,24 +47066,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>29.1</v>
+        <v>31.4</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -46776,13 +47095,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>21</v>
+        <v>20.6</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -46790,10 +47109,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>60</v>
+        <v>69.2</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -46805,24 +47124,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>21.7</v>
+        <v>21</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>58.4</v>
+        <v>56.8</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -46834,13 +47153,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>19.3</v>
+        <v>17.6</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -46848,13 +47167,42 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>17.2</v>
+        <v>13.9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.9</v>
+        <v>10.3</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -46875,7 +47223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48798,13 +49146,13 @@
         <v>46282</v>
       </c>
       <c r="B67" s="4" t="n">
-        <v>12.1</v>
+        <v>13.1</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>1.4</v>
+        <v>0.1</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
@@ -48812,10 +49160,10 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>60.6</v>
+        <v>29</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4.7</v>
+        <v>8.5</v>
       </c>
       <c r="H67" s="10">
         <f>SUM(C61:C67)</f>
@@ -48827,13 +49175,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.2</v>
+        <v>12</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -48841,10 +49189,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>43.2</v>
+        <v>43.9</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -48862,7 +49210,7 @@
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2.5</v>
+        <v>3.6</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -48870,10 +49218,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>38.1</v>
+        <v>70.2</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>7.4</v>
+        <v>3.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -48885,13 +49233,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>13</v>
+        <v>12.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>6.4</v>
+        <v>10.5</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -48899,10 +49247,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>69.90000000000001</v>
+        <v>96.7</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.6</v>
+        <v>0.4</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -48914,13 +49262,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1.5</v>
+        <v>2.3</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -48928,10 +49276,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>45.1</v>
+        <v>31.1</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -48943,13 +49291,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -48957,13 +49305,42 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>57.4</v>
+        <v>59.6</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.1</v>
+        <v>4.8</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H73" s="10">
+        <f>SUM(C67:C73)</f>
         <v/>
       </c>
     </row>
@@ -48984,7 +49361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -54416,13 +54793,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>25.6</v>
+        <v>27</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>5.7</v>
+        <v>7.5</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>4.7</v>
+        <v>6.1</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -54430,10 +54807,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>51.9</v>
+        <v>53.3</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -54445,13 +54822,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>25.9</v>
+        <v>25.7</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>2.9</v>
+        <v>11.9</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -54459,10 +54836,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>69.8</v>
+        <v>68.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -54474,24 +54851,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>5.5</v>
+        <v>8.4</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>73.59999999999999</v>
+        <v>62.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>3.2</v>
+        <v>4.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -54503,24 +54880,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>25.1</v>
+        <v>24.7</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3.4</v>
+        <v>1.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>49.6</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -54532,24 +54909,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>25.4</v>
+        <v>24.9</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0.3</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.9</v>
+        <v>2.6</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>23.2</v>
+        <v>35.1</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -54561,27 +54938,56 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>25.4</v>
+        <v>24.8</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.8</v>
+        <v>6.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>19.7</v>
+        <v>28.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.6</v>
+        <v>8.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -54602,7 +55008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -60034,13 +60440,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>14.6</v>
+        <v>16.5</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -60048,10 +60454,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>53.9</v>
+        <v>4.5</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>5.5</v>
+        <v>11.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -60063,13 +60469,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>14.4</v>
+        <v>13.8</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -60077,10 +60483,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>29.6</v>
+        <v>35.9</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8.4</v>
+        <v>7.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -60092,13 +60498,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>15.2</v>
+        <v>15.6</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -60106,10 +60512,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>5.8</v>
+        <v>18.9</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -60121,13 +60527,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>17.8</v>
+        <v>17.5</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -60135,10 +60541,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>13.3</v>
+        <v>11.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -60150,13 +60556,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.3</v>
+        <v>18.4</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -60164,10 +60570,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>36.5</v>
+        <v>25.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -60179,13 +60585,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>19.6</v>
+        <v>17.8</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -60193,13 +60599,42 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -60220,7 +60655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65652,13 +66087,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>10.4</v>
+        <v>12.2</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>7.4</v>
+        <v>14.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -65666,10 +66101,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>73.5</v>
+        <v>92.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>3.2</v>
+        <v>0.9</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -65681,24 +66116,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>15.7</v>
+        <v>22.9</v>
       </c>
       <c r="D189" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="G189" s="4" t="n">
         <v>0.8</v>
-      </c>
-      <c r="E189" s="4" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="F189" s="4" t="n">
-        <v>94.5</v>
-      </c>
-      <c r="G189" s="4" t="n">
-        <v>0.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -65713,21 +66148,21 @@
         <v>12.8</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>9.6</v>
+        <v>24.3</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>96.8</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -65742,10 +66177,10 @@
         <v>11.7</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>11.2</v>
+        <v>14.7</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -65753,10 +66188,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>93.5</v>
+        <v>96.3</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -65768,13 +66203,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>12.4</v>
+        <v>12.8</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>2.2</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -65782,10 +66217,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>81</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -65797,13 +66232,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>6.6</v>
+        <v>3.9</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -65811,13 +66246,42 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>99.3</v>
+        <v>98.8</v>
       </c>
       <c r="G193" s="4" t="n">
         <v>0.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>99.8</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -65838,7 +66302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -71270,13 +71734,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.3</v>
+        <v>17.1</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>61.3</v>
+        <v>48.2</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -71284,10 +71748,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>87</v>
+        <v>93.2</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -71302,21 +71766,21 @@
         <v>16.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>37.5</v>
+        <v>48</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>89.09999999999999</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -71328,13 +71792,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.6</v>
+        <v>18.1</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>1.6</v>
+        <v>3.1</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -71342,10 +71806,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>66</v>
+        <v>60.9</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.1</v>
+        <v>4.7</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -71357,24 +71821,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>64</v>
+        <v>49.4</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4.3</v>
+        <v>6.1</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -71386,24 +71850,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.4</v>
+        <v>17.9</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>70.09999999999999</v>
+        <v>46.9</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.6</v>
+        <v>6.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -71415,27 +71879,56 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>3.9</v>
+        <v>16</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.5</v>
+        <v>10.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -71456,7 +71949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -76888,13 +77381,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>19.2</v>
+        <v>18.9</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>55.9</v>
+        <v>29.6</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -76902,10 +77395,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>77.5</v>
+        <v>94.3</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>2.7</v>
+        <v>0.7</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -76917,13 +77410,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>32.7</v>
+        <v>21.4</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -76931,10 +77424,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>87.5</v>
+        <v>85.8</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -76946,24 +77439,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>2</v>
+        <v>6.8</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>62.1</v>
+        <v>38.3</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.5</v>
+        <v>7.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -76975,13 +77468,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20.1</v>
+        <v>19.7</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -76989,10 +77482,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>49.2</v>
+        <v>44.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.1</v>
+        <v>6.6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -77004,13 +77497,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>20.9</v>
+        <v>19.3</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -77018,10 +77511,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>71.7</v>
+        <v>48.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.4</v>
+        <v>6.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -77033,7 +77526,7 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>17.6</v>
+        <v>15.4</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
@@ -77043,17 +77536,46 @@
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>8.6</v>
+        <v>13.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11</v>
+        <v>10.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -77074,7 +77596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82506,24 +83028,24 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>17.6</v>
+        <v>18.6</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>5.8</v>
+        <v>8.9</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>28.5</v>
+        <v>49.6</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>8.6</v>
+        <v>6</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -82535,13 +83057,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17</v>
+        <v>17.1</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>10.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -82549,10 +83071,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>60.5</v>
+        <v>61.9</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -82564,24 +83086,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>1.6</v>
+        <v>4.4</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>46.9</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>6.4</v>
+        <v>4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -82593,13 +83115,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>17.6</v>
+        <v>17.1</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -82607,10 +83129,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>5.9</v>
+        <v>4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -82622,13 +83144,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>17.2</v>
+        <v>14.6</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.3</v>
+        <v>4.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -82636,10 +83158,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>72.7</v>
+        <v>39.9</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.3</v>
+        <v>7.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -82651,13 +83173,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>13.2</v>
+        <v>10.4</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -82665,13 +83187,42 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>17.2</v>
+        <v>31.1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>
@@ -82692,7 +83243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -88124,13 +88675,13 @@
         <v>46282</v>
       </c>
       <c r="B188" s="7" t="n">
-        <v>11.6</v>
+        <v>12.4</v>
       </c>
       <c r="C188" s="7" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
@@ -88138,10 +88689,10 @@
         </is>
       </c>
       <c r="F188" s="7" t="n">
-        <v>93</v>
+        <v>87.8</v>
       </c>
       <c r="G188" s="7" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="H188" s="12">
         <f>SUM(C182:C188)</f>
@@ -88153,10 +88704,10 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>0.7</v>
+        <v>2.7</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>1.1</v>
@@ -88167,10 +88718,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>66.5</v>
+        <v>79</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -88182,13 +88733,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>11.9</v>
+        <v>12.4</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -88196,10 +88747,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>63.1</v>
+        <v>55.1</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.4</v>
+        <v>5.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -88211,13 +88762,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>13.8</v>
+        <v>13.6</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -88225,10 +88776,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>75</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -88240,10 +88791,10 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>13.7</v>
+        <v>11.9</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.4</v>
+        <v>1.7</v>
       </c>
       <c r="D192" s="7" t="n">
         <v>0.5</v>
@@ -88254,10 +88805,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>83.40000000000001</v>
+        <v>93</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -88269,27 +88820,56 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>13.1</v>
+        <v>10.2</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>43.6</v>
+        <v>20.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>6.8</v>
+        <v>9.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="C194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="G194" s="7" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H194" s="12">
+        <f>SUM(C188:C194)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-18 10:14 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5974,13 +5974,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>23.5</v>
+        <v>24.8</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -5988,10 +5988,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>37.9</v>
+        <v>15.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.5</v>
+        <v>10.2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -6003,13 +6003,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.3</v>
+        <v>24.2</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -6017,10 +6017,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>21.7</v>
+        <v>22.8</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -6032,24 +6032,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>25.8</v>
+        <v>25.5</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.9</v>
+        <v>3.7</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>34.9</v>
+        <v>17.3</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7.8</v>
+        <v>9.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -6061,13 +6061,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>25.4</v>
+        <v>25.9</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -6075,10 +6075,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>27.9</v>
+        <v>6.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>11.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -6090,24 +6090,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.7</v>
+        <v>6.7</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>23.2</v>
+        <v>34.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -6119,13 +6119,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.8</v>
+        <v>20.3</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -6133,13 +6133,42 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>10.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.8</v>
+        <v>2.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -6160,7 +6189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11621,24 +11650,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.6</v>
+        <v>19.6</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>28.5</v>
+        <v>17.7</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>8.6</v>
+        <v>9.9</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -11650,7 +11679,7 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.6</v>
+        <v>18.9</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
@@ -11664,10 +11693,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>15.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10.1</v>
+        <v>11</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -11679,13 +11708,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>19.3</v>
+        <v>20.6</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -11693,10 +11722,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>6.2</v>
+        <v>0.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -11708,13 +11737,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -11722,10 +11751,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>23</v>
+        <v>49.6</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>6</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -11737,7 +11766,7 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>21.1</v>
+        <v>22.9</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
@@ -11751,10 +11780,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>1</v>
+        <v>38.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.9</v>
+        <v>7.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -11766,27 +11795,56 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.1</v>
+        <v>21.6</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>0.4</v>
+        <v>20.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>12</v>
+        <v>9.5</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -11807,7 +11865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17268,13 +17326,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>22.1</v>
+        <v>22.9</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -17282,10 +17340,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>8.9</v>
+        <v>7</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -17297,13 +17355,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -17311,10 +17369,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>19.5</v>
+        <v>9.6</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -17326,13 +17384,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>5.8</v>
+        <v>7.5</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -17340,10 +17398,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>0.6</v>
+        <v>26</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.9</v>
+        <v>8.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -17355,13 +17413,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>5.3</v>
+        <v>6.7</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -17369,10 +17427,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>43.4</v>
+        <v>6.8</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.8</v>
+        <v>11.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -17384,24 +17442,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>21.8</v>
+        <v>22.8</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>5.2</v>
+        <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5</v>
+        <v>7.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>17.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.9</v>
+        <v>11</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -17413,13 +17471,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19.9</v>
+        <v>21.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.6</v>
+        <v>7.5</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -17427,13 +17485,42 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>1.8</v>
+        <v>10.3</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.8</v>
+        <v>10.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -17454,7 +17541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22915,13 +23002,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>21.5</v>
+        <v>22.6</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>7.1</v>
+        <v>1.3</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -22929,10 +23016,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>47.9</v>
+        <v>36.4</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -22944,13 +23031,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -22958,10 +23045,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>5</v>
+        <v>8.4</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.4</v>
+        <v>11</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -22973,13 +23060,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>22.1</v>
+        <v>23.2</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -22987,10 +23074,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>42.8</v>
+        <v>19.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.9</v>
+        <v>9.6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -23002,24 +23089,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.9</v>
+        <v>22.8</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>70.5</v>
+        <v>86.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.5</v>
+        <v>1.6</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -23031,24 +23118,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>21.5</v>
+        <v>23.8</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>40.8</v>
+        <v>1.9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>7.1</v>
+        <v>11.8</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -23060,13 +23147,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19.2</v>
+        <v>22.2</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -23074,13 +23161,42 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>28.9</v>
+        <v>19.8</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8.5</v>
+        <v>9.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -23101,7 +23217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28562,24 +28678,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>11</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>40.4</v>
+        <v>8</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.2</v>
+        <v>11</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -28591,7 +28707,7 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>10.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
@@ -28601,14 +28717,14 @@
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>10.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -28620,13 +28736,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>11.8</v>
+        <v>12.4</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.1</v>
+        <v>2.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -28634,10 +28750,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>45.5</v>
+        <v>28.3</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.5</v>
+        <v>8.6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -28649,13 +28765,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -28663,10 +28779,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>52</v>
+        <v>51.1</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -28678,21 +28794,21 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>10.3</v>
+        <v>12</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="G193" s="4" t="n">
         <v>11.5</v>
@@ -28707,27 +28823,56 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>9.4</v>
+        <v>11.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>11.7</v>
+        <v>6.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.6</v>
+        <v>11.3</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -28748,7 +28893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30700,24 +30845,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>14.4</v>
+        <v>15.7</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>36.6</v>
+        <v>69.2</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>7.6</v>
+        <v>3.7</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -30729,24 +30874,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.1</v>
+        <v>15.5</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>18.4</v>
+        <v>21.1</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -30758,13 +30903,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.7</v>
+        <v>16.9</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -30772,10 +30917,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>55.3</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>5.4</v>
+        <v>3.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -30787,24 +30932,24 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>13.5</v>
+        <v>13.8</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>68.5</v>
+        <v>44.5</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>3.8</v>
+        <v>6.7</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -30816,24 +30961,24 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>17.2</v>
+        <v>42</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>9.9</v>
+        <v>7</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -30845,27 +30990,56 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>5.4</v>
+        <v>2.9</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>39.6</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>0.4</v>
+        <v>7.2</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="H74" s="12">
+        <f>SUM(C68:C74)</f>
         <v/>
       </c>
     </row>
@@ -30886,7 +31060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32838,13 +33012,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12.8</v>
+        <v>14.9</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -32852,10 +33026,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>50.2</v>
+        <v>41.2</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6</v>
+        <v>7.1</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -32867,7 +33041,7 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>13.9</v>
+        <v>14.1</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
@@ -32881,10 +33055,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>31.2</v>
+        <v>28.6</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -32896,13 +33070,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>14.6</v>
+        <v>15.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.2</v>
+        <v>16.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -32910,10 +33084,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>44.7</v>
+        <v>68.3</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>6.6</v>
+        <v>3.8</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -32925,24 +33099,24 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.3</v>
+        <v>11.5</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>11.7</v>
+        <v>6.8</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>66</v>
+        <v>37.5</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>4.1</v>
+        <v>7.5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -32954,13 +33128,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>3.9</v>
+        <v>6.1</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -32968,10 +33142,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>91.40000000000001</v>
+        <v>54.1</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -32983,27 +33157,56 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C73" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D73" s="4" t="n">
         <v>2.4</v>
       </c>
-      <c r="D73" s="4" t="n">
-        <v>4.4</v>
-      </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>85.90000000000001</v>
+        <v>57.4</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>1.7</v>
+        <v>5.1</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H74" s="12">
+        <f>SUM(C68:C74)</f>
         <v/>
       </c>
     </row>
@@ -33024,7 +33227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34976,24 +35179,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>14</v>
+        <v>15.4</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>30.3</v>
+        <v>47.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>8.4</v>
+        <v>6.3</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -35005,7 +35208,7 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.1</v>
+        <v>15.7</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
@@ -35015,14 +35218,14 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>28.4</v>
+        <v>29.1</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -35034,24 +35237,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.4</v>
+        <v>16.7</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.2</v>
+        <v>10.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>61.5</v>
+        <v>67.7</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.6</v>
+        <v>3.9</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -35063,13 +35266,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>5.7</v>
+        <v>1.9</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -35077,10 +35280,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>55.1</v>
+        <v>37.7</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>5.4</v>
+        <v>7.5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -35092,13 +35295,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.4</v>
+        <v>3.8</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -35106,10 +35309,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>63.9</v>
+        <v>76</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -35121,27 +35324,56 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>5.4</v>
+        <v>3.3</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>95.7</v>
+        <v>44.3</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>0.5</v>
+        <v>6.7</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H74" s="12">
+        <f>SUM(C68:C74)</f>
         <v/>
       </c>
     </row>
@@ -35162,7 +35394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37114,24 +37346,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>13.9</v>
+        <v>14.7</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>48.7</v>
+        <v>74.5</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6.2</v>
+        <v>3.1</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -37143,13 +37375,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -37157,7 +37389,7 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>27.6</v>
+        <v>27.7</v>
       </c>
       <c r="G69" s="4" t="n">
         <v>8.699999999999999</v>
@@ -37172,13 +37404,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.9</v>
+        <v>16.8</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -37186,10 +37418,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>51.6</v>
+        <v>73.5</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>5.8</v>
+        <v>3.2</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -37201,13 +37433,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>3.8</v>
+        <v>0.2</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -37215,10 +37447,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>44.3</v>
+        <v>33.6</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6.7</v>
+        <v>8</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -37230,13 +37462,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -37244,10 +37476,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>42.4</v>
+        <v>47.5</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -37259,27 +37491,56 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>7</v>
+        <v>4.6</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>99.59999999999999</v>
+        <v>53.7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H74" s="12">
+        <f>SUM(C68:C74)</f>
         <v/>
       </c>
     </row>
@@ -37300,7 +37561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39252,24 +39513,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>14.9</v>
+        <v>16.3</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>29.9</v>
+        <v>39.8</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -39281,13 +39542,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.6</v>
+        <v>16.4</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -39295,10 +39556,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>22</v>
+        <v>25.6</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>9.4</v>
+        <v>8.9</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -39310,24 +39571,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.4</v>
+        <v>17</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>50.8</v>
+        <v>63.3</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>5.9</v>
+        <v>4.4</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -39339,13 +39600,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.2</v>
+        <v>12</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>2.6</v>
+        <v>0.2</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -39353,10 +39614,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>41.4</v>
+        <v>35.3</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -39368,10 +39629,10 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>2.3</v>
+        <v>0.3</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>3.6</v>
@@ -39382,10 +39643,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -39397,27 +39658,56 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>10.3</v>
+        <v>10.1</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>4.2</v>
+        <v>2.5</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>85.5</v>
+        <v>35.1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>1.7</v>
+        <v>7.8</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H74" s="12">
+        <f>SUM(C68:C74)</f>
         <v/>
       </c>
     </row>
@@ -39438,7 +39728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41390,24 +41680,24 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>10.4</v>
+        <v>11.8</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>41.6</v>
+        <v>45.3</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -41419,13 +41709,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>11.5</v>
+        <v>12.1</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -41433,10 +41723,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>28.3</v>
+        <v>42.4</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.6</v>
+        <v>6.9</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -41448,13 +41738,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12.5</v>
+        <v>13.1</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.1</v>
+        <v>10.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -41462,10 +41752,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>58</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>5</v>
+        <v>4.1</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -41477,13 +41767,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>7.7</v>
+        <v>7</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>7.5</v>
+        <v>4.8</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.9</v>
+        <v>4.3</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -41491,10 +41781,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>79.5</v>
+        <v>73.2</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -41506,13 +41796,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -41520,10 +41810,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>86.5</v>
+        <v>76.3</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -41538,10 +41828,10 @@
         <v>5.3</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>3.4</v>
+        <v>0.8</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>4.1</v>
+        <v>2.3</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -41549,13 +41839,42 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>97.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>0.3</v>
+        <v>3.8</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H74" s="12">
+        <f>SUM(C68:C74)</f>
         <v/>
       </c>
     </row>
@@ -41576,7 +41895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47037,13 +47356,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>20.5</v>
+        <v>20.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>4.2</v>
+        <v>1.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -47051,10 +47370,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>51</v>
+        <v>44.4</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>5.9</v>
+        <v>6.7</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -47066,24 +47385,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>31.4</v>
+        <v>28.1</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -47095,24 +47414,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20.6</v>
+        <v>21.1</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>69.2</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>3.7</v>
+        <v>4.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -47124,24 +47443,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>56.8</v>
+        <v>70.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.2</v>
+        <v>3.5</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -47153,24 +47472,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>17.6</v>
+        <v>19.9</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>13.9</v>
+        <v>27.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -47182,27 +47501,56 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>16.1</v>
+        <v>18.7</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>31.1</v>
+        <v>80.3</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>2.4</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -47223,7 +47571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49175,13 +49523,13 @@
         <v>46283</v>
       </c>
       <c r="B68" s="7" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
@@ -49189,10 +49537,10 @@
         </is>
       </c>
       <c r="F68" s="7" t="n">
-        <v>43.9</v>
+        <v>49.9</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>6.7</v>
+        <v>6</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(C62:C68)</f>
@@ -49204,13 +49552,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.3</v>
+        <v>12.8</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -49218,10 +49566,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>70.2</v>
+        <v>61</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -49233,13 +49581,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>10.5</v>
+        <v>11.7</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -49247,10 +49595,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>96.7</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>0.4</v>
+        <v>2.4</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -49262,13 +49610,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -49276,10 +49624,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>31.1</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>4.2</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -49291,13 +49639,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -49305,10 +49653,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>59.6</v>
+        <v>66.2</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4.8</v>
+        <v>4.1</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -49320,27 +49668,56 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>5.3</v>
+        <v>2.2</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>49.8</v>
+        <v>11.5</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>6</v>
+        <v>10.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H74" s="12">
+        <f>SUM(C68:C74)</f>
         <v/>
       </c>
     </row>
@@ -49361,7 +49738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -54822,13 +55199,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>25.7</v>
+        <v>26.4</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>11.9</v>
+        <v>6.9</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>6.6</v>
+        <v>6.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -54836,10 +55213,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>68.2</v>
+        <v>55.8</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>3.8</v>
+        <v>5.3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -54851,24 +55228,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>8.4</v>
+        <v>28</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>62.7</v>
+        <v>75</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -54880,24 +55257,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>24.7</v>
+        <v>25.1</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>1.8</v>
+        <v>3.9</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.8</v>
+        <v>4.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>66.40000000000001</v>
+        <v>44.2</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4</v>
+        <v>6.7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -54909,24 +55286,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0.3</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>35.1</v>
+        <v>18.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>7.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -54938,13 +55315,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>24.8</v>
+        <v>25.4</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>6.2</v>
+        <v>3.6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -54952,10 +55329,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>28.3</v>
+        <v>33.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.6</v>
+        <v>8</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -54967,13 +55344,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>23.5</v>
+        <v>25.3</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>6.5</v>
+        <v>5.3</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -54981,13 +55358,42 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -55008,7 +55414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -60469,7 +60875,7 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>13.8</v>
+        <v>16.3</v>
       </c>
       <c r="C189" s="4" t="n">
         <v>0</v>
@@ -60479,14 +60885,14 @@
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>35.9</v>
+        <v>33.2</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -60498,13 +60904,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>15.6</v>
+        <v>15.9</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -60512,10 +60918,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>18.9</v>
+        <v>7.8</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>11.1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -60527,13 +60933,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>17.5</v>
+        <v>17.9</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -60541,10 +60947,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>11.7</v>
+        <v>7.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -60556,13 +60962,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>18.4</v>
+        <v>19.2</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -60570,10 +60976,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>25.4</v>
+        <v>21.3</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -60585,7 +60991,7 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>17.8</v>
+        <v>19.2</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
@@ -60599,10 +61005,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>3.5</v>
+        <v>10.9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.6</v>
+        <v>10.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -60614,7 +61020,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>17.6</v>
+        <v>18.2</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -60628,13 +61034,42 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G194" s="7" t="n">
         <v>12</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -60655,7 +61090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66116,24 +66551,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>11.7</v>
+        <v>10.9</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>22.9</v>
+        <v>14.9</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>93.2</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -66145,24 +66580,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>12.8</v>
+        <v>12.2</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>24.3</v>
+        <v>39.8</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>91.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -66174,13 +66609,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>14.7</v>
+        <v>20</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.3</v>
+        <v>1.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -66188,7 +66623,7 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>96.3</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G191" s="4" t="n">
         <v>0.4</v>
@@ -66203,13 +66638,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>12.8</v>
+        <v>12.3</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -66217,10 +66652,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>76.59999999999999</v>
+        <v>83</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -66235,7 +66670,7 @@
         <v>12.2</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
         <v>0.7</v>
@@ -66246,10 +66681,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>98.8</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -66261,27 +66696,56 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>8.1</v>
+        <v>5.7</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>0.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>99.8</v>
+        <v>100</v>
       </c>
       <c r="G194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -66302,7 +66766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -71763,24 +72227,24 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>16.9</v>
+        <v>18.7</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>48</v>
+        <v>24.8</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>85.09999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -71792,13 +72256,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>3.1</v>
+        <v>11.5</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -71806,10 +72270,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>60.9</v>
+        <v>46.2</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4.7</v>
+        <v>6.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -71821,24 +72285,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18.1</v>
+        <v>18.7</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>49.4</v>
+        <v>55.8</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -71850,24 +72314,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>17.9</v>
+        <v>19.1</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.5</v>
+        <v>2.8</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>46.9</v>
+        <v>65.2</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.4</v>
+        <v>4.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -71879,24 +72343,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>15</v>
+        <v>16.4</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>16</v>
+        <v>24.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -71914,21 +72378,50 @@
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -71949,7 +72442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -77410,13 +77903,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>18.8</v>
+        <v>19.8</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>21.4</v>
+        <v>13.2</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -77424,10 +77917,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>85.8</v>
+        <v>93.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -77442,21 +77935,21 @@
         <v>19.5</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>6.8</v>
+        <v>11.5</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>38.3</v>
+        <v>40.3</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -77468,24 +77961,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>19.7</v>
+        <v>20.5</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>44.9</v>
+        <v>40.1</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.6</v>
+        <v>7.2</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -77497,24 +77990,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.3</v>
+        <v>20.1</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>48.5</v>
+        <v>56.6</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.2</v>
+        <v>5.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -77526,24 +78019,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>15.4</v>
+        <v>17.2</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>13.3</v>
+        <v>21.1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.4</v>
+        <v>9.5</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -77555,27 +78048,56 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.7</v>
+        <v>15.5</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>3.3</v>
+        <v>6.8</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.6</v>
+        <v>11.2</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -77596,7 +78118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83057,13 +83579,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>17.1</v>
+        <v>18.6</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>1.7</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -83071,10 +83593,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>61.9</v>
+        <v>49.5</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>4.6</v>
+        <v>6.1</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -83086,24 +83608,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>17.6</v>
+        <v>16.6</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>4.4</v>
+        <v>67.7</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>66.40000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -83115,24 +83637,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>17.1</v>
+        <v>17.6</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>67</v>
+        <v>45.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4</v>
+        <v>6.5</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -83144,13 +83666,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>14.6</v>
+        <v>16.6</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>2.8</v>
+        <v>0.1</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -83158,10 +83680,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>39.9</v>
+        <v>39.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -83173,13 +83695,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>10.4</v>
+        <v>12.4</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>6.1</v>
+        <v>5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -83187,10 +83709,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>31.1</v>
+        <v>26.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -83202,13 +83724,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>10.7</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>6.1</v>
+        <v>4.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -83216,13 +83738,42 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>55.9</v>
+        <v>6.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>5.3</v>
+        <v>11.3</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>
@@ -83243,7 +83794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -88704,13 +89255,13 @@
         <v>46283</v>
       </c>
       <c r="B189" s="4" t="n">
-        <v>11.8</v>
+        <v>12.3</v>
       </c>
       <c r="C189" s="4" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
@@ -88718,10 +89269,10 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>79</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="G189" s="4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H189" s="10">
         <f>SUM(C183:C189)</f>
@@ -88733,10 +89284,10 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1.2</v>
@@ -88747,10 +89298,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>55.1</v>
+        <v>57.6</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -88762,13 +89313,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>13.6</v>
+        <v>14.8</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -88776,10 +89327,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>81.09999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>2.3</v>
+        <v>3.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -88791,24 +89342,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>11.9</v>
+        <v>12.8</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>1.7</v>
+        <v>0.1</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>93</v>
+        <v>90.8</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -88820,7 +89371,7 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>10.2</v>
+        <v>12.8</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
@@ -88830,14 +89381,14 @@
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>20.3</v>
+        <v>3.9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.6</v>
+        <v>11.5</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -88849,27 +89400,56 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>10.4</v>
+        <v>13.4</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>11.3</v>
+        <v>7.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B195" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H195" s="10">
+        <f>SUM(C189:C195)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-19 09:56 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6003,13 +6003,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.2</v>
+        <v>25.1</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -6017,10 +6017,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>22.8</v>
+        <v>69.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>3.7</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -6032,24 +6032,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>25.5</v>
+        <v>25.2</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>17.3</v>
+        <v>52.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.9</v>
+        <v>5.7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -6061,13 +6061,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>25.9</v>
+        <v>25.4</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -6075,10 +6075,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>6.4</v>
+        <v>10.6</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>11.2</v>
+        <v>10.7</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -6090,24 +6090,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>6.7</v>
+        <v>12.1</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>34.6</v>
+        <v>36.4</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -6119,24 +6119,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.3</v>
+        <v>19.4</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>3</v>
+        <v>0.1</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>2.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>82.59999999999999</v>
+        <v>34</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>2.1</v>
+        <v>7.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -6148,27 +6148,56 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>33.2</v>
+        <v>13.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8</v>
+        <v>10.3</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -6189,7 +6218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11679,13 +11708,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.9</v>
+        <v>20.9</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -11693,10 +11722,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>3.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11</v>
+        <v>11.6</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -11722,10 +11751,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>0.5</v>
+        <v>4.3</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -11737,13 +11766,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.2</v>
+        <v>23.5</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -11751,10 +11780,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>49.6</v>
+        <v>23.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -11766,24 +11795,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>22.9</v>
+        <v>23.1</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>38.3</v>
+        <v>2.1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>7.4</v>
+        <v>11.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -11795,13 +11824,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -11809,10 +11838,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>20.9</v>
+        <v>4.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.5</v>
+        <v>11.4</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -11824,13 +11853,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>21.4</v>
+        <v>21.6</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -11838,13 +11867,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>17</v>
+        <v>21.1</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -11865,7 +11923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17355,13 +17413,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.6</v>
+        <v>23.2</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -17369,10 +17427,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>9.6</v>
+        <v>46.9</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10.8</v>
+        <v>6.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -17390,7 +17448,7 @@
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -17398,10 +17456,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>26</v>
+        <v>55.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>8.9</v>
+        <v>5.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -17413,13 +17471,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.5</v>
+        <v>22.4</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>6.7</v>
+        <v>7.9</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -17427,10 +17485,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>6.8</v>
+        <v>1.9</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>11.2</v>
+        <v>11.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -17442,13 +17500,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>7.2</v>
+        <v>5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -17456,10 +17514,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>17.9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11</v>
+        <v>9.9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -17471,13 +17529,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>21.9</v>
+        <v>19.9</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>7.5</v>
+        <v>8.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -17485,10 +17543,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>10.3</v>
+        <v>10.8</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -17500,13 +17558,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>20.4</v>
+        <v>19.7</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -17521,6 +17579,35 @@
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -17541,7 +17628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23031,24 +23118,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>22.2</v>
+        <v>24.3</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>2.8</v>
+        <v>1.2</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>8.4</v>
+        <v>11.8</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -23060,13 +23147,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>23.2</v>
+        <v>23.3</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -23074,10 +23161,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>19.9</v>
+        <v>39.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>9.6</v>
+        <v>7.2</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -23089,24 +23176,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.8</v>
+        <v>23.8</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.1</v>
+        <v>2.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>86.5</v>
+        <v>84.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -23118,24 +23205,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>1.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.8</v>
+        <v>10.9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -23147,13 +23234,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>22.2</v>
+        <v>22</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -23161,10 +23248,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>19.8</v>
+        <v>58.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.6</v>
+        <v>5</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -23176,13 +23263,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>21</v>
+        <v>20.6</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -23190,13 +23277,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>32.4</v>
+        <v>43</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8.1</v>
+        <v>6.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -23217,7 +23333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28707,24 +28823,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>13</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>15.5</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>10.8</v>
+        <v>10.1</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -28736,7 +28852,7 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>12.4</v>
+        <v>12.2</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
@@ -28746,14 +28862,14 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>28.3</v>
+        <v>55.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>8.6</v>
+        <v>5.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -28765,13 +28881,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -28779,10 +28895,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>51.1</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.9</v>
+        <v>3.7</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -28794,24 +28910,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>4.1</v>
+        <v>12.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.5</v>
+        <v>10.5</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -28823,7 +28939,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>11.9</v>
+        <v>11.6</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -28837,10 +28953,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>6.2</v>
+        <v>10.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.3</v>
+        <v>10.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -28858,21 +28974,50 @@
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -28893,7 +29038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30874,13 +31019,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.5</v>
+        <v>17.6</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -30888,10 +31033,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>21.1</v>
+        <v>35.8</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>9.5</v>
+        <v>7.7</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -30903,13 +31048,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.9</v>
+        <v>16.6</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.3</v>
+        <v>11</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -30917,10 +31062,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>69.90000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -30932,13 +31077,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>13.8</v>
+        <v>12.1</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1.5</v>
+        <v>11.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -30946,10 +31091,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>44.5</v>
+        <v>36.7</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6.7</v>
+        <v>7.6</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -30961,24 +31106,24 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>10</v>
+        <v>9.6</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.8</v>
+        <v>4</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -30990,24 +31135,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>11.1</v>
+        <v>10.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.9</v>
+        <v>2.2</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>39.6</v>
+        <v>11.9</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>7.2</v>
+        <v>10.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -31019,7 +31164,7 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>10.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C74" s="7" t="n">
         <v>0</v>
@@ -31029,17 +31174,46 @@
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>31.6</v>
+        <v>9</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H75" s="10">
+        <f>SUM(C69:C75)</f>
         <v/>
       </c>
     </row>
@@ -31060,7 +31234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33041,13 +33215,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14.1</v>
+        <v>15.9</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -33055,10 +33229,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>28.6</v>
+        <v>46.6</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.6</v>
+        <v>6.4</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -33070,13 +33244,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.5</v>
+        <v>15.1</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>16.2</v>
+        <v>13</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -33084,10 +33258,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>68.3</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -33099,13 +33273,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>6.8</v>
+        <v>22.2</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -33113,10 +33287,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>37.5</v>
+        <v>49.3</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.5</v>
+        <v>6.1</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -33128,13 +33302,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>6.1</v>
+        <v>5.2</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -33142,10 +33316,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>54.1</v>
+        <v>71.3</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.5</v>
+        <v>3.4</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -33157,13 +33331,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -33171,10 +33345,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>57.4</v>
+        <v>45.3</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>5.1</v>
+        <v>6.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -33186,13 +33360,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -33200,13 +33374,42 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>40.6</v>
+        <v>52.9</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>7.1</v>
+        <v>5.7</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H75" s="10">
+        <f>SUM(C69:C75)</f>
         <v/>
       </c>
     </row>
@@ -33227,7 +33430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35208,13 +35411,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15.7</v>
+        <v>16.7</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -35222,10 +35425,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>29.1</v>
+        <v>44.8</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.5</v>
+        <v>6.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -35237,10 +35440,10 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.7</v>
+        <v>16.2</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>10.2</v>
+        <v>11.4</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>2.9</v>
@@ -35251,10 +35454,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>67.7</v>
+        <v>74.3</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -35266,13 +35469,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.1</v>
+        <v>9.5</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -35280,10 +35483,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>37.7</v>
+        <v>40.1</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -35295,13 +35498,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -35309,10 +35512,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>76</v>
+        <v>69.7</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -35324,24 +35527,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>44.3</v>
+        <v>24.6</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>6.7</v>
+        <v>9</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -35353,27 +35556,56 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>27.6</v>
+        <v>67</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H75" s="10">
+        <f>SUM(C69:C75)</f>
         <v/>
       </c>
     </row>
@@ -35394,7 +35626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37375,24 +37607,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>15</v>
+        <v>16.2</v>
       </c>
       <c r="C69" s="4" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="D69" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>27.7</v>
+        <v>41.1</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -37404,13 +37636,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.8</v>
+        <v>16.4</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>1.7</v>
+        <v>11.6</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -37418,10 +37650,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>73.5</v>
+        <v>65.3</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.2</v>
+        <v>4.2</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -37433,13 +37665,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.7</v>
+        <v>11.2</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0.2</v>
+        <v>3.3</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -37447,10 +37679,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>33.6</v>
+        <v>29.5</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -37462,13 +37694,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -37476,10 +37708,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>47.5</v>
+        <v>53.7</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>6.3</v>
+        <v>5.6</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -37491,24 +37723,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>4.6</v>
+        <v>3.3</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>53.7</v>
+        <v>20.1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>5.6</v>
+        <v>9.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -37520,27 +37752,56 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>10</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>25.6</v>
+        <v>23.6</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H75" s="10">
+        <f>SUM(C69:C75)</f>
         <v/>
       </c>
     </row>
@@ -37561,7 +37822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39542,24 +39803,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>16.4</v>
+        <v>17.5</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>25.6</v>
+        <v>28.3</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -39571,13 +39832,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>17</v>
+        <v>16.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>1.5</v>
+        <v>11.5</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -39585,10 +39846,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>63.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -39600,13 +39861,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12</v>
+        <v>10.5</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0.2</v>
+        <v>5.2</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -39614,10 +39875,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>35.3</v>
+        <v>28.8</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -39629,13 +39890,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.6</v>
+        <v>8.9</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -39643,10 +39904,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>52</v>
+        <v>44.5</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -39658,24 +39919,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>10.1</v>
+        <v>10.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>35.1</v>
+        <v>26.8</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>7.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -39687,27 +39948,56 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>29.1</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>8.5</v>
+        <v>3.5</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H75" s="10">
+        <f>SUM(C69:C75)</f>
         <v/>
       </c>
     </row>
@@ -39728,7 +40018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41709,24 +41999,24 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.1</v>
+        <v>13.2</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>42.4</v>
+        <v>58</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>6.9</v>
+        <v>5</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -41738,10 +42028,10 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>10.2</v>
+        <v>11.9</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>2.6</v>
@@ -41752,10 +42042,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>65.59999999999999</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -41767,13 +42057,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>7</v>
+        <v>5.7</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>4.8</v>
+        <v>14.1</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -41781,10 +42071,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>73.2</v>
+        <v>76.8</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -41796,13 +42086,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>5.5</v>
+        <v>7.6</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -41810,10 +42100,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>76.3</v>
+        <v>83.8</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -41825,13 +42115,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -41839,10 +42129,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>68.40000000000001</v>
+        <v>61.9</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>3.8</v>
+        <v>4.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -41854,27 +42144,56 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>5.1</v>
+        <v>6.7</v>
       </c>
       <c r="C74" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>70.3</v>
+        <v>61.9</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.6</v>
+        <v>4.6</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="H75" s="10">
+        <f>SUM(C69:C75)</f>
         <v/>
       </c>
     </row>
@@ -41895,7 +42214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47385,7 +47704,7 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>19.9</v>
+        <v>22.4</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
@@ -47395,14 +47714,14 @@
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>28.1</v>
+        <v>31.2</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -47428,10 +47747,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>64.40000000000001</v>
+        <v>61.1</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -47443,24 +47762,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>21.6</v>
+        <v>21.7</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>70.5</v>
+        <v>74.3</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -47472,13 +47791,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>19.9</v>
+        <v>19.5</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -47486,10 +47805,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>27.3</v>
+        <v>29.9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -47501,13 +47820,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -47515,10 +47834,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>80.3</v>
+        <v>42</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>2.4</v>
+        <v>7</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -47530,13 +47849,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>18.9</v>
+        <v>18</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -47544,13 +47863,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>64.8</v>
+        <v>68.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -47571,7 +47919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49552,13 +49900,13 @@
         <v>46284</v>
       </c>
       <c r="B69" s="4" t="n">
-        <v>12.8</v>
+        <v>14.8</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>3.8</v>
+        <v>4.8</v>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
@@ -49566,10 +49914,10 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>61</v>
+        <v>77.8</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>4.7</v>
+        <v>2.7</v>
       </c>
       <c r="H69" s="10">
         <f>SUM(C63:C69)</f>
@@ -49581,13 +49929,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>11.7</v>
+        <v>7.9</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -49595,10 +49943,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>79.59999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -49610,13 +49958,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1.9</v>
+        <v>9.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.7</v>
+        <v>5.1</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -49624,10 +49972,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>65.40000000000001</v>
+        <v>39.7</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>4.2</v>
+        <v>7.2</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -49639,13 +49987,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -49653,10 +50001,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>66.2</v>
+        <v>77.5</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4.1</v>
+        <v>2.7</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -49668,13 +50016,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -49682,10 +50030,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>11.5</v>
+        <v>59</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>10.6</v>
+        <v>4.9</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -49697,27 +50045,56 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>43.4</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>10.9</v>
+        <v>6.8</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H75" s="10">
+        <f>SUM(C69:C75)</f>
         <v/>
       </c>
     </row>
@@ -49738,7 +50115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -55228,13 +55605,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>24.8</v>
+        <v>24.1</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>28</v>
+        <v>17.5</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>4.7</v>
+        <v>4.1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -55242,7 +55619,7 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>75</v>
+        <v>75.3</v>
       </c>
       <c r="G190" s="7" t="n">
         <v>3</v>
@@ -55257,13 +55634,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>25.1</v>
+        <v>24.1</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>3.9</v>
+        <v>19.2</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -55271,10 +55648,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>44.2</v>
+        <v>57</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.7</v>
+        <v>5.2</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -55286,24 +55663,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.3</v>
+        <v>2.6</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>18.4</v>
+        <v>23.1</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -55315,24 +55692,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>25.4</v>
+        <v>25.1</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>33.6</v>
+        <v>50.4</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -55344,13 +55721,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>25.3</v>
+        <v>24.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -55358,10 +55735,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -55373,13 +55750,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>23.9</v>
+        <v>23.2</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -55387,13 +55764,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>3.3</v>
+        <v>10.6</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>11.6</v>
+        <v>10.7</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -55414,7 +55820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -60904,13 +61310,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>15.9</v>
+        <v>18.1</v>
       </c>
       <c r="C190" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -60918,10 +61324,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>7.8</v>
+        <v>6</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -60933,13 +61339,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -60947,10 +61353,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>7.9</v>
+        <v>6.2</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -60962,24 +61368,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.2</v>
+        <v>20.1</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>21.3</v>
+        <v>24.6</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.4</v>
+        <v>9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -60991,24 +61397,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>19.2</v>
+        <v>18.8</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>10.9</v>
+        <v>0.2</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.7</v>
+        <v>12</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -61020,13 +61426,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -61034,7 +61440,7 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G194" s="7" t="n">
         <v>12</v>
@@ -61049,13 +61455,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>17.7</v>
+        <v>17.9</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -61063,13 +61469,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>3.5</v>
+        <v>0.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>11.6</v>
+        <v>11.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -61090,7 +61525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66580,13 +67015,13 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>12.2</v>
+        <v>11.4</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>39.8</v>
+        <v>15.9</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
@@ -66594,10 +67029,10 @@
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>94.7</v>
+        <v>96.3</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -66609,13 +67044,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>11.6</v>
+        <v>11</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>20</v>
+        <v>29.1</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -66623,10 +67058,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>95</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -66644,18 +67079,18 @@
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>83</v>
+        <v>51.8</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2</v>
+        <v>5.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -66667,24 +67102,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12.2</v>
+        <v>13.1</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>99.59999999999999</v>
+        <v>98.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -66696,21 +67131,21 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>5.7</v>
+        <v>11.1</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>0.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>100</v>
+        <v>99.8</v>
       </c>
       <c r="G194" s="7" t="n">
         <v>0</v>
@@ -66725,13 +67160,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>4.1</v>
+        <v>2.5</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -66739,13 +67174,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>93.09999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -66766,7 +67230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -72256,24 +72720,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>18.2</v>
+        <v>20.1</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>11.5</v>
+        <v>1.5</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>46.2</v>
+        <v>10.4</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>6.5</v>
+        <v>10.8</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -72285,13 +72749,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18.7</v>
+        <v>18.6</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -72299,10 +72763,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>55.8</v>
+        <v>51.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -72317,10 +72781,10 @@
         <v>19.1</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.8</v>
+        <v>4.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -72328,10 +72792,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>65.2</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -72343,13 +72807,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>16.4</v>
+        <v>15.8</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.8</v>
+        <v>4.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -72357,10 +72821,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>24.6</v>
+        <v>23.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -72372,24 +72836,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.3</v>
+        <v>13.8</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.2</v>
+        <v>2.2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.9</v>
+        <v>8.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -72401,13 +72865,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>13.4</v>
+        <v>15.5</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -72415,13 +72879,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>28.7</v>
+        <v>45.3</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8.6</v>
+        <v>6.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -72442,7 +72935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -77932,24 +78425,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>19.5</v>
+        <v>22</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>11.5</v>
+        <v>1.4</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>40.3</v>
+        <v>12.4</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>7.2</v>
+        <v>10.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -77961,13 +78454,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20.5</v>
+        <v>20.7</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -77975,10 +78468,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>40.1</v>
+        <v>49.2</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7.2</v>
+        <v>6.1</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -77990,24 +78483,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>20.1</v>
+        <v>20.6</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>56.6</v>
+        <v>55.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -78019,24 +78512,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>17.2</v>
+        <v>16.4</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>21.1</v>
+        <v>14.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.5</v>
+        <v>10.2</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -78048,13 +78541,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>15.5</v>
+        <v>14.8</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -78062,10 +78555,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>6.8</v>
+        <v>19.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -78077,27 +78570,56 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>14.6</v>
+        <v>17</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>26.8</v>
+        <v>57.6</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>5.1</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -78118,7 +78640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83608,24 +84130,24 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>16.6</v>
+        <v>17.4</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>67.7</v>
+        <v>13.6</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>71.5</v>
+        <v>46.1</v>
       </c>
       <c r="G190" s="7" t="n">
-        <v>3.4</v>
+        <v>6.5</v>
       </c>
       <c r="H190" s="12">
         <f>SUM(C184:C190)</f>
@@ -83637,24 +84159,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>45.7</v>
+        <v>43.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -83666,13 +84188,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>16.6</v>
+        <v>16.4</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -83680,10 +84202,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>39.4</v>
+        <v>55.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>7.3</v>
+        <v>5.3</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -83695,13 +84217,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12.4</v>
+        <v>11.8</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -83709,10 +84231,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>26.6</v>
+        <v>22.1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -83724,13 +84246,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>4.9</v>
+        <v>3.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -83738,10 +84260,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>6.2</v>
+        <v>1.6</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.3</v>
+        <v>11.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -83753,27 +84275,56 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>11.3</v>
+        <v>12.4</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>0</v>
+        <v>31.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>12</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>
@@ -83794,7 +84345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -89284,21 +89835,21 @@
         <v>46284</v>
       </c>
       <c r="B190" s="7" t="n">
-        <v>12.5</v>
+        <v>14.6</v>
       </c>
       <c r="C190" s="7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F190" s="7" t="n">
-        <v>57.6</v>
+        <v>57.1</v>
       </c>
       <c r="G190" s="7" t="n">
         <v>5.1</v>
@@ -89313,13 +89864,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>14.8</v>
+        <v>14.7</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -89327,10 +89878,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>67.7</v>
+        <v>75.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -89342,13 +89893,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -89356,10 +89907,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>90.8</v>
+        <v>78</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>1.1</v>
+        <v>2.6</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -89371,13 +89922,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12.8</v>
+        <v>12.6</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -89385,10 +89936,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>3.9</v>
+        <v>11.9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.5</v>
+        <v>10.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -89400,24 +89951,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.4</v>
+        <v>14.2</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>7.2</v>
+        <v>3.5</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.1</v>
+        <v>11.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -89429,13 +89980,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>15.6</v>
+        <v>14.8</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -89443,13 +89994,42 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>45.5</v>
+        <v>37.3</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="11" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="C196" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="G196" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H196" s="12">
+        <f>SUM(C190:C196)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-20 10:16 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6032,21 +6032,21 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>25.2</v>
+        <v>26.1</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>52.9</v>
+        <v>52.3</v>
       </c>
       <c r="G191" s="4" t="n">
         <v>5.7</v>
@@ -6061,24 +6061,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>25.4</v>
+        <v>25.1</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>10.6</v>
+        <v>16.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>10.7</v>
+        <v>10</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -6090,24 +6090,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>22.9</v>
+        <v>22.4</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>12.1</v>
+        <v>16.1</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>36.4</v>
+        <v>32.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>7.6</v>
+        <v>8.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -6119,13 +6119,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19.4</v>
+        <v>19.5</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -6133,10 +6133,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>34</v>
+        <v>51.5</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>7.9</v>
+        <v>5.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -6148,24 +6148,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19.7</v>
+        <v>19.2</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>13.8</v>
+        <v>30.7</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -6177,13 +6177,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.6</v>
+        <v>19.7</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -6191,13 +6191,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>56.2</v>
+        <v>18.2</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>5.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -6218,7 +6247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11737,13 +11766,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20.6</v>
+        <v>23.2</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -11751,10 +11780,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>4.3</v>
+        <v>5.3</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -11766,13 +11795,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.5</v>
+        <v>23.2</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -11780,10 +11809,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>23.4</v>
+        <v>24.2</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -11795,24 +11824,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23.1</v>
+        <v>23.4</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>2.1</v>
+        <v>8.5</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.7</v>
+        <v>11</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -11824,13 +11853,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -11838,10 +11867,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>4.9</v>
+        <v>0.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -11853,7 +11882,7 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>21.6</v>
+        <v>22.1</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
@@ -11867,10 +11896,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>21.1</v>
+        <v>59.4</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>9.5</v>
+        <v>4.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -11882,13 +11911,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>23.4</v>
+        <v>23.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -11896,13 +11925,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>12</v>
+        <v>10.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -11923,7 +11981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17442,13 +17500,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>22.9</v>
+        <v>23.4</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>8</v>
+        <v>7.1</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -17456,10 +17514,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>55.7</v>
+        <v>49.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>5.3</v>
+        <v>6.1</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -17471,7 +17529,7 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
@@ -17485,10 +17543,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>1.9</v>
+        <v>7.9</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>11.8</v>
+        <v>11.1</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -17500,13 +17558,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>22.9</v>
+        <v>22.7</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -17514,10 +17572,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>17.9</v>
+        <v>5.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.9</v>
+        <v>11.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -17529,13 +17587,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19.9</v>
+        <v>20.8</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>8.1</v>
+        <v>6.6</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -17543,10 +17601,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>10.8</v>
+        <v>0.8</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.7</v>
+        <v>11.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -17558,13 +17616,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19.7</v>
+        <v>20.7</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -17587,13 +17645,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.3</v>
+        <v>21</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -17601,13 +17659,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>22.9</v>
+        <v>0</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>12</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -17628,7 +17715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23147,13 +23234,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>23.3</v>
+        <v>25.6</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -23161,10 +23248,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>39.9</v>
+        <v>49.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>7.2</v>
+        <v>6</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -23179,21 +23266,21 @@
         <v>23.8</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D192" s="7" t="n">
         <v>2.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>84.5</v>
+        <v>76.2</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>1.9</v>
+        <v>2.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -23205,24 +23292,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23.7</v>
+        <v>23.6</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.8</v>
+        <v>5.3</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>4.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.9</v>
+        <v>11.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -23234,13 +23321,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>22</v>
+        <v>21.2</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -23248,10 +23335,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>58.2</v>
+        <v>48.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -23263,13 +23350,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>20.6</v>
+        <v>20.4</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -23277,10 +23364,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>43</v>
+        <v>56.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.8</v>
+        <v>5.2</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -23292,27 +23379,56 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>22.3</v>
+        <v>21.6</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.2</v>
+        <v>4.1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>48.5</v>
+        <v>39.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>6.2</v>
+        <v>7.2</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -23333,7 +23449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28852,24 +28968,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>12.2</v>
+        <v>14.3</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.3</v>
+        <v>3.3</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>55.5</v>
+        <v>55.4</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -28881,13 +28997,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>11.9</v>
+        <v>11.6</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -28895,10 +29011,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>68.90000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.7</v>
+        <v>2.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -28910,24 +29026,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12.1</v>
+        <v>11.6</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>12.3</v>
+        <v>10.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.5</v>
+        <v>10.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -28939,7 +29055,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>11.6</v>
+        <v>10.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -28953,10 +29069,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>10.4</v>
+        <v>3.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.8</v>
+        <v>11.5</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -28968,24 +29084,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>11.3</v>
+        <v>10.6</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.7</v>
+        <v>5.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -28997,27 +29113,56 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.3</v>
+        <v>9.4</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>61.7</v>
+        <v>67.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>4.6</v>
+        <v>3.9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -29038,7 +29183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31048,13 +31193,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.6</v>
+        <v>18.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>11</v>
+        <v>4.8</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -31062,10 +31207,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>69.5</v>
+        <v>68.2</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -31077,13 +31222,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>12.1</v>
+        <v>11.7</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>11.5</v>
+        <v>15.5</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -31091,10 +31236,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>36.7</v>
+        <v>40.7</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.6</v>
+        <v>7.1</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -31106,13 +31251,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>4</v>
+        <v>2.1</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -31120,10 +31265,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>33</v>
+        <v>29.7</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -31135,24 +31280,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>10.6</v>
+        <v>10.2</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>11.9</v>
+        <v>28.3</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>10.6</v>
+        <v>8.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -31170,7 +31315,7 @@
         <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -31178,10 +31323,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>9</v>
+        <v>32.4</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>10.9</v>
+        <v>8.1</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -31193,27 +31338,56 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>11.8</v>
+        <v>10.7</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>62.9</v>
+        <v>24</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>4.5</v>
+        <v>9.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H76" s="12">
+        <f>SUM(C70:C76)</f>
         <v/>
       </c>
     </row>
@@ -31234,7 +31408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33244,24 +33418,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>15.1</v>
+        <v>17.6</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>13</v>
+        <v>20.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>69.09999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -33273,24 +33447,24 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>22.2</v>
+        <v>23.3</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>49.3</v>
+        <v>55.4</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -33302,13 +33476,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>5.2</v>
+        <v>6.9</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -33316,10 +33490,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>71.3</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>3.4</v>
+        <v>2.5</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -33331,24 +33505,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.5</v>
+        <v>9.1</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>45.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>6.6</v>
+        <v>4</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -33360,24 +33534,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9</v>
+        <v>8.1</v>
       </c>
       <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
         <v>1.1</v>
       </c>
-      <c r="D74" s="7" t="n">
-        <v>1.2</v>
-      </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>52.9</v>
+        <v>11.2</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>5.7</v>
+        <v>10.7</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -33389,13 +33563,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.6</v>
+        <v>10.2</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -33403,13 +33577,42 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>62.3</v>
+        <v>15.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>4.5</v>
+        <v>10.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H76" s="12">
+        <f>SUM(C70:C76)</f>
         <v/>
       </c>
     </row>
@@ -33430,7 +33633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35440,24 +35643,24 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.2</v>
+        <v>17.5</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>11.4</v>
+        <v>14.8</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>74.3</v>
+        <v>82.5</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.1</v>
+        <v>2.1</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -35469,13 +35672,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.5</v>
+        <v>9.1</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>17.9</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -35483,10 +35686,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>40.1</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.2</v>
+        <v>3.9</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -35498,13 +35701,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.4</v>
+        <v>8</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>2</v>
+        <v>5.8</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -35512,10 +35715,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>69.7</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>3.6</v>
+        <v>1.8</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -35527,24 +35730,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>24.6</v>
+        <v>60</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>9</v>
+        <v>4.8</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -35556,24 +35759,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>10.2</v>
+        <v>9</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>3.8</v>
+        <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>67</v>
+        <v>11.1</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>4</v>
+        <v>10.7</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -35585,27 +35788,56 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10</v>
+        <v>11.6</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>25.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>8.9</v>
+        <v>10.8</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H76" s="12">
+        <f>SUM(C70:C76)</f>
         <v/>
       </c>
     </row>
@@ -35626,7 +35858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37636,13 +37868,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.4</v>
+        <v>17.9</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>11.6</v>
+        <v>13.5</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -37650,10 +37882,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>65.3</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>4.2</v>
+        <v>3.7</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -37665,10 +37897,10 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>3.3</v>
+        <v>10</v>
       </c>
       <c r="D71" s="4" t="n">
         <v>4.4</v>
@@ -37679,10 +37911,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>29.5</v>
+        <v>41.4</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>8.5</v>
+        <v>7</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -37694,13 +37926,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -37708,10 +37940,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>53.7</v>
+        <v>47</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.6</v>
+        <v>6.4</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -37723,24 +37955,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>20.1</v>
+        <v>48.1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>9.6</v>
+        <v>6.2</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -37752,13 +37984,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -37766,10 +37998,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>23.6</v>
+        <v>28.7</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -37781,27 +38013,56 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.6</v>
+        <v>10.9</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>7.6</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>0.9</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>98.2</v>
+        <v>14.4</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>0.2</v>
+        <v>10.3</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H76" s="12">
+        <f>SUM(C70:C76)</f>
         <v/>
       </c>
     </row>
@@ -37822,7 +38083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39832,10 +40093,10 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>16.5</v>
+        <v>17.9</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>11.5</v>
+        <v>4.3</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>3.1</v>
@@ -39846,10 +40107,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>67.59999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.9</v>
+        <v>2.1</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -39861,13 +40122,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>10.5</v>
+        <v>9.9</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>5.2</v>
+        <v>18</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -39875,10 +40136,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>28.8</v>
+        <v>41.7</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>8.5</v>
+        <v>7</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -39890,13 +40151,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -39904,10 +40165,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>44.5</v>
+        <v>62.5</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>6.7</v>
+        <v>4.5</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -39919,24 +40180,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>10.6</v>
+        <v>9.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>26.8</v>
+        <v>22.7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -39948,24 +40209,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>10.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>70.90000000000001</v>
+        <v>5.1</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.5</v>
+        <v>11.4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -39977,27 +40238,56 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.8</v>
+        <v>11.4</v>
       </c>
       <c r="C75" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>38.3</v>
+        <v>22.7</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>7.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H76" s="12">
+        <f>SUM(C70:C76)</f>
         <v/>
       </c>
     </row>
@@ -40018,7 +40308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42028,13 +42318,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12.7</v>
+        <v>14.6</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>11.9</v>
+        <v>14.1</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -42042,10 +42332,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>70.59999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.5</v>
+        <v>2.2</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -42057,13 +42347,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>14.1</v>
+        <v>15.2</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -42071,10 +42361,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>76.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>2.8</v>
+        <v>1.5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -42086,13 +42376,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="C72" s="7" t="n">
         <v>7.6</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -42100,10 +42390,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>83.8</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>1.9</v>
+        <v>0.9</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -42115,13 +42405,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>5.7</v>
+        <v>5.3</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -42129,10 +42419,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>61.9</v>
+        <v>73.2</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>4.6</v>
+        <v>3.2</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -42144,13 +42434,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="C74" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -42158,10 +42448,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>61.9</v>
+        <v>9.9</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>4.6</v>
+        <v>10.8</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -42173,27 +42463,56 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>6.9</v>
+        <v>7.6</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>68.90000000000001</v>
+        <v>13.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>3.7</v>
+        <v>10.3</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="H76" s="12">
+        <f>SUM(C70:C76)</f>
         <v/>
       </c>
     </row>
@@ -42214,7 +42533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47733,24 +48052,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>21.1</v>
+        <v>23.9</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>61.1</v>
+        <v>56.9</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4.7</v>
+        <v>5.2</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -47762,13 +48081,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -47776,10 +48095,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>74.3</v>
+        <v>75.7</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -47791,24 +48110,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>29.9</v>
+        <v>25.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.4</v>
+        <v>9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -47820,13 +48139,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.4</v>
+        <v>18.8</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -47834,10 +48153,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>42</v>
+        <v>44.7</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -47849,13 +48168,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>18</v>
+        <v>17.8</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -47863,10 +48182,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>68.2</v>
+        <v>48</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>3.8</v>
+        <v>6.2</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -47878,13 +48197,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>18.8</v>
+        <v>17.7</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -47892,13 +48211,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>25.6</v>
+        <v>44.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.9</v>
+        <v>6.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -47919,7 +48267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49929,13 +50277,13 @@
         <v>46285</v>
       </c>
       <c r="B70" s="7" t="n">
-        <v>12.1</v>
+        <v>14</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>7.9</v>
+        <v>20.2</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
@@ -49943,10 +50291,10 @@
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>69.8</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="H70" s="12">
         <f>SUM(C64:C70)</f>
@@ -49958,13 +50306,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>9.5</v>
+        <v>11.3</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -49972,10 +50320,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>39.7</v>
+        <v>54.2</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.2</v>
+        <v>5.5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -49987,13 +50335,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0.2</v>
+        <v>4.6</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -50001,10 +50349,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>77.5</v>
+        <v>51.3</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>2.7</v>
+        <v>5.8</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -50016,24 +50364,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>1.5</v>
+        <v>2.3</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>59</v>
+        <v>37.3</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>4.9</v>
+        <v>7.5</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -50045,24 +50393,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>43.4</v>
+        <v>55.3</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>6.8</v>
+        <v>5.4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -50074,27 +50422,56 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>68.40000000000001</v>
+        <v>17</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>3.8</v>
+        <v>10</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H76" s="12">
+        <f>SUM(C70:C76)</f>
         <v/>
       </c>
     </row>
@@ -50115,7 +50492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -55634,24 +56011,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>24.1</v>
+        <v>24.7</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>19.2</v>
+        <v>5.6</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>57</v>
+        <v>37.5</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>5.2</v>
+        <v>7.5</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -55663,24 +56040,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>2.6</v>
+        <v>6.3</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>23.1</v>
+        <v>15.6</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -55692,24 +56069,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>25.1</v>
+        <v>24.9</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>50.4</v>
+        <v>21.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>6</v>
+        <v>9.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -55721,24 +56098,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>24.9</v>
+        <v>24.4</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>5.7</v>
+        <v>2.6</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>1</v>
+        <v>10.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.9</v>
+        <v>10.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -55750,24 +56127,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>23.2</v>
+        <v>23.4</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>10.6</v>
+        <v>12.5</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -55779,27 +56156,56 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>23.5</v>
+        <v>22.4</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>3.4</v>
+        <v>10.7</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3.6</v>
+        <v>4.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>15.6</v>
+        <v>65.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.1</v>
+        <v>4.1</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -55820,7 +56226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61339,24 +61745,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18</v>
+        <v>19.9</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>6.2</v>
+        <v>5.1</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -61368,24 +61774,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>20.1</v>
+        <v>19.6</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>24.6</v>
+        <v>27.1</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -61397,13 +61803,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>18.8</v>
+        <v>18.4</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.2</v>
+        <v>3.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -61411,10 +61817,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>0.2</v>
+        <v>3.4</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -61426,13 +61832,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.1</v>
+        <v>18.6</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -61440,10 +61846,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -61455,13 +61861,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>17.9</v>
+        <v>19</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -61469,10 +61875,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>0.8</v>
+        <v>12.3</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>11.9</v>
+        <v>10.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -61484,13 +61890,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>19.4</v>
+        <v>19.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -61498,13 +61904,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>1.9</v>
+        <v>5.5</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.8</v>
+        <v>11.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -61525,7 +61960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67044,13 +67479,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>29.1</v>
+        <v>5.4</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -67058,10 +67493,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>95</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -67073,13 +67508,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>12.3</v>
+        <v>11.6</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -67087,10 +67522,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>51.8</v>
+        <v>43</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -67102,24 +67537,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>98.8</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -67131,21 +67566,21 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>11.1</v>
+        <v>8.4</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>0.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>99.8</v>
+        <v>100</v>
       </c>
       <c r="G194" s="7" t="n">
         <v>0</v>
@@ -67160,24 +67595,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>13.2</v>
+        <v>12</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D195" s="4" t="n">
         <v>0.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>99.09999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -67189,27 +67624,56 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>12.3</v>
+        <v>12</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>92.40000000000001</v>
+        <v>98</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -67230,7 +67694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -72749,7 +73213,7 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18.6</v>
+        <v>20.9</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
@@ -72759,14 +73223,14 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>51.9</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>5.8</v>
+        <v>3.8</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -72778,13 +73242,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.1</v>
+        <v>19.4</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -72792,10 +73256,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>65.90000000000001</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -72813,7 +73277,7 @@
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -72821,10 +73285,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>23.8</v>
+        <v>10.7</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.1</v>
+        <v>10.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -72836,13 +73300,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.8</v>
+        <v>13.5</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -72850,10 +73314,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>26</v>
+        <v>32.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8.9</v>
+        <v>8.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -72865,24 +73329,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>15.5</v>
+        <v>15.1</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0.3</v>
+        <v>2.9</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>45.3</v>
+        <v>75.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.6</v>
+        <v>2.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -72894,13 +73358,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>16</v>
+        <v>14.9</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -72908,13 +73372,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.9</v>
+        <v>10.2</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -72935,7 +73428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -78454,24 +78947,24 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>20.7</v>
+        <v>22.5</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>49.2</v>
+        <v>61</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -78483,24 +78976,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>55.4</v>
+        <v>66.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.4</v>
+        <v>4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -78512,13 +79005,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -78526,10 +79019,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>14.8</v>
+        <v>7.4</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.2</v>
+        <v>11.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -78541,7 +79034,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -78555,10 +79048,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>19.4</v>
+        <v>28.1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -78570,13 +79063,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>17</v>
+        <v>16.4</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>1.2</v>
+        <v>3.5</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -78584,10 +79077,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>57.6</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5.1</v>
+        <v>2.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -78599,13 +79092,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>17.2</v>
+        <v>15.8</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -78613,13 +79106,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>31.2</v>
+        <v>13.1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -78640,7 +79162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84159,13 +84681,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>18</v>
+        <v>19.8</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -84173,10 +84695,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>43.7</v>
+        <v>42.7</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -84188,7 +84710,7 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>16.4</v>
+        <v>16.8</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
@@ -84202,10 +84724,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>55.5</v>
+        <v>63.9</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -84217,13 +84739,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -84231,10 +84753,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>22.1</v>
+        <v>10.8</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -84252,7 +84774,7 @@
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -84260,10 +84782,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -84275,13 +84797,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0.1</v>
+        <v>4.5</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -84289,10 +84811,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>31.2</v>
+        <v>26.6</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -84304,13 +84826,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>6.1</v>
+        <v>2.4</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -84318,13 +84840,42 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>41</v>
+        <v>67.2</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.1</v>
+        <v>3.9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>
@@ -84345,7 +84896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -89864,13 +90415,13 @@
         <v>46285</v>
       </c>
       <c r="B191" s="4" t="n">
-        <v>14.7</v>
+        <v>16.1</v>
       </c>
       <c r="C191" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
@@ -89878,10 +90429,10 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>75.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="H191" s="10">
         <f>SUM(C185:C191)</f>
@@ -89893,13 +90444,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>12.9</v>
+        <v>12.6</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -89907,10 +90458,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>78</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -89922,13 +90473,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12.6</v>
+        <v>11.5</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -89936,7 +90487,7 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="G193" s="4" t="n">
         <v>10.6</v>
@@ -89951,13 +90502,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.2</v>
+        <v>13.1</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -89965,10 +90516,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>3.5</v>
+        <v>2.1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -89980,24 +90531,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>14.8</v>
+        <v>13</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.8</v>
+        <v>1.3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>37.3</v>
+        <v>45.7</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -90009,7 +90560,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>14</v>
+        <v>11.8</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -90019,17 +90570,46 @@
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G196" s="7" t="n">
         <v>9.9</v>
-      </c>
-      <c r="G196" s="7" t="n">
-        <v>10.8</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B197" s="4" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H197" s="10">
+        <f>SUM(C191:C197)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-21 11:25 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6061,13 +6061,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>25.1</v>
+        <v>26.2</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.1</v>
+        <v>2.6</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -6075,10 +6075,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>16.4</v>
+        <v>11.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>10</v>
+        <v>10.6</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -6090,13 +6090,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>22.4</v>
+        <v>21.9</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>16.1</v>
+        <v>34.4</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -6104,10 +6104,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>32.8</v>
+        <v>51.2</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.1</v>
+        <v>5.9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -6119,13 +6119,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19.5</v>
+        <v>19.2</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>13</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.7</v>
+        <v>3.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -6133,10 +6133,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>51.5</v>
+        <v>53.1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -6148,13 +6148,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -6162,10 +6162,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>30.7</v>
+        <v>25.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -6177,13 +6177,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -6191,10 +6191,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>18.2</v>
+        <v>27.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -6206,27 +6206,56 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21</v>
+        <v>19.9</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>0</v>
+        <v>6.3</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>24.2</v>
+        <v>55.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.1</v>
+        <v>5.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -6247,7 +6276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11795,24 +11824,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.2</v>
+        <v>25.3</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>24.2</v>
+        <v>56.4</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>9.1</v>
+        <v>5.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -11824,13 +11853,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23.4</v>
+        <v>23.1</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -11838,10 +11867,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>8.5</v>
+        <v>11.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -11853,24 +11882,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>21.2</v>
+        <v>22</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>0.4</v>
+        <v>32.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>12</v>
+        <v>8.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -11882,13 +11911,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -11896,10 +11925,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>59.4</v>
+        <v>58.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -11911,7 +11940,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -11921,14 +11950,14 @@
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>10.5</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.7</v>
+        <v>3.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -11940,13 +11969,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21.1</v>
+        <v>22.4</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -11954,13 +11983,42 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>37.9</v>
+        <v>79.3</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -11981,7 +12039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17529,13 +17587,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>22.3</v>
+        <v>23.3</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>7.9</v>
+        <v>7.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -17543,10 +17601,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>7.9</v>
+        <v>4.5</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -17558,7 +17616,7 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
@@ -17572,10 +17630,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>5.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.4</v>
+        <v>10.8</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -17587,13 +17645,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.8</v>
+        <v>20.6</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>6.6</v>
+        <v>7.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -17601,10 +17659,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>0.8</v>
+        <v>2.6</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -17616,13 +17674,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -17645,13 +17703,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>21</v>
+        <v>20.6</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -17674,13 +17732,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.8</v>
+        <v>4.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -17688,13 +17746,42 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>33.2</v>
+        <v>49.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8</v>
+        <v>6.1</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -17715,7 +17802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23263,24 +23350,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>23.8</v>
+        <v>25.1</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>76.2</v>
+        <v>77.8</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -23292,13 +23379,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23.6</v>
+        <v>24</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -23306,7 +23393,7 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="G193" s="4" t="n">
         <v>11.4</v>
@@ -23321,13 +23408,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>21.2</v>
+        <v>20.7</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -23335,10 +23422,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>48.4</v>
+        <v>41</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>6.2</v>
+        <v>7.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -23350,7 +23437,7 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>20.4</v>
+        <v>20.5</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
@@ -23364,10 +23451,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>56.8</v>
+        <v>49</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -23379,13 +23466,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>21.6</v>
+        <v>20.7</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4.1</v>
+        <v>2.9</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -23393,10 +23480,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>39.8</v>
+        <v>53.1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.2</v>
+        <v>5.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -23408,27 +23495,56 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21.4</v>
+        <v>20.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.6</v>
+        <v>2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>58.6</v>
+        <v>0.4</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -23449,7 +23565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28997,24 +29113,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>11.6</v>
+        <v>13.8</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>76.90000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.8</v>
+        <v>1.7</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -29026,7 +29142,7 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
@@ -29040,10 +29156,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="G193" s="4" t="n">
         <v>10.8</v>
-      </c>
-      <c r="G193" s="4" t="n">
-        <v>10.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -29055,24 +29171,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.2</v>
+        <v>2.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>3.9</v>
+        <v>20.8</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -29084,7 +29200,7 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>10.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
@@ -29098,10 +29214,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>51</v>
+        <v>58.4</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5.9</v>
+        <v>5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -29113,7 +29229,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>9.4</v>
+        <v>10.5</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -29123,14 +29239,14 @@
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>67.8</v>
+        <v>53.5</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>3.9</v>
+        <v>5.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -29142,7 +29258,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>10.2</v>
+        <v>10.7</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -29152,17 +29268,46 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>29.1</v>
+        <v>28.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -29183,7 +29328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31222,24 +31367,24 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11.7</v>
+        <v>11.3</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>15.5</v>
+        <v>1.5</v>
       </c>
       <c r="D71" s="4" t="n">
         <v>3.4</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>40.7</v>
+        <v>58.4</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7.1</v>
+        <v>5</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -31251,13 +31396,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.9</v>
+        <v>9.5</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>2.1</v>
+        <v>12.6</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -31265,10 +31410,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>29.7</v>
+        <v>52.8</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>8.4</v>
+        <v>5.7</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -31280,24 +31425,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>10.2</v>
+        <v>9.9</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.2</v>
+        <v>1.7</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>28.3</v>
+        <v>24</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -31309,24 +31454,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>32.4</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>8.1</v>
+        <v>3.5</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -31338,24 +31483,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>24</v>
+        <v>42.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>9.1</v>
+        <v>6.9</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -31367,27 +31512,56 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>13.4</v>
+        <v>13.1</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>28.1</v>
+        <v>56.9</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8.6</v>
+        <v>5.2</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H77" s="10">
+        <f>SUM(C71:C77)</f>
         <v/>
       </c>
     </row>
@@ -31408,7 +31582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33447,24 +33621,24 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.4</v>
+        <v>9.1</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>23.3</v>
+        <v>10.6</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>55.4</v>
+        <v>58.8</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>5.4</v>
+        <v>4.9</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -33476,10 +33650,10 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>6.9</v>
+        <v>15.6</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>3.3</v>
@@ -33490,10 +33664,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>79.40000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -33505,24 +33679,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.5</v>
+        <v>4.7</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>66.40000000000001</v>
+        <v>44.7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>4</v>
+        <v>6.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -33534,13 +33708,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.1</v>
+        <v>8.6</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -33548,10 +33722,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>11.2</v>
+        <v>80.3</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>10.7</v>
+        <v>2.4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -33563,24 +33737,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>15.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>10.1</v>
+        <v>1.7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -33592,13 +33766,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.2</v>
+        <v>10.6</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -33606,13 +33780,42 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>8.6</v>
+        <v>72.7</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>11</v>
+        <v>3.3</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H77" s="10">
+        <f>SUM(C71:C77)</f>
         <v/>
       </c>
     </row>
@@ -33633,7 +33836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35672,13 +35875,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.1</v>
+        <v>8.5</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>17.9</v>
+        <v>6.4</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -35686,10 +35889,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>67.40000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -35701,13 +35904,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>5.8</v>
+        <v>11.5</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -35715,10 +35918,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>84.90000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -35730,13 +35933,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -35744,10 +35947,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>60</v>
+        <v>46.7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>4.8</v>
+        <v>6.4</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -35759,24 +35962,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>11.1</v>
+        <v>73.8</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>10.7</v>
+        <v>3.1</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -35788,24 +35991,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>11.6</v>
+        <v>10.3</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.1</v>
+        <v>2.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>67</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>10.8</v>
+        <v>4</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -35817,27 +36020,56 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>13.3</v>
+        <v>12</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>10.2</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>10.8</v>
+        <v>3.2</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H77" s="10">
+        <f>SUM(C71:C77)</f>
         <v/>
       </c>
     </row>
@@ -35858,7 +36090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37897,10 +38129,10 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>11</v>
+        <v>10.3</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>10</v>
+        <v>3.4</v>
       </c>
       <c r="D71" s="4" t="n">
         <v>4.4</v>
@@ -37911,10 +38143,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>41.4</v>
+        <v>57.1</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7</v>
+        <v>5.1</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -37926,13 +38158,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>2.4</v>
+        <v>8.1</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -37940,10 +38172,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>47</v>
+        <v>53.4</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -37955,13 +38187,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -37969,10 +38201,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>48.1</v>
+        <v>25.6</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>6.2</v>
+        <v>8.9</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -37984,13 +38216,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -37998,10 +38230,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>28.7</v>
+        <v>76.8</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>8.6</v>
+        <v>2.8</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -38013,24 +38245,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.9</v>
+        <v>9.9</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>0.9</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>14.4</v>
+        <v>79.5</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>10.3</v>
+        <v>2.5</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -38042,27 +38274,56 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>13.2</v>
+        <v>12</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>28.1</v>
+        <v>56.1</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8.6</v>
+        <v>5.3</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H77" s="10">
+        <f>SUM(C71:C77)</f>
         <v/>
       </c>
     </row>
@@ -38083,7 +38344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40122,13 +40383,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9.9</v>
+        <v>9.1</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>18</v>
+        <v>2.6</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -40136,10 +40397,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>41.7</v>
+        <v>48.1</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>7</v>
+        <v>6.2</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -40151,13 +40412,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>13</v>
+        <v>6.2</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -40165,10 +40426,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>62.5</v>
+        <v>65.2</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -40180,24 +40441,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.6</v>
+        <v>9.4</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.8</v>
+        <v>3.5</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>22.7</v>
+        <v>21.3</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -40209,13 +40470,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>0.9</v>
+        <v>2.6</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -40223,10 +40484,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>5.1</v>
+        <v>69.3</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>11.4</v>
+        <v>3.7</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -40238,24 +40499,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>11.4</v>
+        <v>10.5</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>22.7</v>
+        <v>53.5</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -40267,13 +40528,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>13</v>
+        <v>11.8</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -40281,13 +40542,42 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>18.4</v>
+        <v>68</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>3.8</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H77" s="10">
+        <f>SUM(C71:C77)</f>
         <v/>
       </c>
     </row>
@@ -40308,7 +40598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42347,13 +42637,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>5.5</v>
+        <v>4.6</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>15.2</v>
+        <v>8.1</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>4.3</v>
+        <v>3.9</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -42361,10 +42651,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>87.90000000000001</v>
+        <v>84.3</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -42379,10 +42669,10 @@
         <v>4.2</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>7.6</v>
+        <v>11</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -42390,10 +42680,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>92.09999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -42405,13 +42695,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>5.3</v>
+        <v>4.9</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.3</v>
+        <v>3.2</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -42419,10 +42709,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>73.2</v>
+        <v>53.2</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>3.2</v>
+        <v>5.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -42434,13 +42724,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -42448,10 +42738,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>9.9</v>
+        <v>73.8</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>10.8</v>
+        <v>3.1</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -42463,24 +42753,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>13.8</v>
+        <v>65.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>10.3</v>
+        <v>4.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -42492,13 +42782,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>9.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -42506,13 +42796,42 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>13.9</v>
+        <v>86.5</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>10.3</v>
+        <v>1.6</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H77" s="10">
+        <f>SUM(C71:C77)</f>
         <v/>
       </c>
     </row>
@@ -42533,7 +42852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48081,24 +48400,24 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>21.5</v>
+        <v>22.8</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>75.7</v>
+        <v>70.8</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -48110,13 +48429,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>19</v>
+        <v>18.7</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -48124,10 +48443,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>25.3</v>
+        <v>31.3</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -48139,24 +48458,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.8</v>
+        <v>18.3</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>44.7</v>
+        <v>47.8</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -48168,10 +48487,10 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>17.8</v>
+        <v>17.5</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="D195" s="4" t="n">
         <v>0.4</v>
@@ -48182,10 +48501,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>48</v>
+        <v>51.4</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -48197,13 +48516,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>17.7</v>
+        <v>16.8</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -48211,10 +48530,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>44.7</v>
+        <v>37.9</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>6.6</v>
+        <v>7.5</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -48226,7 +48545,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>18.3</v>
+        <v>18.1</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -48236,17 +48555,46 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>60.4</v>
+        <v>5.7</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>4.8</v>
+        <v>11.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -48267,7 +48615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -50306,13 +50654,13 @@
         <v>46286</v>
       </c>
       <c r="B71" s="4" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C71" s="4" t="n">
-        <v>11.3</v>
+        <v>3.3</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
@@ -50320,10 +50668,10 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>54.2</v>
+        <v>31.5</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>5.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H71" s="10">
         <f>SUM(C65:C71)</f>
@@ -50335,10 +50683,10 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>4.6</v>
+        <v>3.1</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>4.8</v>
@@ -50349,10 +50697,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>51.3</v>
+        <v>49.4</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -50364,13 +50712,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -50378,10 +50726,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>37.3</v>
+        <v>36.5</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -50393,24 +50741,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.1</v>
+        <v>7.5</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>55.3</v>
+        <v>82.2</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>5.4</v>
+        <v>2.1</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -50422,24 +50770,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>17</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>10</v>
+        <v>0.3</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -50451,27 +50799,56 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>18.8</v>
+        <v>65.8</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>4.1</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H77" s="10">
+        <f>SUM(C71:C77)</f>
         <v/>
       </c>
     </row>
@@ -50492,7 +50869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56040,13 +56417,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>25</v>
+        <v>25.3</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>6.3</v>
+        <v>0.9</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -56054,10 +56431,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>15.6</v>
+        <v>29.6</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>10.1</v>
+        <v>8.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -56069,10 +56446,10 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.3</v>
+        <v>3.5</v>
       </c>
       <c r="D193" s="4" t="n">
         <v>3.3</v>
@@ -56083,10 +56460,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>21.3</v>
+        <v>26.7</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -56098,24 +56475,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>24.4</v>
+        <v>24.5</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.6</v>
+        <v>5.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -56127,24 +56504,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>12.5</v>
+        <v>3.1</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10.5</v>
+        <v>11.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -56156,24 +56533,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>22.4</v>
+        <v>23.6</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>10.7</v>
+        <v>4.5</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4.3</v>
+        <v>4.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>65.8</v>
+        <v>35.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>4.1</v>
+        <v>7.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -56185,27 +56562,56 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21</v>
+        <v>23.1</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>15</v>
+        <v>1.5</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.7</v>
+        <v>5.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>75.59999999999999</v>
+        <v>11.9</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>2.9</v>
+        <v>10.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -56226,7 +56632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61774,13 +62180,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.6</v>
+        <v>22.6</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -61788,10 +62194,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>27.1</v>
+        <v>37.1</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -61803,13 +62209,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -61817,10 +62223,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>3.4</v>
+        <v>20.1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.6</v>
+        <v>9.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -61832,13 +62238,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.6</v>
+        <v>19</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.3</v>
+        <v>3.2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -61846,10 +62252,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>8.4</v>
+        <v>16.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11</v>
+        <v>10.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -61861,13 +62267,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19</v>
+        <v>18.8</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -61875,10 +62281,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>12.3</v>
+        <v>14.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -61896,7 +62302,7 @@
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -61904,10 +62310,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>5.5</v>
+        <v>59.6</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.3</v>
+        <v>4.8</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -61919,13 +62325,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.1</v>
+        <v>19.4</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -61933,13 +62339,42 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>24.4</v>
+        <v>15</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.1</v>
+        <v>10.2</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -61960,7 +62395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67508,13 +67943,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>11.6</v>
+        <v>12.5</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -67522,10 +67957,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>43</v>
+        <v>33.8</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -67537,10 +67972,10 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>12.6</v>
+        <v>13.2</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>2.2</v>
+        <v>5.5</v>
       </c>
       <c r="D193" s="4" t="n">
         <v>0.6</v>
@@ -67551,10 +67986,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>96.40000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -67566,17 +68001,17 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.8</v>
+        <v>14</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>8.4</v>
+        <v>49</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
@@ -67595,13 +68030,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -67609,10 +68044,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>94.7</v>
+        <v>64.5</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>0.6</v>
+        <v>4.3</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -67624,13 +68059,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>12</v>
+        <v>12.6</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -67638,10 +68073,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>98</v>
+        <v>98.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -67653,13 +68088,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>12.7</v>
+        <v>13.1</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>5.6</v>
+        <v>3.7</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -67667,13 +68102,42 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>94.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -67694,7 +68158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -73242,13 +73706,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>19.4</v>
+        <v>19.7</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4.1</v>
+        <v>6.1</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -73256,10 +73720,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>73.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3.2</v>
+        <v>5.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -73271,13 +73735,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -73285,10 +73749,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>10.7</v>
+        <v>9</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -73300,13 +73764,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -73314,10 +73778,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>32.2</v>
+        <v>19.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8.1</v>
+        <v>9.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -73329,24 +73793,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>15.1</v>
+        <v>14.6</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>75.8</v>
+        <v>63.1</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>2.9</v>
+        <v>4.4</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -73358,13 +73822,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>14.9</v>
+        <v>14.4</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3.5</v>
+        <v>2.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -73372,10 +73836,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>15</v>
+        <v>4.9</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.2</v>
+        <v>11.4</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -73387,13 +73851,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>16.4</v>
+        <v>14.6</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -73401,13 +73865,42 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>56.2</v>
+        <v>3.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>5.3</v>
+        <v>11.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -73428,7 +73921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -78979,10 +79472,10 @@
         <v>20.7</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2.3</v>
+        <v>3.2</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -78990,10 +79483,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>66.5</v>
+        <v>56.6</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>4</v>
+        <v>5.2</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -79011,7 +79504,7 @@
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -79019,10 +79512,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>7.4</v>
+        <v>4.1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -79034,7 +79527,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -79044,14 +79537,14 @@
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>28.1</v>
+        <v>20.5</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8.6</v>
+        <v>9.5</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -79063,24 +79556,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>3.5</v>
+        <v>2.3</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>78.09999999999999</v>
+        <v>40.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>2.6</v>
+        <v>7.2</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -79092,13 +79585,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>15.8</v>
+        <v>15.3</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -79106,10 +79599,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>13.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.4</v>
+        <v>10.9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -79121,13 +79614,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.2</v>
+        <v>15.6</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -79135,13 +79628,42 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>54.7</v>
+        <v>2.4</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>5.4</v>
+        <v>11.7</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -79162,7 +79684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84710,13 +85232,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>16.8</v>
+        <v>16.1</v>
       </c>
       <c r="C192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -84724,10 +85246,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>63.9</v>
+        <v>38</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>4.3</v>
+        <v>7.4</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -84739,13 +85261,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -84753,10 +85275,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>10.8</v>
+        <v>11.5</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -84774,7 +85296,7 @@
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -84782,10 +85304,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>2.1</v>
+        <v>5.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.7</v>
+        <v>11.4</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -84797,17 +85319,17 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>4.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
@@ -84826,13 +85348,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>12.7</v>
+        <v>11.1</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.9</v>
+        <v>4.1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -84840,10 +85362,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>67.2</v>
+        <v>36.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>3.9</v>
+        <v>7.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -84855,27 +85377,56 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>13.9</v>
+        <v>12.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.9</v>
+        <v>3.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>30.9</v>
+        <v>12.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>
@@ -84896,7 +85447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -90444,13 +90995,13 @@
         <v>46286</v>
       </c>
       <c r="B192" s="7" t="n">
-        <v>12.6</v>
+        <v>13.5</v>
       </c>
       <c r="C192" s="7" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
@@ -90458,10 +91009,10 @@
         </is>
       </c>
       <c r="F192" s="7" t="n">
-        <v>75.59999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="G192" s="7" t="n">
-        <v>2.9</v>
+        <v>0.9</v>
       </c>
       <c r="H192" s="12">
         <f>SUM(C186:C192)</f>
@@ -90473,7 +91024,7 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
@@ -90487,10 +91038,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>11.5</v>
+        <v>6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.6</v>
+        <v>11.3</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -90502,13 +91053,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.1</v>
+        <v>13.8</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -90516,10 +91067,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>2.1</v>
+        <v>21.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.7</v>
+        <v>9.4</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -90534,21 +91085,21 @@
         <v>13</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>45.7</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.5</v>
+        <v>3.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -90560,24 +91111,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.8</v>
+        <v>12.2</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>17.2</v>
+        <v>30.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>9.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -90589,27 +91140,56 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.2</v>
+        <v>15.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>29.5</v>
+        <v>0</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.5</v>
+        <v>12</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="11" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B198" s="7" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="C198" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G198" s="7" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H198" s="12">
+        <f>SUM(C192:C198)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-22 10:33 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6090,24 +6090,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>21.9</v>
+        <v>20.9</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>34.4</v>
+        <v>22.8</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>51.2</v>
+        <v>87.5</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>5.9</v>
+        <v>1.5</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -6119,13 +6119,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>13</v>
+        <v>11.3</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -6133,10 +6133,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>53.1</v>
+        <v>61.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>5.6</v>
+        <v>4.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -6148,24 +6148,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19.1</v>
+        <v>18.8</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.6</v>
+        <v>3.3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>25.2</v>
+        <v>23.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -6177,13 +6177,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0.1</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -6191,10 +6191,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>27.7</v>
+        <v>10</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -6206,13 +6206,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>19.9</v>
+        <v>20.5</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -6220,10 +6220,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>55.5</v>
+        <v>38.8</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>5.3</v>
+        <v>7.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -6235,27 +6235,56 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21</v>
+        <v>21.3</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>5.2</v>
+        <v>2.6</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>69.90000000000001</v>
+        <v>8</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3.6</v>
+        <v>11</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -6276,7 +6305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11853,13 +11882,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>23.1</v>
+        <v>24.7</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -11867,10 +11896,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>11.6</v>
+        <v>4.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.6</v>
+        <v>11.4</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -11882,24 +11911,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>22</v>
+        <v>21.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>32.4</v>
+        <v>28.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8.1</v>
+        <v>8.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -11911,13 +11940,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>22.2</v>
+        <v>22.5</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -11925,10 +11954,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>58.2</v>
+        <v>43.9</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5</v>
+        <v>6.7</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -11940,13 +11969,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>23.4</v>
+        <v>23.2</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -11954,10 +11983,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>68.90000000000001</v>
+        <v>45.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>3.7</v>
+        <v>6.5</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -11969,13 +11998,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>22.4</v>
+        <v>21.5</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -11983,10 +12012,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>79.3</v>
+        <v>22.6</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>2.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -11998,13 +12027,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.8</v>
+        <v>20.3</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -12012,13 +12041,42 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>59.2</v>
+        <v>87.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>4.9</v>
+        <v>1.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>94.3</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -12039,7 +12097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17616,13 +17674,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>22.9</v>
+        <v>22.6</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -17630,10 +17688,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -17645,13 +17703,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.6</v>
+        <v>20.1</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -17659,10 +17717,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>2.6</v>
+        <v>11.5</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.7</v>
+        <v>10.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -17674,13 +17732,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>20.6</v>
+        <v>19.9</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -17703,13 +17761,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.6</v>
+        <v>20.4</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -17732,13 +17790,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>20.8</v>
+        <v>21.1</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.3</v>
+        <v>5.7</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -17746,10 +17804,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>49.2</v>
+        <v>18.8</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>6.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -17761,27 +17819,56 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>22.2</v>
+        <v>21.6</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3</v>
+        <v>7.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>51.2</v>
+        <v>0</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>5.9</v>
+        <v>12</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -17802,7 +17889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23379,24 +23466,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>24</v>
+        <v>25.3</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>4.9</v>
+        <v>2.2</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -23408,13 +23495,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>2.3</v>
+        <v>1.1</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -23422,10 +23509,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>41</v>
+        <v>36.3</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>7.1</v>
+        <v>7.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -23437,13 +23524,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>20.5</v>
+        <v>21.2</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.9</v>
+        <v>3.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -23451,10 +23538,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.1</v>
+        <v>3.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -23466,24 +23553,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>53.1</v>
+        <v>73</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>5.6</v>
+        <v>3.2</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -23495,7 +23582,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>20.8</v>
+        <v>19.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -23505,14 +23592,14 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>0.4</v>
+        <v>6.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -23524,13 +23611,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>22.3</v>
+        <v>20</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.9</v>
+        <v>1.3</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -23538,13 +23625,42 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>27.2</v>
+        <v>18</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -23565,7 +23681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29142,24 +29258,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>11.4</v>
+        <v>13.6</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>0</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -29171,7 +29287,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -29185,10 +29301,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>20.8</v>
+        <v>14.1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.5</v>
+        <v>10.3</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -29200,13 +29316,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -29214,10 +29330,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>58.4</v>
+        <v>60.5</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -29229,13 +29345,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>10.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -29258,13 +29374,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -29272,10 +29388,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>28.1</v>
+        <v>25</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -29287,13 +29403,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>11.2</v>
+        <v>10.6</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -29301,13 +29417,42 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>63.9</v>
+        <v>42.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>4.3</v>
+        <v>6.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -29328,7 +29473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31396,10 +31541,10 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.5</v>
+        <v>10.1</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>12.6</v>
+        <v>2</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>3.5</v>
@@ -31410,10 +31555,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>52.8</v>
+        <v>50</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.7</v>
+        <v>6</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -31425,10 +31570,10 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>1.7</v>
+        <v>5.4</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>3.1</v>
@@ -31439,10 +31584,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>24</v>
+        <v>36.6</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>9.1</v>
+        <v>7.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -31454,13 +31599,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.4</v>
+        <v>2.7</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -31468,10 +31613,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>71.09999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -31483,13 +31628,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.3</v>
+        <v>4.4</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -31497,10 +31642,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>42.8</v>
+        <v>49.2</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>6.9</v>
+        <v>6.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -31512,24 +31657,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>13.1</v>
+        <v>11.1</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>56.9</v>
+        <v>80.3</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5.2</v>
+        <v>2.4</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -31541,27 +31686,56 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>13.9</v>
+        <v>12.9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>18.9</v>
+        <v>19.4</v>
       </c>
       <c r="G77" s="4" t="n">
         <v>9.699999999999999</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H78" s="12">
+        <f>SUM(C72:C78)</f>
         <v/>
       </c>
     </row>
@@ -31582,7 +31756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33650,13 +33824,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>15.6</v>
+        <v>9.4</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -33664,10 +33838,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>77.3</v>
+        <v>82.8</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -33679,24 +33853,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>4.7</v>
+        <v>3</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>2.3</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>44.7</v>
+        <v>55.1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>6.6</v>
+        <v>5.4</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -33708,13 +33882,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>2.2</v>
+        <v>11.2</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -33722,10 +33896,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>80.3</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -33737,13 +33911,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -33751,10 +33925,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>86.09999999999999</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>1.7</v>
+        <v>3.6</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -33766,24 +33940,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>72.7</v>
+        <v>49.4</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>3.3</v>
+        <v>6.1</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -33795,13 +33969,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -33809,13 +33983,42 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>16.2</v>
+        <v>17.6</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>10.1</v>
+        <v>9.9</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H78" s="12">
+        <f>SUM(C72:C78)</f>
         <v/>
       </c>
     </row>
@@ -33836,7 +34039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35904,13 +36107,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>7.8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>11.5</v>
+        <v>3.7</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -35918,10 +36121,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>83.59999999999999</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -35933,10 +36136,10 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>3.6</v>
@@ -35947,10 +36150,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>46.7</v>
+        <v>55.1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>6.4</v>
+        <v>5.4</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -35962,13 +36165,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.3</v>
+        <v>7.5</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -35976,10 +36179,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>73.8</v>
+        <v>69.8</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -35991,13 +36194,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.3</v>
+        <v>9</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.3</v>
+        <v>2.1</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -36005,10 +36208,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>67</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -36020,24 +36223,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>12</v>
+        <v>10.7</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>73.59999999999999</v>
+        <v>50.6</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>3.2</v>
+        <v>5.9</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -36049,27 +36252,56 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>13.9</v>
+        <v>12.9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>30.5</v>
+        <v>4.5</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>11.5</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H78" s="12">
+        <f>SUM(C72:C78)</f>
         <v/>
       </c>
     </row>
@@ -36090,7 +36322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38158,13 +38390,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>8.1</v>
+        <v>2.2</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -38172,10 +38404,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>53.4</v>
+        <v>63</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5.6</v>
+        <v>4.4</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -38190,10 +38422,10 @@
         <v>9.6</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -38201,10 +38433,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>25.6</v>
+        <v>27.4</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>8.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -38216,24 +38448,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.8</v>
+        <v>6.8</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>76.8</v>
+        <v>64.5</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>2.8</v>
+        <v>4.3</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -38245,24 +38477,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1.6</v>
+        <v>7.5</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>79.5</v>
+        <v>51.2</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>2.5</v>
+        <v>5.9</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -38274,24 +38506,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>12</v>
+        <v>10.3</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="D76" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="G76" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="E76" s="7" t="inlineStr">
-        <is>
-          <t>JV</t>
-        </is>
-      </c>
-      <c r="F76" s="7" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="G76" s="7" t="n">
-        <v>5.3</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -38303,13 +38535,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>14</v>
+        <v>12.3</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -38317,13 +38549,42 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>44.9</v>
+        <v>30.6</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>6.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H78" s="12">
+        <f>SUM(C72:C78)</f>
         <v/>
       </c>
     </row>
@@ -38344,7 +38605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40412,13 +40673,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.6</v>
+        <v>9.5</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>6.2</v>
+        <v>1.8</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.8</v>
+        <v>4.4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -40426,10 +40687,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>65.2</v>
+        <v>49.9</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -40441,7 +40702,7 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
@@ -40455,10 +40716,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>21.3</v>
+        <v>23.7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>9.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -40470,13 +40731,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.3</v>
+        <v>3.3</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -40484,10 +40745,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>69.3</v>
+        <v>63.4</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -40499,24 +40760,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.5</v>
+        <v>9.5</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>53.5</v>
+        <v>48.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -40528,7 +40789,7 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.8</v>
+        <v>11</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
@@ -40538,14 +40799,14 @@
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>68</v>
+        <v>59.5</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>3.8</v>
+        <v>4.9</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -40557,13 +40818,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>14.1</v>
+        <v>13.3</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -40571,13 +40832,42 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>29.7</v>
+        <v>1.4</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.4</v>
+        <v>11.8</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H78" s="12">
+        <f>SUM(C72:C78)</f>
         <v/>
       </c>
     </row>
@@ -40598,7 +40888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42666,10 +42956,10 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>11</v>
+        <v>5.6</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>3.5</v>
@@ -42695,10 +42985,10 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>2.9</v>
@@ -42709,10 +42999,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>53.2</v>
+        <v>62.3</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>5.6</v>
+        <v>4.5</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -42724,24 +43014,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>0.2</v>
+        <v>11.5</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>73.8</v>
+        <v>77.3</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -42753,13 +43043,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1.7</v>
+        <v>4.1</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -42767,10 +43057,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>65.8</v>
+        <v>71.7</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -42782,24 +43072,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>86.5</v>
+        <v>64.3</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>1.6</v>
+        <v>4.3</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -42811,7 +43101,7 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>10.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
@@ -42821,17 +43111,46 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>24.6</v>
+        <v>14.6</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9</v>
+        <v>10.2</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H78" s="12">
+        <f>SUM(C72:C78)</f>
         <v/>
       </c>
     </row>
@@ -42852,7 +43171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48429,24 +48748,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>18.7</v>
+        <v>20.7</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>31.3</v>
+        <v>18.5</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -48458,13 +48777,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.3</v>
+        <v>17.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -48472,10 +48791,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>47.8</v>
+        <v>56.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>6.3</v>
+        <v>5.2</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -48487,13 +48806,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -48501,10 +48820,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>51.4</v>
+        <v>46.6</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -48522,7 +48841,7 @@
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -48530,10 +48849,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>37.9</v>
+        <v>25.4</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -48545,7 +48864,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -48555,14 +48874,14 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>5.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.3</v>
+        <v>10.9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -48574,27 +48893,56 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.4</v>
+        <v>20</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>5.3</v>
+        <v>32.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.4</v>
+        <v>8.1</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -48615,7 +48963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -50683,13 +51031,13 @@
         <v>46287</v>
       </c>
       <c r="B72" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -50697,10 +51045,10 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>49.4</v>
+        <v>33.1</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>6.1</v>
+        <v>8</v>
       </c>
       <c r="H72" s="12">
         <f>SUM(C66:C72)</f>
@@ -50712,7 +51060,7 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
@@ -50726,10 +51074,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>36.5</v>
+        <v>52</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>7.6</v>
+        <v>5.8</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -50741,13 +51089,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>5.2</v>
+        <v>16.1</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -50755,10 +51103,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>82.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -50770,13 +51118,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.1</v>
+        <v>9.6</v>
       </c>
       <c r="C75" s="4" t="n">
         <v>1.9</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -50799,24 +51147,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>2.6</v>
+        <v>1.9</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>65.8</v>
+        <v>29.3</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>4.1</v>
+        <v>8.5</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -50828,27 +51176,56 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>15.6</v>
+        <v>7.8</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>10.1</v>
+        <v>11.1</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H78" s="12">
+        <f>SUM(C72:C78)</f>
         <v/>
       </c>
     </row>
@@ -50869,7 +51246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56446,24 +56823,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>24.8</v>
+        <v>25.3</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>26.7</v>
+        <v>10.2</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>10.8</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -56475,13 +56852,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>4.3</v>
+        <v>0.4</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -56489,10 +56866,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>9.4</v>
+        <v>4.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.9</v>
+        <v>11.4</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -56504,21 +56881,21 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>23.5</v>
+        <v>23.6</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>3.1</v>
+        <v>3.7</v>
       </c>
       <c r="G195" s="4" t="n">
         <v>11.6</v>
@@ -56533,24 +56910,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>23.6</v>
+        <v>22.4</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>4.5</v>
+        <v>7.6</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>35.8</v>
+        <v>47.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.7</v>
+        <v>6.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -56562,13 +56939,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>23.1</v>
+        <v>22.7</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>5.6</v>
+        <v>4.1</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -56576,10 +56953,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>11.9</v>
+        <v>17.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.6</v>
+        <v>9.9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -56591,13 +56968,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>24.1</v>
+        <v>23.2</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>7.8</v>
+        <v>3.2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -56605,13 +56982,42 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>10.2</v>
+        <v>6.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.8</v>
+        <v>11.2</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -56632,7 +57038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62209,24 +62615,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>18.3</v>
+        <v>20.2</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>20.1</v>
+        <v>24</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>9.6</v>
+        <v>9.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -62238,7 +62644,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -62252,10 +62658,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>16.2</v>
+        <v>20.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.1</v>
+        <v>9.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -62267,13 +62673,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -62281,10 +62687,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>14.2</v>
+        <v>10.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10.3</v>
+        <v>10.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -62296,7 +62702,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>19.9</v>
+        <v>19.4</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -62310,10 +62716,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>59.6</v>
+        <v>28.6</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>4.8</v>
+        <v>8.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -62325,13 +62731,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>19.4</v>
+        <v>17.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -62339,10 +62745,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>15</v>
+        <v>10.3</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.2</v>
+        <v>10.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -62354,13 +62760,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.5</v>
+        <v>17.1</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -62368,13 +62774,42 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>51.4</v>
+        <v>75</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>5.8</v>
+        <v>3</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>87.7</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -62395,7 +62830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67972,13 +68407,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="C193" s="4" t="n">
-        <v>5.5</v>
+        <v>6.8</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -67986,10 +68421,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>96.2</v>
+        <v>97.7</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -68001,17 +68436,17 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14</v>
+        <v>13.7</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>49</v>
+        <v>36.9</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
@@ -68030,13 +68465,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>12.3</v>
+        <v>14</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -68044,10 +68479,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>64.5</v>
+        <v>92</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -68059,13 +68494,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>12.6</v>
+        <v>12.9</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -68073,10 +68508,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>98.8</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -68088,24 +68523,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>13.1</v>
+        <v>12.9</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>96.5</v>
+        <v>85.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -68117,10 +68552,10 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="D198" s="7" t="n">
         <v>1.2</v>
@@ -68131,13 +68566,42 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>72.2</v>
+        <v>87.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3.3</v>
+        <v>1.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -68158,7 +68622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -73735,13 +74199,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>15.7</v>
+        <v>16.5</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>4.7</v>
+        <v>3.9</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -73749,10 +74213,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>9</v>
+        <v>3.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -73764,7 +74228,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -73778,10 +74242,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>19.9</v>
+        <v>16</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -73793,24 +74257,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>14.6</v>
+        <v>15.6</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>3.9</v>
+        <v>14.4</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>63.1</v>
+        <v>60.4</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -73822,13 +74286,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>14.4</v>
+        <v>14.8</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -73836,10 +74300,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>4.9</v>
+        <v>1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -73851,24 +74315,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>14.6</v>
+        <v>14.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>3.5</v>
+        <v>7.8</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.6</v>
+        <v>11.1</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -73886,21 +74350,50 @@
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -73921,7 +74414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -79498,13 +79991,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>16.3</v>
+        <v>17</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -79512,10 +80005,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -79527,7 +80020,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.6</v>
+        <v>14.5</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -79541,10 +80034,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>20.5</v>
+        <v>17.6</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -79556,24 +80049,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>16.2</v>
+        <v>16.9</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>2.3</v>
+        <v>11.4</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>40.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>7.2</v>
+        <v>4.2</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -79585,13 +80078,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>15.3</v>
+        <v>15.5</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -79599,10 +80092,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>1.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.9</v>
+        <v>11.8</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -79614,13 +80107,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.6</v>
+        <v>16.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -79628,10 +80121,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -79643,13 +80136,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.9</v>
+        <v>18.4</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -79657,13 +80150,42 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>12</v>
+        <v>10.6</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -79684,7 +80206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -85261,13 +85783,13 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>11.5</v>
+        <v>11.9</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
@@ -85275,10 +85797,10 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>11.5</v>
+        <v>7.6</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -85290,7 +85812,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -85304,10 +85826,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>5.2</v>
+        <v>9.9</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.4</v>
+        <v>10.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -85319,13 +85841,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>12.2</v>
+        <v>13</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>13.6</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -85333,10 +85855,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>26.6</v>
+        <v>45.9</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -85348,13 +85870,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.1</v>
+        <v>11.7</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4.1</v>
+        <v>4.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -85362,10 +85884,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>36.7</v>
+        <v>30.1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.6</v>
+        <v>8.4</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -85383,7 +85905,7 @@
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.4</v>
+        <v>2.2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -85391,10 +85913,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>12.5</v>
+        <v>6.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.5</v>
+        <v>11.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -85406,27 +85928,56 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>13.9</v>
+        <v>15.3</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>10.3</v>
+        <v>7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.8</v>
+        <v>11.2</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>
@@ -85447,7 +85998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -91024,24 +91575,24 @@
         <v>46287</v>
       </c>
       <c r="B193" s="4" t="n">
-        <v>11.8</v>
+        <v>12.7</v>
       </c>
       <c r="C193" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>6</v>
+        <v>1.1</v>
       </c>
       <c r="G193" s="4" t="n">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="H193" s="10">
         <f>SUM(C187:C193)</f>
@@ -91053,7 +91604,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.8</v>
+        <v>13.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -91067,10 +91618,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>21.9</v>
+        <v>12</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.4</v>
+        <v>10.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -91082,13 +91633,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -91096,10 +91647,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>67.40000000000001</v>
+        <v>58.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>3.9</v>
+        <v>4.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -91111,7 +91662,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -91125,10 +91676,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>30.8</v>
+        <v>11.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>10.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -91140,7 +91691,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -91150,14 +91701,14 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>12</v>
+        <v>11.4</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -91169,7 +91720,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>16.4</v>
+        <v>15.9</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -91179,17 +91730,46 @@
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>6.2</v>
+        <v>34.4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.3</v>
+        <v>7.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B199" s="4" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="C199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H199" s="10">
+        <f>SUM(C193:C199)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-23 10:27 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6119,24 +6119,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>11.3</v>
+        <v>0.9</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>61.9</v>
+        <v>37.1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>4.6</v>
+        <v>7.5</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -6154,7 +6154,7 @@
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -6162,10 +6162,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>23.8</v>
+        <v>18</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>9.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -6177,24 +6177,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>10</v>
+        <v>10.9</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -6206,13 +6206,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>20.5</v>
+        <v>19.7</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>1</v>
+        <v>4.8</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -6220,10 +6220,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>38.8</v>
+        <v>72.3</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>7.3</v>
+        <v>3.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -6235,24 +6235,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21.3</v>
+        <v>18.3</v>
       </c>
       <c r="C198" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="G198" s="7" t="n">
         <v>0.1</v>
-      </c>
-      <c r="D198" s="7" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E198" s="7" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="F198" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="G198" s="7" t="n">
-        <v>11</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -6264,13 +6264,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>21.8</v>
+        <v>19.7</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.3</v>
+        <v>4.5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -6278,13 +6278,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>2.4</v>
+        <v>57</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.7</v>
+        <v>5.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -6305,7 +6334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11911,13 +11940,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>21.9</v>
+        <v>24.3</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -11925,10 +11954,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>28.2</v>
+        <v>33.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8.6</v>
+        <v>8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -11940,13 +11969,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>22.5</v>
+        <v>23.2</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -11954,10 +11983,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>43.9</v>
+        <v>16.7</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.7</v>
+        <v>10</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -11969,13 +11998,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>23.2</v>
+        <v>24.3</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -11983,10 +12012,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>45.7</v>
+        <v>13.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>6.5</v>
+        <v>10.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -11998,13 +12027,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -12012,10 +12041,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>22.6</v>
+        <v>25</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -12027,13 +12056,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -12041,10 +12070,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>87.5</v>
+        <v>46.1</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>1.5</v>
+        <v>6.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -12056,27 +12085,56 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>18.4</v>
+        <v>19.4</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>94.3</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.7</v>
+        <v>1.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -12097,7 +12155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17703,13 +17761,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>7.1</v>
+        <v>8.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -17717,10 +17775,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>11.5</v>
+        <v>24.3</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.6</v>
+        <v>9.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -17732,13 +17790,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -17761,13 +17819,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.4</v>
+        <v>20.1</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>7.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -17775,10 +17833,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -17790,13 +17848,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21.1</v>
+        <v>20.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>5.7</v>
+        <v>4.5</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -17804,10 +17862,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>18.8</v>
+        <v>44.3</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>6.7</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -17819,13 +17877,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21.6</v>
+        <v>21.3</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>7.8</v>
+        <v>2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -17833,10 +17891,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>0</v>
+        <v>75.8</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>12</v>
+        <v>2.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -17848,27 +17906,56 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>21.8</v>
+        <v>21</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>7.7</v>
+        <v>3.5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0</v>
+        <v>14.8</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>12</v>
+        <v>10.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -17889,7 +17976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23495,24 +23582,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>20.9</v>
+        <v>21.7</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>36.3</v>
+        <v>28.3</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>7.6</v>
+        <v>8.6</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -23530,7 +23617,7 @@
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -23538,10 +23625,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>68</v>
+        <v>58.3</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>3.8</v>
+        <v>5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -23553,24 +23640,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.9</v>
+        <v>21.5</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>73</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -23582,24 +23669,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>19.8</v>
+        <v>20.4</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>6.2</v>
+        <v>19.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -23611,24 +23698,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20</v>
+        <v>21.3</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.3</v>
+        <v>2.2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>18</v>
+        <v>22.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -23640,13 +23727,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.4</v>
+        <v>21.3</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -23654,13 +23741,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>2.9</v>
+        <v>7.8</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -23681,7 +23797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29287,24 +29403,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>11.1</v>
+        <v>12.7</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>14.1</v>
+        <v>5.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.3</v>
+        <v>11.4</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -29316,13 +29432,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>10.8</v>
+        <v>10.4</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -29330,10 +29446,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>60.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.7</v>
+        <v>3.7</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -29345,24 +29461,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>53.5</v>
+        <v>57.6</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>5.6</v>
+        <v>5.1</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -29374,24 +29490,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>25</v>
+        <v>28.7</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9</v>
+        <v>8.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -29403,7 +29519,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>10.6</v>
+        <v>10.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -29417,10 +29533,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>42.6</v>
+        <v>31.1</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>6.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -29432,13 +29548,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -29446,13 +29562,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>96.09999999999999</v>
+        <v>14.7</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.5</v>
+        <v>10.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -29473,7 +29618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31570,13 +31715,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>5.4</v>
+        <v>1.7</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -31584,10 +31729,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>36.6</v>
+        <v>28.7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>7.6</v>
+        <v>8.6</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -31599,24 +31744,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>2.7</v>
+        <v>11.3</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>66.7</v>
+        <v>76</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -31628,24 +31773,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>4.4</v>
+        <v>1.4</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>49.2</v>
+        <v>53.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>6.1</v>
+        <v>5.5</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -31657,13 +31802,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.1</v>
+        <v>10.1</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -31671,10 +31816,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>80.3</v>
+        <v>39.6</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>2.4</v>
+        <v>7.2</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -31686,24 +31831,24 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.9</v>
+        <v>12.4</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>19.4</v>
+        <v>43.8</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>6.7</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -31715,27 +31860,56 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>14.3</v>
+        <v>12.8</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>9.4</v>
+        <v>0</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>10.9</v>
+        <v>12</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H79" s="10">
+        <f>SUM(C73:C79)</f>
         <v/>
       </c>
     </row>
@@ -31756,7 +31930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33853,24 +34027,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>55.1</v>
+        <v>21.5</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>5.4</v>
+        <v>9.4</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -33882,13 +34056,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>11.2</v>
+        <v>13.9</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -33896,10 +34070,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>79.40000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>2.5</v>
+        <v>3.4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -33911,24 +34085,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>3.1</v>
+        <v>8.5</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>70.09999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>3.6</v>
+        <v>2.4</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -33940,24 +34114,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>49.4</v>
+        <v>64.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>6.1</v>
+        <v>4.3</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -33969,13 +34143,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.4</v>
+        <v>10.8</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -33983,10 +34157,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>17.6</v>
+        <v>75.8</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9.9</v>
+        <v>2.9</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -33998,13 +34172,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.4</v>
+        <v>11.2</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -34012,13 +34186,42 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>40.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>7.1</v>
+        <v>10.8</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H79" s="10">
+        <f>SUM(C73:C79)</f>
         <v/>
       </c>
     </row>
@@ -34039,7 +34242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36136,24 +36339,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>55.1</v>
+        <v>31.1</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>5.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -36165,13 +36368,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>8</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>7.5</v>
+        <v>15.5</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -36179,10 +36382,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>69.8</v>
+        <v>63.7</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -36194,24 +36397,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>64.40000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -36223,24 +36426,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>10.7</v>
+        <v>11.1</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>50.6</v>
+        <v>39.1</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5.9</v>
+        <v>7.3</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -36252,24 +36455,24 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.9</v>
+        <v>12.2</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>4.5</v>
+        <v>71.5</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>11.5</v>
+        <v>3.4</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -36281,13 +36484,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>14.6</v>
+        <v>12.8</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -36295,13 +36498,42 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>30.1</v>
+        <v>7.6</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>8.4</v>
+        <v>11.1</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H79" s="10">
+        <f>SUM(C73:C79)</f>
         <v/>
       </c>
     </row>
@@ -36322,7 +36554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38419,10 +38651,10 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.6</v>
+        <v>10.2</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>3.6</v>
@@ -38433,10 +38665,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>27.4</v>
+        <v>16.4</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -38448,24 +38680,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>6.8</v>
+        <v>12.4</v>
       </c>
       <c r="D74" s="7" t="n">
         <v>2.4</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>64.5</v>
+        <v>71.8</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -38477,24 +38709,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>51.2</v>
+        <v>53.3</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -38506,24 +38738,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>10.3</v>
+        <v>10.6</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>83.2</v>
+        <v>49.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>2</v>
+        <v>6.1</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -38535,13 +38767,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.3</v>
+        <v>11.9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -38549,10 +38781,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>30.6</v>
+        <v>43.4</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>6.8</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -38564,13 +38796,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.9</v>
+        <v>12.9</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -38578,13 +38810,42 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H79" s="10">
+        <f>SUM(C73:C79)</f>
         <v/>
       </c>
     </row>
@@ -38605,7 +38866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40702,24 +40963,24 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>23.7</v>
+        <v>27.4</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -40731,13 +40992,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>8</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>3.3</v>
+        <v>6.3</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -40745,10 +41006,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>63.4</v>
+        <v>54.4</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>4.4</v>
+        <v>5.5</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -40760,24 +41021,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>2.2</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>48.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>6.1</v>
+        <v>3.8</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -40789,24 +41050,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>59.5</v>
+        <v>36.7</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>4.9</v>
+        <v>7.6</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -40818,13 +41079,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>13.3</v>
+        <v>12</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.7</v>
+        <v>1.9</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -40832,10 +41093,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>1.4</v>
+        <v>61.7</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>11.8</v>
+        <v>4.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -40847,13 +41108,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>14.4</v>
+        <v>12.9</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -40861,13 +41122,42 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>26.3</v>
+        <v>3.5</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>11.6</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H79" s="10">
+        <f>SUM(C73:C79)</f>
         <v/>
       </c>
     </row>
@@ -40888,7 +41178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42985,10 +43275,10 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="C73" s="4" t="n">
-        <v>3.4</v>
+        <v>0.5</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>2.9</v>
@@ -42999,10 +43289,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>62.3</v>
+        <v>46.7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>4.5</v>
+        <v>6.4</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -43017,10 +43307,10 @@
         <v>5.3</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>11.5</v>
+        <v>7.7</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -43028,10 +43318,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>77.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -43043,13 +43333,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>4.1</v>
+        <v>6.5</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -43057,10 +43347,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>71.7</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -43072,24 +43362,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>7.5</v>
+        <v>6.8</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>64.3</v>
+        <v>56.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>4.3</v>
+        <v>5.3</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -43101,24 +43391,24 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>14.6</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>10.2</v>
+        <v>1.2</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -43130,13 +43420,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>10.5</v>
+        <v>8.9</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -43144,13 +43434,42 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>16.6</v>
+        <v>11.7</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>10</v>
+        <v>10.6</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H79" s="10">
+        <f>SUM(C73:C79)</f>
         <v/>
       </c>
     </row>
@@ -43171,7 +43490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48777,7 +49096,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>17.9</v>
+        <v>18.5</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -48787,14 +49106,14 @@
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>56.4</v>
+        <v>49.3</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -48806,13 +49125,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>17.6</v>
+        <v>17.7</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -48820,10 +49139,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>46.6</v>
+        <v>46.2</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -48835,13 +49154,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -48849,10 +49168,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>25.4</v>
+        <v>40.6</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>9</v>
+        <v>7.1</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -48864,24 +49183,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>18.2</v>
+        <v>17.1</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>15</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.9</v>
+        <v>10.2</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -48893,7 +49212,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20</v>
+        <v>18.3</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -48907,10 +49226,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>32.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>8.1</v>
+        <v>11</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -48922,7 +49241,7 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.3</v>
+        <v>18.7</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
@@ -48932,17 +49251,46 @@
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>52.1</v>
+        <v>36.5</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>5.7</v>
+        <v>7.6</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -48963,7 +49311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51060,13 +51408,13 @@
         <v>46288</v>
       </c>
       <c r="B73" s="4" t="n">
-        <v>8.4</v>
+        <v>9.4</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
@@ -51074,10 +51422,10 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>52</v>
+        <v>51.2</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H73" s="10">
         <f>SUM(C67:C73)</f>
@@ -51089,13 +51437,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>16.1</v>
+        <v>17.2</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -51103,10 +51451,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>85.90000000000001</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>1.7</v>
+        <v>4.3</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -51118,13 +51466,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1.9</v>
+        <v>6.6</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -51132,10 +51480,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>97.09999999999999</v>
+        <v>99.3</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -51147,24 +51495,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>9</v>
+        <v>10.1</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>29.3</v>
+        <v>79.7</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8.5</v>
+        <v>2.4</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -51176,13 +51524,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>2.3</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -51190,10 +51538,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>7.8</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>11.1</v>
+        <v>3.2</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -51205,13 +51553,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.3</v>
+        <v>12.3</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.8</v>
+        <v>3.4</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -51219,13 +51567,42 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>44.5</v>
+        <v>3.1</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>6.7</v>
+        <v>11.6</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H79" s="10">
+        <f>SUM(C73:C79)</f>
         <v/>
       </c>
     </row>
@@ -51246,7 +51623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56852,13 +57229,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>24.6</v>
+        <v>24.2</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>5.8</v>
+        <v>7.1</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -56866,10 +57243,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>4.9</v>
+        <v>0.5</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -56881,13 +57258,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>23.6</v>
+        <v>23.1</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -56895,10 +57272,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -56910,13 +57287,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>22.4</v>
+        <v>22.1</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>7.6</v>
+        <v>39</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -56924,10 +57301,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>47.3</v>
+        <v>56.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>6.3</v>
+        <v>5.2</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -56939,13 +57316,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>22.7</v>
+        <v>22.3</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -56953,10 +57330,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>17.2</v>
+        <v>6.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.9</v>
+        <v>11.2</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -56968,13 +57345,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>23.2</v>
+        <v>23</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3.2</v>
+        <v>5.2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -56982,10 +57359,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>6.6</v>
+        <v>12.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.2</v>
+        <v>10.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -56997,13 +57374,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>23.1</v>
+        <v>22.5</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -57011,13 +57388,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>3.1</v>
+        <v>48</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.6</v>
+        <v>6.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -57038,7 +57444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62644,13 +63050,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>18.6</v>
+        <v>20.6</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -62658,10 +63064,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>20.2</v>
+        <v>14.7</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.6</v>
+        <v>10.2</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -62673,13 +63079,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19</v>
+        <v>19.4</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -62687,10 +63093,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>10.2</v>
+        <v>20.9</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10.8</v>
+        <v>9.5</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -62702,24 +63108,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>19.4</v>
+        <v>20.2</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>28.6</v>
+        <v>13.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.6</v>
+        <v>10.4</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -62731,7 +63137,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -62745,10 +63151,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="G197" s="4" t="n">
         <v>10.3</v>
-      </c>
-      <c r="G197" s="4" t="n">
-        <v>10.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -62760,13 +63166,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.1</v>
+        <v>17.5</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0.1</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -62774,10 +63180,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>75</v>
+        <v>69.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -62789,13 +63195,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -62803,13 +63209,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>87.7</v>
+        <v>86.7</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -62830,7 +63265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68436,17 +68871,17 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.7</v>
+        <v>12.7</v>
       </c>
       <c r="C194" s="7" t="n">
-        <v>36.9</v>
+        <v>23.7</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>0.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
@@ -68465,24 +68900,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>14</v>
+        <v>12.4</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>3</v>
+        <v>0.9</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>92</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>1</v>
+        <v>3.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -68494,24 +68929,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>12.9</v>
+        <v>11.9</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>2.6</v>
+        <v>6.5</v>
       </c>
       <c r="D196" s="7" t="n">
         <v>0.7</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>98.40000000000001</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -68523,24 +68958,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>12.9</v>
+        <v>12.6</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="D197" s="4" t="n">
         <v>0.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>85.2</v>
+        <v>67.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>1.8</v>
+        <v>3.9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -68552,24 +68987,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>12.5</v>
+        <v>12.2</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>87.2</v>
+        <v>71.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>1.5</v>
+        <v>3.4</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -68581,13 +69016,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>13.3</v>
+        <v>13.1</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -68595,13 +69030,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>97</v>
+        <v>95.7</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -68622,7 +69086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -74228,24 +74692,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.1</v>
+        <v>15</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>16</v>
+        <v>22.1</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -74257,10 +74721,10 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>14.4</v>
+        <v>8.1</v>
       </c>
       <c r="D195" s="4" t="n">
         <v>2.8</v>
@@ -74271,7 +74735,7 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>60.4</v>
+        <v>59.7</v>
       </c>
       <c r="G195" s="4" t="n">
         <v>4.8</v>
@@ -74286,13 +74750,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>14.8</v>
+        <v>14.2</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -74300,10 +74764,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>1</v>
+        <v>5.6</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.9</v>
+        <v>11.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -74315,24 +74779,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>14.2</v>
+        <v>14</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>7.8</v>
+        <v>4.3</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -74344,24 +74808,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.9</v>
+        <v>14.9</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>2.7</v>
+        <v>9.4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.7</v>
+        <v>10.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -74373,13 +74837,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>16.4</v>
+        <v>15.1</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -74387,13 +74851,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>25.8</v>
+        <v>0.4</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>8.9</v>
+        <v>12</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -74414,7 +74907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80020,7 +80513,7 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>14.5</v>
+        <v>15.9</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
@@ -80030,14 +80523,14 @@
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -80049,13 +80542,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>16.9</v>
+        <v>16.6</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -80063,10 +80556,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>59.1</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.2</v>
+        <v>4.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -80078,13 +80571,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>15.5</v>
+        <v>15.2</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -80092,10 +80585,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>1.8</v>
+        <v>5.9</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.8</v>
+        <v>11.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -80107,21 +80600,21 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>16.2</v>
+        <v>14.9</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="G197" s="4" t="n">
         <v>11.6</v>
@@ -80136,13 +80629,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>18.4</v>
+        <v>16.2</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -80150,10 +80643,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>11.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.6</v>
+        <v>10.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -80165,13 +80658,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>19.1</v>
+        <v>16.7</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -80179,13 +80672,42 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>28.7</v>
+        <v>0.4</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>8.6</v>
+        <v>12</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -80206,7 +80728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -85812,13 +86334,13 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>10.9</v>
+        <v>12</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>3.7</v>
+        <v>2.7</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
@@ -85826,10 +86348,10 @@
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>9.9</v>
+        <v>11.2</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -85841,13 +86363,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>13</v>
+        <v>12.8</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>13.6</v>
+        <v>24.3</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -85855,10 +86377,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>45.9</v>
+        <v>53.5</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.5</v>
+        <v>5.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -85870,13 +86392,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.7</v>
+        <v>10.1</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -85884,10 +86406,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>30.1</v>
+        <v>23</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -85899,13 +86421,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>12.2</v>
+        <v>10.9</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -85913,10 +86435,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>6.1</v>
+        <v>3.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -85928,21 +86450,21 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.3</v>
+        <v>12</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>7</v>
+        <v>6.4</v>
       </c>
       <c r="G198" s="7" t="n">
         <v>11.2</v>
@@ -85957,27 +86479,56 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>17.2</v>
+        <v>13</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>3.1</v>
+        <v>5.9</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.6</v>
+        <v>11.3</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>
@@ -85998,7 +86549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -91604,24 +92155,24 @@
         <v>46288</v>
       </c>
       <c r="B194" s="7" t="n">
-        <v>13.9</v>
+        <v>15.1</v>
       </c>
       <c r="C194" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F194" s="7" t="n">
-        <v>12</v>
+        <v>1.7</v>
       </c>
       <c r="G194" s="7" t="n">
-        <v>10.6</v>
+        <v>11.8</v>
       </c>
       <c r="H194" s="12">
         <f>SUM(C188:C194)</f>
@@ -91633,7 +92184,7 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>13.3</v>
+        <v>13</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
@@ -91647,10 +92198,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>58.8</v>
+        <v>61.7</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.9</v>
+        <v>4.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -91662,13 +92213,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.9</v>
+        <v>13</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -91676,10 +92227,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>11.3</v>
+        <v>26.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -91691,7 +92242,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.7</v>
+        <v>15.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -91701,14 +92252,14 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>4.7</v>
+        <v>0.6</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -91720,7 +92271,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -91734,10 +92285,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>34.4</v>
+        <v>0</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>7.9</v>
+        <v>12</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -91749,27 +92300,56 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>78.3</v>
+        <v>32</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>2.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="11" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="C200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="G200" s="7" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H200" s="12">
+        <f>SUM(C194:C200)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-24 10:44 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6148,13 +6148,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>18.8</v>
+        <v>20.1</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3.5</v>
+        <v>3.9</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -6162,10 +6162,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>18</v>
+        <v>13.3</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -6177,13 +6177,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -6191,10 +6191,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>10.9</v>
+        <v>44.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.7</v>
+        <v>6.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -6206,24 +6206,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>19.7</v>
+        <v>18.5</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>4.8</v>
+        <v>37.8</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.9</v>
+        <v>3.8</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>72.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>3.3</v>
+        <v>1.1</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -6235,13 +6235,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>11.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4</v>
+        <v>5.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -6249,10 +6249,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>99.2</v>
+        <v>77.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>0.1</v>
+        <v>2.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -6264,13 +6264,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>19.7</v>
+        <v>20.7</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -6278,10 +6278,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>57</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>5.2</v>
+        <v>11</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -6293,13 +6293,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -6307,13 +6307,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>10.9</v>
+        <v>11.3</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -6334,7 +6363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11969,13 +11998,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>23.2</v>
+        <v>25.6</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -11983,10 +12012,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>16.7</v>
+        <v>26.7</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>10</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -11998,13 +12027,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -12012,10 +12041,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>13.8</v>
+        <v>2.1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -12027,13 +12056,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21.6</v>
+        <v>22</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -12041,10 +12070,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>25</v>
+        <v>33.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -12056,13 +12085,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.4</v>
+        <v>20.6</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -12070,10 +12099,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>46.1</v>
+        <v>68.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>6.5</v>
+        <v>3.8</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -12085,10 +12114,10 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>19.4</v>
+        <v>18.6</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="D199" s="4" t="n">
         <v>2.6</v>
@@ -12099,10 +12128,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>84.40000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>1.9</v>
+        <v>3.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -12114,27 +12143,56 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>15.2</v>
+        <v>17.1</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>18.6</v>
+        <v>4.6</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>97.5</v>
+        <v>70.5</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>0.3</v>
+        <v>3.5</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -12155,7 +12213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17790,13 +17848,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>10.3</v>
+        <v>10.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -17819,13 +17877,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -17833,10 +17891,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>0.7</v>
+        <v>1.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -17848,13 +17906,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>20.8</v>
+        <v>20.3</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -17862,10 +17920,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>44.3</v>
+        <v>43.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -17877,24 +17935,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21.3</v>
+        <v>20.7</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2</v>
+        <v>2.9</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>75.8</v>
+        <v>71.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -17906,24 +17964,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>21</v>
+        <v>21.2</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.5</v>
+        <v>5.2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>14.8</v>
+        <v>11.3</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.2</v>
+        <v>10.6</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -17935,17 +17993,17 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>21.8</v>
+        <v>21.1</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>7.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
@@ -17956,6 +18014,35 @@
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -17976,7 +18063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23611,24 +23698,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>21.2</v>
+        <v>22.9</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.8</v>
+        <v>4.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>58.3</v>
+        <v>93.5</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5</v>
+        <v>0.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -23640,24 +23727,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>21.5</v>
+        <v>21.7</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>64.09999999999999</v>
+        <v>74.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>4.3</v>
+        <v>3.1</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -23669,24 +23756,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>20.4</v>
+        <v>21.1</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -23698,13 +23785,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -23712,10 +23799,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>22.2</v>
+        <v>20.3</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -23727,13 +23814,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>21.3</v>
+        <v>21</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -23741,10 +23828,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>35</v>
+        <v>4.7</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>7.8</v>
+        <v>11.4</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -23756,27 +23843,56 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>20.8</v>
+        <v>20.9</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="n">
         <v>1.6</v>
       </c>
-      <c r="E200" s="7" t="inlineStr">
-        <is>
-          <t>JV</t>
-        </is>
-      </c>
-      <c r="F200" s="7" t="n">
-        <v>3.1</v>
-      </c>
       <c r="G200" s="7" t="n">
-        <v>11.6</v>
+        <v>11.8</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -23797,7 +23913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29432,24 +29548,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>10.4</v>
+        <v>13.4</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>69.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>3.7</v>
+        <v>1.1</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -29461,13 +29577,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -29475,7 +29591,7 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>57.6</v>
+        <v>57.9</v>
       </c>
       <c r="G196" s="7" t="n">
         <v>5.1</v>
@@ -29490,13 +29606,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>10.3</v>
+        <v>11</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -29504,10 +29620,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>28.7</v>
+        <v>29.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -29519,13 +29635,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -29533,10 +29649,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>31.1</v>
+        <v>22.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -29548,7 +29664,7 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>10.5</v>
+        <v>10.8</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
@@ -29562,10 +29678,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>14.7</v>
+        <v>10.3</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.2</v>
+        <v>10.8</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -29583,7 +29699,7 @@
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -29591,13 +29707,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>61.6</v>
+        <v>32.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>4.6</v>
+        <v>8.1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -29618,7 +29763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31744,24 +31889,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.4</v>
+        <v>11</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>11.3</v>
+        <v>5.5</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>76</v>
+        <v>93.3</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>2.9</v>
+        <v>0.8</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -31773,24 +31918,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.6</v>
+        <v>10.2</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1.4</v>
+        <v>4.4</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>53.8</v>
+        <v>65.7</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>5.5</v>
+        <v>4.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -31802,13 +31947,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>10.1</v>
+        <v>11.9</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -31816,10 +31961,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>39.6</v>
+        <v>56.3</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>7.2</v>
+        <v>5.2</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -31831,24 +31976,24 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.4</v>
+        <v>13</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>43.8</v>
+        <v>27.6</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>6.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -31860,13 +32005,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.8</v>
+        <v>13.3</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -31874,10 +32019,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -31889,13 +32034,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13</v>
+        <v>11.8</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -31903,13 +32048,42 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H80" s="12">
+        <f>SUM(C74:C80)</f>
         <v/>
       </c>
     </row>
@@ -31930,7 +32104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34056,24 +34230,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>7.7</v>
+        <v>10.5</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>71.7</v>
+        <v>98.3</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.4</v>
+        <v>0.2</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -34085,13 +34259,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.4</v>
+        <v>10.3</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -34099,10 +34273,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>79.90000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -34114,24 +34288,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>64.2</v>
+        <v>54.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>4.3</v>
+        <v>5.5</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -34149,7 +34323,7 @@
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -34157,10 +34331,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>75.8</v>
+        <v>24.6</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>2.9</v>
+        <v>9</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -34172,13 +34346,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -34186,10 +34360,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>0</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -34201,27 +34375,56 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>15.4</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>10.2</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H80" s="12">
+        <f>SUM(C74:C80)</f>
         <v/>
       </c>
     </row>
@@ -34242,7 +34445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36368,13 +36571,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8</v>
+        <v>9.4</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>15.5</v>
+        <v>11.7</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -36382,10 +36585,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>63.7</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>4.4</v>
+        <v>0.8</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -36397,13 +36600,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -36411,10 +36614,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>71.3</v>
+        <v>66.7</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -36426,24 +36629,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>39.1</v>
+        <v>51</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>7.3</v>
+        <v>5.9</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -36455,13 +36658,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.2</v>
+        <v>12.5</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -36469,10 +36672,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>71.5</v>
+        <v>17.8</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>3.4</v>
+        <v>9.9</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -36484,24 +36687,24 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.8</v>
+        <v>13.8</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>7.6</v>
+        <v>1</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.1</v>
+        <v>11.9</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -36513,27 +36716,56 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
         <v>14.7</v>
       </c>
-      <c r="C79" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D79" s="4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>JZ</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>10.2</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="H80" s="12">
+        <f>SUM(C74:C80)</f>
         <v/>
       </c>
     </row>
@@ -36554,7 +36786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38680,24 +38912,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>12.4</v>
+        <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>71.8</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.4</v>
+        <v>1.3</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -38709,24 +38941,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.4</v>
+        <v>10.3</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>5.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>53.3</v>
+        <v>58</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>5.6</v>
+        <v>5</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -38738,10 +38970,10 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>10.6</v>
+        <v>11.4</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="D76" s="7" t="n">
         <v>1.5</v>
@@ -38752,10 +38984,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>49.2</v>
+        <v>61.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -38767,13 +38999,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.9</v>
+        <v>12.7</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -38781,10 +39013,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>43.4</v>
+        <v>36.1</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>6.8</v>
+        <v>7.7</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -38796,21 +39028,21 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.9</v>
+        <v>13.2</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>12</v>
@@ -38825,27 +39057,56 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.1</v>
+        <v>11.7</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>0.7</v>
+        <v>2.2</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H80" s="12">
+        <f>SUM(C74:C80)</f>
         <v/>
       </c>
     </row>
@@ -38866,7 +39127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40992,24 +41253,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>8</v>
+        <v>9.6</v>
       </c>
       <c r="C74" s="7" t="n">
         <v>6.3</v>
       </c>
       <c r="D74" s="7" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="G74" s="7" t="n">
         <v>2.9</v>
-      </c>
-      <c r="E74" s="7" t="inlineStr">
-        <is>
-          <t>JV</t>
-        </is>
-      </c>
-      <c r="F74" s="7" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="G74" s="7" t="n">
-        <v>5.5</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -41021,13 +41282,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9</v>
+        <v>10.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -41035,10 +41296,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>68.59999999999999</v>
+        <v>59.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>3.8</v>
+        <v>4.8</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -41050,24 +41311,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>36.7</v>
+        <v>53</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>7.6</v>
+        <v>5.6</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -41079,13 +41340,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -41093,10 +41354,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>61.7</v>
+        <v>17.2</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>4.6</v>
+        <v>9.9</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -41108,13 +41369,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.9</v>
+        <v>13.8</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -41122,10 +41383,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>3.5</v>
+        <v>4.7</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -41137,13 +41398,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.5</v>
+        <v>13</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -41151,13 +41412,42 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H80" s="12">
+        <f>SUM(C74:C80)</f>
         <v/>
       </c>
     </row>
@@ -41178,7 +41468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43304,13 +43594,13 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>5.3</v>
+        <v>6.9</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>7.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
@@ -43318,10 +43608,10 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>70.09999999999999</v>
+        <v>96</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>3.6</v>
+        <v>0.5</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -43333,13 +43623,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>5.7</v>
+        <v>6.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>6.5</v>
+        <v>1.9</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -43347,10 +43637,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>76.40000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>2.8</v>
+        <v>3.9</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -43362,24 +43652,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>6.8</v>
+        <v>7.7</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>56.2</v>
+        <v>66.7</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5.3</v>
+        <v>4</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -43391,24 +43681,24 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>89.59999999999999</v>
+        <v>42.8</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>1.2</v>
+        <v>6.9</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -43420,13 +43710,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>8.9</v>
+        <v>10</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -43434,10 +43724,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>11.7</v>
+        <v>4.7</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>10.6</v>
+        <v>11.4</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -43449,27 +43739,56 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>9.9</v>
+        <v>8.9</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>4.9</v>
+        <v>1</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H80" s="12">
+        <f>SUM(C74:C80)</f>
         <v/>
       </c>
     </row>
@@ -43490,7 +43809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49125,24 +49444,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>17.7</v>
+        <v>20</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>46.2</v>
+        <v>58.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>6.5</v>
+        <v>4.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -49154,7 +49473,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>17.2</v>
+        <v>16.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -49164,14 +49483,14 @@
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>40.6</v>
+        <v>24.2</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.1</v>
+        <v>9.1</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -49183,24 +49502,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.1</v>
+        <v>18</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>15</v>
+        <v>16.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -49212,7 +49531,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>18.3</v>
+        <v>19.6</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -49222,14 +49541,14 @@
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>3.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11</v>
+        <v>11.6</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -49241,13 +49560,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>18.7</v>
+        <v>20.3</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -49255,10 +49574,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>36.5</v>
+        <v>5.1</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>7.6</v>
+        <v>11.4</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -49270,13 +49589,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>19.6</v>
+        <v>20.5</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -49284,13 +49603,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>27.4</v>
+        <v>7.2</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>11.1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -49311,7 +49659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51437,24 +51785,24 @@
         <v>46289</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>7.8</v>
+        <v>9.1</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>17.2</v>
+        <v>1.1</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>64.40000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="H74" s="12">
         <f>SUM(C68:C74)</f>
@@ -51466,13 +51814,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>6.6</v>
+        <v>2.1</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -51480,10 +51828,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>99.3</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>0.1</v>
+        <v>1.1</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -51495,24 +51843,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>10.1</v>
+        <v>9.5</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
         <v>2.2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>79.7</v>
+        <v>33.4</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>2.4</v>
+        <v>8</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -51524,13 +51872,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>2.3</v>
+        <v>1.4</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -51538,10 +51886,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>73.59999999999999</v>
+        <v>53.5</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>3.2</v>
+        <v>5.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -51559,7 +51907,7 @@
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>3.4</v>
+        <v>2.3</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -51567,10 +51915,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>3.1</v>
+        <v>0.2</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -51582,27 +51930,56 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H80" s="12">
+        <f>SUM(C74:C80)</f>
         <v/>
       </c>
     </row>
@@ -51623,7 +52000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -57258,13 +57635,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>23.1</v>
+        <v>23.8</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -57272,10 +57649,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>3.9</v>
+        <v>6.4</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>11.5</v>
+        <v>11.2</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -57287,13 +57664,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>22.1</v>
+        <v>23.5</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>39</v>
+        <v>14.7</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -57301,10 +57678,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>56.3</v>
+        <v>47.1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>5.2</v>
+        <v>6.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -57316,13 +57693,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>22.3</v>
+        <v>23</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.9</v>
+        <v>7.2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -57330,10 +57707,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>6.5</v>
+        <v>29</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.2</v>
+        <v>8.5</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -57345,13 +57722,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>5.2</v>
+        <v>6</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -57359,10 +57736,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>12.5</v>
+        <v>26.1</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.5</v>
+        <v>8.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -57374,13 +57751,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>22.5</v>
+        <v>22.7</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.3</v>
+        <v>2.6</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -57388,10 +57765,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>48</v>
+        <v>57.8</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>6.2</v>
+        <v>5.1</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -57403,13 +57780,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>22.5</v>
+        <v>22.8</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -57417,13 +57794,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -57444,7 +57850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63079,13 +63485,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>19.4</v>
+        <v>21.3</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -63093,10 +63499,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>20.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>9.5</v>
+        <v>10.8</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -63114,7 +63520,7 @@
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -63122,10 +63528,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>13.7</v>
+        <v>14.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -63137,13 +63543,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.6</v>
+        <v>18.3</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.3</v>
+        <v>4.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -63151,10 +63557,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>14.4</v>
+        <v>35.3</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.3</v>
+        <v>7.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -63166,10 +63572,10 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.5</v>
+        <v>17.3</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
         <v>4.5</v>
@@ -63180,10 +63586,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>69.5</v>
+        <v>58.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -63195,13 +63601,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>17.4</v>
+        <v>16.8</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.7</v>
+        <v>1.7</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -63209,10 +63615,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>86.7</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -63224,10 +63630,10 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>15.2</v>
+        <v>16.9</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>15.8</v>
+        <v>1.8</v>
       </c>
       <c r="D200" s="7" t="n">
         <v>3.8</v>
@@ -63238,13 +63644,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>95.90000000000001</v>
+        <v>59.4</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>0.5</v>
+        <v>4.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -63265,7 +63700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68900,24 +69335,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>12.4</v>
+        <v>11.8</v>
       </c>
       <c r="C195" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="D195" s="4" t="n">
-        <v>0.8</v>
-      </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>67.90000000000001</v>
+        <v>36.4</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>3.9</v>
+        <v>7.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -68929,10 +69364,10 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.9</v>
+        <v>10.8</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="D196" s="7" t="n">
         <v>0.7</v>
@@ -68943,10 +69378,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>96.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>0.4</v>
+        <v>2.5</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -68958,24 +69393,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>12.6</v>
+        <v>10.4</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>67.2</v>
+        <v>53.8</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>3.9</v>
+        <v>5.5</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -68987,24 +69422,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>12.2</v>
+        <v>13</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>71.5</v>
+        <v>83.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3.4</v>
+        <v>2</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -69016,24 +69451,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>13.1</v>
+        <v>12.8</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>95.7</v>
+        <v>97.2</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -69045,27 +69480,56 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>13</v>
+        <v>11.6</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>93.2</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -69086,7 +69550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -74721,13 +75185,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>15.5</v>
+        <v>16.6</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>8.1</v>
+        <v>29.7</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -74735,10 +75199,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>59.7</v>
+        <v>83.8</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.8</v>
+        <v>1.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -74750,13 +75214,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>14.2</v>
+        <v>13.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -74764,10 +75228,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -74779,13 +75243,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>14</v>
+        <v>14.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2.4</v>
+        <v>3.7</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -74793,10 +75257,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>4.3</v>
+        <v>1.6</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -74808,24 +75272,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>14.9</v>
+        <v>15.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>9.4</v>
+        <v>1.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.9</v>
+        <v>11.8</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -74837,13 +75301,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>15.1</v>
+        <v>16</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -74851,7 +75315,7 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="G199" s="4" t="n">
         <v>12</v>
@@ -74866,7 +75330,7 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>16.7</v>
+        <v>17.2</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
@@ -74880,13 +75344,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -74907,7 +75400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80542,13 +81035,13 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>16.6</v>
+        <v>17.7</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>11.1</v>
+        <v>29.6</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
@@ -80556,10 +81049,10 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>59.1</v>
+        <v>78.7</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.9</v>
+        <v>2.6</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -80571,13 +81064,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>15.2</v>
+        <v>14.7</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -80585,10 +81078,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>5.9</v>
+        <v>3.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -80600,13 +81093,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>14.9</v>
+        <v>15.7</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -80614,10 +81107,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>3.1</v>
+        <v>1.7</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.6</v>
+        <v>11.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -80629,13 +81122,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>16.2</v>
+        <v>16.8</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -80643,10 +81136,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.9</v>
+        <v>11.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -80658,7 +81151,7 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>16.7</v>
+        <v>17.8</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
@@ -80672,7 +81165,7 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="G199" s="4" t="n">
         <v>12</v>
@@ -80687,7 +81180,7 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>18.1</v>
+        <v>18.8</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
@@ -80701,13 +81194,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G200" s="7" t="n">
         <v>12</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -80728,7 +81250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -86363,24 +86885,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>12.8</v>
+        <v>14.5</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>24.3</v>
+        <v>42.3</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>53.5</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>5.6</v>
+        <v>0.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -86392,13 +86914,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>10.1</v>
+        <v>10.2</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -86406,10 +86928,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>23</v>
+        <v>36.1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -86421,24 +86943,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G197" s="4" t="n">
         <v>10.9</v>
-      </c>
-      <c r="C197" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D197" s="4" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E197" s="4" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F197" s="4" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="G197" s="4" t="n">
-        <v>11.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -86450,13 +86972,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>12</v>
+        <v>12.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -86464,10 +86986,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>6.4</v>
+        <v>23.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -86479,13 +87001,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>13</v>
+        <v>13.8</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -86493,10 +87015,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>5.9</v>
+        <v>18.4</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -86514,7 +87036,7 @@
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -86522,13 +87044,42 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>25</v>
+        <v>4.3</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>9</v>
+        <v>11.5</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>
@@ -86549,7 +87100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -92184,24 +92735,24 @@
         <v>46289</v>
       </c>
       <c r="B195" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C195" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>61.7</v>
+        <v>76</v>
       </c>
       <c r="G195" s="4" t="n">
-        <v>4.6</v>
+        <v>2.9</v>
       </c>
       <c r="H195" s="10">
         <f>SUM(C189:C195)</f>
@@ -92219,7 +92770,7 @@
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -92227,10 +92778,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>26.3</v>
+        <v>34.2</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -92242,24 +92793,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.2</v>
+        <v>15.9</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>0.6</v>
+        <v>14.4</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.9</v>
+        <v>10.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -92271,13 +92822,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -92285,10 +92836,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -92300,13 +92851,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>15.3</v>
+        <v>15.8</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -92314,10 +92865,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>32</v>
+        <v>49.2</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -92329,27 +92880,56 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>15</v>
+        <v>14.8</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>32.2</v>
+        <v>19.1</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>8.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B201" s="4" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="C201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H201" s="10">
+        <f>SUM(C195:C201)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-25 10:48 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6177,7 +6177,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20</v>
+        <v>20.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -6191,10 +6191,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>44.7</v>
+        <v>46.2</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -6206,24 +6206,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>18.5</v>
+        <v>17.9</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>37.8</v>
+        <v>35.4</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.8</v>
+        <v>4.5</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>90.59999999999999</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -6235,24 +6235,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>18.4</v>
+        <v>19.4</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>7.4</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>5.8</v>
+        <v>8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>77.7</v>
+        <v>49.3</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>2.7</v>
+        <v>6.1</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -6264,13 +6264,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.7</v>
+        <v>20.4</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -6278,7 +6278,7 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="G199" s="4" t="n">
         <v>11</v>
@@ -6293,24 +6293,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>20.3</v>
+        <v>20</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.4</v>
+        <v>3.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>5.8</v>
+        <v>2.9</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.3</v>
+        <v>11.7</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -6322,27 +6322,56 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.1</v>
+        <v>4.6</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>18.6</v>
+        <v>5.3</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>11.4</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -6363,7 +6392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12027,24 +12056,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>24.4</v>
+        <v>26.3</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.3</v>
+        <v>3.2</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>2.1</v>
+        <v>6.9</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.7</v>
+        <v>11.2</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -12056,24 +12085,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>22</v>
+        <v>21.7</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>33.5</v>
+        <v>23</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -12085,13 +12114,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.6</v>
+        <v>20.4</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.4</v>
+        <v>3.3</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -12099,10 +12128,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>68.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -12114,13 +12143,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>18.6</v>
+        <v>19.6</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -12128,10 +12157,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>70.5</v>
+        <v>86.3</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>3.5</v>
+        <v>1.6</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -12143,13 +12172,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>17.1</v>
+        <v>18.6</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>4.6</v>
+        <v>1.1</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -12157,10 +12186,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>70.5</v>
+        <v>42.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>3.5</v>
+        <v>6.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -12172,13 +12201,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>0.9</v>
+        <v>8.4</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -12186,13 +12215,42 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>63.3</v>
+        <v>52.3</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>4.4</v>
+        <v>5.7</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -12213,7 +12271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17877,13 +17935,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>8.4</v>
+        <v>7.3</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -17891,10 +17949,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>1.7</v>
+        <v>2.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -17912,7 +17970,7 @@
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -17920,10 +17978,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>43.5</v>
+        <v>74.8</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>6.8</v>
+        <v>3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -17935,13 +17993,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.7</v>
+        <v>21.3</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -17949,10 +18007,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>71.7</v>
+        <v>65.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -17967,21 +18025,21 @@
         <v>21.2</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>5.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>11.3</v>
+        <v>0.6</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.6</v>
+        <v>11.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -17993,13 +18051,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>21.1</v>
+        <v>21</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -18022,17 +18080,17 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>20.5</v>
+        <v>21.3</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
@@ -18043,6 +18101,35 @@
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -18063,7 +18150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23727,7 +23814,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>21.7</v>
+        <v>22.6</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -23737,14 +23824,14 @@
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>74.3</v>
+        <v>54.3</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>3.1</v>
+        <v>5.5</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -23762,7 +23849,7 @@
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -23770,10 +23857,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>16.5</v>
+        <v>18.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -23785,24 +23872,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21.2</v>
+        <v>21.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.4</v>
+        <v>3.7</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>20.3</v>
+        <v>4.4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>9.6</v>
+        <v>11.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -23814,13 +23901,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>21</v>
+        <v>20.9</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -23828,10 +23915,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>4.7</v>
+        <v>1.3</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -23849,7 +23936,7 @@
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -23857,10 +23944,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>1.6</v>
+        <v>42.6</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.8</v>
+        <v>6.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -23872,27 +23959,56 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>21.3</v>
+        <v>21.8</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>22.8</v>
+        <v>8.6</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>11</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -23913,7 +24029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29577,24 +29693,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>11.1</v>
+        <v>13.1</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>57.9</v>
+        <v>38.1</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>5.1</v>
+        <v>7.4</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -29612,7 +29728,7 @@
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -29620,10 +29736,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>29.1</v>
+        <v>32.4</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.5</v>
+        <v>8.1</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -29635,13 +29751,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>10.6</v>
+        <v>11</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.8</v>
+        <v>1.7</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -29649,10 +29765,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>22.6</v>
+        <v>13.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -29664,7 +29780,7 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
@@ -29678,10 +29794,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>10.3</v>
+        <v>89.5</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.8</v>
+        <v>1.3</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -29693,13 +29809,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>10.7</v>
+        <v>11</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -29707,10 +29823,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>32.8</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>8.1</v>
+        <v>2.2</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -29722,13 +29838,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -29736,13 +29852,42 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>41</v>
+        <v>33.4</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>7.1</v>
+        <v>8</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>97.7</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -29763,7 +29908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31918,24 +32063,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.2</v>
+        <v>11.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>65.7</v>
+        <v>36.1</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>4.1</v>
+        <v>7.7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -31947,13 +32092,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.9</v>
+        <v>12.2</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -31961,10 +32106,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>56.3</v>
+        <v>38.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5.2</v>
+        <v>7.4</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -31976,13 +32121,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -31990,10 +32135,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>27.6</v>
+        <v>28.3</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -32005,13 +32150,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.3</v>
+        <v>12.5</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -32019,10 +32164,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -32034,24 +32179,24 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>11.8</v>
+        <v>13.1</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2.6</v>
+        <v>1.1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -32063,13 +32208,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.1</v>
+        <v>13.7</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>3.1</v>
+        <v>1.4</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -32077,13 +32222,42 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="G80" s="7" t="n">
         <v>11.8</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H81" s="10">
+        <f>SUM(C75:C81)</f>
         <v/>
       </c>
     </row>
@@ -32104,7 +32278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34259,13 +34433,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.3</v>
+        <v>10.7</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -34273,10 +34447,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>89.90000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>1.2</v>
+        <v>3.3</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -34294,7 +34468,7 @@
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -34302,10 +34476,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>54.2</v>
+        <v>40.8</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -34317,13 +34491,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>10.8</v>
+        <v>11.1</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -34331,10 +34505,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>24.6</v>
+        <v>36.4</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -34346,13 +34520,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -34360,10 +34534,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -34375,24 +34549,24 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>15.4</v>
+        <v>0</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>10.2</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -34404,13 +34578,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>11.3</v>
+        <v>11.7</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.9</v>
+        <v>1</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -34418,13 +34592,42 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>1.6</v>
+        <v>3.5</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="H81" s="10">
+        <f>SUM(C75:C81)</f>
         <v/>
       </c>
     </row>
@@ -34445,7 +34648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36600,17 +36803,17 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10</v>
+        <v>10.8</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>2.7</v>
+        <v>0.8</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
@@ -36629,7 +36832,7 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
@@ -36643,10 +36846,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>51</v>
+        <v>28.8</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5.9</v>
+        <v>8.5</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -36658,13 +36861,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -36672,10 +36875,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>17.8</v>
+        <v>34</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9.9</v>
+        <v>7.9</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -36687,24 +36890,24 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.8</v>
+        <v>13.4</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>1</v>
+        <v>2.4</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -36716,13 +36919,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>14.1</v>
+        <v>13.6</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -36730,10 +36933,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>14.7</v>
+        <v>0.2</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>10.2</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -36745,27 +36948,56 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.5</v>
+        <v>13.9</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>14.7</v>
+        <v>3.1</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>10.2</v>
+        <v>11.6</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H81" s="10">
+        <f>SUM(C75:C81)</f>
         <v/>
       </c>
     </row>
@@ -36786,7 +37018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38941,24 +39173,24 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.3</v>
+        <v>11.3</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>58</v>
+        <v>42.4</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>5</v>
+        <v>6.9</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -38970,24 +39202,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.4</v>
+        <v>11.6</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>2.4</v>
+        <v>1.1</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>61.2</v>
+        <v>50.3</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>4.7</v>
+        <v>6</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -38999,13 +39231,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.7</v>
+        <v>12.5</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -39013,10 +39245,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>36.1</v>
+        <v>31.3</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -39028,17 +39260,17 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.2</v>
+        <v>12.6</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
@@ -39057,13 +39289,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>11.7</v>
+        <v>13.3</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2.2</v>
+        <v>0.7</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -39071,10 +39303,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>5.8</v>
+        <v>1.4</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.3</v>
+        <v>11.8</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -39086,13 +39318,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>11.7</v>
+        <v>13.8</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>2.4</v>
+        <v>1.1</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -39100,13 +39332,42 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>15.8</v>
+        <v>0.2</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>10.1</v>
+        <v>12</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H81" s="10">
+        <f>SUM(C75:C81)</f>
         <v/>
       </c>
     </row>
@@ -39127,7 +39388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41282,13 +41543,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>10.4</v>
+        <v>12.1</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -41296,10 +41557,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>59.8</v>
+        <v>78.5</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>4.8</v>
+        <v>2.6</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -41311,7 +41572,7 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
@@ -41325,10 +41586,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>53</v>
+        <v>23.6</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -41340,7 +41601,7 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
@@ -41354,10 +41615,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>17.2</v>
+        <v>31.3</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -41369,13 +41630,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.8</v>
+        <v>12.9</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -41383,10 +41644,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>4.7</v>
+        <v>2.5</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -41398,13 +41659,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13</v>
+        <v>13.1</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -41412,10 +41673,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>4.3</v>
+        <v>1.8</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -41427,13 +41688,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.1</v>
+        <v>13.3</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -41441,13 +41702,42 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>15.8</v>
+        <v>1.6</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>10.1</v>
+        <v>11.8</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H81" s="10">
+        <f>SUM(C75:C81)</f>
         <v/>
       </c>
     </row>
@@ -41468,7 +41758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43623,13 +43913,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1.9</v>
+        <v>0.3</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -43637,10 +43927,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>67.5</v>
+        <v>89.2</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>3.9</v>
+        <v>1.3</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -43652,13 +43942,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -43666,10 +43956,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>66.7</v>
+        <v>44.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>4</v>
+        <v>6.7</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -43681,13 +43971,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -43695,10 +43985,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>42.8</v>
+        <v>28.3</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>6.9</v>
+        <v>8.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -43710,24 +44000,24 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>10</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>4.7</v>
+        <v>1.4</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -43739,21 +44029,21 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="G79" s="4" t="n">
         <v>11.9</v>
@@ -43768,27 +44058,56 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>2.5</v>
+        <v>1.4</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>10.2</v>
+        <v>1.6</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>10.8</v>
+        <v>11.8</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H81" s="10">
+        <f>SUM(C75:C81)</f>
         <v/>
       </c>
     </row>
@@ -43809,7 +44128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49473,13 +49792,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>16.9</v>
+        <v>18.4</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -49487,10 +49806,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>24.2</v>
+        <v>41.7</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>9.1</v>
+        <v>7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -49502,7 +49821,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>18</v>
+        <v>17.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -49516,10 +49835,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>16.2</v>
+        <v>31.3</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -49531,13 +49850,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -49545,10 +49864,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>3.5</v>
+        <v>4.8</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -49560,7 +49879,7 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.3</v>
+        <v>19.7</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
@@ -49574,10 +49893,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>5.1</v>
+        <v>9</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.4</v>
+        <v>10.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -49589,7 +49908,7 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>20.5</v>
+        <v>19.6</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
@@ -49603,10 +49922,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>7.2</v>
+        <v>11.1</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.1</v>
+        <v>10.7</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -49618,27 +49937,56 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.7</v>
+        <v>19</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>28.9</v>
+        <v>20.1</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>8.5</v>
+        <v>9.6</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -49659,7 +50007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51814,13 +52162,13 @@
         <v>46290</v>
       </c>
       <c r="B75" s="4" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
@@ -51828,10 +52176,10 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>91.09999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(C69:C75)</f>
@@ -51849,7 +52197,7 @@
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -51857,10 +52205,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>33.4</v>
+        <v>44.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8</v>
+        <v>6.7</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -51872,24 +52220,24 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11</v>
+        <v>11.9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>53.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>5.6</v>
+        <v>3.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -51901,13 +52249,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.3</v>
+        <v>12.7</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -51915,10 +52263,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0.2</v>
+        <v>12.9</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>12</v>
+        <v>10.5</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -51930,24 +52278,24 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>12.7</v>
+        <v>13.1</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.2</v>
+        <v>2.6</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>4.5</v>
+        <v>7.6</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.5</v>
+        <v>11.1</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -51959,27 +52307,56 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>11.3</v>
+        <v>12.4</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>3.1</v>
+        <v>1.7</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>0.2</v>
+        <v>2.5</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H81" s="10">
+        <f>SUM(C75:C81)</f>
         <v/>
       </c>
     </row>
@@ -52000,7 +52377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -57664,24 +58041,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>23.5</v>
+        <v>24.3</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>14.7</v>
+        <v>6</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>47.1</v>
+        <v>30.5</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>6.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -57693,13 +58070,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>2.8</v>
+        <v>5.4</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -57707,10 +58084,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>29</v>
+        <v>23.7</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -57722,13 +58099,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>23.4</v>
+        <v>23.2</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>6</v>
+        <v>4.9</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -57736,10 +58113,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>26.1</v>
+        <v>8.1</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>8.9</v>
+        <v>11</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -57751,24 +58128,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>22.7</v>
+        <v>22.5</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>57.8</v>
+        <v>20.7</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>5.1</v>
+        <v>9.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -57780,13 +58157,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -57794,10 +58171,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -57809,27 +58186,56 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>22.6</v>
+        <v>23</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G201" s="4" t="n">
         <v>12</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -57850,7 +58256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63514,13 +63920,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>20.2</v>
+        <v>21.9</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.8</v>
+        <v>4.1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -63528,10 +63934,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>14.3</v>
+        <v>1.8</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>10.3</v>
+        <v>11.8</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -63543,13 +63949,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>18.3</v>
+        <v>17.6</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -63557,10 +63963,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>35.3</v>
+        <v>46.6</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>7.8</v>
+        <v>6.4</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -63572,13 +63978,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.3</v>
+        <v>17.6</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4.5</v>
+        <v>5.2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -63586,10 +63992,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>58.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>5</v>
+        <v>1.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -63601,24 +64007,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="C199" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="G199" s="4" t="n">
         <v>1.7</v>
-      </c>
-      <c r="D199" s="4" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E199" s="4" t="inlineStr">
-        <is>
-          <t>JZ</t>
-        </is>
-      </c>
-      <c r="F199" s="4" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="G199" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -63630,13 +64036,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>16.9</v>
+        <v>17</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -63644,10 +64050,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>59.4</v>
+        <v>32.6</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>4.9</v>
+        <v>8.1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -63659,13 +64065,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>17.7</v>
+        <v>18.4</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -63673,13 +64079,42 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>72.2</v>
+        <v>40.8</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>3.3</v>
+        <v>7.1</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>91</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -63700,7 +64135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69364,24 +69799,24 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>10.8</v>
+        <v>10.3</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>79.2</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -69393,13 +69828,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>3.6</v>
+        <v>5.7</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -69407,10 +69842,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>53.8</v>
+        <v>61.9</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>5.5</v>
+        <v>4.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -69422,7 +69857,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>13</v>
+        <v>11.4</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -69432,11 +69867,11 @@
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>83.2</v>
+        <v>83</v>
       </c>
       <c r="G198" s="7" t="n">
         <v>2</v>
@@ -69451,13 +69886,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>12.8</v>
+        <v>13.1</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -69465,10 +69900,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>97.2</v>
+        <v>98.5</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -69480,7 +69915,7 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>11.6</v>
+        <v>11.1</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
@@ -69494,10 +69929,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>87.40000000000001</v>
+        <v>82</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -69509,13 +69944,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>13.8</v>
+        <v>13.3</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -69523,13 +69958,42 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -69550,7 +70014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -75214,13 +75678,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>13.9</v>
+        <v>15</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -75228,10 +75692,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>5.3</v>
+        <v>10.9</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.4</v>
+        <v>10.7</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -75249,7 +75713,7 @@
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -75257,10 +75721,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>1.6</v>
+        <v>0.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -75272,24 +75736,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>1.6</v>
+        <v>0.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -75301,13 +75765,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>16</v>
+        <v>15.8</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -75315,7 +75779,7 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G199" s="4" t="n">
         <v>12</v>
@@ -75330,7 +75794,7 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>17.2</v>
+        <v>16.9</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
@@ -75344,10 +75808,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -75359,13 +75823,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>16.8</v>
+        <v>16.2</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -75373,13 +75837,42 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>5.1</v>
+        <v>0</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -75400,7 +75893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81064,13 +81557,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>14.7</v>
+        <v>16</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -81078,10 +81571,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>3.7</v>
+        <v>9.9</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>11.6</v>
+        <v>10.8</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -81093,13 +81586,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -81107,10 +81600,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>1.7</v>
+        <v>0.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -81122,13 +81615,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -81136,10 +81629,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -81151,13 +81644,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -81180,7 +81673,7 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>18.8</v>
+        <v>18.2</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
@@ -81194,10 +81687,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -81209,27 +81702,56 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>17.1</v>
+        <v>16.9</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>11.3</v>
+        <v>12</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -81250,7 +81772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -86914,13 +87436,13 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>10.2</v>
+        <v>11</v>
       </c>
       <c r="C196" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
@@ -86928,10 +87450,10 @@
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>36.1</v>
+        <v>22.6</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -86943,13 +87465,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -86957,10 +87479,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>9.5</v>
+        <v>16.4</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.9</v>
+        <v>10</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -86972,13 +87494,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>12.7</v>
+        <v>13</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -86986,10 +87508,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>23.2</v>
+        <v>9.4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -87001,13 +87523,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>13.8</v>
+        <v>13.6</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -87015,10 +87537,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>18.4</v>
+        <v>17.4</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -87030,13 +87552,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>14.1</v>
+        <v>13.8</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -87044,10 +87566,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>4.3</v>
+        <v>13.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.5</v>
+        <v>10.3</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -87059,13 +87581,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>3.6</v>
+        <v>2.7</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -87073,13 +87595,42 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>
@@ -87100,7 +87651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -92764,7 +93315,7 @@
         <v>46290</v>
       </c>
       <c r="B196" s="7" t="n">
-        <v>13</v>
+        <v>15.3</v>
       </c>
       <c r="C196" s="7" t="n">
         <v>0</v>
@@ -92774,14 +93325,14 @@
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F196" s="7" t="n">
-        <v>34.2</v>
+        <v>5.6</v>
       </c>
       <c r="G196" s="7" t="n">
-        <v>7.9</v>
+        <v>11.3</v>
       </c>
       <c r="H196" s="12">
         <f>SUM(C190:C196)</f>
@@ -92807,10 +93358,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>14.4</v>
+        <v>5.2</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10.3</v>
+        <v>11.4</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -92822,24 +93373,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.7</v>
+        <v>16.6</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -92851,24 +93402,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>49.2</v>
+        <v>46.1</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -92880,24 +93431,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>14.8</v>
+        <v>15.6</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>19.1</v>
+        <v>40.6</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -92909,13 +93460,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>15.9</v>
+        <v>14.5</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -92923,13 +93474,42 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>49.6</v>
+        <v>23.8</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>6</v>
+        <v>9.1</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="11" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B202" s="7" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C202" s="7" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="G202" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H202" s="12">
+        <f>SUM(C196:C202)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-26 10:29 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6206,24 +6206,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.9</v>
+        <v>18.2</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>35.4</v>
+        <v>12.8</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>83.90000000000001</v>
+        <v>99.5</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>1.9</v>
+        <v>0.1</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -6235,13 +6235,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>19.4</v>
+        <v>18.8</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>7.4</v>
+        <v>22.7</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -6249,10 +6249,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>49.3</v>
+        <v>60.8</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -6264,24 +6264,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.4</v>
+        <v>20.2</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>8.6</v>
+        <v>10.6</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11</v>
+        <v>10.7</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -6293,13 +6293,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>20</v>
+        <v>19.7</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>3.9</v>
+        <v>4.1</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -6307,10 +6307,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>2.9</v>
+        <v>7.2</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.7</v>
+        <v>11.1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -6322,13 +6322,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.9</v>
+        <v>19.4</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>4.6</v>
+        <v>5.6</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -6336,10 +6336,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>5.3</v>
+        <v>32.2</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>11.4</v>
+        <v>8.1</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -6351,27 +6351,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>19.3</v>
+        <v>18.7</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>3.4</v>
+        <v>6.1</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>11.1</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>10.7</v>
+        <v>2.8</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -6392,7 +6421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12085,13 +12114,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21.7</v>
+        <v>23.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -12099,10 +12128,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>23</v>
+        <v>14.4</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -12114,13 +12143,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.4</v>
+        <v>20.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -12128,10 +12157,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>73.40000000000001</v>
+        <v>58.8</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3.2</v>
+        <v>4.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -12143,13 +12172,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>19.6</v>
+        <v>19</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.8</v>
+        <v>15.5</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -12157,10 +12186,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>86.3</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -12172,13 +12201,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>18.6</v>
+        <v>17.9</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>1.1</v>
+        <v>6.6</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -12186,10 +12215,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>42.8</v>
+        <v>67.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>6.9</v>
+        <v>3.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -12201,24 +12230,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.1</v>
+        <v>19.7</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>8.4</v>
+        <v>3.5</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>52.3</v>
+        <v>95.3</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>5.7</v>
+        <v>0.6</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -12230,27 +12259,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>16.8</v>
+        <v>18.4</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>11.4</v>
+        <v>3.8</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>0.7</v>
+        <v>1.9</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>79.3</v>
+        <v>85</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -12271,7 +12329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17964,24 +18022,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.9</v>
+        <v>3.8</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>74.8</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -17993,24 +18051,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21.3</v>
+        <v>19.2</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0</v>
+        <v>16.8</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>65.5</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>4.1</v>
+        <v>1.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -18022,24 +18080,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>21.2</v>
+        <v>20.5</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0.6</v>
+        <v>5.1</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.9</v>
+        <v>11.4</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -18057,7 +18115,7 @@
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>8.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -18080,7 +18138,7 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>21.3</v>
+        <v>20.7</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
@@ -18090,11 +18148,11 @@
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G201" s="4" t="n">
         <v>12</v>
@@ -18109,27 +18167,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>20.3</v>
+        <v>20.8</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>7.1</v>
+        <v>5.2</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>12</v>
+        <v>9.1</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -18150,7 +18237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23843,24 +23930,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>21.1</v>
+        <v>22.8</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>18.1</v>
+        <v>18.9</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -23872,13 +23959,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>21.7</v>
+        <v>22.1</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -23886,7 +23973,7 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="G198" s="7" t="n">
         <v>11.5</v>
@@ -23901,13 +23988,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.9</v>
+        <v>22.3</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2.1</v>
+        <v>3.3</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -23915,10 +24002,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -23930,24 +24017,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>20.9</v>
+        <v>21.8</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>42.6</v>
+        <v>9</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>6.9</v>
+        <v>10.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -23959,13 +24046,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>21.8</v>
+        <v>22.1</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -23973,10 +24060,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>8.6</v>
+        <v>17</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -23988,27 +24075,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>22.3</v>
+        <v>22.7</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>66.2</v>
+        <v>72.3</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>4.1</v>
+        <v>3.3</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -24029,7 +24145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29722,24 +29838,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>11</v>
+        <v>13.3</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>32.4</v>
+        <v>31.6</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -29751,13 +29867,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -29765,10 +29881,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>13.7</v>
+        <v>9</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.4</v>
+        <v>10.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -29780,13 +29896,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>10.6</v>
+        <v>11.5</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -29794,10 +29910,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>89.5</v>
+        <v>56.7</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>1.3</v>
+        <v>5.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -29809,13 +29925,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -29823,10 +29939,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>81.59999999999999</v>
+        <v>92</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>2.2</v>
+        <v>1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -29838,13 +29954,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -29852,10 +29968,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>33.4</v>
+        <v>47.2</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>8</v>
+        <v>6.3</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -29867,27 +29983,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.9</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>12.9</v>
+        <v>0.1</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>97.7</v>
+        <v>86.5</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>0.3</v>
+        <v>1.6</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>78.7</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -29908,7 +30053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32092,24 +32237,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>12.2</v>
+        <v>13.9</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>38.2</v>
+        <v>24</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>7.4</v>
+        <v>9.1</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -32135,10 +32280,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>28.3</v>
+        <v>27.4</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -32150,21 +32295,21 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.5</v>
+        <v>12.2</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.3</v>
+        <v>2.2</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>12</v>
@@ -32179,24 +32324,24 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.1</v>
+        <v>12.9</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -32208,24 +32353,24 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>13.7</v>
+        <v>13.2</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -32237,27 +32382,56 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>13</v>
+        <v>12.7</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>1.9</v>
+        <v>0.9</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>2.5</v>
+        <v>35.5</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>11.7</v>
+        <v>7.7</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H82" s="12">
+        <f>SUM(C76:C82)</f>
         <v/>
       </c>
     </row>
@@ -32278,7 +32452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34462,24 +34636,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>10</v>
+        <v>12.2</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>40.8</v>
+        <v>27.7</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>7.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -34491,13 +34665,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -34505,10 +34679,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -34520,13 +34694,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>11.6</v>
+        <v>11.8</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -34534,10 +34708,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>6.2</v>
+        <v>0.9</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -34549,13 +34723,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -34563,10 +34737,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -34578,24 +34752,24 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>11.7</v>
+        <v>11.3</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.6</v>
+        <v>11.9</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -34607,13 +34781,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -34621,13 +34795,42 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>15.2</v>
+        <v>13.5</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="H82" s="12">
+        <f>SUM(C76:C82)</f>
         <v/>
       </c>
     </row>
@@ -34648,7 +34851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36832,24 +37035,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.3</v>
+        <v>12.2</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>28.8</v>
+        <v>28.1</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -36861,13 +37064,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -36875,10 +37078,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>34</v>
+        <v>28.5</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -36890,13 +37093,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -36904,10 +37107,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>2.4</v>
+        <v>1.3</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -36919,21 +37122,21 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.6</v>
+        <v>13</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G79" s="4" t="n">
         <v>12</v>
@@ -36948,24 +37151,24 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>13.9</v>
+        <v>12.6</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1</v>
+        <v>2.1</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>3.1</v>
+        <v>5.1</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -36977,27 +37180,56 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>12.3</v>
+        <v>13.9</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>2.6</v>
+        <v>0.9</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>2.1</v>
+        <v>15.8</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>11.7</v>
+        <v>10.1</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H82" s="12">
+        <f>SUM(C76:C82)</f>
         <v/>
       </c>
     </row>
@@ -37018,7 +37250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39202,24 +39434,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.6</v>
+        <v>12.9</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>50.3</v>
+        <v>35.4</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>6</v>
+        <v>7.8</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -39241,14 +39473,14 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>31.3</v>
+        <v>30.6</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -39260,21 +39492,21 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>12</v>
@@ -39289,24 +39521,24 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.3</v>
+        <v>12.9</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -39318,24 +39550,24 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>13.8</v>
+        <v>13.1</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>0.2</v>
+        <v>3.1</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -39347,27 +39579,56 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>12.5</v>
+        <v>13.6</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>24.2</v>
+        <v>25.2</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H82" s="12">
+        <f>SUM(C76:C82)</f>
         <v/>
       </c>
     </row>
@@ -39388,7 +39649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41572,13 +41833,13 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
@@ -41586,10 +41847,10 @@
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>23.6</v>
+        <v>22</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -41601,13 +41862,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.7</v>
+        <v>12.6</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -41615,10 +41876,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>31.3</v>
+        <v>21.6</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -41630,13 +41891,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.9</v>
+        <v>13.1</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -41644,10 +41905,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.7</v>
+        <v>11.3</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -41659,24 +41920,24 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.1</v>
+        <v>12.8</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>1.8</v>
+        <v>0.2</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -41688,13 +41949,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -41702,10 +41963,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -41717,27 +41978,56 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>12.4</v>
+        <v>13.3</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>6.2</v>
+        <v>6.9</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H82" s="12">
+        <f>SUM(C76:C82)</f>
         <v/>
       </c>
     </row>
@@ -41758,7 +42048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43942,24 +44232,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>8.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>44.2</v>
+        <v>40.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>6.7</v>
+        <v>7.2</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -43977,7 +44267,7 @@
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -43985,10 +44275,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>28.3</v>
+        <v>39.9</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -44000,13 +44290,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -44014,10 +44304,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>1.4</v>
+        <v>3.1</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -44029,13 +44319,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>9.4</v>
+        <v>8.9</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -44043,10 +44333,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -44058,13 +44348,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -44072,10 +44362,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>1.6</v>
+        <v>5.7</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.8</v>
+        <v>11.3</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -44087,13 +44377,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>8.6</v>
+        <v>9.5</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>2.3</v>
+        <v>0.8</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -44101,13 +44391,42 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>19.6</v>
+        <v>11.9</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>9.6</v>
+        <v>10.6</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H82" s="12">
+        <f>SUM(C76:C82)</f>
         <v/>
       </c>
     </row>
@@ -44128,7 +44447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49821,7 +50140,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.8</v>
+        <v>20.9</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -49831,14 +50150,14 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>31.3</v>
+        <v>12.8</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>8.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -49850,7 +50169,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -49864,10 +50183,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -49879,13 +50198,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>19.7</v>
+        <v>20.4</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -49893,7 +50212,7 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G199" s="4" t="n">
         <v>10.9</v>
@@ -49908,24 +50227,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>11.1</v>
+        <v>27.7</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>10.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -49937,24 +50256,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>20.1</v>
+        <v>21.1</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -49966,7 +50285,7 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
@@ -49980,13 +50299,42 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>41.6</v>
+        <v>8.6</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -50007,7 +50355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -52191,24 +52539,24 @@
         <v>46291</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>9.5</v>
+        <v>11.9</v>
       </c>
       <c r="C76" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F76" s="7" t="n">
-        <v>44.2</v>
+        <v>41.2</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="H76" s="12">
         <f>SUM(C70:C76)</f>
@@ -52220,13 +52568,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -52234,10 +52582,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>69.59999999999999</v>
+        <v>67</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -52249,13 +52597,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.7</v>
+        <v>12.1</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>3.5</v>
+        <v>3.9</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -52263,10 +52611,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>12.9</v>
+        <v>4.1</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -52278,13 +52626,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13.1</v>
+        <v>12.2</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -52292,10 +52640,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>7.6</v>
+        <v>6.4</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -52307,13 +52655,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.4</v>
+        <v>11.8</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -52321,10 +52669,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>2.5</v>
+        <v>52.5</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.7</v>
+        <v>5.7</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -52336,7 +52684,7 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>12.2</v>
+        <v>12.6</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
@@ -52350,13 +52698,42 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>0</v>
+        <v>35.9</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>12</v>
+        <v>7.7</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H82" s="12">
+        <f>SUM(C76:C82)</f>
         <v/>
       </c>
     </row>
@@ -52377,7 +52754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -58070,13 +58447,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>22.9</v>
+        <v>23.5</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -58084,10 +58461,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>23.7</v>
+        <v>1.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>11.9</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -58099,13 +58476,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>23.2</v>
+        <v>23.5</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4.9</v>
+        <v>6.7</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -58113,10 +58490,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>8.1</v>
+        <v>26.1</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11</v>
+        <v>8.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -58128,24 +58505,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>22.5</v>
+        <v>22.7</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>20.7</v>
+        <v>9.9</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>9.5</v>
+        <v>10.8</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -58163,7 +58540,7 @@
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -58171,10 +58548,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -58186,21 +58563,21 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="G201" s="4" t="n">
         <v>12</v>
@@ -58215,27 +58592,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>10.8</v>
+        <v>0.2</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>10.7</v>
+        <v>12</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -58256,7 +58662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63949,13 +64355,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>17.6</v>
+        <v>19.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>4.2</v>
+        <v>5.1</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -63963,10 +64369,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>46.6</v>
+        <v>15.1</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>6.4</v>
+        <v>10.2</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -63978,13 +64384,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.6</v>
+        <v>17.7</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -63992,10 +64398,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>83.90000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -64007,10 +64413,10 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>17.2</v>
+        <v>16.9</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.5</v>
+        <v>10</v>
       </c>
       <c r="D199" s="4" t="n">
         <v>4.2</v>
@@ -64021,10 +64427,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>85.5</v>
+        <v>93.2</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -64036,13 +64442,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>17</v>
+        <v>16.3</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>0.9</v>
+        <v>2.4</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -64050,10 +64456,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>32.6</v>
+        <v>51.4</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>8.1</v>
+        <v>5.8</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -64065,13 +64471,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>18.4</v>
+        <v>17.8</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>3.5</v>
+        <v>2.2</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -64079,10 +64485,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>40.8</v>
+        <v>97.5</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>7.1</v>
+        <v>0.3</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -64094,27 +64500,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>17.6</v>
+        <v>16.8</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>1.2</v>
+        <v>4.3</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>91</v>
+        <v>89.2</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>98.59999999999999</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -64135,7 +64570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69828,13 +70263,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>5.7</v>
+        <v>2.4</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -69842,10 +70277,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>61.9</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>4.6</v>
+        <v>2.1</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -69857,13 +70292,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>11.4</v>
+        <v>12.9</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -69871,10 +70306,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>83</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>2</v>
+        <v>0.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -69886,24 +70321,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>13.1</v>
+        <v>14.8</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>7.2</v>
+        <v>2.7</v>
       </c>
       <c r="D199" s="4" t="n">
         <v>1.3</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>98.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.2</v>
+        <v>3.3</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -69915,13 +70350,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>11.1</v>
+        <v>10.9</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -69929,10 +70364,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>2.2</v>
+        <v>3.8</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -69944,13 +70379,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -69958,10 +70393,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>92</v>
+        <v>64.8</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -69973,13 +70408,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>15.1</v>
+        <v>14.9</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -69987,13 +70422,42 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>74.2</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>3.1</v>
+        <v>1.2</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -70014,7 +70478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -75707,13 +76171,13 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>14.8</v>
+        <v>17.1</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
@@ -75736,24 +76200,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>0.2</v>
+        <v>4.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>12</v>
+        <v>11.4</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -75765,24 +76229,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>15.8</v>
+        <v>16.4</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0.2</v>
+        <v>4.9</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>12</v>
+        <v>11.4</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -75794,13 +76258,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>16.9</v>
+        <v>16.5</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -75823,13 +76287,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>16.2</v>
+        <v>15.8</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -75852,27 +76316,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>0.6</v>
+        <v>13.3</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>11.9</v>
+        <v>10.4</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -75893,7 +76386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81586,17 +82079,17 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.6</v>
+        <v>18.2</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
@@ -81615,13 +82108,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.2</v>
+        <v>17</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -81629,10 +82122,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>0.4</v>
+        <v>2.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -81644,13 +82137,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>17.4</v>
+        <v>17.9</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -81658,10 +82151,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -81673,13 +82166,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>18.2</v>
+        <v>17.2</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -81687,10 +82180,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -81708,11 +82201,11 @@
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
@@ -81737,21 +82230,50 @@
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -81772,7 +82294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -87465,7 +87987,7 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>11.3</v>
+        <v>13</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
@@ -87479,10 +88001,10 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>16.4</v>
+        <v>1.7</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>10</v>
+        <v>11.8</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -87494,13 +88016,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>13</v>
+        <v>12.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -87508,10 +88030,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>9.4</v>
+        <v>6.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -87523,13 +88045,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>13.6</v>
+        <v>13.4</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -87537,10 +88059,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>17.4</v>
+        <v>16.1</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>9.9</v>
+        <v>10.1</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -87552,13 +88074,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>13.8</v>
+        <v>12.9</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -87566,10 +88088,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>13.8</v>
+        <v>6.5</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>10.3</v>
+        <v>11.2</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -87581,13 +88103,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -87595,10 +88117,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>2.1</v>
+        <v>0.8</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -87610,13 +88132,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.5</v>
+        <v>3.1</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -87624,13 +88146,42 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>0.6</v>
+        <v>21.1</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>11.9</v>
+        <v>9.5</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>
@@ -87651,7 +88202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -93344,24 +93895,24 @@
         <v>46291</v>
       </c>
       <c r="B197" s="4" t="n">
-        <v>15.9</v>
+        <v>16.3</v>
       </c>
       <c r="C197" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>5.2</v>
+        <v>11.7</v>
       </c>
       <c r="G197" s="4" t="n">
-        <v>11.4</v>
+        <v>10.6</v>
       </c>
       <c r="H197" s="10">
         <f>SUM(C191:C197)</f>
@@ -93373,7 +93924,7 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>16.6</v>
+        <v>16.7</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
@@ -93387,10 +93938,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>3.3</v>
+        <v>1.3</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.6</v>
+        <v>11.8</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -93402,24 +93953,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>15.7</v>
+        <v>16.9</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>0.7</v>
+        <v>1.6</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>46.1</v>
+        <v>20.5</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -93431,24 +93982,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>15.6</v>
+        <v>14.8</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>40.6</v>
+        <v>46.5</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>7.1</v>
+        <v>6.4</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -93460,13 +94011,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -93474,10 +94025,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>23.8</v>
+        <v>51.6</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>9.1</v>
+        <v>5.8</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -93489,27 +94040,56 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>14.8</v>
+        <v>14.1</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>3.7</v>
+        <v>2.7</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>95.5</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B203" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C203" s="4" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H203" s="10">
+        <f>SUM(C197:C203)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-27 11:01 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6235,13 +6235,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>18.8</v>
+        <v>19.7</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>22.7</v>
+        <v>7.6</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -6249,10 +6249,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>60.8</v>
+        <v>26.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>4.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -6267,10 +6267,10 @@
         <v>20.2</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>1.5</v>
+        <v>0.4</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -6278,10 +6278,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>10.6</v>
+        <v>12.2</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -6293,24 +6293,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>1</v>
+        <v>3.1</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>4.1</v>
+        <v>5.3</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>7.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.1</v>
+        <v>10.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -6322,13 +6322,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.4</v>
+        <v>19.5</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>3.2</v>
+        <v>5.3</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>5.6</v>
+        <v>6.3</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -6336,10 +6336,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>32.2</v>
+        <v>38.3</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -6351,13 +6351,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>18.7</v>
+        <v>18.3</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>6.1</v>
+        <v>7</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -6365,10 +6365,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>76.40000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -6380,13 +6380,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>18.8</v>
+        <v>18.4</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>2</v>
+        <v>5.8</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -6394,13 +6394,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>58.2</v>
+        <v>63.6</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>5</v>
+        <v>4.4</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -6421,7 +6450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12143,24 +12172,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>20.7</v>
+        <v>22.1</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>58.8</v>
+        <v>94.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>4.9</v>
+        <v>0.6</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -12172,13 +12201,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>15.5</v>
+        <v>30.2</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -12186,10 +12215,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>93.90000000000001</v>
+        <v>95</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -12201,13 +12230,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>17.9</v>
+        <v>16.3</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>6.6</v>
+        <v>22.8</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -12215,10 +12244,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>67.8</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>3.9</v>
+        <v>0.1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -12230,24 +12259,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.7</v>
+        <v>18.4</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>3.5</v>
+        <v>1.7</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>0.8</v>
+        <v>1.9</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>95.3</v>
+        <v>98.5</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -12262,21 +12291,21 @@
         <v>18.4</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>3.8</v>
+        <v>4.6</v>
       </c>
       <c r="D202" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="G202" s="7" t="n">
         <v>1.9</v>
-      </c>
-      <c r="E202" s="7" t="inlineStr">
-        <is>
-          <t>JV</t>
-        </is>
-      </c>
-      <c r="F202" s="7" t="n">
-        <v>85</v>
-      </c>
-      <c r="G202" s="7" t="n">
-        <v>1.8</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -12288,27 +12317,56 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>17.6</v>
+        <v>16.5</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>2.5</v>
+        <v>20</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>95.90000000000001</v>
+        <v>97.8</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -12329,7 +12387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18051,24 +18109,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>16.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4.5</v>
+        <v>5.6</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>87.09999999999999</v>
+        <v>59.4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>1.5</v>
+        <v>4.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -18080,24 +18138,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.5</v>
+        <v>20.3</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>10.2</v>
+        <v>10.8</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>5.1</v>
+        <v>6.8</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.4</v>
+        <v>11.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -18109,13 +18167,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>21</v>
+        <v>20.2</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -18123,7 +18181,7 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="G200" s="7" t="n">
         <v>12</v>
@@ -18138,21 +18196,21 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="G201" s="4" t="n">
         <v>12</v>
@@ -18167,13 +18225,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>20.8</v>
+        <v>20.6</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>5.2</v>
+        <v>4</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -18181,10 +18239,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>24</v>
+        <v>28.9</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>9.1</v>
+        <v>8.5</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -18196,13 +18254,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>20.8</v>
+        <v>20.4</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>7.8</v>
+        <v>3.6</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -18210,13 +18268,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>1.8</v>
+        <v>49.4</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>11.8</v>
+        <v>6.1</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -18237,7 +18324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23959,24 +24046,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>22.1</v>
+        <v>22.9</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>3.9</v>
+        <v>0.1</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -23988,13 +24075,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>22.3</v>
+        <v>22</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -24002,10 +24089,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -24017,24 +24104,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>21.8</v>
+        <v>22.4</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.4</v>
+        <v>3.8</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>9</v>
+        <v>33.5</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>10.9</v>
+        <v>8</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -24046,13 +24133,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>22.1</v>
+        <v>22.5</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -24060,10 +24147,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>17</v>
+        <v>61.9</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>10</v>
+        <v>4.6</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -24075,24 +24162,24 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>72.3</v>
+        <v>54.9</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>3.3</v>
+        <v>5.4</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -24104,13 +24191,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -24118,13 +24205,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>61.9</v>
+        <v>90.2</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>4.6</v>
+        <v>1.2</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -24145,7 +24261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29867,24 +29983,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>11.1</v>
+        <v>13.2</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>9</v>
+        <v>12.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>10.9</v>
+        <v>10.5</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -29896,13 +30012,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -29910,10 +30026,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>56.7</v>
+        <v>71</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>5.2</v>
+        <v>3.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -29925,13 +30041,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>10.9</v>
+        <v>11.4</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.5</v>
+        <v>2.7</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -29939,10 +30055,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>92</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -29954,24 +30070,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>10.9</v>
+        <v>11.4</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>47.2</v>
+        <v>67.8</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>6.3</v>
+        <v>3.9</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -29983,24 +30099,24 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>10.9</v>
+        <v>10.4</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>0.1</v>
+        <v>3.8</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>86.5</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>1.6</v>
+        <v>0.2</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -30012,13 +30128,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -30026,13 +30142,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>78.7</v>
+        <v>99.2</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>2.6</v>
+        <v>0.1</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -30053,7 +30198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32266,13 +32411,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12</v>
+        <v>12.9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -32280,10 +32425,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>27.4</v>
+        <v>21.5</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -32309,7 +32454,7 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>12</v>
@@ -32330,15 +32475,15 @@
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="G79" s="4" t="n">
         <v>11.9</v>
@@ -32353,13 +32498,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>13.2</v>
+        <v>13</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -32367,10 +32512,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>12</v>
+        <v>11.4</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -32382,7 +32527,7 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
@@ -32392,14 +32537,14 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>35.5</v>
+        <v>96.5</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>7.7</v>
+        <v>0.4</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -32417,21 +32562,50 @@
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>21.3</v>
+        <v>0</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>9.4</v>
+        <v>12</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H83" s="10">
+        <f>SUM(C77:C83)</f>
         <v/>
       </c>
     </row>
@@ -32452,7 +32626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34665,7 +34839,7 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.2</v>
+        <v>13.6</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
@@ -34679,10 +34853,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>38.4</v>
+        <v>16.1</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>7.4</v>
+        <v>10.1</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -34694,7 +34868,7 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
@@ -34708,7 +34882,7 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>11.9</v>
@@ -34723,13 +34897,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -34737,10 +34911,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -34752,13 +34926,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>11.3</v>
+        <v>10.8</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -34766,10 +34940,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>1.2</v>
+        <v>14.4</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.9</v>
+        <v>10.3</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -34781,13 +34955,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>11.6</v>
+        <v>11</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -34795,10 +34969,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>13.5</v>
+        <v>77</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>10.4</v>
+        <v>2.8</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -34810,13 +34984,13 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>11.9</v>
+        <v>11.3</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
@@ -34824,13 +34998,42 @@
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>14.9</v>
+        <v>0</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>10.2</v>
+        <v>12</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H83" s="10">
+        <f>SUM(C77:C83)</f>
         <v/>
       </c>
     </row>
@@ -34851,7 +35054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37064,13 +37267,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.8</v>
+        <v>13.9</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -37078,10 +37281,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>28.5</v>
+        <v>23.9</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -37093,7 +37296,7 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
@@ -37107,10 +37310,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>1.3</v>
+        <v>2.8</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -37122,13 +37325,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>13</v>
+        <v>12.9</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -37151,7 +37354,7 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.6</v>
+        <v>12.1</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
@@ -37165,10 +37368,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>5.1</v>
+        <v>31.4</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -37180,24 +37383,24 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>13.9</v>
+        <v>12.5</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>15.8</v>
+        <v>90</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>10.1</v>
+        <v>1.2</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -37209,13 +37412,13 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>14.8</v>
+        <v>13.9</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
@@ -37223,13 +37426,42 @@
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>13.5</v>
+        <v>0</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H83" s="10">
+        <f>SUM(C77:C83)</f>
         <v/>
       </c>
     </row>
@@ -37250,7 +37482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39463,13 +39695,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.5</v>
+        <v>13.7</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -39477,10 +39709,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>30.6</v>
+        <v>26.4</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -39492,7 +39724,7 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.5</v>
+        <v>12.6</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
@@ -39502,11 +39734,11 @@
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>12</v>
@@ -39521,17 +39753,17 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>12.9</v>
+        <v>12.6</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
@@ -39550,13 +39782,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>13.1</v>
+        <v>12.4</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -39564,10 +39796,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>3.1</v>
+        <v>13.3</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.6</v>
+        <v>10.4</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -39579,7 +39811,7 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>13.6</v>
+        <v>13</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
@@ -39593,10 +39825,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>25.2</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -39608,7 +39840,7 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
@@ -39622,13 +39854,42 @@
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>29.1</v>
+        <v>0</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>8.5</v>
+        <v>12</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H83" s="10">
+        <f>SUM(C77:C83)</f>
         <v/>
       </c>
     </row>
@@ -39649,7 +39910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41862,7 +42123,7 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>12.6</v>
+        <v>14</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
@@ -41876,10 +42137,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>21.6</v>
+        <v>24.5</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>9.4</v>
+        <v>9.1</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -41905,10 +42166,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -41926,7 +42187,7 @@
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -41934,7 +42195,7 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G79" s="4" t="n">
         <v>12</v>
@@ -41949,13 +42210,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.8</v>
+        <v>12.4</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -41963,10 +42224,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>2.6</v>
+        <v>9</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.7</v>
+        <v>10.9</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -41978,13 +42239,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -41992,10 +42253,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>6.9</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>11.2</v>
+        <v>0.9</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -42007,13 +42268,13 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>13.4</v>
+        <v>12.8</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
@@ -42021,13 +42282,42 @@
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>17.2</v>
+        <v>0</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>9.9</v>
+        <v>12</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H83" s="10">
+        <f>SUM(C77:C83)</f>
         <v/>
       </c>
     </row>
@@ -42048,7 +42338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44261,13 +44551,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>9</v>
+        <v>10.7</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -44275,10 +44565,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>39.9</v>
+        <v>28</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>7.2</v>
+        <v>8.6</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -44300,11 +44590,11 @@
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>11.6</v>
@@ -44325,7 +44615,7 @@
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -44333,10 +44623,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -44348,7 +44638,7 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>8.6</v>
+        <v>8</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
@@ -44362,10 +44652,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>5.7</v>
+        <v>32.2</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.3</v>
+        <v>8.1</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -44377,13 +44667,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>9.5</v>
+        <v>9.1</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -44391,10 +44681,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>11.9</v>
+        <v>90</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>10.6</v>
+        <v>1.2</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -44406,27 +44696,56 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>10.2</v>
+        <v>9.5</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>17.6</v>
+        <v>0</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>9.9</v>
+        <v>12</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H83" s="10">
+        <f>SUM(C77:C83)</f>
         <v/>
       </c>
     </row>
@@ -44447,7 +44766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -50169,24 +50488,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>19.8</v>
+        <v>22.1</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>4</v>
+        <v>1.6</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -50212,10 +50531,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>9.300000000000001</v>
+        <v>6.3</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -50227,13 +50546,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -50241,10 +50560,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>27.7</v>
+        <v>13</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>8.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -50256,24 +50575,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>21.1</v>
+        <v>19.9</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>9.5</v>
+        <v>9.6</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -50285,7 +50604,7 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>19.4</v>
+        <v>19.6</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
@@ -50299,10 +50618,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>8.6</v>
+        <v>44</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>11</v>
+        <v>6.7</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -50314,27 +50633,56 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>19.9</v>
+        <v>20.8</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>39.8</v>
+        <v>59.4</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>7.2</v>
+        <v>4.9</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -50355,7 +50703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -52568,13 +52916,13 @@
         <v>46292</v>
       </c>
       <c r="B77" s="4" t="n">
-        <v>11.7</v>
+        <v>13.2</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
@@ -52582,10 +52930,10 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>67</v>
+        <v>6.5</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>4</v>
+        <v>11.2</v>
       </c>
       <c r="H77" s="10">
         <f>SUM(C71:C77)</f>
@@ -52597,13 +52945,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -52611,10 +52959,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>4.1</v>
+        <v>1.2</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.5</v>
+        <v>11.9</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -52626,13 +52974,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -52640,10 +52988,10 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>6.4</v>
+        <v>15</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.2</v>
+        <v>10.2</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -52655,13 +53003,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -52669,10 +53017,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>52.5</v>
+        <v>65.2</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>5.7</v>
+        <v>4.2</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -52684,24 +53032,24 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>12.6</v>
+        <v>12.3</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>35.9</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>7.7</v>
+        <v>1</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -52723,17 +53071,46 @@
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>12</v>
+        <v>7.9</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B83" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H83" s="10">
+        <f>SUM(C77:C83)</f>
         <v/>
       </c>
     </row>
@@ -52754,7 +53131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -58476,13 +58853,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>23.5</v>
+        <v>23.1</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>6.7</v>
+        <v>6.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -58490,10 +58867,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>26.1</v>
+        <v>17.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>8.9</v>
+        <v>9.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -58505,24 +58882,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>9.9</v>
+        <v>15.5</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.8</v>
+        <v>10.1</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -58534,21 +58911,21 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>22.9</v>
+        <v>23.1</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.7</v>
+        <v>4.1</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="G200" s="7" t="n">
         <v>12</v>
@@ -58563,13 +58940,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>22.9</v>
+        <v>22.7</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.7</v>
+        <v>4.1</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -58592,24 +58969,24 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>22.7</v>
+        <v>23.2</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>3.1</v>
+        <v>3.7</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -58621,13 +58998,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>23.1</v>
+        <v>23.2</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -58635,13 +59012,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -58662,7 +59068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64384,13 +64790,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17.7</v>
+        <v>18.5</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -64398,10 +64804,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>77.3</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>2.7</v>
+        <v>0.6</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -64413,10 +64819,10 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>16.9</v>
+        <v>17</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>10</v>
+        <v>6.4</v>
       </c>
       <c r="D199" s="4" t="n">
         <v>4.2</v>
@@ -64427,10 +64833,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>93.2</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -64445,10 +64851,10 @@
         <v>16.3</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>2.4</v>
+        <v>11.5</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -64456,10 +64862,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>51.4</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>5.8</v>
+        <v>2.7</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -64471,13 +64877,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>17.8</v>
+        <v>17.9</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -64485,10 +64891,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>97.5</v>
+        <v>87.5</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>0.3</v>
+        <v>1.5</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -64500,13 +64906,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>16.8</v>
+        <v>18.2</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>4.3</v>
+        <v>2.6</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -64514,10 +64920,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>89.2</v>
+        <v>94.5</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -64529,13 +64935,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>15.4</v>
+        <v>16</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>2.7</v>
+        <v>16.3</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -64543,13 +64949,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>98.59999999999999</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -64570,7 +65005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -70292,24 +70727,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>12.9</v>
+        <v>14.5</v>
       </c>
       <c r="C198" s="7" t="n">
-        <v>5.2</v>
+        <v>7</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>94.09999999999999</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -70321,13 +70756,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>14.8</v>
+        <v>13.1</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>2.7</v>
+        <v>10.4</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -70335,10 +70770,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>72.40000000000001</v>
+        <v>56.8</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>3.3</v>
+        <v>5.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -70350,24 +70785,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>10.9</v>
+        <v>11.5</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>68</v>
+        <v>57.1</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>3.8</v>
+        <v>5.1</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -70379,24 +70814,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>13.2</v>
+        <v>12.5</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>64.8</v>
+        <v>54.2</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>4.2</v>
+        <v>5.5</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -70408,13 +70843,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>14.9</v>
+        <v>14.6</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -70422,10 +70857,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>90.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>1.2</v>
+        <v>3.3</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -70440,10 +70875,10 @@
         <v>14.6</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -70451,13 +70886,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>85.40000000000001</v>
+        <v>97.8</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>1.8</v>
+        <v>0.3</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -70478,7 +70942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -76200,13 +76664,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>15.9</v>
+        <v>17.8</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -76214,10 +76678,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>4.6</v>
+        <v>1.5</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -76229,13 +76693,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -76243,10 +76707,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>4.9</v>
+        <v>0.9</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -76258,21 +76722,21 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>16.5</v>
+        <v>16.9</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="G200" s="7" t="n">
         <v>12</v>
@@ -76287,7 +76751,7 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
@@ -76297,7 +76761,7 @@
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
@@ -76316,13 +76780,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>16.2</v>
+        <v>15.9</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -76330,10 +76794,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>13.3</v>
+        <v>40.2</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>10.4</v>
+        <v>7.2</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -76345,13 +76809,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>16.5</v>
+        <v>16.1</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -76359,13 +76823,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>18.8</v>
+        <v>49.2</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>9.699999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -76386,7 +76879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82108,24 +82601,24 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>17</v>
+        <v>19.2</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>2.5</v>
+        <v>0.7</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -82151,10 +82644,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -82166,13 +82659,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>17.2</v>
+        <v>18</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -82195,13 +82688,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -82224,13 +82717,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>16.5</v>
+        <v>16.7</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -82238,10 +82731,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>3.7</v>
+        <v>37.7</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>11.6</v>
+        <v>7.5</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -82253,7 +82746,7 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
@@ -82267,13 +82760,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>7.8</v>
+        <v>51.8</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>11.1</v>
+        <v>5.8</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -82294,7 +82816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -88016,13 +88538,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>12.7</v>
+        <v>14.9</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -88030,10 +88552,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>6.5</v>
+        <v>0.4</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -88051,7 +88573,7 @@
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -88059,10 +88581,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>16.1</v>
+        <v>15.2</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.1</v>
+        <v>10.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -88074,13 +88596,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>12.9</v>
+        <v>13.1</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -88088,10 +88610,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -88103,13 +88625,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -88117,10 +88639,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -88138,7 +88660,7 @@
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>3.1</v>
+        <v>2.5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -88146,10 +88668,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>21.1</v>
+        <v>55.6</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>9.5</v>
+        <v>5.3</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -88161,13 +88683,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>13.4</v>
+        <v>13.2</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -88175,13 +88697,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>5.1</v>
+        <v>50.8</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>11.4</v>
+        <v>5.9</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>
@@ -88202,7 +88753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H203"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -93924,13 +94475,13 @@
         <v>46292</v>
       </c>
       <c r="B198" s="7" t="n">
-        <v>16.7</v>
+        <v>17.6</v>
       </c>
       <c r="C198" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E198" s="7" t="inlineStr">
         <is>
@@ -93938,10 +94489,10 @@
         </is>
       </c>
       <c r="F198" s="7" t="n">
-        <v>1.3</v>
+        <v>5.2</v>
       </c>
       <c r="G198" s="7" t="n">
-        <v>11.8</v>
+        <v>11.4</v>
       </c>
       <c r="H198" s="12">
         <f>SUM(C192:C198)</f>
@@ -93953,24 +94504,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>16.9</v>
+        <v>16.4</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>20.5</v>
+        <v>17.8</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -93982,13 +94533,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>14.8</v>
+        <v>16.1</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -93996,10 +94547,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>46.5</v>
+        <v>67.2</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>6.4</v>
+        <v>3.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -94011,13 +94562,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -94025,10 +94576,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>51.6</v>
+        <v>84</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>5.8</v>
+        <v>1.9</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -94040,24 +94591,24 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>14.1</v>
+        <v>14.6</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="D202" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>90.40000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>1.2</v>
+        <v>0.2</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -94069,10 +94620,10 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>13.5</v>
+        <v>14.2</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="D203" s="4" t="n">
         <v>0.7</v>
@@ -94083,13 +94634,42 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="11" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B204" s="7" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C204" s="7" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H204" s="12">
+        <f>SUM(C198:C204)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
WeatherHistory update – 2026-09-28 12:20 UTC
</commit_message>
<xml_diff>
--- a/WeatherHistory.xlsx
+++ b/WeatherHistory.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6264,24 +6264,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.2</v>
+        <v>20.7</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>5.1</v>
+        <v>3.2</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>12.2</v>
+        <v>40.4</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>10.5</v>
+        <v>7.2</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -6293,24 +6293,24 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>3.1</v>
+        <v>6.3</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>17.5</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>10.9</v>
+        <v>9.9</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -6322,13 +6322,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>19.5</v>
+        <v>18.9</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>5.3</v>
+        <v>16.3</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>6.3</v>
+        <v>8.4</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -6336,10 +6336,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>38.3</v>
+        <v>49.9</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>7.4</v>
+        <v>6</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -6351,13 +6351,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -6365,10 +6365,10 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>76.2</v>
+        <v>51</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>2.9</v>
+        <v>5.9</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -6383,10 +6383,10 @@
         <v>18.4</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>5.8</v>
+        <v>3.9</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -6394,10 +6394,10 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>63.6</v>
+        <v>53.1</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>4.4</v>
+        <v>5.6</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
@@ -6409,27 +6409,56 @@
         <v>46298</v>
       </c>
       <c r="B204" s="7" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="C204" s="7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D204" s="7" t="n">
         <v>6</v>
       </c>
       <c r="E204" s="7" t="inlineStr">
         <is>
-          <t>JV</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="F204" s="7" t="n">
-        <v>46.5</v>
+        <v>36.5</v>
       </c>
       <c r="G204" s="7" t="n">
-        <v>6.4</v>
+        <v>7.6</v>
       </c>
       <c r="H204" s="12">
         <f>SUM(C198:C204)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="9" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B205" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="C205" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D205" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E205" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F205" s="4" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H205" s="10">
+        <f>SUM(C199:C205)</f>
         <v/>
       </c>
     </row>
@@ -6450,7 +6479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12201,24 +12230,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>19.1</v>
+        <v>20.3</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>30.2</v>
+        <v>15</v>
       </c>
       <c r="D199" s="4" t="n">
         <v>3.6</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>95</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -12230,13 +12259,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>16.3</v>
+        <v>17.7</v>
       </c>
       <c r="C200" s="7" t="n">
-        <v>22.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -12244,10 +12273,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>98.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>0.1</v>
+        <v>2.6</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -12259,24 +12288,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>18.4</v>
+        <v>19.7</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>1.7</v>
+        <v>3.6</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>98.5</v>
+        <v>75.7</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>0.2</v>
+        <v>2.9</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -12288,24 +12317,24 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>18.4</v>
+        <v>19.2</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>4.6</v>
+        <v>5.7</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>83.8</v>
+        <v>72.7</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>1.9</v>
+        <v>3.3</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -12317,13 +12346,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>16.5</v>
+        <v>15.9</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -12331,10 +12360,10 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>97.8</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
@@ -12346,27 +12375,56 @@
         <v>46298</v>
       </c>
       <c r="B204" s="7" t="n">
-        <v>16.6</v>
+        <v>17</v>
       </c>
       <c r="C204" s="7" t="n">
-        <v>14.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="D204" s="7" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="E204" s="7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F204" s="7" t="n">
-        <v>83.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G204" s="7" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="H204" s="12">
         <f>SUM(C198:C204)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="9" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B205" s="4" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="C205" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D205" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E205" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F205" s="4" t="n">
+        <v>87.7</v>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H205" s="10">
+        <f>SUM(C199:C205)</f>
         <v/>
       </c>
     </row>
@@ -12387,7 +12445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18138,13 +18196,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>20.3</v>
+        <v>20.7</v>
       </c>
       <c r="C199" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>10.8</v>
+        <v>11.6</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -18152,10 +18210,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>6.8</v>
+        <v>0.1</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -18167,13 +18225,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -18181,7 +18239,7 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G200" s="7" t="n">
         <v>12</v>
@@ -18202,7 +18260,7 @@
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -18210,10 +18268,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -18225,24 +18283,24 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>20.6</v>
+        <v>20.4</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>28.9</v>
+        <v>48.1</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>8.5</v>
+        <v>6.2</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -18254,24 +18312,24 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>3.6</v>
+        <v>4.3</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>49.4</v>
+        <v>59.8</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>6.1</v>
+        <v>4.8</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
@@ -18283,13 +18341,13 @@
         <v>46298</v>
       </c>
       <c r="B204" s="7" t="n">
-        <v>20.8</v>
+        <v>21.2</v>
       </c>
       <c r="C204" s="7" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D204" s="7" t="n">
-        <v>2.8</v>
+        <v>5.8</v>
       </c>
       <c r="E204" s="7" t="inlineStr">
         <is>
@@ -18297,13 +18355,42 @@
         </is>
       </c>
       <c r="F204" s="7" t="n">
-        <v>46.9</v>
+        <v>18.2</v>
       </c>
       <c r="G204" s="7" t="n">
-        <v>6.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H204" s="12">
         <f>SUM(C198:C204)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="9" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B205" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C205" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D205" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="E205" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F205" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H205" s="10">
+        <f>SUM(C199:C205)</f>
         <v/>
       </c>
     </row>
@@ -18324,7 +18411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24075,13 +24162,13 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
@@ -24089,10 +24176,10 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>2.1</v>
+        <v>12.9</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>11.7</v>
+        <v>10.5</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -24104,13 +24191,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -24118,10 +24205,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>33.5</v>
+        <v>69.8</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>8</v>
+        <v>3.6</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -24133,24 +24220,24 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>22.5</v>
+        <v>22.4</v>
       </c>
       <c r="C201" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>2.5</v>
+        <v>4.2</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>61.9</v>
+        <v>56.4</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>4.6</v>
+        <v>5.2</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -24162,24 +24249,24 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="C202" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>54.9</v>
+        <v>67.2</v>
       </c>
       <c r="G202" s="7" t="n">
-        <v>5.4</v>
+        <v>3.9</v>
       </c>
       <c r="H202" s="12">
         <f>SUM(C196:C202)</f>
@@ -24191,13 +24278,13 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>23</v>
+        <v>22.5</v>
       </c>
       <c r="C203" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
@@ -24205,10 +24292,10 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>90.2</v>
+        <v>81.8</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
@@ -24220,13 +24307,13 @@
         <v>46298</v>
       </c>
       <c r="B204" s="7" t="n">
-        <v>22.6</v>
+        <v>22.2</v>
       </c>
       <c r="C204" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D204" s="7" t="n">
-        <v>2.9</v>
+        <v>2.3</v>
       </c>
       <c r="E204" s="7" t="inlineStr">
         <is>
@@ -24234,13 +24321,42 @@
         </is>
       </c>
       <c r="F204" s="7" t="n">
-        <v>47.6</v>
+        <v>46.1</v>
       </c>
       <c r="G204" s="7" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="H204" s="12">
         <f>SUM(C198:C204)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="9" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B205" s="4" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C205" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D205" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" s="4" t="inlineStr">
+        <is>
+          <t>JV</t>
+        </is>
+      </c>
+      <c r="F205" s="4" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H205" s="10">
+        <f>SUM(C199:C205)</f>
         <v/>
       </c>
     </row>
@@ -24261,7 +24377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30012,24 +30128,24 @@
         <v>46293</v>
       </c>
       <c r="B199" s="4" t="n">
-        <v>11.4</v>
+        <v>13.2</v>
       </c>
       <c r="C199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D199" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>71</v>
+        <v>97.2</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>3.5</v>
+        <v>0.3</v>
       </c>
       <c r="H199" s="10">
         <f>SUM(C193:C199)</f>
@@ -30041,13 +30157,13 @@
         <v>46294</v>
       </c>
       <c r="B200" s="7" t="n">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="C200" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
@@ -30055,10 +30171,10 @@
         </is>
       </c>
       <c r="F200" s="7" t="n">
-        <v>72.59999999999999</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G200" s="7" t="n">
-        <v>3.3</v>
+        <v>1.2</v>
       </c>
       <c r="H200" s="12">
         <f>SUM(C194:C200)</f>
@@ -30070,13 +30186,13 @@
         <v>46295</v>
       </c>
       <c r="B201" s="4" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="C201" s="4" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>1.6</v>
+        <v>3.1</v>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
@@ -30084,10 +30200,10 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>67.8</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="G201" s="4" t="n">
-        <v>3.9</v>
+        <v>0.6</v>
       </c>
       <c r="H201" s="10">
         <f>SUM(C195:C201)</f>
@@ -30099,13 +30215,13 @@
         <v>46296</v>
       </c>
       <c r="B202" s="7" t="n">
-        <v>10.4</v>
+        <v>9.5</v>
       </c>
       <c r="C202" s="7" t="n">
-        <v>3.8</v>
+        <v>7.7</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
@@ -30113,7 +30229,7 @@
         </is>
       </c>
       <c r="F202" s="7" t="n">
-        <v>98.40000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="G202" s="7" t="n">
         <v>0.2</v>
@@ -30128,24 +30244,24 @@
         <v>46297</v>
       </c>
       <c r="B203" s="4" t="n">
-        <v>10.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>99.2</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G203" s="4" t="n">
-        <v>0.1</v>
+        <v>2.4</v>
       </c>
       <c r="H203" s="10">
         <f>SUM(C197:C203)</f>
@@ -30157,27 +30273,56 @@
         <v>46298</v>
       </c>
       <c r="B204" s="7" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="C204" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D204" s="7" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E204" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F204" s="7" t="n">
-        <v>80.5</v>
+        <v>45.7</v>
       </c>
       <c r="G204" s="7" t="n">
-        <v>2.3</v>
+        <v>6.5</v>
       </c>
       <c r="H204" s="12">
         <f>SUM(C198:C204)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="9" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B205" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C205" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D205" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E205" s="4" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="F205" s="4" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H205" s="10">
+        <f>SUM(C199:C205)</f>
         <v/>
       </c>
     </row>
@@ -30198,7 +30343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32440,17 +32585,17 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.2</v>
+        <v>13.6</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
@@ -32469,24 +32614,24 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>12.9</v>
+        <v>12.6</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="H79" s="10">
         <f>SUM(C73:C79)</f>
@@ -32498,24 +32643,24 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>13</v>
+        <v>12.7</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>4.9</v>
+        <v>0.5</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>11.4</v>
+        <v>11.9</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -32527,13 +32672,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>12.4</v>
+        <v>12.2</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -32541,10 +32686,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>96.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>0.4</v>
+        <v>3</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -32556,7 +32701,7 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>12.3</v>
+        <v>12.8</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
@@ -32570,10 +32715,10 @@
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
@@ -32591,7 +32736,7 @@
         <v>0</v>
       </c>
       <c r="D83" s="4" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
@@ -32599,13 +32744,42 @@
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>28.1</v>
+        <v>0</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>8.6</v>
+        <v>12</v>
       </c>
       <c r="H83" s="10">
         <f>SUM(C77:C83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B84" s="7" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="G84" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H84" s="12">
+        <f>SUM(C78:C84)</f>
         <v/>
       </c>
     </row>
@@ -32626,7 +32800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34868,7 +35042,7 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12</v>
+        <v>13.7</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
@@ -34882,10 +35056,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -34897,13 +35071,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -34911,7 +35085,7 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G79" s="4" t="n">
         <v>12</v>
@@ -34926,13 +35100,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>10.8</v>
+        <v>11.8</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -34940,10 +35114,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>14.4</v>
+        <v>0.2</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>10.3</v>
+        <v>12</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -34955,13 +35129,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -34969,10 +35143,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>2.8</v>
+        <v>4.8</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -34984,13 +35158,13 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
@@ -34998,10 +35172,10 @@
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>12</v>
+        <v>10.1</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
@@ -35013,27 +35187,56 @@
         <v>46298</v>
       </c>
       <c r="B83" s="4" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="C83" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D83" s="4" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JZ</t>
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>12</v>
+        <v>11.4</v>
       </c>
       <c r="H83" s="10">
         <f>SUM(C77:C83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B84" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C84" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="G84" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" s="12">
+        <f>SUM(C78:C84)</f>
         <v/>
       </c>
     </row>
@@ -35054,7 +35257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37296,13 +37499,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.9</v>
+        <v>14.2</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -37310,10 +37513,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>2.8</v>
+        <v>7.3</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.7</v>
+        <v>11.1</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -37325,13 +37528,13 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>12.9</v>
+        <v>12.6</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
@@ -37354,13 +37557,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.1</v>
+        <v>12.8</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -37368,10 +37571,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>31.4</v>
+        <v>0</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>8.199999999999999</v>
+        <v>12</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -37389,7 +37592,7 @@
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -37397,10 +37600,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>90</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>1.2</v>
+        <v>4</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -37418,18 +37621,18 @@
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>0</v>
+        <v>20.9</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>12</v>
+        <v>9.5</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
@@ -37441,17 +37644,17 @@
         <v>46298</v>
       </c>
       <c r="B83" s="4" t="n">
-        <v>14.2</v>
+        <v>14</v>
       </c>
       <c r="C83" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D83" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F83" s="4" t="n">
@@ -37462,6 +37665,35 @@
       </c>
       <c r="H83" s="10">
         <f>SUM(C77:C83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B84" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="C84" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="G84" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H84" s="12">
+        <f>SUM(C78:C84)</f>
         <v/>
       </c>
     </row>
@@ -37482,7 +37714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39724,7 +39956,7 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>12.6</v>
+        <v>13.5</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
@@ -39734,11 +39966,11 @@
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>12</v>
@@ -39753,7 +39985,7 @@
         <v>46294</v>
       </c>
       <c r="B79" s="4" t="n">
-        <v>12.6</v>
+        <v>12.4</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>0</v>
@@ -39763,11 +39995,11 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G79" s="4" t="n">
         <v>12</v>
@@ -39782,13 +40014,13 @@
         <v>46295</v>
       </c>
       <c r="B80" s="7" t="n">
-        <v>12.4</v>
+        <v>12.6</v>
       </c>
       <c r="C80" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -39796,10 +40028,10 @@
         </is>
       </c>
       <c r="F80" s="7" t="n">
-        <v>13.3</v>
+        <v>1.2</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>10.4</v>
+        <v>11.9</v>
       </c>
       <c r="H80" s="12">
         <f>SUM(C74:C80)</f>
@@ -39811,13 +40043,13 @@
         <v>46296</v>
       </c>
       <c r="B81" s="4" t="n">
-        <v>13</v>
+        <v>12.8</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
@@ -39825,10 +40057,10 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>91.59999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="H81" s="10">
         <f>SUM(C75:C81)</f>
@@ -39840,13 +40072,13 @@
         <v>46297</v>
       </c>
       <c r="B82" s="7" t="n">
-        <v>13</v>
+        <v>13.1</v>
       </c>
       <c r="C82" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
@@ -39854,10 +40086,10 @@
         </is>
       </c>
       <c r="F82" s="7" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="H82" s="12">
         <f>SUM(C76:C82)</f>
@@ -39869,27 +40101,56 @@
         <v>46298</v>
       </c>
       <c r="B83" s="4" t="n">
-        <v>13.6</v>
+        <v>13</v>
       </c>
       <c r="C83" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D83" s="4" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>JV</t>
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>20.9</v>
+        <v>0</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="H83" s="10">
         <f>SUM(C77:C83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B84" s="7" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="C84" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="G84" s="7" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H84" s="12">
+        <f>SUM(C78:C84)</f>
         <v/>
       </c>
     </row>
@@ -39910,7 +40171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42152,13 +42413,13 @@
         <v>46293</v>
       </c>
       <c r="B78" s="7" t="n">
-        <v>13.1</v>
+        <v>14</v>
       </c>
       <c r="C78" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
@@ -42166,10 +42427,10 @@
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>7.5</v>
+        <v>10.8</v>
       </c>
       <c r="G78" s="7" t="n">
-        <v>11.1</v>
+        <v>10.7</v>
       </c>
       <c r="H78" s="12">
         <f>SUM(C72:C78)</f>
@@ -42181,13 +42442,13 @@
         <v>46